<commit_message>
feat(product): add START HERE guide tab, interactive tab showcase, and high-intent results callout
</commit_message>
<xml_diff>
--- a/public/downloads/NetWorth_FIRE_Master_Vault_2026.xlsx
+++ b/public/downloads/NetWorth_FIRE_Master_Vault_2026.xlsx
@@ -4,20 +4,135 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="⚡ 2-Min Quick Check-In" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="📊 Executive Dashboard" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="💸 Smart Budget (50-30-20)" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="🎯 Sinking Funds Shield" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="🔥 FIRE Freedom Engine" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="💳 Debt Avalanche &amp; Snowball" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="🏛️ Fed Benchmarks (SCF)" state="visible" r:id="rId10"/>
+    <sheet sheetId="1" name="🟢 START HERE (60-Sec Guide)" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="⚡ 2-Min Quick Check-In" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="📊 Executive Dashboard" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="💸 Smart Budget (50-30-20)" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="🎯 Sinking Funds Shield" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="🔥 FIRE Freedom Engine" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="💳 Debt Avalanche &amp; Snowball" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="🏛️ Fed Benchmarks (SCF)" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="188">
+  <si>
+    <t>👋 WELCOME TO YOUR PRIVATE WEALTH &amp; BUDGET OPERATING SYSTEM</t>
+  </si>
+  <si>
+    <t>Designed for normal humans, not CPAs. Zero homework, zero broken formulas, 100% private &amp; offline.</t>
+  </si>
+  <si>
+    <t>🚀 THE 3-STEP MONTHLY ROUTINE (TAKES 2 MINUTES ON THE 1ST OF EACH MONTH)</t>
+  </si>
+  <si>
+    <t>Step 1: Open Tab 2</t>
+  </si>
+  <si>
+    <t>Click '⚡ 2-Min Quick Check-In'</t>
+  </si>
+  <si>
+    <t>On the 1st of every month, open the second tab.</t>
+  </si>
+  <si>
+    <t>Step 2: Enter 4 Numbers</t>
+  </si>
+  <si>
+    <t>Fill the Green Cells Only</t>
+  </si>
+  <si>
+    <t>Type your: (1) Cash, (2) Invested Portfolio, (3) Property Value, (4) Total Debts.</t>
+  </si>
+  <si>
+    <t>Step 3: You Are Done!</t>
+  </si>
+  <si>
+    <t>Relax &amp; Enjoy Your Life</t>
+  </si>
+  <si>
+    <t>All formulas, Fed Reserve Percentile rankings, FIRE retirement dates, and Safe-to-Spend buffers calculate automatically!</t>
+  </si>
+  <si>
+    <t>🎨 VISUAL COLOR CODES (HOW TO NEVER BREAK A FORMULA)</t>
+  </si>
+  <si>
+    <t>🟩 GREEN CELLS</t>
+  </si>
+  <si>
+    <t>Your Input Area</t>
+  </si>
+  <si>
+    <t>Safe to edit and type your monthly numbers here.</t>
+  </si>
+  <si>
+    <t>⬛ DARK / SLATE CELLS</t>
+  </si>
+  <si>
+    <t>Automated Math Engine</t>
+  </si>
+  <si>
+    <t>Formulas do all the work here. Never edit or delete these.</t>
+  </si>
+  <si>
+    <t>🟨 GOLD / AMBER CELLS</t>
+  </si>
+  <si>
+    <t>Key Benchmarks &amp; Goals</t>
+  </si>
+  <si>
+    <t>Shows your Federal Reserve percentile, Coast FIRE, and Safe-to-Spend limit.</t>
+  </si>
+  <si>
+    <t>📖 WHAT EACH TAB DOES (CHOOSE YOUR PURPOSE)</t>
+  </si>
+  <si>
+    <t>⚡ 2-Min Quick Check-In</t>
+  </si>
+  <si>
+    <t>For 90% of months: Type 4 numbers once a month in 90 seconds. Zero homework.</t>
+  </si>
+  <si>
+    <t>📊 Executive Dashboard</t>
+  </si>
+  <si>
+    <t>Bloomberg-style visual terminal showing Net Worth, Fed rank, and quarterly progress.</t>
+  </si>
+  <si>
+    <t>💸 Smart Budget (50/30/20)</t>
+  </si>
+  <si>
+    <t>Answers: 'How much can I spend today guilt-free?' (Needs 50%, Wants 30%, Wealth 20%).</t>
+  </si>
+  <si>
+    <t>🎯 Sinking Funds Shield</t>
+  </si>
+  <si>
+    <t>Prevents budget shock from car repairs, holiday travel, and annual insurance renewals.</t>
+  </si>
+  <si>
+    <t>🔥 FIRE Freedom Engine</t>
+  </si>
+  <si>
+    <t>Trinity 4% rule calculator showing your Coast FIRE milestone and exact retirement date.</t>
+  </si>
+  <si>
+    <t>💳 Debt Accelerator</t>
+  </si>
+  <si>
+    <t>Side-by-side Avalanche (interest saver) vs Snowball (momentum builder) payoff rank.</t>
+  </si>
+  <si>
+    <t>🏛️ Fed Benchmarks (SCF)</t>
+  </si>
+  <si>
+    <t>Official US Federal Reserve Survey of Consumer Finances raw microdata tables.</t>
+  </si>
+  <si>
+    <t>💡 Using Google Sheets? Just drag and drop this file into Google Drive and click "Open with Google Sheets". It converts in 2 seconds with 100% of formulas intact.</t>
+  </si>
   <si>
     <t>⚡ 2-MINUTE MONTHLY QUICK CHECK-IN (NO HOMEWORK, NO OVERWHELM)</t>
   </si>
@@ -480,13 +595,49 @@
     <numFmt numFmtId="167" formatCode="$#,##0/day"/>
     <numFmt numFmtId="168" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="29" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
       <scheme val="minor"/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="13"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FFCBD5E1"/>
+      <sz val="9.5"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF065F46"/>
+    </font>
+    <font>
+      <b/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <sz val="9"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF065F46"/>
+      <sz val="9"/>
     </font>
     <font>
       <b/>
@@ -520,12 +671,6 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="13"/>
-      <name val="Arial"/>
     </font>
     <font>
       <i/>
@@ -588,14 +733,6 @@
       <sz val="15"/>
     </font>
     <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b/>
-    </font>
-    <font>
       <i/>
       <color rgb="FF64748B"/>
       <sz val="9"/>
@@ -607,7 +744,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -616,7 +753,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF065F46"/>
+        <fgColor rgb="FF0F172A"/>
       </patternFill>
     </fill>
     <fill>
@@ -626,7 +763,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0F172A"/>
+        <fgColor rgb="FF065F46"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCFCE7"/>
       </patternFill>
     </fill>
     <fill>
@@ -677,7 +819,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -685,85 +827,96 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="14" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="17" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="167" fontId="19" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="18" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="26" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="14" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="14" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="21" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="21" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="14" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="14" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1103,6 +1256,210 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B2:D24"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="4" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="32" customWidth="1"/>
+    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="5" max="5" width="4" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="32" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B6" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B8" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B10" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+    </row>
+    <row r="11" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B11" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B12" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B13" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B15" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B16" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="10"/>
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B17" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D17" s="10"/>
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B18" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="10"/>
+    </row>
+    <row r="19" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B19" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D19" s="10"/>
+    </row>
+    <row r="20" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B20" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D20" s="10"/>
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B21" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D21" s="10"/>
+    </row>
+    <row r="22" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B22" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D22" s="10"/>
+    </row>
+    <row r="24" ht="26" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B24" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="B24:D24"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:I18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -1118,390 +1475,390 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B3" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+    </row>
+    <row r="5" ht="24" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B5" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G5" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="H5" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="I5" s="14" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B6" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" s="17">
+        <v>25000</v>
+      </c>
+      <c r="D6" s="17">
+        <v>185000</v>
+      </c>
+      <c r="E6" s="17">
+        <v>350000</v>
+      </c>
+      <c r="F6" s="17">
+        <v>245000</v>
+      </c>
+      <c r="G6" s="18">
+        <f>=(C6+D6+E6)-F6</f>
+      </c>
+      <c r="H6" s="19">
         <v>0</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-    </row>
-    <row r="3" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-    </row>
-    <row r="5" ht="24" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B5" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B6" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="6">
-        <v>25000</v>
-      </c>
-      <c r="D6" s="6">
-        <v>185000</v>
-      </c>
-      <c r="E6" s="6">
+      <c r="I6" s="20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B7" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="22">
+        <v>26200</v>
+      </c>
+      <c r="D7" s="22">
+        <v>189500</v>
+      </c>
+      <c r="E7" s="22">
         <v>350000</v>
       </c>
-      <c r="F6" s="6">
-        <v>245000</v>
-      </c>
-      <c r="G6" s="7">
-        <f>=(C6+D6+E6)-F6</f>
-      </c>
-      <c r="H6" s="8">
-        <v>0</v>
-      </c>
-      <c r="I6" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="11">
-        <v>26200</v>
-      </c>
-      <c r="D7" s="11">
-        <v>189500</v>
-      </c>
-      <c r="E7" s="11">
+      <c r="F7" s="22">
+        <v>243800</v>
+      </c>
+      <c r="G7" s="18">
+        <f>=(C7+D7+E7)-F7</f>
+      </c>
+      <c r="H7" s="23">
+        <f>=G7-G6</f>
+      </c>
+      <c r="I7" s="24">
+        <f>=(G7-G6)/G6</f>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B8" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="17">
+        <v>25800</v>
+      </c>
+      <c r="D8" s="17">
+        <v>194200</v>
+      </c>
+      <c r="E8" s="17">
         <v>350000</v>
       </c>
-      <c r="F7" s="11">
-        <v>243800</v>
-      </c>
-      <c r="G7" s="7">
-        <f>=(C7+D7+E7)-F7</f>
-      </c>
-      <c r="H7" s="12">
-        <f>=G7-G6</f>
-      </c>
-      <c r="I7" s="13">
-        <f>=(G7-G6)/G6</f>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B8" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="6">
-        <v>25800</v>
-      </c>
-      <c r="D8" s="6">
-        <v>194200</v>
-      </c>
-      <c r="E8" s="6">
+      <c r="F8" s="17">
+        <v>242600</v>
+      </c>
+      <c r="G8" s="18">
+        <f>=(C8+D8+E8)-F8</f>
+      </c>
+      <c r="H8" s="19">
+        <f>=G8-G7</f>
+      </c>
+      <c r="I8" s="20">
+        <f>=(G8-G7)/G7</f>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B9" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="22">
+        <v>27100</v>
+      </c>
+      <c r="D9" s="22">
+        <v>191000</v>
+      </c>
+      <c r="E9" s="22">
         <v>350000</v>
       </c>
-      <c r="F8" s="6">
-        <v>242600</v>
-      </c>
-      <c r="G8" s="7">
-        <f>=(C8+D8+E8)-F8</f>
-      </c>
-      <c r="H8" s="8">
-        <f>=G8-G7</f>
-      </c>
-      <c r="I8" s="9">
-        <f>=(G8-G7)/G7</f>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B9" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="11">
-        <v>27100</v>
-      </c>
-      <c r="D9" s="11">
-        <v>191000</v>
-      </c>
-      <c r="E9" s="11">
-        <v>350000</v>
-      </c>
-      <c r="F9" s="11">
+      <c r="F9" s="22">
         <v>241400</v>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="18">
         <f>=(C9+D9+E9)-F9</f>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="23">
         <f>=G9-G8</f>
       </c>
-      <c r="I9" s="13">
+      <c r="I9" s="24">
         <f>=(G9-G8)/G8</f>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B10" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="6">
+      <c r="B10" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" s="17">
         <v>26900</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="17">
         <v>198500</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="17">
         <v>352000</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="17">
         <v>240100</v>
       </c>
-      <c r="G10" s="7">
+      <c r="G10" s="18">
         <f>=(C10+D10+E10)-F10</f>
       </c>
-      <c r="H10" s="8">
+      <c r="H10" s="19">
         <f>=G10-G9</f>
       </c>
-      <c r="I10" s="9">
+      <c r="I10" s="20">
         <f>=(G10-G9)/G9</f>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B11" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" s="11">
+      <c r="B11" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="22">
         <v>28400</v>
       </c>
-      <c r="D11" s="11">
+      <c r="D11" s="22">
         <v>204000</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="22">
         <v>352000</v>
       </c>
-      <c r="F11" s="11">
+      <c r="F11" s="22">
         <v>238800</v>
       </c>
-      <c r="G11" s="7">
+      <c r="G11" s="18">
         <f>=(C11+D11+E11)-F11</f>
       </c>
-      <c r="H11" s="12">
+      <c r="H11" s="23">
         <f>=G11-G10</f>
       </c>
-      <c r="I11" s="13">
+      <c r="I11" s="24">
         <f>=(G11-G10)/G10</f>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B12" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="6">
+      <c r="B12" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" s="17">
         <v>29000</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="17">
         <v>209500</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="17">
         <v>352000</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="17">
         <v>237500</v>
       </c>
-      <c r="G12" s="7">
+      <c r="G12" s="18">
         <f>=(C12+D12+E12)-F12</f>
       </c>
-      <c r="H12" s="8">
+      <c r="H12" s="19">
         <f>=G12-G11</f>
       </c>
-      <c r="I12" s="9">
+      <c r="I12" s="20">
         <f>=(G12-G11)/G11</f>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B13" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="11">
+      <c r="B13" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13" s="22">
         <v>28500</v>
       </c>
-      <c r="D13" s="11">
+      <c r="D13" s="22">
         <v>215000</v>
       </c>
-      <c r="E13" s="11">
+      <c r="E13" s="22">
         <v>355000</v>
       </c>
-      <c r="F13" s="11">
+      <c r="F13" s="22">
         <v>236100</v>
       </c>
-      <c r="G13" s="7">
+      <c r="G13" s="18">
         <f>=(C13+D13+E13)-F13</f>
       </c>
-      <c r="H13" s="12">
+      <c r="H13" s="23">
         <f>=G13-G12</f>
       </c>
-      <c r="I13" s="13">
+      <c r="I13" s="24">
         <f>=(G13-G12)/G12</f>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B14" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" s="6">
+      <c r="B14" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" s="17">
         <v>30200</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="17">
         <v>221000</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="17">
         <v>355000</v>
       </c>
-      <c r="F14" s="6">
+      <c r="F14" s="17">
         <v>234700</v>
       </c>
-      <c r="G14" s="7">
+      <c r="G14" s="18">
         <f>=(C14+D14+E14)-F14</f>
       </c>
-      <c r="H14" s="8">
+      <c r="H14" s="19">
         <f>=G14-G13</f>
       </c>
-      <c r="I14" s="9">
+      <c r="I14" s="20">
         <f>=(G14-G13)/G13</f>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B15" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="11">
+      <c r="B15" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" s="22">
         <v>31000</v>
       </c>
-      <c r="D15" s="11">
+      <c r="D15" s="22">
         <v>228000</v>
       </c>
-      <c r="E15" s="11">
+      <c r="E15" s="22">
         <v>355000</v>
       </c>
-      <c r="F15" s="11">
+      <c r="F15" s="22">
         <v>233200</v>
       </c>
-      <c r="G15" s="7">
+      <c r="G15" s="18">
         <f>=(C15+D15+E15)-F15</f>
       </c>
-      <c r="H15" s="12">
+      <c r="H15" s="23">
         <f>=G15-G14</f>
       </c>
-      <c r="I15" s="13">
+      <c r="I15" s="24">
         <f>=(G15-G14)/G14</f>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B16" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C16" s="6">
+      <c r="B16" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16" s="17">
         <v>31500</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="17">
         <v>234500</v>
       </c>
-      <c r="E16" s="6">
+      <c r="E16" s="17">
         <v>358000</v>
       </c>
-      <c r="F16" s="6">
+      <c r="F16" s="17">
         <v>231700</v>
       </c>
-      <c r="G16" s="7">
+      <c r="G16" s="18">
         <f>=(C16+D16+E16)-F16</f>
       </c>
-      <c r="H16" s="8">
+      <c r="H16" s="19">
         <f>=G16-G15</f>
       </c>
-      <c r="I16" s="9">
+      <c r="I16" s="20">
         <f>=(G16-G15)/G15</f>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B17" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="C17" s="11">
+      <c r="B17" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="C17" s="22">
         <v>33000</v>
       </c>
-      <c r="D17" s="11">
+      <c r="D17" s="22">
         <v>242000</v>
       </c>
-      <c r="E17" s="11">
+      <c r="E17" s="22">
         <v>358000</v>
       </c>
-      <c r="F17" s="11">
+      <c r="F17" s="22">
         <v>230100</v>
       </c>
-      <c r="G17" s="7">
+      <c r="G17" s="18">
         <f>=(C17+D17+E17)-F17</f>
       </c>
-      <c r="H17" s="12">
+      <c r="H17" s="23">
         <f>=G17-G16</f>
       </c>
-      <c r="I17" s="13">
+      <c r="I17" s="24">
         <f>=(G17-G16)/G16</f>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B18" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="C18" s="15">
+      <c r="B18" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="C18" s="26">
         <f>=C17</f>
       </c>
-      <c r="D18" s="15">
+      <c r="D18" s="26">
         <f>=D17</f>
       </c>
-      <c r="E18" s="15">
+      <c r="E18" s="26">
         <f>=E17</f>
       </c>
-      <c r="F18" s="15">
+      <c r="F18" s="26">
         <f>=F17</f>
       </c>
-      <c r="G18" s="15">
+      <c r="G18" s="26">
         <f>=G17</f>
       </c>
-      <c r="H18" s="15">
+      <c r="H18" s="26">
         <f>=G17-G6</f>
       </c>
-      <c r="I18" s="16">
+      <c r="I18" s="27">
         <f>=(G17-G6)/G6</f>
       </c>
     </row>
@@ -1515,7 +1872,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:F20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1528,211 +1885,211 @@
   </cols>
   <sheetData>
     <row r="2" ht="30" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
+      <c r="B2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="B3" s="28" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
     </row>
     <row r="5" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19" t="s">
-        <v>27</v>
+      <c r="B5" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="20">
+      <c r="B6" s="30">
         <f>='⚡ 2-Min Quick Check-In'!G18</f>
       </c>
-      <c r="C6" s="20"/>
-      <c r="D6" s="21">
+      <c r="C6" s="30"/>
+      <c r="D6" s="31">
         <f>='⚡ 2-Min Quick Check-In'!C18+'⚡ 2-Min Quick Check-In'!D18</f>
       </c>
-      <c r="E6" s="21"/>
-      <c r="F6" s="22" t="s">
-        <v>28</v>
+      <c r="E6" s="31"/>
+      <c r="F6" s="32" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="23">
+      <c r="B7" s="33">
         <f>="▲ Annual Growth: " &amp; TEXT('⚡ 2-Min Quick Check-In'!I18, "+0.0%") &amp; " (+$" &amp; TEXT('⚡ 2-Min Quick Check-In'!H18, "#,##0") &amp; ")"</f>
       </c>
-      <c r="C7" s="23"/>
-      <c r="D7" s="24">
+      <c r="C7" s="33"/>
+      <c r="D7" s="34">
         <f>="Liquid Ratio: " &amp; TEXT(('⚡ 2-Min Quick Check-In'!C18+'⚡ 2-Min Quick Check-In'!D18)/('⚡ 2-Min Quick Check-In'!G18+'⚡ 2-Min Quick Check-In'!F18), "0.0%") &amp; " of total assets"</f>
       </c>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24" t="s">
-        <v>29</v>
+      <c r="E7" s="34"/>
+      <c r="F7" s="34" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="25" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
+      <c r="B9" s="35" t="s">
+        <v>68</v>
+      </c>
+      <c r="C9" s="35"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="35"/>
+      <c r="F9" s="35"/>
     </row>
     <row r="10" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B10" s="26" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" s="26" t="s">
-        <v>32</v>
-      </c>
-      <c r="D10" s="26" t="s">
-        <v>33</v>
-      </c>
-      <c r="E10" s="26" t="s">
-        <v>34</v>
-      </c>
-      <c r="F10" s="26" t="s">
-        <v>35</v>
+      <c r="B10" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="C10" s="36" t="s">
+        <v>70</v>
+      </c>
+      <c r="D10" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="E10" s="36" t="s">
+        <v>72</v>
+      </c>
+      <c r="F10" s="36" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B11" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="C11" s="6">
+      <c r="B11" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C11" s="17">
         <f>='⚡ 2-Min Quick Check-In'!G6</f>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="17">
         <f>='⚡ 2-Min Quick Check-In'!D6</f>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="17">
         <f>='⚡ 2-Min Quick Check-In'!F6</f>
       </c>
-      <c r="F11" s="27" t="s">
-        <v>37</v>
+      <c r="F11" s="6" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B12" s="28" t="s">
-        <v>38</v>
-      </c>
-      <c r="C12" s="11">
+      <c r="B12" s="37" t="s">
+        <v>76</v>
+      </c>
+      <c r="C12" s="22">
         <f>='⚡ 2-Min Quick Check-In'!G9</f>
       </c>
-      <c r="D12" s="11">
+      <c r="D12" s="22">
         <f>='⚡ 2-Min Quick Check-In'!D9</f>
       </c>
-      <c r="E12" s="11">
+      <c r="E12" s="22">
         <f>='⚡ 2-Min Quick Check-In'!F9</f>
       </c>
-      <c r="F12" s="28" t="s">
-        <v>39</v>
+      <c r="F12" s="37" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B13" s="27" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="6">
+      <c r="B13" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C13" s="17">
         <f>='⚡ 2-Min Quick Check-In'!G12</f>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="17">
         <f>='⚡ 2-Min Quick Check-In'!D12</f>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="17">
         <f>='⚡ 2-Min Quick Check-In'!F12</f>
       </c>
-      <c r="F13" s="27" t="s">
-        <v>41</v>
+      <c r="F13" s="6" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="28" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14" s="11">
+      <c r="B14" s="37" t="s">
+        <v>80</v>
+      </c>
+      <c r="C14" s="22">
         <f>='⚡ 2-Min Quick Check-In'!G15</f>
       </c>
-      <c r="D14" s="11">
+      <c r="D14" s="22">
         <f>='⚡ 2-Min Quick Check-In'!D15</f>
       </c>
-      <c r="E14" s="11">
+      <c r="E14" s="22">
         <f>='⚡ 2-Min Quick Check-In'!F15</f>
       </c>
-      <c r="F14" s="28" t="s">
-        <v>43</v>
+      <c r="F14" s="37" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B15" s="27" t="s">
-        <v>44</v>
-      </c>
-      <c r="C15" s="6">
+      <c r="B15" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C15" s="17">
         <f>='⚡ 2-Min Quick Check-In'!G17</f>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="17">
         <f>='⚡ 2-Min Quick Check-In'!D17</f>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="17">
         <f>='⚡ 2-Min Quick Check-In'!F17</f>
       </c>
-      <c r="F15" s="27" t="s">
-        <v>45</v>
+      <c r="F15" s="6" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B18" s="25" t="s">
-        <v>46</v>
-      </c>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
+      <c r="B18" s="35" t="s">
+        <v>84</v>
+      </c>
+      <c r="C18" s="35"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="35"/>
+      <c r="F18" s="35"/>
     </row>
     <row r="19" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B19" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="C19" s="29" t="s">
-        <v>48</v>
-      </c>
-      <c r="D19" s="29" t="s">
-        <v>49</v>
-      </c>
-      <c r="E19" s="29" t="s">
-        <v>50</v>
-      </c>
-      <c r="F19" s="29"/>
+      <c r="B19" s="38" t="s">
+        <v>85</v>
+      </c>
+      <c r="C19" s="38" t="s">
+        <v>86</v>
+      </c>
+      <c r="D19" s="38" t="s">
+        <v>87</v>
+      </c>
+      <c r="E19" s="38" t="s">
+        <v>88</v>
+      </c>
+      <c r="F19" s="38"/>
     </row>
     <row r="20" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B20" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="C20" s="30" t="s">
-        <v>52</v>
-      </c>
-      <c r="D20" s="30" t="s">
-        <v>53</v>
-      </c>
-      <c r="E20" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="F20" s="30"/>
+      <c r="B20" s="39" t="s">
+        <v>89</v>
+      </c>
+      <c r="C20" s="39" t="s">
+        <v>90</v>
+      </c>
+      <c r="D20" s="39" t="s">
+        <v>91</v>
+      </c>
+      <c r="E20" s="39" t="s">
+        <v>92</v>
+      </c>
+      <c r="F20" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -1754,7 +2111,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:F30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1768,401 +2125,401 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="31" t="s">
-        <v>55</v>
-      </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
+      <c r="B2" s="40" t="s">
+        <v>93</v>
+      </c>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="B3" s="28" t="s">
+        <v>94</v>
+      </c>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="F5" s="19"/>
+      <c r="B5" s="33" t="s">
+        <v>95</v>
+      </c>
+      <c r="C5" s="33"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="29" t="s">
+        <v>96</v>
+      </c>
+      <c r="F5" s="29"/>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="32">
+      <c r="B6" s="41">
         <f>=E24</f>
       </c>
-      <c r="C6" s="32"/>
-      <c r="D6" s="32"/>
-      <c r="E6" s="33">
+      <c r="C6" s="41"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="42">
         <f>=E24/30</f>
       </c>
-      <c r="F6" s="33"/>
+      <c r="F6" s="42"/>
     </row>
     <row r="8" ht="22" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="34" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" s="34" t="s">
-        <v>60</v>
-      </c>
-      <c r="D8" s="34" t="s">
-        <v>61</v>
-      </c>
-      <c r="E8" s="34" t="s">
-        <v>62</v>
-      </c>
-      <c r="F8" s="34" t="s">
-        <v>63</v>
+      <c r="B8" s="43" t="s">
+        <v>97</v>
+      </c>
+      <c r="C8" s="43" t="s">
+        <v>98</v>
+      </c>
+      <c r="D8" s="43" t="s">
+        <v>99</v>
+      </c>
+      <c r="E8" s="43" t="s">
+        <v>100</v>
+      </c>
+      <c r="F8" s="43" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="35" t="s">
-        <v>64</v>
-      </c>
-      <c r="C9" s="35"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="35"/>
+      <c r="B9" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
     </row>
     <row r="10" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B10" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="C10" s="6">
+      <c r="B10" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C10" s="17">
         <v>6800</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="17">
         <v>6800</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="17">
         <f>=D10-C10</f>
       </c>
-      <c r="F10" s="27" t="s">
-        <v>66</v>
+      <c r="F10" s="6" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B11" s="27" t="s">
-        <v>67</v>
-      </c>
-      <c r="C11" s="6">
+      <c r="B11" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C11" s="17">
         <v>2200</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="17">
         <v>2200</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="17">
         <f>=D11-C11</f>
       </c>
-      <c r="F11" s="27" t="s">
-        <v>66</v>
+      <c r="F11" s="6" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B12" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="C12" s="6">
+      <c r="B12" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C12" s="17">
         <v>500</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="17">
         <v>650</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="17">
         <f>=D12-C12</f>
       </c>
-      <c r="F12" s="27" t="s">
-        <v>66</v>
+      <c r="F12" s="6" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B13" s="36" t="s">
-        <v>69</v>
-      </c>
-      <c r="C13" s="37">
+      <c r="B13" s="44" t="s">
+        <v>107</v>
+      </c>
+      <c r="C13" s="45">
         <f>=SUM(C10:C12)</f>
       </c>
-      <c r="D13" s="37">
+      <c r="D13" s="45">
         <f>=SUM(D10:D12)</f>
       </c>
-      <c r="E13" s="37">
+      <c r="E13" s="45">
         <f>=D13-C13</f>
       </c>
-      <c r="F13" s="36" t="s">
-        <v>70</v>
+      <c r="F13" s="44" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="38" t="s">
-        <v>71</v>
-      </c>
-      <c r="C14" s="38"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="38"/>
-      <c r="F14" s="38"/>
+      <c r="B14" s="46" t="s">
+        <v>109</v>
+      </c>
+      <c r="C14" s="46"/>
+      <c r="D14" s="46"/>
+      <c r="E14" s="46"/>
+      <c r="F14" s="46"/>
     </row>
     <row r="15" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B15" s="27" t="s">
-        <v>72</v>
-      </c>
-      <c r="C15" s="6">
+      <c r="B15" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="C15" s="17">
         <v>2400</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="17">
         <v>2400</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="17">
         <f>=C15-D15</f>
       </c>
-      <c r="F15" s="27">
+      <c r="F15" s="6">
         <f>=TEXT(D15/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B16" s="27" t="s">
-        <v>73</v>
-      </c>
-      <c r="C16" s="6">
+      <c r="B16" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C16" s="17">
         <v>750</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="17">
         <v>820</v>
       </c>
-      <c r="E16" s="6">
+      <c r="E16" s="17">
         <f>=C16-D16</f>
       </c>
-      <c r="F16" s="27">
+      <c r="F16" s="6">
         <f>=TEXT(D16/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B17" s="27" t="s">
-        <v>74</v>
-      </c>
-      <c r="C17" s="6">
+      <c r="B17" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="C17" s="17">
         <v>320</v>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="17">
         <v>310</v>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="17">
         <f>=C17-D17</f>
       </c>
-      <c r="F17" s="27">
+      <c r="F17" s="6">
         <f>=TEXT(D17/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B18" s="27" t="s">
-        <v>75</v>
-      </c>
-      <c r="C18" s="6">
+      <c r="B18" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C18" s="17">
         <v>450</v>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="17">
         <v>450</v>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="17">
         <f>=C18-D18</f>
       </c>
-      <c r="F18" s="27">
+      <c r="F18" s="6">
         <f>=TEXT(D18/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B19" s="27" t="s">
-        <v>76</v>
-      </c>
-      <c r="C19" s="6">
+      <c r="B19" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C19" s="17">
         <v>400</v>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="17">
         <v>380</v>
       </c>
-      <c r="E19" s="6">
+      <c r="E19" s="17">
         <f>=C19-D19</f>
       </c>
-      <c r="F19" s="27">
+      <c r="F19" s="6">
         <f>=TEXT(D19/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B20" s="39" t="s">
-        <v>77</v>
-      </c>
-      <c r="C20" s="40">
+      <c r="B20" s="47" t="s">
+        <v>115</v>
+      </c>
+      <c r="C20" s="48">
         <f>=SUM(C15:C19)</f>
       </c>
-      <c r="D20" s="40">
+      <c r="D20" s="48">
         <f>=SUM(D15:D19)</f>
       </c>
-      <c r="E20" s="40">
+      <c r="E20" s="48">
         <f>=C20-D20</f>
       </c>
-      <c r="F20" s="39">
+      <c r="F20" s="47">
         <f>="Actual: " &amp; TEXT(D20/D13, "0.0%") &amp; " (Target: ≤50%)"</f>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B21" s="41" t="s">
-        <v>78</v>
-      </c>
-      <c r="C21" s="41"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="41"/>
+      <c r="B21" s="49" t="s">
+        <v>116</v>
+      </c>
+      <c r="C21" s="49"/>
+      <c r="D21" s="49"/>
+      <c r="E21" s="49"/>
+      <c r="F21" s="49"/>
     </row>
     <row r="22" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B22" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="C22" s="6">
+      <c r="B22" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="C22" s="17">
         <v>650</v>
       </c>
-      <c r="D22" s="6">
+      <c r="D22" s="17">
         <v>520</v>
       </c>
-      <c r="E22" s="6">
+      <c r="E22" s="17">
         <f>=C22-D22</f>
       </c>
-      <c r="F22" s="27">
+      <c r="F22" s="6">
         <f>=TEXT(D22/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="23" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B23" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="C23" s="6">
+      <c r="B23" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C23" s="17">
         <v>120</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="17">
         <v>115</v>
       </c>
-      <c r="E23" s="6">
+      <c r="E23" s="17">
         <f>=C23-D23</f>
       </c>
-      <c r="F23" s="27">
+      <c r="F23" s="6">
         <f>=TEXT(D23/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="24" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B24" s="27" t="s">
-        <v>81</v>
-      </c>
-      <c r="C24" s="6">
+      <c r="B24" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="C24" s="17">
         <v>450</v>
       </c>
-      <c r="D24" s="6">
+      <c r="D24" s="17">
         <v>380</v>
       </c>
-      <c r="E24" s="6">
+      <c r="E24" s="17">
         <f>=C24-D24</f>
       </c>
-      <c r="F24" s="27">
+      <c r="F24" s="6">
         <f>=TEXT(D24/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B25" s="42" t="s">
-        <v>82</v>
-      </c>
-      <c r="C25" s="43">
+      <c r="B25" s="50" t="s">
+        <v>120</v>
+      </c>
+      <c r="C25" s="51">
         <f>=SUM(C22:C24)</f>
       </c>
-      <c r="D25" s="43">
+      <c r="D25" s="51">
         <f>=SUM(D22:D24)</f>
       </c>
-      <c r="E25" s="43">
+      <c r="E25" s="51">
         <f>=C25-D25</f>
       </c>
-      <c r="F25" s="42">
+      <c r="F25" s="50">
         <f>="Actual: " &amp; TEXT(D25/D13, "0.0%") &amp; " (Target: ≤30%)"</f>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B26" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="C26" s="35"/>
-      <c r="D26" s="35"/>
-      <c r="E26" s="35"/>
-      <c r="F26" s="35"/>
+      <c r="B26" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
     </row>
     <row r="27" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B27" s="27" t="s">
-        <v>84</v>
-      </c>
-      <c r="C27" s="6">
+      <c r="B27" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C27" s="17">
         <v>2200</v>
       </c>
-      <c r="D27" s="6">
+      <c r="D27" s="17">
         <v>2200</v>
       </c>
-      <c r="E27" s="6">
+      <c r="E27" s="17">
         <f>=D27-C27</f>
       </c>
-      <c r="F27" s="27">
+      <c r="F27" s="6">
         <f>=TEXT(D27/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="28" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B28" s="27" t="s">
-        <v>85</v>
-      </c>
-      <c r="C28" s="6">
+      <c r="B28" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="C28" s="17">
         <v>500</v>
       </c>
-      <c r="D28" s="6">
+      <c r="D28" s="17">
         <v>500</v>
       </c>
-      <c r="E28" s="6">
+      <c r="E28" s="17">
         <f>=D28-C28</f>
       </c>
-      <c r="F28" s="27">
+      <c r="F28" s="6">
         <f>=TEXT(D28/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="29" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B29" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="C29" s="6">
+      <c r="B29" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C29" s="17">
         <v>600</v>
       </c>
-      <c r="D29" s="6">
+      <c r="D29" s="17">
         <v>750</v>
       </c>
-      <c r="E29" s="6">
+      <c r="E29" s="17">
         <f>=D29-C29</f>
       </c>
-      <c r="F29" s="27">
+      <c r="F29" s="6">
         <f>=TEXT(D29/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B30" s="44" t="s">
-        <v>87</v>
-      </c>
-      <c r="C30" s="45">
+      <c r="B30" s="52" t="s">
+        <v>125</v>
+      </c>
+      <c r="C30" s="53">
         <f>=SUM(C27:C29)</f>
       </c>
-      <c r="D30" s="45">
+      <c r="D30" s="53">
         <f>=SUM(D27:D29)</f>
       </c>
-      <c r="E30" s="45">
+      <c r="E30" s="53">
         <f>=D30-C30</f>
       </c>
-      <c r="F30" s="44">
+      <c r="F30" s="52">
         <f>="Savings Rate: " &amp; TEXT(D30/D13, "0.0%") &amp; " (FIRE Speed)"</f>
       </c>
     </row>
@@ -2184,7 +2541,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:H11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -2197,185 +2554,185 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="46" t="s">
-        <v>88</v>
-      </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
+      <c r="B2" s="54" t="s">
+        <v>126</v>
+      </c>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B3" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
+      <c r="B3" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
     </row>
     <row r="5" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B5" s="34" t="s">
-        <v>90</v>
-      </c>
-      <c r="C5" s="34" t="s">
-        <v>91</v>
-      </c>
-      <c r="D5" s="34" t="s">
-        <v>92</v>
-      </c>
-      <c r="E5" s="34" t="s">
-        <v>93</v>
-      </c>
-      <c r="F5" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="G5" s="34" t="s">
-        <v>95</v>
-      </c>
-      <c r="H5" s="34" t="s">
-        <v>96</v>
+      <c r="B5" s="43" t="s">
+        <v>128</v>
+      </c>
+      <c r="C5" s="43" t="s">
+        <v>129</v>
+      </c>
+      <c r="D5" s="43" t="s">
+        <v>130</v>
+      </c>
+      <c r="E5" s="43" t="s">
+        <v>131</v>
+      </c>
+      <c r="F5" s="43" t="s">
+        <v>132</v>
+      </c>
+      <c r="G5" s="43" t="s">
+        <v>133</v>
+      </c>
+      <c r="H5" s="43" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B6" s="27" t="s">
-        <v>97</v>
-      </c>
-      <c r="C6" s="6">
+      <c r="B6" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="C6" s="17">
         <v>25000</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="17">
         <v>21500</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="17">
         <f>=C6-D6</f>
       </c>
-      <c r="F6" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" s="6">
+      <c r="F6" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G6" s="17">
         <v>700</v>
       </c>
-      <c r="H6" s="47">
+      <c r="H6" s="55">
         <f>=D6/C6</f>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B7" s="28" t="s">
-        <v>98</v>
-      </c>
-      <c r="C7" s="11">
+      <c r="B7" s="37" t="s">
+        <v>136</v>
+      </c>
+      <c r="C7" s="22">
         <v>2000</v>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="22">
         <v>1400</v>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="22">
         <f>=C7-D7</f>
       </c>
-      <c r="F7" s="28" t="s">
-        <v>17</v>
-      </c>
-      <c r="G7" s="11">
+      <c r="F7" s="37" t="s">
+        <v>55</v>
+      </c>
+      <c r="G7" s="22">
         <v>150</v>
       </c>
-      <c r="H7" s="48">
+      <c r="H7" s="56">
         <f>=D7/C7</f>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="27" t="s">
-        <v>99</v>
-      </c>
-      <c r="C8" s="6">
+      <c r="B8" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="C8" s="17">
         <v>4500</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="17">
         <v>2800</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="17">
         <f>=C8-D8</f>
       </c>
-      <c r="F8" s="27" t="s">
-        <v>21</v>
-      </c>
-      <c r="G8" s="6">
+      <c r="F8" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="G8" s="17">
         <v>250</v>
       </c>
-      <c r="H8" s="47">
+      <c r="H8" s="55">
         <f>=D8/C8</f>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="28" t="s">
-        <v>100</v>
-      </c>
-      <c r="C9" s="11">
+      <c r="B9" s="37" t="s">
+        <v>138</v>
+      </c>
+      <c r="C9" s="22">
         <v>1500</v>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="22">
         <v>750</v>
       </c>
-      <c r="E9" s="11">
+      <c r="E9" s="22">
         <f>=C9-D9</f>
       </c>
-      <c r="F9" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="G9" s="11">
+      <c r="F9" s="37" t="s">
+        <v>58</v>
+      </c>
+      <c r="G9" s="22">
         <v>125</v>
       </c>
-      <c r="H9" s="48">
+      <c r="H9" s="56">
         <f>=D9/C9</f>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="27" t="s">
-        <v>101</v>
-      </c>
-      <c r="C10" s="6">
+      <c r="B10" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="C10" s="17">
         <v>3500</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="17">
         <v>1800</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="17">
         <f>=C10-D10</f>
       </c>
-      <c r="F10" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="G10" s="6">
+      <c r="F10" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="G10" s="17">
         <v>250</v>
       </c>
-      <c r="H10" s="47">
+      <c r="H10" s="55">
         <f>=D10/C10</f>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="C11" s="15">
+      <c r="B11" s="25" t="s">
+        <v>140</v>
+      </c>
+      <c r="C11" s="26">
         <f>=SUM(C6:C10)</f>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="26">
         <f>=SUM(D6:D10)</f>
       </c>
-      <c r="E11" s="15">
+      <c r="E11" s="26">
         <f>=SUM(E6:E10)</f>
       </c>
-      <c r="F11" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="G11" s="15">
+      <c r="F11" s="25" t="s">
+        <v>141</v>
+      </c>
+      <c r="G11" s="26">
         <f>=SUM(G6:G10)</f>
       </c>
-      <c r="H11" s="49">
+      <c r="H11" s="57">
         <f>=D11/C11</f>
       </c>
     </row>
@@ -2389,7 +2746,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:E16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -2403,119 +2760,119 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B2" s="31" t="s">
-        <v>104</v>
-      </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
+      <c r="B2" s="40" t="s">
+        <v>142</v>
+      </c>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B4" s="50" t="s">
-        <v>105</v>
-      </c>
-      <c r="C4" s="50"/>
-      <c r="D4" s="50"/>
-      <c r="E4" s="50"/>
+      <c r="B4" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
     </row>
     <row r="5" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="C5" s="51">
+      <c r="B5" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="C5" s="58">
         <v>32</v>
       </c>
     </row>
     <row r="6" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="27" t="s">
-        <v>107</v>
-      </c>
-      <c r="C6" s="52">
+      <c r="B6" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="C6" s="59">
         <v>66000</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7" s="27" t="s">
-        <v>108</v>
-      </c>
-      <c r="C7" s="53">
+      <c r="B7" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C7" s="60">
         <v>0.04</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="27" t="s">
-        <v>109</v>
-      </c>
-      <c r="C8" s="53">
+      <c r="B8" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="C8" s="60">
         <v>0.07</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B9" s="27" t="s">
-        <v>110</v>
-      </c>
-      <c r="C9" s="52">
+      <c r="B9" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="C9" s="59">
         <f>'⚡ 2-Min Quick Check-In'!D18</f>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B10" s="27" t="s">
-        <v>111</v>
-      </c>
-      <c r="C10" s="52">
+      <c r="B10" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="C10" s="59">
         <f>'💸 Smart Budget (50-30-20)'!D27</f>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B12" s="35" t="s">
-        <v>112</v>
-      </c>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="35"/>
+      <c r="B12" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B13" s="27" t="s">
-        <v>113</v>
-      </c>
-      <c r="C13" s="52">
+      <c r="B13" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="C13" s="59">
         <f>C6*0.65/C7</f>
       </c>
-      <c r="D13" s="54" t="s">
-        <v>114</v>
+      <c r="D13" s="61" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B14" s="27" t="s">
-        <v>115</v>
-      </c>
-      <c r="C14" s="52">
+      <c r="B14" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="C14" s="59">
         <f>C6/C7</f>
       </c>
-      <c r="D14" s="54" t="s">
-        <v>116</v>
+      <c r="D14" s="61" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B15" s="27" t="s">
-        <v>117</v>
-      </c>
-      <c r="C15" s="52">
+      <c r="B15" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="C15" s="59">
         <f>C6*1.4/C7</f>
       </c>
-      <c r="D15" s="54" t="s">
-        <v>118</v>
+      <c r="D15" s="61" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B16" s="27" t="s">
-        <v>119</v>
-      </c>
-      <c r="C16" s="52">
+      <c r="B16" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="C16" s="59">
         <f>(C6/C7)/(1+C8)^(60-C5)</f>
       </c>
-      <c r="D16" s="54" t="s">
-        <v>120</v>
+      <c r="D16" s="61" t="s">
+        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -2529,7 +2886,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:F9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -2544,114 +2901,114 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="55" t="s">
-        <v>121</v>
-      </c>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
+      <c r="B2" s="62" t="s">
+        <v>159</v>
+      </c>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
     </row>
     <row r="4" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="26" t="s">
-        <v>122</v>
-      </c>
-      <c r="C4" s="26" t="s">
-        <v>92</v>
-      </c>
-      <c r="D4" s="26" t="s">
-        <v>123</v>
-      </c>
-      <c r="E4" s="26" t="s">
-        <v>124</v>
-      </c>
-      <c r="F4" s="26" t="s">
-        <v>125</v>
+      <c r="B4" s="36" t="s">
+        <v>160</v>
+      </c>
+      <c r="C4" s="36" t="s">
+        <v>130</v>
+      </c>
+      <c r="D4" s="36" t="s">
+        <v>161</v>
+      </c>
+      <c r="E4" s="36" t="s">
+        <v>162</v>
+      </c>
+      <c r="F4" s="36" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="5" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="27" t="s">
-        <v>126</v>
-      </c>
-      <c r="C5" s="6">
+      <c r="B5" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="C5" s="17">
         <v>4200</v>
       </c>
-      <c r="D5" s="56">
+      <c r="D5" s="63">
         <v>0.2499</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="17">
         <v>140</v>
       </c>
-      <c r="F5" s="27" t="s">
-        <v>127</v>
+      <c r="F5" s="6" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="6" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="27" t="s">
-        <v>128</v>
-      </c>
-      <c r="C6" s="6">
+      <c r="B6" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="C6" s="17">
         <v>8500</v>
       </c>
-      <c r="D6" s="56">
+      <c r="D6" s="63">
         <v>0.115</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="17">
         <v>210</v>
       </c>
-      <c r="F6" s="27" t="s">
-        <v>129</v>
+      <c r="F6" s="6" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="27" t="s">
-        <v>130</v>
-      </c>
-      <c r="C7" s="6">
+      <c r="B7" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="C7" s="17">
         <v>17400</v>
       </c>
-      <c r="D7" s="56">
+      <c r="D7" s="63">
         <v>0.059</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="17">
         <v>380</v>
       </c>
-      <c r="F7" s="27" t="s">
-        <v>131</v>
+      <c r="F7" s="6" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="27" t="s">
-        <v>132</v>
-      </c>
-      <c r="C8" s="6">
+      <c r="B8" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="C8" s="17">
         <v>200000</v>
       </c>
-      <c r="D8" s="56">
+      <c r="D8" s="63">
         <v>0.035</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="17">
         <v>1670</v>
       </c>
-      <c r="F8" s="27" t="s">
-        <v>133</v>
+      <c r="F8" s="6" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="36" t="s">
-        <v>134</v>
-      </c>
-      <c r="C9" s="37">
+      <c r="B9" s="44" t="s">
+        <v>172</v>
+      </c>
+      <c r="C9" s="45">
         <f>=SUM(C5:C8)</f>
       </c>
-      <c r="D9" s="57">
+      <c r="D9" s="64">
         <f>=AVERAGE(D5:D8)</f>
       </c>
-      <c r="E9" s="37">
+      <c r="E9" s="45">
         <f>=SUM(E5:E8)</f>
       </c>
-      <c r="F9" s="36" t="s">
-        <v>135</v>
+      <c r="F9" s="44" t="s">
+        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -2663,7 +3020,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:H10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -2675,174 +3032,174 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="55" t="s">
-        <v>136</v>
-      </c>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
+      <c r="B2" s="62" t="s">
+        <v>174</v>
+      </c>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
     </row>
     <row r="4" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B4" s="26" t="s">
-        <v>137</v>
-      </c>
-      <c r="C4" s="26" t="s">
-        <v>138</v>
-      </c>
-      <c r="D4" s="26" t="s">
-        <v>139</v>
-      </c>
-      <c r="E4" s="26" t="s">
-        <v>140</v>
-      </c>
-      <c r="F4" s="26" t="s">
-        <v>141</v>
-      </c>
-      <c r="G4" s="26" t="s">
-        <v>142</v>
-      </c>
-      <c r="H4" s="26" t="s">
-        <v>143</v>
+      <c r="B4" s="36" t="s">
+        <v>175</v>
+      </c>
+      <c r="C4" s="36" t="s">
+        <v>176</v>
+      </c>
+      <c r="D4" s="36" t="s">
+        <v>177</v>
+      </c>
+      <c r="E4" s="36" t="s">
+        <v>178</v>
+      </c>
+      <c r="F4" s="36" t="s">
+        <v>179</v>
+      </c>
+      <c r="G4" s="36" t="s">
+        <v>180</v>
+      </c>
+      <c r="H4" s="36" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="5" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B5" s="27" t="s">
-        <v>144</v>
-      </c>
-      <c r="C5" s="6">
+      <c r="B5" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="C5" s="17">
         <v>4800</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="17">
         <v>39000</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="17">
         <v>145000</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="17">
         <v>380000</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="17">
         <v>750000</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H5" s="17">
         <v>2800000</v>
       </c>
     </row>
     <row r="6" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B6" s="28" t="s">
-        <v>145</v>
-      </c>
-      <c r="C6" s="11">
+      <c r="B6" s="37" t="s">
+        <v>183</v>
+      </c>
+      <c r="C6" s="22">
         <v>35000</v>
       </c>
-      <c r="D6" s="11">
+      <c r="D6" s="22">
         <v>135600</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="22">
         <v>420000</v>
       </c>
-      <c r="F6" s="11">
+      <c r="F6" s="22">
         <v>980000</v>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="22">
         <v>1850000</v>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="22">
         <v>5500000</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B7" s="27" t="s">
-        <v>146</v>
-      </c>
-      <c r="C7" s="6">
+      <c r="B7" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="C7" s="17">
         <v>68000</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="17">
         <v>247200</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="17">
         <v>780000</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="17">
         <v>1950000</v>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="17">
         <v>3400000</v>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="17">
         <v>10200000</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="28" t="s">
-        <v>147</v>
-      </c>
-      <c r="C8" s="11">
+      <c r="B8" s="37" t="s">
+        <v>185</v>
+      </c>
+      <c r="C8" s="22">
         <v>95000</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="22">
         <v>364500</v>
       </c>
-      <c r="E8" s="11">
+      <c r="E8" s="22">
         <v>1150000</v>
       </c>
-      <c r="F8" s="11">
+      <c r="F8" s="22">
         <v>2800000</v>
       </c>
-      <c r="G8" s="11">
+      <c r="G8" s="22">
         <v>4900000</v>
       </c>
-      <c r="H8" s="11">
+      <c r="H8" s="22">
         <v>14500000</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="27" t="s">
-        <v>148</v>
-      </c>
-      <c r="C9" s="6">
+      <c r="B9" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="C9" s="17">
         <v>110000</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="17">
         <v>409900</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="17">
         <v>1350000</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="17">
         <v>3200000</v>
       </c>
-      <c r="G9" s="6">
+      <c r="G9" s="17">
         <v>5600000</v>
       </c>
-      <c r="H9" s="6">
+      <c r="H9" s="17">
         <v>16800000</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="28" t="s">
-        <v>149</v>
-      </c>
-      <c r="C10" s="11">
+      <c r="B10" s="37" t="s">
+        <v>187</v>
+      </c>
+      <c r="C10" s="22">
         <v>92000</v>
       </c>
-      <c r="D10" s="11">
+      <c r="D10" s="22">
         <v>335600</v>
       </c>
-      <c r="E10" s="11">
+      <c r="E10" s="22">
         <v>1050000</v>
       </c>
-      <c r="F10" s="11">
+      <c r="F10" s="22">
         <v>2600000</v>
       </c>
-      <c r="G10" s="11">
+      <c r="G10" s="22">
         <v>4700000</v>
       </c>
-      <c r="H10" s="11">
+      <c r="H10" s="22">
         <v>13200000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(product): add live reactive Vault Simulator widget and official GetNetWorth touch
</commit_message>
<xml_diff>
--- a/public/downloads/NetWorth_FIRE_Master_Vault_2026.xlsx
+++ b/public/downloads/NetWorth_FIRE_Master_Vault_2026.xlsx
@@ -20,10 +20,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="188">
   <si>
-    <t>👋 WELCOME TO YOUR PRIVATE WEALTH &amp; BUDGET OPERATING SYSTEM</t>
-  </si>
-  <si>
-    <t>Designed for normal humans, not CPAs. Zero homework, zero broken formulas, 100% private &amp; offline.</t>
+    <t>🏛️ GETNETWORTHCALCULATOR.COM • OFFICIAL WEALTH &amp; BUDGET OPERATING SYSTEM</t>
+  </si>
+  <si>
+    <t>Researched &amp; Modeled by Yash Jha | Benchmarked Against US Federal Reserve SCF Microdata (2026)</t>
   </si>
   <si>
     <t>🚀 THE 3-STEP MONTHLY ROUTINE (TAKES 2 MINUTES ON THE 1ST OF EACH MONTH)</t>
@@ -131,10 +131,10 @@
     <t>Official US Federal Reserve Survey of Consumer Finances raw microdata tables.</t>
   </si>
   <si>
-    <t>💡 Using Google Sheets? Just drag and drop this file into Google Drive and click "Open with Google Sheets". It converts in 2 seconds with 100% of formulas intact.</t>
-  </si>
-  <si>
-    <t>⚡ 2-MINUTE MONTHLY QUICK CHECK-IN (NO HOMEWORK, NO OVERWHELM)</t>
+    <t>🌐 GetNetWorthCalculator.com • 100% Private, Anonymous &amp; Offline • Curated by Yash Jha</t>
+  </si>
+  <si>
+    <t>⚡ 2-MINUTE MONTHLY QUICK CHECK-IN • GETNETWORTHCALCULATOR.COM</t>
   </si>
   <si>
     <t>Rule of Thumb: On the 1st of each month, type just 4 numbers (green headers). Everything else calculates automatically.</t>
@@ -203,7 +203,7 @@
     <t>LATEST / ANNUAL</t>
   </si>
   <si>
-    <t>🏛️ NET WORTH &amp; FINANCIAL INDEPENDENCE MASTER VAULT (2026 EDITION)</t>
+    <t>🏛️ EXECUTIVE WEALTH COMMAND CENTER • GETNETWORTHCALCULATOR.COM</t>
   </si>
   <si>
     <t>Private Wealth Dashboard • Federal Reserve SCF Percentile Engine • Trinity Study FIRE Calculator</t>
@@ -299,7 +299,7 @@
     <t>October 2038</t>
   </si>
   <si>
-    <t>💸 SMART MONTHLY CASH FLOW &amp; 50/30/20 BUDGET ENGINE</t>
+    <t>💸 SMART MONTHLY CASH FLOW &amp; 50/30/20 BUDGET • GETNETWORTHCALCULATOR.COM</t>
   </si>
   <si>
     <t>Answers: "How much can I safely spend guilt-free?" • 50% Needs, 30% Wants, 20% Wealth Surplus.</t>
@@ -398,7 +398,7 @@
     <t>TOTAL WEALTH SURPLUS</t>
   </si>
   <si>
-    <t>🎯 SINKING FUNDS &amp; IRREGULAR EXPENSE DEFENSE SHIELD</t>
+    <t>🎯 SINKING FUNDS &amp; IRREGULAR EXPENSE DEFENSE SHIELD • GETNETWORTHCALCULATOR.COM</t>
   </si>
   <si>
     <t>Prevents budget shock from annual car insurance, holiday gifts, unexpected home repairs, and vacations.</t>
@@ -446,7 +446,7 @@
     <t>Multiple</t>
   </si>
   <si>
-    <t>🔥 FINANCIAL INDEPENDENCE &amp; EARLY RETIREMENT CALCULATOR (TRINITY STUDY)</t>
+    <t>🔥 FINANCIAL INDEPENDENCE &amp; EARLY RETIREMENT CALCULATOR • GETNETWORTHCALCULATOR.COM</t>
   </si>
   <si>
     <t>1. CORE ASSUMPTIONS &amp; SAFE WITHDRAWAL RATE (SWR)</t>
@@ -497,7 +497,7 @@
     <t>Compounding does all remaining work</t>
   </si>
   <si>
-    <t>💳 DEBT PAYOFF ACCELERATOR: MATHEMATICAL AVALANCHE VS BEHAVIORAL SNOWBALL</t>
+    <t>💳 DEBT PAYOFF ACCELERATOR: AVALANCHE VS SNOWBALL • GETNETWORTHCALCULATOR.COM</t>
   </si>
   <si>
     <t>Debt Name</t>
@@ -542,7 +542,7 @@
     <t>Blended APR</t>
   </si>
   <si>
-    <t>🏛️ OFFICIAL US FEDERAL RESERVE SURVEY OF CONSUMER FINANCES (SCF) BENCHMARK DATA</t>
+    <t>🏛️ OFFICIAL US FEDERAL RESERVE SCF BENCHMARK DATA • GETNETWORTHCALCULATOR.COM</t>
   </si>
   <si>
     <t>Age Bracket</t>
@@ -595,7 +595,7 @@
     <numFmt numFmtId="167" formatCode="$#,##0/day"/>
     <numFmt numFmtId="168" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="29" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -606,13 +606,13 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
-      <sz val="13"/>
+      <sz val="12"/>
       <name val="Arial"/>
     </font>
     <font>
       <i/>
       <color rgb="FFCBD5E1"/>
-      <sz val="9.5"/>
+      <sz val="9"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -635,21 +635,9 @@
       <sz val="9"/>
     </font>
     <font>
-      <i/>
+      <b/>
       <color rgb="FF065F46"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FFCBD5E1"/>
-      <sz val="9"/>
-      <name val="Arial"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <b/>
@@ -733,23 +721,28 @@
       <sz val="15"/>
     </font>
     <font>
-      <i/>
-      <color rgb="FF64748B"/>
-      <sz val="9"/>
-    </font>
-    <font>
       <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <i/>
+      <color rgb="FF64748B"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF047857"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -763,17 +756,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF065F46"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFDCFCE7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF047857"/>
       </patternFill>
     </fill>
     <fill>
@@ -819,7 +802,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -832,91 +815,85 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="14" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="17" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="20" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="25" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="24" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="12" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="12" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="167" fontId="26" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="14" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="14" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="14" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="168" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="14" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1261,12 +1238,12 @@
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="32" customWidth="1"/>
-    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="30" customWidth="1"/>
     <col min="5" max="5" width="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" ht="32" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="2" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1321,11 +1298,11 @@
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
     </row>
     <row r="11" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B11" s="5" t="s">
@@ -1361,81 +1338,81 @@
       </c>
     </row>
     <row r="15" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
     </row>
     <row r="16" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D16" s="10"/>
+      <c r="D16" s="9"/>
     </row>
     <row r="17" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D17" s="10"/>
+      <c r="D17" s="9"/>
     </row>
     <row r="18" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D18" s="10"/>
+      <c r="D18" s="9"/>
     </row>
     <row r="19" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D19" s="10"/>
+      <c r="D19" s="9"/>
     </row>
     <row r="20" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D20" s="10"/>
+      <c r="D20" s="9"/>
     </row>
     <row r="21" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D21" s="10"/>
+      <c r="D21" s="9"/>
     </row>
     <row r="22" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D22" s="10"/>
+      <c r="D22" s="9"/>
     </row>
     <row r="24" ht="26" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B24" s="11" t="s">
+      <c r="B24" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -1475,390 +1452,390 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
     </row>
     <row r="3" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
     </row>
     <row r="5" ht="24" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="E5" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="F5" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="G5" s="14" t="s">
+      <c r="G5" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="H5" s="14" t="s">
+      <c r="H5" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="I5" s="14" t="s">
+      <c r="I5" s="12" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="17">
+      <c r="C6" s="15">
         <v>25000</v>
       </c>
-      <c r="D6" s="17">
+      <c r="D6" s="15">
         <v>185000</v>
       </c>
-      <c r="E6" s="17">
+      <c r="E6" s="15">
         <v>350000</v>
       </c>
-      <c r="F6" s="17">
+      <c r="F6" s="15">
         <v>245000</v>
       </c>
-      <c r="G6" s="18">
+      <c r="G6" s="16">
         <f>=(C6+D6+E6)-F6</f>
       </c>
-      <c r="H6" s="19">
+      <c r="H6" s="17">
         <v>0</v>
       </c>
-      <c r="I6" s="20">
+      <c r="I6" s="18">
         <v>0</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="C7" s="22">
+      <c r="C7" s="20">
         <v>26200</v>
       </c>
-      <c r="D7" s="22">
+      <c r="D7" s="20">
         <v>189500</v>
       </c>
-      <c r="E7" s="22">
+      <c r="E7" s="20">
         <v>350000</v>
       </c>
-      <c r="F7" s="22">
+      <c r="F7" s="20">
         <v>243800</v>
       </c>
-      <c r="G7" s="18">
+      <c r="G7" s="16">
         <f>=(C7+D7+E7)-F7</f>
       </c>
-      <c r="H7" s="23">
+      <c r="H7" s="21">
         <f>=G7-G6</f>
       </c>
-      <c r="I7" s="24">
+      <c r="I7" s="22">
         <f>=(G7-G6)/G6</f>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="C8" s="17">
+      <c r="C8" s="15">
         <v>25800</v>
       </c>
-      <c r="D8" s="17">
+      <c r="D8" s="15">
         <v>194200</v>
       </c>
-      <c r="E8" s="17">
+      <c r="E8" s="15">
         <v>350000</v>
       </c>
-      <c r="F8" s="17">
+      <c r="F8" s="15">
         <v>242600</v>
       </c>
-      <c r="G8" s="18">
+      <c r="G8" s="16">
         <f>=(C8+D8+E8)-F8</f>
       </c>
-      <c r="H8" s="19">
+      <c r="H8" s="17">
         <f>=G8-G7</f>
       </c>
-      <c r="I8" s="20">
+      <c r="I8" s="18">
         <f>=(G8-G7)/G7</f>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="20">
         <v>27100</v>
       </c>
-      <c r="D9" s="22">
+      <c r="D9" s="20">
         <v>191000</v>
       </c>
-      <c r="E9" s="22">
+      <c r="E9" s="20">
         <v>350000</v>
       </c>
-      <c r="F9" s="22">
+      <c r="F9" s="20">
         <v>241400</v>
       </c>
-      <c r="G9" s="18">
+      <c r="G9" s="16">
         <f>=(C9+D9+E9)-F9</f>
       </c>
-      <c r="H9" s="23">
+      <c r="H9" s="21">
         <f>=G9-G8</f>
       </c>
-      <c r="I9" s="24">
+      <c r="I9" s="22">
         <f>=(G9-G8)/G8</f>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="17">
+      <c r="C10" s="15">
         <v>26900</v>
       </c>
-      <c r="D10" s="17">
+      <c r="D10" s="15">
         <v>198500</v>
       </c>
-      <c r="E10" s="17">
+      <c r="E10" s="15">
         <v>352000</v>
       </c>
-      <c r="F10" s="17">
+      <c r="F10" s="15">
         <v>240100</v>
       </c>
-      <c r="G10" s="18">
+      <c r="G10" s="16">
         <f>=(C10+D10+E10)-F10</f>
       </c>
-      <c r="H10" s="19">
+      <c r="H10" s="17">
         <f>=G10-G9</f>
       </c>
-      <c r="I10" s="20">
+      <c r="I10" s="18">
         <f>=(G10-G9)/G9</f>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="C11" s="22">
+      <c r="C11" s="20">
         <v>28400</v>
       </c>
-      <c r="D11" s="22">
+      <c r="D11" s="20">
         <v>204000</v>
       </c>
-      <c r="E11" s="22">
+      <c r="E11" s="20">
         <v>352000</v>
       </c>
-      <c r="F11" s="22">
+      <c r="F11" s="20">
         <v>238800</v>
       </c>
-      <c r="G11" s="18">
+      <c r="G11" s="16">
         <f>=(C11+D11+E11)-F11</f>
       </c>
-      <c r="H11" s="23">
+      <c r="H11" s="21">
         <f>=G11-G10</f>
       </c>
-      <c r="I11" s="24">
+      <c r="I11" s="22">
         <f>=(G11-G10)/G10</f>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="17">
+      <c r="C12" s="15">
         <v>29000</v>
       </c>
-      <c r="D12" s="17">
+      <c r="D12" s="15">
         <v>209500</v>
       </c>
-      <c r="E12" s="17">
+      <c r="E12" s="15">
         <v>352000</v>
       </c>
-      <c r="F12" s="17">
+      <c r="F12" s="15">
         <v>237500</v>
       </c>
-      <c r="G12" s="18">
+      <c r="G12" s="16">
         <f>=(C12+D12+E12)-F12</f>
       </c>
-      <c r="H12" s="19">
+      <c r="H12" s="17">
         <f>=G12-G11</f>
       </c>
-      <c r="I12" s="20">
+      <c r="I12" s="18">
         <f>=(G12-G11)/G11</f>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="22">
+      <c r="C13" s="20">
         <v>28500</v>
       </c>
-      <c r="D13" s="22">
+      <c r="D13" s="20">
         <v>215000</v>
       </c>
-      <c r="E13" s="22">
+      <c r="E13" s="20">
         <v>355000</v>
       </c>
-      <c r="F13" s="22">
+      <c r="F13" s="20">
         <v>236100</v>
       </c>
-      <c r="G13" s="18">
+      <c r="G13" s="16">
         <f>=(C13+D13+E13)-F13</f>
       </c>
-      <c r="H13" s="23">
+      <c r="H13" s="21">
         <f>=G13-G12</f>
       </c>
-      <c r="I13" s="24">
+      <c r="I13" s="22">
         <f>=(G13-G12)/G12</f>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="17">
+      <c r="C14" s="15">
         <v>30200</v>
       </c>
-      <c r="D14" s="17">
+      <c r="D14" s="15">
         <v>221000</v>
       </c>
-      <c r="E14" s="17">
+      <c r="E14" s="15">
         <v>355000</v>
       </c>
-      <c r="F14" s="17">
+      <c r="F14" s="15">
         <v>234700</v>
       </c>
-      <c r="G14" s="18">
+      <c r="G14" s="16">
         <f>=(C14+D14+E14)-F14</f>
       </c>
-      <c r="H14" s="19">
+      <c r="H14" s="17">
         <f>=G14-G13</f>
       </c>
-      <c r="I14" s="20">
+      <c r="I14" s="18">
         <f>=(G14-G13)/G13</f>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B15" s="21" t="s">
+      <c r="B15" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="22">
+      <c r="C15" s="20">
         <v>31000</v>
       </c>
-      <c r="D15" s="22">
+      <c r="D15" s="20">
         <v>228000</v>
       </c>
-      <c r="E15" s="22">
+      <c r="E15" s="20">
         <v>355000</v>
       </c>
-      <c r="F15" s="22">
+      <c r="F15" s="20">
         <v>233200</v>
       </c>
-      <c r="G15" s="18">
+      <c r="G15" s="16">
         <f>=(C15+D15+E15)-F15</f>
       </c>
-      <c r="H15" s="23">
+      <c r="H15" s="21">
         <f>=G15-G14</f>
       </c>
-      <c r="I15" s="24">
+      <c r="I15" s="22">
         <f>=(G15-G14)/G14</f>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="C16" s="17">
+      <c r="C16" s="15">
         <v>31500</v>
       </c>
-      <c r="D16" s="17">
+      <c r="D16" s="15">
         <v>234500</v>
       </c>
-      <c r="E16" s="17">
+      <c r="E16" s="15">
         <v>358000</v>
       </c>
-      <c r="F16" s="17">
+      <c r="F16" s="15">
         <v>231700</v>
       </c>
-      <c r="G16" s="18">
+      <c r="G16" s="16">
         <f>=(C16+D16+E16)-F16</f>
       </c>
-      <c r="H16" s="19">
+      <c r="H16" s="17">
         <f>=G16-G15</f>
       </c>
-      <c r="I16" s="20">
+      <c r="I16" s="18">
         <f>=(G16-G15)/G15</f>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B17" s="21" t="s">
+      <c r="B17" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="C17" s="22">
+      <c r="C17" s="20">
         <v>33000</v>
       </c>
-      <c r="D17" s="22">
+      <c r="D17" s="20">
         <v>242000</v>
       </c>
-      <c r="E17" s="22">
+      <c r="E17" s="20">
         <v>358000</v>
       </c>
-      <c r="F17" s="22">
+      <c r="F17" s="20">
         <v>230100</v>
       </c>
-      <c r="G17" s="18">
+      <c r="G17" s="16">
         <f>=(C17+D17+E17)-F17</f>
       </c>
-      <c r="H17" s="23">
+      <c r="H17" s="21">
         <f>=G17-G16</f>
       </c>
-      <c r="I17" s="24">
+      <c r="I17" s="22">
         <f>=(G17-G16)/G16</f>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B18" s="25" t="s">
+      <c r="B18" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="C18" s="26">
+      <c r="C18" s="24">
         <f>=C17</f>
       </c>
-      <c r="D18" s="26">
+      <c r="D18" s="24">
         <f>=D17</f>
       </c>
-      <c r="E18" s="26">
+      <c r="E18" s="24">
         <f>=E17</f>
       </c>
-      <c r="F18" s="26">
+      <c r="F18" s="24">
         <f>=F17</f>
       </c>
-      <c r="G18" s="26">
+      <c r="G18" s="24">
         <f>=G17</f>
       </c>
-      <c r="H18" s="26">
+      <c r="H18" s="24">
         <f>=G17-G6</f>
       </c>
-      <c r="I18" s="27">
+      <c r="I18" s="25">
         <f>=(G17-G6)/G6</f>
       </c>
     </row>
@@ -1885,85 +1862,85 @@
   </cols>
   <sheetData>
     <row r="2" ht="30" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="27"/>
     </row>
     <row r="5" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="28" t="s">
         <v>63</v>
       </c>
-      <c r="C5" s="29"/>
-      <c r="D5" s="29" t="s">
+      <c r="C5" s="28"/>
+      <c r="D5" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="E5" s="29"/>
-      <c r="F5" s="29" t="s">
+      <c r="E5" s="28"/>
+      <c r="F5" s="28" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="30">
+      <c r="B6" s="29">
         <f>='⚡ 2-Min Quick Check-In'!G18</f>
       </c>
-      <c r="C6" s="30"/>
-      <c r="D6" s="31">
+      <c r="C6" s="29"/>
+      <c r="D6" s="30">
         <f>='⚡ 2-Min Quick Check-In'!C18+'⚡ 2-Min Quick Check-In'!D18</f>
       </c>
-      <c r="E6" s="31"/>
-      <c r="F6" s="32" t="s">
+      <c r="E6" s="30"/>
+      <c r="F6" s="31" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="33">
+      <c r="B7" s="32">
         <f>="▲ Annual Growth: " &amp; TEXT('⚡ 2-Min Quick Check-In'!I18, "+0.0%") &amp; " (+$" &amp; TEXT('⚡ 2-Min Quick Check-In'!H18, "#,##0") &amp; ")"</f>
       </c>
-      <c r="C7" s="33"/>
-      <c r="D7" s="34">
+      <c r="C7" s="32"/>
+      <c r="D7" s="33">
         <f>="Liquid Ratio: " &amp; TEXT(('⚡ 2-Min Quick Check-In'!C18+'⚡ 2-Min Quick Check-In'!D18)/('⚡ 2-Min Quick Check-In'!G18+'⚡ 2-Min Quick Check-In'!F18), "0.0%") &amp; " of total assets"</f>
       </c>
-      <c r="E7" s="34"/>
-      <c r="F7" s="34" t="s">
+      <c r="E7" s="33"/>
+      <c r="F7" s="33" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="C9" s="35"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="35"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="34"/>
+      <c r="F9" s="34"/>
     </row>
     <row r="10" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B10" s="36" t="s">
+      <c r="B10" s="35" t="s">
         <v>69</v>
       </c>
-      <c r="C10" s="36" t="s">
+      <c r="C10" s="35" t="s">
         <v>70</v>
       </c>
-      <c r="D10" s="36" t="s">
+      <c r="D10" s="35" t="s">
         <v>71</v>
       </c>
-      <c r="E10" s="36" t="s">
+      <c r="E10" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F10" s="36" t="s">
+      <c r="F10" s="35" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1971,13 +1948,13 @@
       <c r="B11" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="C11" s="17">
+      <c r="C11" s="15">
         <f>='⚡ 2-Min Quick Check-In'!G6</f>
       </c>
-      <c r="D11" s="17">
+      <c r="D11" s="15">
         <f>='⚡ 2-Min Quick Check-In'!D6</f>
       </c>
-      <c r="E11" s="17">
+      <c r="E11" s="15">
         <f>='⚡ 2-Min Quick Check-In'!F6</f>
       </c>
       <c r="F11" s="6" t="s">
@@ -1985,19 +1962,19 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B12" s="37" t="s">
+      <c r="B12" s="36" t="s">
         <v>76</v>
       </c>
-      <c r="C12" s="22">
+      <c r="C12" s="20">
         <f>='⚡ 2-Min Quick Check-In'!G9</f>
       </c>
-      <c r="D12" s="22">
+      <c r="D12" s="20">
         <f>='⚡ 2-Min Quick Check-In'!D9</f>
       </c>
-      <c r="E12" s="22">
+      <c r="E12" s="20">
         <f>='⚡ 2-Min Quick Check-In'!F9</f>
       </c>
-      <c r="F12" s="37" t="s">
+      <c r="F12" s="36" t="s">
         <v>77</v>
       </c>
     </row>
@@ -2005,13 +1982,13 @@
       <c r="B13" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="C13" s="17">
+      <c r="C13" s="15">
         <f>='⚡ 2-Min Quick Check-In'!G12</f>
       </c>
-      <c r="D13" s="17">
+      <c r="D13" s="15">
         <f>='⚡ 2-Min Quick Check-In'!D12</f>
       </c>
-      <c r="E13" s="17">
+      <c r="E13" s="15">
         <f>='⚡ 2-Min Quick Check-In'!F12</f>
       </c>
       <c r="F13" s="6" t="s">
@@ -2019,19 +1996,19 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="37" t="s">
+      <c r="B14" s="36" t="s">
         <v>80</v>
       </c>
-      <c r="C14" s="22">
+      <c r="C14" s="20">
         <f>='⚡ 2-Min Quick Check-In'!G15</f>
       </c>
-      <c r="D14" s="22">
+      <c r="D14" s="20">
         <f>='⚡ 2-Min Quick Check-In'!D15</f>
       </c>
-      <c r="E14" s="22">
+      <c r="E14" s="20">
         <f>='⚡ 2-Min Quick Check-In'!F15</f>
       </c>
-      <c r="F14" s="37" t="s">
+      <c r="F14" s="36" t="s">
         <v>81</v>
       </c>
     </row>
@@ -2039,13 +2016,13 @@
       <c r="B15" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="C15" s="17">
+      <c r="C15" s="15">
         <f>='⚡ 2-Min Quick Check-In'!G17</f>
       </c>
-      <c r="D15" s="17">
+      <c r="D15" s="15">
         <f>='⚡ 2-Min Quick Check-In'!D17</f>
       </c>
-      <c r="E15" s="17">
+      <c r="E15" s="15">
         <f>='⚡ 2-Min Quick Check-In'!F17</f>
       </c>
       <c r="F15" s="6" t="s">
@@ -2053,43 +2030,43 @@
       </c>
     </row>
     <row r="18" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B18" s="35" t="s">
+      <c r="B18" s="34" t="s">
         <v>84</v>
       </c>
-      <c r="C18" s="35"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="35"/>
-      <c r="F18" s="35"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="34"/>
     </row>
     <row r="19" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B19" s="38" t="s">
+      <c r="B19" s="37" t="s">
         <v>85</v>
       </c>
-      <c r="C19" s="38" t="s">
+      <c r="C19" s="37" t="s">
         <v>86</v>
       </c>
-      <c r="D19" s="38" t="s">
+      <c r="D19" s="37" t="s">
         <v>87</v>
       </c>
-      <c r="E19" s="38" t="s">
+      <c r="E19" s="37" t="s">
         <v>88</v>
       </c>
-      <c r="F19" s="38"/>
+      <c r="F19" s="37"/>
     </row>
     <row r="20" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B20" s="39" t="s">
+      <c r="B20" s="38" t="s">
         <v>89</v>
       </c>
-      <c r="C20" s="39" t="s">
+      <c r="C20" s="38" t="s">
         <v>90</v>
       </c>
-      <c r="D20" s="39" t="s">
+      <c r="D20" s="38" t="s">
         <v>91</v>
       </c>
-      <c r="E20" s="39" t="s">
+      <c r="E20" s="38" t="s">
         <v>92</v>
       </c>
-      <c r="F20" s="39"/>
+      <c r="F20" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -2125,82 +2102,82 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="40" t="s">
+      <c r="B2" s="26" t="s">
         <v>93</v>
       </c>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="27" t="s">
         <v>94</v>
       </c>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="27"/>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="33" t="s">
+      <c r="B5" s="32" t="s">
         <v>95</v>
       </c>
-      <c r="C5" s="33"/>
-      <c r="D5" s="33"/>
-      <c r="E5" s="29" t="s">
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="28" t="s">
         <v>96</v>
       </c>
-      <c r="F5" s="29"/>
+      <c r="F5" s="28"/>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="41">
+      <c r="B6" s="39">
         <f>=E24</f>
       </c>
-      <c r="C6" s="41"/>
-      <c r="D6" s="41"/>
-      <c r="E6" s="42">
+      <c r="C6" s="39"/>
+      <c r="D6" s="39"/>
+      <c r="E6" s="40">
         <f>=E24/30</f>
       </c>
-      <c r="F6" s="42"/>
+      <c r="F6" s="40"/>
     </row>
     <row r="8" ht="22" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="43" t="s">
+      <c r="B8" s="41" t="s">
         <v>97</v>
       </c>
-      <c r="C8" s="43" t="s">
+      <c r="C8" s="41" t="s">
         <v>98</v>
       </c>
-      <c r="D8" s="43" t="s">
+      <c r="D8" s="41" t="s">
         <v>99</v>
       </c>
-      <c r="E8" s="43" t="s">
+      <c r="E8" s="41" t="s">
         <v>100</v>
       </c>
-      <c r="F8" s="43" t="s">
+      <c r="F8" s="41" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="42" t="s">
         <v>102</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="42"/>
+      <c r="F9" s="42"/>
     </row>
     <row r="10" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="C10" s="17">
+      <c r="C10" s="15">
         <v>6800</v>
       </c>
-      <c r="D10" s="17">
+      <c r="D10" s="15">
         <v>6800</v>
       </c>
-      <c r="E10" s="17">
+      <c r="E10" s="15">
         <f>=D10-C10</f>
       </c>
       <c r="F10" s="6" t="s">
@@ -2211,13 +2188,13 @@
       <c r="B11" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="C11" s="17">
+      <c r="C11" s="15">
         <v>2200</v>
       </c>
-      <c r="D11" s="17">
+      <c r="D11" s="15">
         <v>2200</v>
       </c>
-      <c r="E11" s="17">
+      <c r="E11" s="15">
         <f>=D11-C11</f>
       </c>
       <c r="F11" s="6" t="s">
@@ -2228,13 +2205,13 @@
       <c r="B12" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="C12" s="17">
+      <c r="C12" s="15">
         <v>500</v>
       </c>
-      <c r="D12" s="17">
+      <c r="D12" s="15">
         <v>650</v>
       </c>
-      <c r="E12" s="17">
+      <c r="E12" s="15">
         <f>=D12-C12</f>
       </c>
       <c r="F12" s="6" t="s">
@@ -2242,42 +2219,42 @@
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B13" s="44" t="s">
+      <c r="B13" s="43" t="s">
         <v>107</v>
       </c>
-      <c r="C13" s="45">
+      <c r="C13" s="44">
         <f>=SUM(C10:C12)</f>
       </c>
-      <c r="D13" s="45">
+      <c r="D13" s="44">
         <f>=SUM(D10:D12)</f>
       </c>
-      <c r="E13" s="45">
+      <c r="E13" s="44">
         <f>=D13-C13</f>
       </c>
-      <c r="F13" s="44" t="s">
+      <c r="F13" s="43" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="46" t="s">
+      <c r="B14" s="45" t="s">
         <v>109</v>
       </c>
-      <c r="C14" s="46"/>
-      <c r="D14" s="46"/>
-      <c r="E14" s="46"/>
-      <c r="F14" s="46"/>
+      <c r="C14" s="45"/>
+      <c r="D14" s="45"/>
+      <c r="E14" s="45"/>
+      <c r="F14" s="45"/>
     </row>
     <row r="15" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="C15" s="17">
+      <c r="C15" s="15">
         <v>2400</v>
       </c>
-      <c r="D15" s="17">
+      <c r="D15" s="15">
         <v>2400</v>
       </c>
-      <c r="E15" s="17">
+      <c r="E15" s="15">
         <f>=C15-D15</f>
       </c>
       <c r="F15" s="6">
@@ -2288,13 +2265,13 @@
       <c r="B16" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="C16" s="17">
+      <c r="C16" s="15">
         <v>750</v>
       </c>
-      <c r="D16" s="17">
+      <c r="D16" s="15">
         <v>820</v>
       </c>
-      <c r="E16" s="17">
+      <c r="E16" s="15">
         <f>=C16-D16</f>
       </c>
       <c r="F16" s="6">
@@ -2305,13 +2282,13 @@
       <c r="B17" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="C17" s="17">
+      <c r="C17" s="15">
         <v>320</v>
       </c>
-      <c r="D17" s="17">
+      <c r="D17" s="15">
         <v>310</v>
       </c>
-      <c r="E17" s="17">
+      <c r="E17" s="15">
         <f>=C17-D17</f>
       </c>
       <c r="F17" s="6">
@@ -2322,13 +2299,13 @@
       <c r="B18" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="C18" s="17">
+      <c r="C18" s="15">
         <v>450</v>
       </c>
-      <c r="D18" s="17">
+      <c r="D18" s="15">
         <v>450</v>
       </c>
-      <c r="E18" s="17">
+      <c r="E18" s="15">
         <f>=C18-D18</f>
       </c>
       <c r="F18" s="6">
@@ -2339,13 +2316,13 @@
       <c r="B19" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="C19" s="17">
+      <c r="C19" s="15">
         <v>400</v>
       </c>
-      <c r="D19" s="17">
+      <c r="D19" s="15">
         <v>380</v>
       </c>
-      <c r="E19" s="17">
+      <c r="E19" s="15">
         <f>=C19-D19</f>
       </c>
       <c r="F19" s="6">
@@ -2353,42 +2330,42 @@
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B20" s="47" t="s">
+      <c r="B20" s="46" t="s">
         <v>115</v>
       </c>
-      <c r="C20" s="48">
+      <c r="C20" s="47">
         <f>=SUM(C15:C19)</f>
       </c>
-      <c r="D20" s="48">
+      <c r="D20" s="47">
         <f>=SUM(D15:D19)</f>
       </c>
-      <c r="E20" s="48">
+      <c r="E20" s="47">
         <f>=C20-D20</f>
       </c>
-      <c r="F20" s="47">
+      <c r="F20" s="46">
         <f>="Actual: " &amp; TEXT(D20/D13, "0.0%") &amp; " (Target: ≤50%)"</f>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B21" s="49" t="s">
+      <c r="B21" s="48" t="s">
         <v>116</v>
       </c>
-      <c r="C21" s="49"/>
-      <c r="D21" s="49"/>
-      <c r="E21" s="49"/>
-      <c r="F21" s="49"/>
+      <c r="C21" s="48"/>
+      <c r="D21" s="48"/>
+      <c r="E21" s="48"/>
+      <c r="F21" s="48"/>
     </row>
     <row r="22" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="C22" s="17">
+      <c r="C22" s="15">
         <v>650</v>
       </c>
-      <c r="D22" s="17">
+      <c r="D22" s="15">
         <v>520</v>
       </c>
-      <c r="E22" s="17">
+      <c r="E22" s="15">
         <f>=C22-D22</f>
       </c>
       <c r="F22" s="6">
@@ -2399,13 +2376,13 @@
       <c r="B23" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="C23" s="17">
+      <c r="C23" s="15">
         <v>120</v>
       </c>
-      <c r="D23" s="17">
+      <c r="D23" s="15">
         <v>115</v>
       </c>
-      <c r="E23" s="17">
+      <c r="E23" s="15">
         <f>=C23-D23</f>
       </c>
       <c r="F23" s="6">
@@ -2416,13 +2393,13 @@
       <c r="B24" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="C24" s="17">
+      <c r="C24" s="15">
         <v>450</v>
       </c>
-      <c r="D24" s="17">
+      <c r="D24" s="15">
         <v>380</v>
       </c>
-      <c r="E24" s="17">
+      <c r="E24" s="15">
         <f>=C24-D24</f>
       </c>
       <c r="F24" s="6">
@@ -2430,42 +2407,42 @@
       </c>
     </row>
     <row r="25" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B25" s="50" t="s">
+      <c r="B25" s="49" t="s">
         <v>120</v>
       </c>
-      <c r="C25" s="51">
+      <c r="C25" s="50">
         <f>=SUM(C22:C24)</f>
       </c>
-      <c r="D25" s="51">
+      <c r="D25" s="50">
         <f>=SUM(D22:D24)</f>
       </c>
-      <c r="E25" s="51">
+      <c r="E25" s="50">
         <f>=C25-D25</f>
       </c>
-      <c r="F25" s="50">
+      <c r="F25" s="49">
         <f>="Actual: " &amp; TEXT(D25/D13, "0.0%") &amp; " (Target: ≤30%)"</f>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="42" t="s">
         <v>121</v>
       </c>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
+      <c r="C26" s="42"/>
+      <c r="D26" s="42"/>
+      <c r="E26" s="42"/>
+      <c r="F26" s="42"/>
     </row>
     <row r="27" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="C27" s="17">
+      <c r="C27" s="15">
         <v>2200</v>
       </c>
-      <c r="D27" s="17">
+      <c r="D27" s="15">
         <v>2200</v>
       </c>
-      <c r="E27" s="17">
+      <c r="E27" s="15">
         <f>=D27-C27</f>
       </c>
       <c r="F27" s="6">
@@ -2476,13 +2453,13 @@
       <c r="B28" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="C28" s="17">
+      <c r="C28" s="15">
         <v>500</v>
       </c>
-      <c r="D28" s="17">
+      <c r="D28" s="15">
         <v>500</v>
       </c>
-      <c r="E28" s="17">
+      <c r="E28" s="15">
         <f>=D28-C28</f>
       </c>
       <c r="F28" s="6">
@@ -2493,13 +2470,13 @@
       <c r="B29" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="C29" s="17">
+      <c r="C29" s="15">
         <v>600</v>
       </c>
-      <c r="D29" s="17">
+      <c r="D29" s="15">
         <v>750</v>
       </c>
-      <c r="E29" s="17">
+      <c r="E29" s="15">
         <f>=D29-C29</f>
       </c>
       <c r="F29" s="6">
@@ -2507,19 +2484,19 @@
       </c>
     </row>
     <row r="30" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B30" s="52" t="s">
+      <c r="B30" s="51" t="s">
         <v>125</v>
       </c>
-      <c r="C30" s="53">
+      <c r="C30" s="52">
         <f>=SUM(C27:C29)</f>
       </c>
-      <c r="D30" s="53">
+      <c r="D30" s="52">
         <f>=SUM(D27:D29)</f>
       </c>
-      <c r="E30" s="53">
+      <c r="E30" s="52">
         <f>=D30-C30</f>
       </c>
-      <c r="F30" s="52">
+      <c r="F30" s="51">
         <f>="Savings Rate: " &amp; TEXT(D30/D13, "0.0%") &amp; " (FIRE Speed)"</f>
       </c>
     </row>
@@ -2554,47 +2531,47 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="54" t="s">
+      <c r="B2" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
     </row>
     <row r="5" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B5" s="43" t="s">
+      <c r="B5" s="41" t="s">
         <v>128</v>
       </c>
-      <c r="C5" s="43" t="s">
+      <c r="C5" s="41" t="s">
         <v>129</v>
       </c>
-      <c r="D5" s="43" t="s">
+      <c r="D5" s="41" t="s">
         <v>130</v>
       </c>
-      <c r="E5" s="43" t="s">
+      <c r="E5" s="41" t="s">
         <v>131</v>
       </c>
-      <c r="F5" s="43" t="s">
+      <c r="F5" s="41" t="s">
         <v>132</v>
       </c>
-      <c r="G5" s="43" t="s">
+      <c r="G5" s="41" t="s">
         <v>133</v>
       </c>
-      <c r="H5" s="43" t="s">
+      <c r="H5" s="41" t="s">
         <v>134</v>
       </c>
     </row>
@@ -2602,45 +2579,45 @@
       <c r="B6" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="C6" s="17">
+      <c r="C6" s="15">
         <v>25000</v>
       </c>
-      <c r="D6" s="17">
+      <c r="D6" s="15">
         <v>21500</v>
       </c>
-      <c r="E6" s="17">
+      <c r="E6" s="15">
         <f>=C6-D6</f>
       </c>
       <c r="F6" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="G6" s="17">
+      <c r="G6" s="15">
         <v>700</v>
       </c>
-      <c r="H6" s="55">
+      <c r="H6" s="53">
         <f>=D6/C6</f>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B7" s="37" t="s">
+      <c r="B7" s="36" t="s">
         <v>136</v>
       </c>
-      <c r="C7" s="22">
+      <c r="C7" s="20">
         <v>2000</v>
       </c>
-      <c r="D7" s="22">
+      <c r="D7" s="20">
         <v>1400</v>
       </c>
-      <c r="E7" s="22">
+      <c r="E7" s="20">
         <f>=C7-D7</f>
       </c>
-      <c r="F7" s="37" t="s">
+      <c r="F7" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="G7" s="22">
+      <c r="G7" s="20">
         <v>150</v>
       </c>
-      <c r="H7" s="56">
+      <c r="H7" s="54">
         <f>=D7/C7</f>
       </c>
     </row>
@@ -2648,45 +2625,45 @@
       <c r="B8" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="C8" s="17">
+      <c r="C8" s="15">
         <v>4500</v>
       </c>
-      <c r="D8" s="17">
+      <c r="D8" s="15">
         <v>2800</v>
       </c>
-      <c r="E8" s="17">
+      <c r="E8" s="15">
         <f>=C8-D8</f>
       </c>
       <c r="F8" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="G8" s="17">
+      <c r="G8" s="15">
         <v>250</v>
       </c>
-      <c r="H8" s="55">
+      <c r="H8" s="53">
         <f>=D8/C8</f>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="37" t="s">
+      <c r="B9" s="36" t="s">
         <v>138</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="20">
         <v>1500</v>
       </c>
-      <c r="D9" s="22">
+      <c r="D9" s="20">
         <v>750</v>
       </c>
-      <c r="E9" s="22">
+      <c r="E9" s="20">
         <f>=C9-D9</f>
       </c>
-      <c r="F9" s="37" t="s">
+      <c r="F9" s="36" t="s">
         <v>58</v>
       </c>
-      <c r="G9" s="22">
+      <c r="G9" s="20">
         <v>125</v>
       </c>
-      <c r="H9" s="56">
+      <c r="H9" s="54">
         <f>=D9/C9</f>
       </c>
     </row>
@@ -2694,45 +2671,45 @@
       <c r="B10" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="C10" s="17">
+      <c r="C10" s="15">
         <v>3500</v>
       </c>
-      <c r="D10" s="17">
+      <c r="D10" s="15">
         <v>1800</v>
       </c>
-      <c r="E10" s="17">
+      <c r="E10" s="15">
         <f>=C10-D10</f>
       </c>
       <c r="F10" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="G10" s="17">
+      <c r="G10" s="15">
         <v>250</v>
       </c>
-      <c r="H10" s="55">
+      <c r="H10" s="53">
         <f>=D10/C10</f>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="25" t="s">
+      <c r="B11" s="23" t="s">
         <v>140</v>
       </c>
-      <c r="C11" s="26">
+      <c r="C11" s="24">
         <f>=SUM(C6:C10)</f>
       </c>
-      <c r="D11" s="26">
+      <c r="D11" s="24">
         <f>=SUM(D6:D10)</f>
       </c>
-      <c r="E11" s="26">
+      <c r="E11" s="24">
         <f>=SUM(E6:E10)</f>
       </c>
-      <c r="F11" s="25" t="s">
+      <c r="F11" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="G11" s="26">
+      <c r="G11" s="24">
         <f>=SUM(G6:G10)</f>
       </c>
-      <c r="H11" s="57">
+      <c r="H11" s="55">
         <f>=D11/C11</f>
       </c>
     </row>
@@ -2760,26 +2737,26 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B2" s="40" t="s">
+      <c r="B2" s="56" t="s">
         <v>142</v>
       </c>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
     </row>
     <row r="5" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B5" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="C5" s="58">
+      <c r="C5" s="57">
         <v>32</v>
       </c>
     </row>
@@ -2787,7 +2764,7 @@
       <c r="B6" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="C6" s="59">
+      <c r="C6" s="58">
         <v>66000</v>
       </c>
     </row>
@@ -2795,7 +2772,7 @@
       <c r="B7" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="C7" s="60">
+      <c r="C7" s="59">
         <v>0.04</v>
       </c>
     </row>
@@ -2803,7 +2780,7 @@
       <c r="B8" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="C8" s="60">
+      <c r="C8" s="59">
         <v>0.07</v>
       </c>
     </row>
@@ -2811,7 +2788,7 @@
       <c r="B9" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="C9" s="59">
+      <c r="C9" s="58">
         <f>'⚡ 2-Min Quick Check-In'!D18</f>
       </c>
     </row>
@@ -2819,26 +2796,26 @@
       <c r="B10" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="C10" s="59">
+      <c r="C10" s="58">
         <f>'💸 Smart Budget (50-30-20)'!D27</f>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="42" t="s">
         <v>150</v>
       </c>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
+      <c r="C12" s="42"/>
+      <c r="D12" s="42"/>
+      <c r="E12" s="42"/>
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="C13" s="59">
+      <c r="C13" s="58">
         <f>C6*0.65/C7</f>
       </c>
-      <c r="D13" s="61" t="s">
+      <c r="D13" s="60" t="s">
         <v>152</v>
       </c>
     </row>
@@ -2846,10 +2823,10 @@
       <c r="B14" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="C14" s="59">
+      <c r="C14" s="58">
         <f>C6/C7</f>
       </c>
-      <c r="D14" s="61" t="s">
+      <c r="D14" s="60" t="s">
         <v>154</v>
       </c>
     </row>
@@ -2857,10 +2834,10 @@
       <c r="B15" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="C15" s="59">
+      <c r="C15" s="58">
         <f>C6*1.4/C7</f>
       </c>
-      <c r="D15" s="61" t="s">
+      <c r="D15" s="60" t="s">
         <v>156</v>
       </c>
     </row>
@@ -2868,10 +2845,10 @@
       <c r="B16" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="C16" s="59">
+      <c r="C16" s="58">
         <f>(C6/C7)/(1+C8)^(60-C5)</f>
       </c>
-      <c r="D16" s="61" t="s">
+      <c r="D16" s="60" t="s">
         <v>158</v>
       </c>
     </row>
@@ -2901,28 +2878,28 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="62" t="s">
+      <c r="B2" s="56" t="s">
         <v>159</v>
       </c>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
     </row>
     <row r="4" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="35" t="s">
         <v>160</v>
       </c>
-      <c r="C4" s="36" t="s">
+      <c r="C4" s="35" t="s">
         <v>130</v>
       </c>
-      <c r="D4" s="36" t="s">
+      <c r="D4" s="35" t="s">
         <v>161</v>
       </c>
-      <c r="E4" s="36" t="s">
+      <c r="E4" s="35" t="s">
         <v>162</v>
       </c>
-      <c r="F4" s="36" t="s">
+      <c r="F4" s="35" t="s">
         <v>163</v>
       </c>
     </row>
@@ -2930,13 +2907,13 @@
       <c r="B5" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="C5" s="17">
+      <c r="C5" s="15">
         <v>4200</v>
       </c>
-      <c r="D5" s="63">
+      <c r="D5" s="61">
         <v>0.2499</v>
       </c>
-      <c r="E5" s="17">
+      <c r="E5" s="15">
         <v>140</v>
       </c>
       <c r="F5" s="6" t="s">
@@ -2947,13 +2924,13 @@
       <c r="B6" s="6" t="s">
         <v>166</v>
       </c>
-      <c r="C6" s="17">
+      <c r="C6" s="15">
         <v>8500</v>
       </c>
-      <c r="D6" s="63">
+      <c r="D6" s="61">
         <v>0.115</v>
       </c>
-      <c r="E6" s="17">
+      <c r="E6" s="15">
         <v>210</v>
       </c>
       <c r="F6" s="6" t="s">
@@ -2964,13 +2941,13 @@
       <c r="B7" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="C7" s="17">
+      <c r="C7" s="15">
         <v>17400</v>
       </c>
-      <c r="D7" s="63">
+      <c r="D7" s="61">
         <v>0.059</v>
       </c>
-      <c r="E7" s="17">
+      <c r="E7" s="15">
         <v>380</v>
       </c>
       <c r="F7" s="6" t="s">
@@ -2981,13 +2958,13 @@
       <c r="B8" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="C8" s="17">
+      <c r="C8" s="15">
         <v>200000</v>
       </c>
-      <c r="D8" s="63">
+      <c r="D8" s="61">
         <v>0.035</v>
       </c>
-      <c r="E8" s="17">
+      <c r="E8" s="15">
         <v>1670</v>
       </c>
       <c r="F8" s="6" t="s">
@@ -2995,19 +2972,19 @@
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="44" t="s">
+      <c r="B9" s="43" t="s">
         <v>172</v>
       </c>
-      <c r="C9" s="45">
+      <c r="C9" s="44">
         <f>=SUM(C5:C8)</f>
       </c>
-      <c r="D9" s="64">
+      <c r="D9" s="62">
         <f>=AVERAGE(D5:D8)</f>
       </c>
-      <c r="E9" s="45">
+      <c r="E9" s="44">
         <f>=SUM(E5:E8)</f>
       </c>
-      <c r="F9" s="44" t="s">
+      <c r="F9" s="43" t="s">
         <v>173</v>
       </c>
     </row>
@@ -3032,36 +3009,36 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="62" t="s">
+      <c r="B2" s="56" t="s">
         <v>174</v>
       </c>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
     </row>
     <row r="4" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="35" t="s">
         <v>175</v>
       </c>
-      <c r="C4" s="36" t="s">
+      <c r="C4" s="35" t="s">
         <v>176</v>
       </c>
-      <c r="D4" s="36" t="s">
+      <c r="D4" s="35" t="s">
         <v>177</v>
       </c>
-      <c r="E4" s="36" t="s">
+      <c r="E4" s="35" t="s">
         <v>178</v>
       </c>
-      <c r="F4" s="36" t="s">
+      <c r="F4" s="35" t="s">
         <v>179</v>
       </c>
-      <c r="G4" s="36" t="s">
+      <c r="G4" s="35" t="s">
         <v>180</v>
       </c>
-      <c r="H4" s="36" t="s">
+      <c r="H4" s="35" t="s">
         <v>181</v>
       </c>
     </row>
@@ -3069,45 +3046,45 @@
       <c r="B5" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="C5" s="17">
+      <c r="C5" s="15">
         <v>4800</v>
       </c>
-      <c r="D5" s="17">
+      <c r="D5" s="15">
         <v>39000</v>
       </c>
-      <c r="E5" s="17">
+      <c r="E5" s="15">
         <v>145000</v>
       </c>
-      <c r="F5" s="17">
+      <c r="F5" s="15">
         <v>380000</v>
       </c>
-      <c r="G5" s="17">
+      <c r="G5" s="15">
         <v>750000</v>
       </c>
-      <c r="H5" s="17">
+      <c r="H5" s="15">
         <v>2800000</v>
       </c>
     </row>
     <row r="6" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="36" t="s">
         <v>183</v>
       </c>
-      <c r="C6" s="22">
+      <c r="C6" s="20">
         <v>35000</v>
       </c>
-      <c r="D6" s="22">
+      <c r="D6" s="20">
         <v>135600</v>
       </c>
-      <c r="E6" s="22">
+      <c r="E6" s="20">
         <v>420000</v>
       </c>
-      <c r="F6" s="22">
+      <c r="F6" s="20">
         <v>980000</v>
       </c>
-      <c r="G6" s="22">
+      <c r="G6" s="20">
         <v>1850000</v>
       </c>
-      <c r="H6" s="22">
+      <c r="H6" s="20">
         <v>5500000</v>
       </c>
     </row>
@@ -3115,45 +3092,45 @@
       <c r="B7" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="C7" s="17">
+      <c r="C7" s="15">
         <v>68000</v>
       </c>
-      <c r="D7" s="17">
+      <c r="D7" s="15">
         <v>247200</v>
       </c>
-      <c r="E7" s="17">
+      <c r="E7" s="15">
         <v>780000</v>
       </c>
-      <c r="F7" s="17">
+      <c r="F7" s="15">
         <v>1950000</v>
       </c>
-      <c r="G7" s="17">
+      <c r="G7" s="15">
         <v>3400000</v>
       </c>
-      <c r="H7" s="17">
+      <c r="H7" s="15">
         <v>10200000</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="37" t="s">
+      <c r="B8" s="36" t="s">
         <v>185</v>
       </c>
-      <c r="C8" s="22">
+      <c r="C8" s="20">
         <v>95000</v>
       </c>
-      <c r="D8" s="22">
+      <c r="D8" s="20">
         <v>364500</v>
       </c>
-      <c r="E8" s="22">
+      <c r="E8" s="20">
         <v>1150000</v>
       </c>
-      <c r="F8" s="22">
+      <c r="F8" s="20">
         <v>2800000</v>
       </c>
-      <c r="G8" s="22">
+      <c r="G8" s="20">
         <v>4900000</v>
       </c>
-      <c r="H8" s="22">
+      <c r="H8" s="20">
         <v>14500000</v>
       </c>
     </row>
@@ -3161,45 +3138,45 @@
       <c r="B9" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="C9" s="17">
+      <c r="C9" s="15">
         <v>110000</v>
       </c>
-      <c r="D9" s="17">
+      <c r="D9" s="15">
         <v>409900</v>
       </c>
-      <c r="E9" s="17">
+      <c r="E9" s="15">
         <v>1350000</v>
       </c>
-      <c r="F9" s="17">
+      <c r="F9" s="15">
         <v>3200000</v>
       </c>
-      <c r="G9" s="17">
+      <c r="G9" s="15">
         <v>5600000</v>
       </c>
-      <c r="H9" s="17">
+      <c r="H9" s="15">
         <v>16800000</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="37" t="s">
+      <c r="B10" s="36" t="s">
         <v>187</v>
       </c>
-      <c r="C10" s="22">
+      <c r="C10" s="20">
         <v>92000</v>
       </c>
-      <c r="D10" s="22">
+      <c r="D10" s="20">
         <v>335600</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="20">
         <v>1050000</v>
       </c>
-      <c r="F10" s="22">
+      <c r="F10" s="20">
         <v>2600000</v>
       </c>
-      <c r="G10" s="22">
+      <c r="G10" s="20">
         <v>4700000</v>
       </c>
-      <c r="H10" s="22">
+      <c r="H10" s="20">
         <v>13200000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(vault): integrate website signatures (PAW engine, 50 states, liquid net worth) and enforce institutional identity on vault
</commit_message>
<xml_diff>
--- a/public/downloads/NetWorth_FIRE_Master_Vault_2026.xlsx
+++ b/public/downloads/NetWorth_FIRE_Master_Vault_2026.xlsx
@@ -11,19 +11,19 @@
     <sheet sheetId="5" name="🎯 Sinking Funds Shield" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="🔥 FIRE Freedom Engine" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="💳 Debt Avalanche &amp; Snowball" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="🏛️ Fed Benchmarks (SCF)" state="visible" r:id="rId11"/>
+    <sheet sheetId="8" name="🏛️ Fed &amp; State Benchmarks" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="281">
   <si>
     <t>🏛️ GETNETWORTHCALCULATOR.COM • OFFICIAL WEALTH &amp; BUDGET OPERATING SYSTEM</t>
   </si>
   <si>
-    <t>Researched &amp; Modeled by Yash Jha | Benchmarked Against US Federal Reserve SCF Microdata (2026)</t>
+    <t>Modeled by GetNetWorth Analytics | Benchmarked Against US Federal Reserve SCF Microdata (2026)</t>
   </si>
   <si>
     <t>🚀 THE 3-STEP MONTHLY ROUTINE (TAKES 2 MINUTES ON THE 1ST OF EACH MONTH)</t>
@@ -98,7 +98,7 @@
     <t>📊 Executive Dashboard</t>
   </si>
   <si>
-    <t>Bloomberg-style visual terminal showing Net Worth, Fed rank, and quarterly progress.</t>
+    <t>Bloomberg-style visual terminal with Stanley &amp; Danko Wealth Class (PAW/UAW) Engine.</t>
   </si>
   <si>
     <t>💸 Smart Budget (50/30/20)</t>
@@ -125,19 +125,19 @@
     <t>Side-by-side Avalanche (interest saver) vs Snowball (momentum builder) payoff rank.</t>
   </si>
   <si>
-    <t>🏛️ Fed Benchmarks (SCF)</t>
-  </si>
-  <si>
-    <t>Official US Federal Reserve Survey of Consumer Finances raw microdata tables.</t>
-  </si>
-  <si>
-    <t>🌐 GetNetWorthCalculator.com • 100% Private, Anonymous &amp; Offline • Curated by Yash Jha</t>
+    <t>🏛️ Fed &amp; State Benchmarks</t>
+  </si>
+  <si>
+    <t>Official US Federal Reserve SCF microdata + 50 US States Median Wealth Index.</t>
+  </si>
+  <si>
+    <t>🌐 GetNetWorthCalculator.com • 100% Private, Anonymous &amp; Offline • Official 2026 Edition</t>
   </si>
   <si>
     <t>⚡ 2-MINUTE MONTHLY QUICK CHECK-IN • GETNETWORTHCALCULATOR.COM</t>
   </si>
   <si>
-    <t>Rule of Thumb: On the 1st of each month, type just 4 numbers (green headers). Everything else calculates automatically.</t>
+    <t>Rule of Thumb: On the 1st of each month, type just 4 numbers (green headers). Net Worth, Liquid Ratio &amp; Deltas compute automatically.</t>
   </si>
   <si>
     <t>Month</t>
@@ -155,7 +155,7 @@
     <t>💳 Total Debts</t>
   </si>
   <si>
-    <t>🏛️ NET WORTH</t>
+    <t>🏛️ TOTAL NET WORTH</t>
   </si>
   <si>
     <t>MoM Gain ($)</t>
@@ -164,6 +164,12 @@
     <t>MoM Growth (%)</t>
   </si>
   <si>
+    <t>💧 LIQUID NET WORTH</t>
+  </si>
+  <si>
+    <t>Liquid Ratio (%)</t>
+  </si>
+  <si>
     <t>Jan 2026</t>
   </si>
   <si>
@@ -299,6 +305,90 @@
     <t>October 2038</t>
   </si>
   <si>
+    <t>🏆 STANLEY &amp; DANKO WEALTH ACCUMULATION CLASS (PAW / AAW / UAW ENGINE)</t>
+  </si>
+  <si>
+    <t>Your Age (Green Input)</t>
+  </si>
+  <si>
+    <t>Pre-Tax Income (Green Input)</t>
+  </si>
+  <si>
+    <t>Expected NW (Age×Income/10)</t>
+  </si>
+  <si>
+    <t>Accumulation Multiplier</t>
+  </si>
+  <si>
+    <t>Wealth Class Status</t>
+  </si>
+  <si>
+    <t>🎯 WEALTH ACCELERATION MILESTONES (CHARLIE MUNGER COMPOUNDING CURVE)</t>
+  </si>
+  <si>
+    <t>Milestone Tier</t>
+  </si>
+  <si>
+    <t>Target ($)</t>
+  </si>
+  <si>
+    <t>Progress (%)</t>
+  </si>
+  <si>
+    <t>Remaining Gap ($)</t>
+  </si>
+  <si>
+    <t>Compounding Dynamics &amp; Insights</t>
+  </si>
+  <si>
+    <t>$100,000 (Base Foundation)</t>
+  </si>
+  <si>
+    <t>The hardest milestone — 100% savings driven (Charlie Munger rule)</t>
+  </si>
+  <si>
+    <t>$250,000 (Tipping Point)</t>
+  </si>
+  <si>
+    <t>Compounding returns begin matching your monthly cash savings</t>
+  </si>
+  <si>
+    <t>$500,000 (Half-Million)</t>
+  </si>
+  <si>
+    <t>Investment gains frequently exceed annual take-home salary</t>
+  </si>
+  <si>
+    <t>$1,000,000 (Two-Comma Club)</t>
+  </si>
+  <si>
+    <t>Top 7% of US households — Full Financial Sovereignty</t>
+  </si>
+  <si>
+    <t>💧 LIQUID NET WORTH &amp; EMERGENCY RUNWAY SHIELD • GETNETWORTHCALCULATOR.COM</t>
+  </si>
+  <si>
+    <t>Liquid Assets (Cash+Invested)</t>
+  </si>
+  <si>
+    <t>Monthly Baseline Needs</t>
+  </si>
+  <si>
+    <t>Emergency Runway (Months)</t>
+  </si>
+  <si>
+    <t>Liquid to Total NW Ratio</t>
+  </si>
+  <si>
+    <t>Safe Liquidity Benchmark</t>
+  </si>
+  <si>
+    <t>3-6 Mo for W2 • 12+ Mo for 1099/FIRE</t>
+  </si>
+  <si>
+    <t>🌐 LIVE TOOLS ON GETNETWORTHCALCULATOR.COM: /wealth-class-calculator • /liquid-net-worth-calculator • /state • /coast-fire</t>
+  </si>
+  <si>
     <t>💸 SMART MONTHLY CASH FLOW &amp; 50/30/20 BUDGET • GETNETWORTHCALCULATOR.COM</t>
   </si>
   <si>
@@ -582,20 +672,212 @@
   </si>
   <si>
     <t>75+</t>
+  </si>
+  <si>
+    <t>📍 TOP 10 US STATES WEALTH &amp; COST-OF-LIVING INDEX • GETNETWORTHCALCULATOR.COM/STATE</t>
+  </si>
+  <si>
+    <t>US State</t>
+  </si>
+  <si>
+    <t>Median NW</t>
+  </si>
+  <si>
+    <t>Top 10% NW</t>
+  </si>
+  <si>
+    <t>COL Index</t>
+  </si>
+  <si>
+    <t>Median Home</t>
+  </si>
+  <si>
+    <t>Wealth Tier</t>
+  </si>
+  <si>
+    <t>Website State Hub</t>
+  </si>
+  <si>
+    <t>California (CA)</t>
+  </si>
+  <si>
+    <t>138.5 (HCOL)</t>
+  </si>
+  <si>
+    <t>Top Tier</t>
+  </si>
+  <si>
+    <t>getnetworthcalculator.com/state/california</t>
+  </si>
+  <si>
+    <t>New York (NY)</t>
+  </si>
+  <si>
+    <t>134.2 (HCOL)</t>
+  </si>
+  <si>
+    <t>getnetworthcalculator.com/state/new-york</t>
+  </si>
+  <si>
+    <t>Washington (WA)</t>
+  </si>
+  <si>
+    <t>115.1 (MCOL+)</t>
+  </si>
+  <si>
+    <t>getnetworthcalculator.com/state/washington</t>
+  </si>
+  <si>
+    <t>Texas (TX)</t>
+  </si>
+  <si>
+    <t>92.5 (LCOL)</t>
+  </si>
+  <si>
+    <t>High Value</t>
+  </si>
+  <si>
+    <t>getnetworthcalculator.com/state/texas</t>
+  </si>
+  <si>
+    <t>Florida (FL)</t>
+  </si>
+  <si>
+    <t>102.8 (Avg)</t>
+  </si>
+  <si>
+    <t>Growing</t>
+  </si>
+  <si>
+    <t>getnetworthcalculator.com/state/florida</t>
+  </si>
+  <si>
+    <t>Massachusetts (MA)</t>
+  </si>
+  <si>
+    <t>148.0 (HCOL)</t>
+  </si>
+  <si>
+    <t>getnetworthcalculator.com/state/massachusetts</t>
+  </si>
+  <si>
+    <t>Illinois (IL)</t>
+  </si>
+  <si>
+    <t>91.8 (LCOL)</t>
+  </si>
+  <si>
+    <t>getnetworthcalculator.com/state/illinois</t>
+  </si>
+  <si>
+    <t>Colorado (CO)</t>
+  </si>
+  <si>
+    <t>105.4 (Avg)</t>
+  </si>
+  <si>
+    <t>High Growth</t>
+  </si>
+  <si>
+    <t>getnetworthcalculator.com/state/colorado</t>
+  </si>
+  <si>
+    <t>📊 FIDELITY RETIREMENT SAVINGS BENCHMARKS BY AGE • GETNETWORTHCALCULATOR.COM</t>
+  </si>
+  <si>
+    <t>Age Milestone</t>
+  </si>
+  <si>
+    <t>Salary Multiplier</t>
+  </si>
+  <si>
+    <t>Target ($100k Sal)</t>
+  </si>
+  <si>
+    <t>Target ($150k Sal)</t>
+  </si>
+  <si>
+    <t>Fidelity Rule of Thumb</t>
+  </si>
+  <si>
+    <t>Online Calculator Tool</t>
+  </si>
+  <si>
+    <t>Website Hub</t>
+  </si>
+  <si>
+    <t>Age 30</t>
+  </si>
+  <si>
+    <t>Have 1x annual salary saved in invested portfolio</t>
+  </si>
+  <si>
+    <t>savings-multiplier-by-age</t>
+  </si>
+  <si>
+    <t>getnetworthcalculator.com</t>
+  </si>
+  <si>
+    <t>Age 35</t>
+  </si>
+  <si>
+    <t>Have 2x annual salary saved (tipping point)</t>
+  </si>
+  <si>
+    <t>Age 40</t>
+  </si>
+  <si>
+    <t>Have 3x annual salary saved</t>
+  </si>
+  <si>
+    <t>Age 45</t>
+  </si>
+  <si>
+    <t>Have 4x annual salary saved</t>
+  </si>
+  <si>
+    <t>Age 50</t>
+  </si>
+  <si>
+    <t>Have 6x annual salary saved</t>
+  </si>
+  <si>
+    <t>Age 55</t>
+  </si>
+  <si>
+    <t>Have 7x annual salary saved</t>
+  </si>
+  <si>
+    <t>Age 60</t>
+  </si>
+  <si>
+    <t>Have 8x annual salary saved</t>
+  </si>
+  <si>
+    <t>Age 67</t>
+  </si>
+  <si>
+    <t>Full retirement baseline target (10x income)</t>
+  </si>
+  <si>
+    <t>🌐 Explore live interactive tools: getnetworthcalculator.com/savings-multiplier-by-age • /wealth-class-calculator • /state</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="5">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="+$#,##0;-$#,##0;$0"/>
     <numFmt numFmtId="166" formatCode="+0.0%;-0.0%;0.0%"/>
-    <numFmt numFmtId="167" formatCode="$#,##0/day"/>
-    <numFmt numFmtId="168" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="169" formatCode="0.0&quot; Months&quot;"/>
+    <numFmt numFmtId="170" formatCode="$#,##0/day"/>
+    <numFmt numFmtId="171" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="35" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -642,7 +924,7 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
+      <sz val="9.5"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -653,6 +935,12 @@
     <font>
       <b/>
       <color rgb="FF065F46"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF10B981"/>
       <sz val="10"/>
       <name val="Arial"/>
     </font>
@@ -718,6 +1006,36 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF10B981"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="FF475569"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFF59E0B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <color rgb="FF10B981"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="15"/>
     </font>
     <font>
@@ -730,6 +1048,12 @@
       <i/>
       <color rgb="FF64748B"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="9">
@@ -802,7 +1126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -836,64 +1160,103 @@
     <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="17" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="23" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="167" fontId="24" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="27" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="19" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="19" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="28" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="26" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="27" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="26" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="29" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="170" fontId="31" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="12" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="13" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="12" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="13" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="171" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1437,7 +1800,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:I18"/>
+  <dimension ref="B2:K18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1448,10 +1811,12 @@
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="20" customWidth="1"/>
     <col min="8" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="4" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" ht="28" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="2" ht="28" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>38</v>
       </c>
@@ -1462,8 +1827,10 @@
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
-    </row>
-    <row r="3" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="11" t="s">
         <v>39</v>
       </c>
@@ -1474,8 +1841,10 @@
       <c r="G3" s="11"/>
       <c r="H3" s="11"/>
       <c r="I3" s="11"/>
-    </row>
-    <row r="5" ht="24" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
+    </row>
+    <row r="5" ht="24" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" s="12" t="s">
         <v>40</v>
       </c>
@@ -1500,10 +1869,16 @@
       <c r="I5" s="12" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="J5" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="K5" s="12" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C6" s="15">
         <v>25000</v>
@@ -1526,36 +1901,48 @@
       <c r="I6" s="18">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="C7" s="20">
+      <c r="J6" s="19">
+        <f>=C6+D6</f>
+      </c>
+      <c r="K6" s="20">
+        <f>=(C6+D6)/G6</f>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B7" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="22">
         <v>26200</v>
       </c>
-      <c r="D7" s="20">
+      <c r="D7" s="22">
         <v>189500</v>
       </c>
-      <c r="E7" s="20">
+      <c r="E7" s="22">
         <v>350000</v>
       </c>
-      <c r="F7" s="20">
+      <c r="F7" s="22">
         <v>243800</v>
       </c>
       <c r="G7" s="16">
         <f>=(C7+D7+E7)-F7</f>
       </c>
-      <c r="H7" s="21">
+      <c r="H7" s="23">
         <f>=G7-G6</f>
       </c>
-      <c r="I7" s="22">
+      <c r="I7" s="24">
         <f>=(G7-G6)/G6</f>
       </c>
-    </row>
-    <row r="8" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="J7" s="19">
+        <f>=C7+D7</f>
+      </c>
+      <c r="K7" s="25">
+        <f>=(C7+D7)/G7</f>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B8" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C8" s="15">
         <v>25800</v>
@@ -1578,36 +1965,48 @@
       <c r="I8" s="18">
         <f>=(G8-G7)/G7</f>
       </c>
-    </row>
-    <row r="9" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B9" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="C9" s="20">
+      <c r="J8" s="19">
+        <f>=C8+D8</f>
+      </c>
+      <c r="K8" s="20">
+        <f>=(C8+D8)/G8</f>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B9" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" s="22">
         <v>27100</v>
       </c>
-      <c r="D9" s="20">
+      <c r="D9" s="22">
         <v>191000</v>
       </c>
-      <c r="E9" s="20">
+      <c r="E9" s="22">
         <v>350000</v>
       </c>
-      <c r="F9" s="20">
+      <c r="F9" s="22">
         <v>241400</v>
       </c>
       <c r="G9" s="16">
         <f>=(C9+D9+E9)-F9</f>
       </c>
-      <c r="H9" s="21">
+      <c r="H9" s="23">
         <f>=G9-G8</f>
       </c>
-      <c r="I9" s="22">
+      <c r="I9" s="24">
         <f>=(G9-G8)/G8</f>
       </c>
-    </row>
-    <row r="10" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="J9" s="19">
+        <f>=C9+D9</f>
+      </c>
+      <c r="K9" s="25">
+        <f>=(C9+D9)/G9</f>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B10" s="14" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C10" s="15">
         <v>26900</v>
@@ -1630,36 +2029,48 @@
       <c r="I10" s="18">
         <f>=(G10-G9)/G9</f>
       </c>
-    </row>
-    <row r="11" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B11" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="C11" s="20">
+      <c r="J10" s="19">
+        <f>=C10+D10</f>
+      </c>
+      <c r="K10" s="20">
+        <f>=(C10+D10)/G10</f>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B11" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="C11" s="22">
         <v>28400</v>
       </c>
-      <c r="D11" s="20">
+      <c r="D11" s="22">
         <v>204000</v>
       </c>
-      <c r="E11" s="20">
+      <c r="E11" s="22">
         <v>352000</v>
       </c>
-      <c r="F11" s="20">
+      <c r="F11" s="22">
         <v>238800</v>
       </c>
       <c r="G11" s="16">
         <f>=(C11+D11+E11)-F11</f>
       </c>
-      <c r="H11" s="21">
+      <c r="H11" s="23">
         <f>=G11-G10</f>
       </c>
-      <c r="I11" s="22">
+      <c r="I11" s="24">
         <f>=(G11-G10)/G10</f>
       </c>
-    </row>
-    <row r="12" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="J11" s="19">
+        <f>=C11+D11</f>
+      </c>
+      <c r="K11" s="25">
+        <f>=(C11+D11)/G11</f>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B12" s="14" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C12" s="15">
         <v>29000</v>
@@ -1682,36 +2093,48 @@
       <c r="I12" s="18">
         <f>=(G12-G11)/G11</f>
       </c>
-    </row>
-    <row r="13" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B13" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="C13" s="20">
+      <c r="J12" s="19">
+        <f>=C12+D12</f>
+      </c>
+      <c r="K12" s="20">
+        <f>=(C12+D12)/G12</f>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B13" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="C13" s="22">
         <v>28500</v>
       </c>
-      <c r="D13" s="20">
+      <c r="D13" s="22">
         <v>215000</v>
       </c>
-      <c r="E13" s="20">
+      <c r="E13" s="22">
         <v>355000</v>
       </c>
-      <c r="F13" s="20">
+      <c r="F13" s="22">
         <v>236100</v>
       </c>
       <c r="G13" s="16">
         <f>=(C13+D13+E13)-F13</f>
       </c>
-      <c r="H13" s="21">
+      <c r="H13" s="23">
         <f>=G13-G12</f>
       </c>
-      <c r="I13" s="22">
+      <c r="I13" s="24">
         <f>=(G13-G12)/G12</f>
       </c>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="J13" s="19">
+        <f>=C13+D13</f>
+      </c>
+      <c r="K13" s="25">
+        <f>=(C13+D13)/G13</f>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B14" s="14" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C14" s="15">
         <v>30200</v>
@@ -1734,36 +2157,48 @@
       <c r="I14" s="18">
         <f>=(G14-G13)/G13</f>
       </c>
-    </row>
-    <row r="15" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B15" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="C15" s="20">
+      <c r="J14" s="19">
+        <f>=C14+D14</f>
+      </c>
+      <c r="K14" s="20">
+        <f>=(C14+D14)/G14</f>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B15" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" s="22">
         <v>31000</v>
       </c>
-      <c r="D15" s="20">
+      <c r="D15" s="22">
         <v>228000</v>
       </c>
-      <c r="E15" s="20">
+      <c r="E15" s="22">
         <v>355000</v>
       </c>
-      <c r="F15" s="20">
+      <c r="F15" s="22">
         <v>233200</v>
       </c>
       <c r="G15" s="16">
         <f>=(C15+D15+E15)-F15</f>
       </c>
-      <c r="H15" s="21">
+      <c r="H15" s="23">
         <f>=G15-G14</f>
       </c>
-      <c r="I15" s="22">
+      <c r="I15" s="24">
         <f>=(G15-G14)/G14</f>
       </c>
-    </row>
-    <row r="16" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="J15" s="19">
+        <f>=C15+D15</f>
+      </c>
+      <c r="K15" s="25">
+        <f>=(C15+D15)/G15</f>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B16" s="14" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C16" s="15">
         <v>31500</v>
@@ -1786,63 +2221,81 @@
       <c r="I16" s="18">
         <f>=(G16-G15)/G15</f>
       </c>
-    </row>
-    <row r="17" ht="20" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B17" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="C17" s="20">
+      <c r="J16" s="19">
+        <f>=C16+D16</f>
+      </c>
+      <c r="K16" s="20">
+        <f>=(C16+D16)/G16</f>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B17" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" s="22">
         <v>33000</v>
       </c>
-      <c r="D17" s="20">
+      <c r="D17" s="22">
         <v>242000</v>
       </c>
-      <c r="E17" s="20">
+      <c r="E17" s="22">
         <v>358000</v>
       </c>
-      <c r="F17" s="20">
+      <c r="F17" s="22">
         <v>230100</v>
       </c>
       <c r="G17" s="16">
         <f>=(C17+D17+E17)-F17</f>
       </c>
-      <c r="H17" s="21">
+      <c r="H17" s="23">
         <f>=G17-G16</f>
       </c>
-      <c r="I17" s="22">
+      <c r="I17" s="24">
         <f>=(G17-G16)/G16</f>
       </c>
-    </row>
-    <row r="18" ht="22" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B18" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="C18" s="24">
+      <c r="J17" s="19">
+        <f>=C17+D17</f>
+      </c>
+      <c r="K17" s="25">
+        <f>=(C17+D17)/G17</f>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B18" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="C18" s="27">
         <f>=C17</f>
       </c>
-      <c r="D18" s="24">
+      <c r="D18" s="27">
         <f>=D17</f>
       </c>
-      <c r="E18" s="24">
+      <c r="E18" s="27">
         <f>=E17</f>
       </c>
-      <c r="F18" s="24">
+      <c r="F18" s="27">
         <f>=F17</f>
       </c>
-      <c r="G18" s="24">
+      <c r="G18" s="27">
         <f>=G17</f>
       </c>
-      <c r="H18" s="24">
+      <c r="H18" s="27">
         <f>=G17-G6</f>
       </c>
-      <c r="I18" s="25">
+      <c r="I18" s="28">
         <f>=(G17-G6)/G6</f>
+      </c>
+      <c r="J18" s="27">
+        <f>=C17+D17</f>
+      </c>
+      <c r="K18" s="28">
+        <f>=(C17+D17)/G17</f>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="B3:K3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1851,7 +2304,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:F20"/>
+  <dimension ref="B2:F37"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1862,91 +2315,91 @@
   </cols>
   <sheetData>
     <row r="2" ht="30" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="26" t="s">
-        <v>61</v>
-      </c>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
+      <c r="B2" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="27" t="s">
-        <v>62</v>
-      </c>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="27"/>
+      <c r="B3" s="30" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
     </row>
     <row r="5" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="28" t="s">
-        <v>63</v>
-      </c>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28" t="s">
+      <c r="B5" s="31" t="s">
         <v>65</v>
       </c>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="E5" s="31"/>
+      <c r="F5" s="31" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="6" ht="28" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="29">
+      <c r="B6" s="32">
         <f>='⚡ 2-Min Quick Check-In'!G18</f>
       </c>
-      <c r="C6" s="29"/>
-      <c r="D6" s="30">
+      <c r="C6" s="32"/>
+      <c r="D6" s="33">
         <f>='⚡ 2-Min Quick Check-In'!C18+'⚡ 2-Min Quick Check-In'!D18</f>
       </c>
-      <c r="E6" s="30"/>
-      <c r="F6" s="31" t="s">
-        <v>66</v>
+      <c r="E6" s="33"/>
+      <c r="F6" s="34" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="32">
+      <c r="B7" s="35">
         <f>="▲ Annual Growth: " &amp; TEXT('⚡ 2-Min Quick Check-In'!I18, "+0.0%") &amp; " (+$" &amp; TEXT('⚡ 2-Min Quick Check-In'!H18, "#,##0") &amp; ")"</f>
       </c>
-      <c r="C7" s="32"/>
-      <c r="D7" s="33">
+      <c r="C7" s="35"/>
+      <c r="D7" s="36">
         <f>="Liquid Ratio: " &amp; TEXT(('⚡ 2-Min Quick Check-In'!C18+'⚡ 2-Min Quick Check-In'!D18)/('⚡ 2-Min Quick Check-In'!G18+'⚡ 2-Min Quick Check-In'!F18), "0.0%") &amp; " of total assets"</f>
       </c>
-      <c r="E7" s="33"/>
-      <c r="F7" s="33" t="s">
-        <v>67</v>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="34" t="s">
-        <v>68</v>
-      </c>
-      <c r="C9" s="34"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="34"/>
-      <c r="F9" s="34"/>
+      <c r="B9" s="37" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
     </row>
     <row r="10" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B10" s="35" t="s">
-        <v>69</v>
-      </c>
-      <c r="C10" s="35" t="s">
-        <v>70</v>
-      </c>
-      <c r="D10" s="35" t="s">
+      <c r="B10" s="38" t="s">
         <v>71</v>
       </c>
-      <c r="E10" s="35" t="s">
+      <c r="C10" s="38" t="s">
         <v>72</v>
       </c>
-      <c r="F10" s="35" t="s">
+      <c r="D10" s="38" t="s">
         <v>73</v>
+      </c>
+      <c r="E10" s="38" t="s">
+        <v>74</v>
+      </c>
+      <c r="F10" s="38" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" s="6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C11" s="15">
         <f>='⚡ 2-Min Quick Check-In'!G6</f>
@@ -1958,29 +2411,29 @@
         <f>='⚡ 2-Min Quick Check-In'!F6</f>
       </c>
       <c r="F11" s="6" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B12" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="C12" s="20">
+      <c r="B12" s="39" t="s">
+        <v>78</v>
+      </c>
+      <c r="C12" s="22">
         <f>='⚡ 2-Min Quick Check-In'!G9</f>
       </c>
-      <c r="D12" s="20">
+      <c r="D12" s="22">
         <f>='⚡ 2-Min Quick Check-In'!D9</f>
       </c>
-      <c r="E12" s="20">
+      <c r="E12" s="22">
         <f>='⚡ 2-Min Quick Check-In'!F9</f>
       </c>
-      <c r="F12" s="36" t="s">
-        <v>77</v>
+      <c r="F12" s="39" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" s="6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C13" s="15">
         <f>='⚡ 2-Min Quick Check-In'!G12</f>
@@ -1992,29 +2445,29 @@
         <f>='⚡ 2-Min Quick Check-In'!F12</f>
       </c>
       <c r="F13" s="6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="36" t="s">
-        <v>80</v>
-      </c>
-      <c r="C14" s="20">
+      <c r="B14" s="39" t="s">
+        <v>82</v>
+      </c>
+      <c r="C14" s="22">
         <f>='⚡ 2-Min Quick Check-In'!G15</f>
       </c>
-      <c r="D14" s="20">
+      <c r="D14" s="22">
         <f>='⚡ 2-Min Quick Check-In'!D15</f>
       </c>
-      <c r="E14" s="20">
+      <c r="E14" s="22">
         <f>='⚡ 2-Min Quick Check-In'!F15</f>
       </c>
-      <c r="F14" s="36" t="s">
-        <v>81</v>
+      <c r="F14" s="39" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" s="6" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C15" s="15">
         <f>='⚡ 2-Min Quick Check-In'!G17</f>
@@ -2026,50 +2479,239 @@
         <f>='⚡ 2-Min Quick Check-In'!F17</f>
       </c>
       <c r="F15" s="6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B18" s="34" t="s">
-        <v>84</v>
-      </c>
-      <c r="C18" s="34"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="34"/>
-      <c r="F18" s="34"/>
+      <c r="B18" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="37"/>
     </row>
     <row r="19" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B19" s="37" t="s">
-        <v>85</v>
-      </c>
-      <c r="C19" s="37" t="s">
-        <v>86</v>
-      </c>
-      <c r="D19" s="37" t="s">
+      <c r="B19" s="40" t="s">
         <v>87</v>
       </c>
-      <c r="E19" s="37" t="s">
+      <c r="C19" s="40" t="s">
         <v>88</v>
       </c>
-      <c r="F19" s="37"/>
+      <c r="D19" s="40" t="s">
+        <v>89</v>
+      </c>
+      <c r="E19" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="F19" s="40"/>
     </row>
     <row r="20" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B20" s="38" t="s">
-        <v>89</v>
-      </c>
-      <c r="C20" s="38" t="s">
-        <v>90</v>
-      </c>
-      <c r="D20" s="38" t="s">
+      <c r="B20" s="41" t="s">
         <v>91</v>
       </c>
-      <c r="E20" s="38" t="s">
+      <c r="C20" s="41" t="s">
         <v>92</v>
       </c>
-      <c r="F20" s="38"/>
+      <c r="D20" s="41" t="s">
+        <v>93</v>
+      </c>
+      <c r="E20" s="41" t="s">
+        <v>94</v>
+      </c>
+      <c r="F20" s="41"/>
+    </row>
+    <row r="22" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B22" s="42" t="s">
+        <v>95</v>
+      </c>
+      <c r="C22" s="42"/>
+      <c r="D22" s="42"/>
+      <c r="E22" s="42"/>
+      <c r="F22" s="42"/>
+    </row>
+    <row r="23" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B23" s="43" t="s">
+        <v>96</v>
+      </c>
+      <c r="C23" s="43" t="s">
+        <v>97</v>
+      </c>
+      <c r="D23" s="43" t="s">
+        <v>98</v>
+      </c>
+      <c r="E23" s="43" t="s">
+        <v>99</v>
+      </c>
+      <c r="F23" s="43" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B24" s="44">
+        <v>32</v>
+      </c>
+      <c r="C24" s="45">
+        <v>108000</v>
+      </c>
+      <c r="D24" s="46">
+        <f>=(B24*C24)/10</f>
+      </c>
+      <c r="E24" s="47">
+        <f>='⚡ 2-Min Quick Check-In'!G18/D24</f>
+      </c>
+      <c r="F24" s="48">
+        <f>=IF('⚡ 2-Min Quick Check-In'!G18&gt;=2*D24, "🏆 PAW (Top 10% Accumulator)", IF('⚡ 2-Min Quick Check-In'!G18&gt;=D24, "⚡ AAW (Solid Average)", "⚠️ UAW (Under Accumulator)"))</f>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B26" s="49" t="s">
+        <v>101</v>
+      </c>
+      <c r="C26" s="49"/>
+      <c r="D26" s="49"/>
+      <c r="E26" s="49"/>
+      <c r="F26" s="49"/>
+    </row>
+    <row r="27" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B27" s="43" t="s">
+        <v>102</v>
+      </c>
+      <c r="C27" s="43" t="s">
+        <v>103</v>
+      </c>
+      <c r="D27" s="43" t="s">
+        <v>104</v>
+      </c>
+      <c r="E27" s="43" t="s">
+        <v>105</v>
+      </c>
+      <c r="F27" s="43" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="28" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B28" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="C28" s="50">
+        <v>100000</v>
+      </c>
+      <c r="D28" s="51">
+        <f>=MIN(1, '⚡ 2-Min Quick Check-In'!G18/C28)</f>
+      </c>
+      <c r="E28" s="50">
+        <f>=MAX(0, C28-'⚡ 2-Min Quick Check-In'!G18)</f>
+      </c>
+      <c r="F28" s="52" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="29" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B29" s="53" t="s">
+        <v>109</v>
+      </c>
+      <c r="C29" s="54">
+        <v>250000</v>
+      </c>
+      <c r="D29" s="55">
+        <f>=MIN(1, '⚡ 2-Min Quick Check-In'!G18/C29)</f>
+      </c>
+      <c r="E29" s="54">
+        <f>=MAX(0, C29-'⚡ 2-Min Quick Check-In'!G18)</f>
+      </c>
+      <c r="F29" s="56" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="30" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B30" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="C30" s="50">
+        <v>500000</v>
+      </c>
+      <c r="D30" s="51">
+        <f>=MIN(1, '⚡ 2-Min Quick Check-In'!G18/C30)</f>
+      </c>
+      <c r="E30" s="50">
+        <f>=MAX(0, C30-'⚡ 2-Min Quick Check-In'!G18)</f>
+      </c>
+      <c r="F30" s="52" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="31" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B31" s="53" t="s">
+        <v>113</v>
+      </c>
+      <c r="C31" s="54">
+        <v>1000000</v>
+      </c>
+      <c r="D31" s="55">
+        <f>=MIN(1, '⚡ 2-Min Quick Check-In'!G18/C31)</f>
+      </c>
+      <c r="E31" s="54">
+        <f>=MAX(0, C31-'⚡ 2-Min Quick Check-In'!G18)</f>
+      </c>
+      <c r="F31" s="56" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="33" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B33" s="42" t="s">
+        <v>115</v>
+      </c>
+      <c r="C33" s="42"/>
+      <c r="D33" s="42"/>
+      <c r="E33" s="42"/>
+      <c r="F33" s="42"/>
+    </row>
+    <row r="34" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B34" s="43" t="s">
+        <v>116</v>
+      </c>
+      <c r="C34" s="43" t="s">
+        <v>117</v>
+      </c>
+      <c r="D34" s="43" t="s">
+        <v>118</v>
+      </c>
+      <c r="E34" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="F34" s="43" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="35" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B35" s="57">
+        <f>='⚡ 2-Min Quick Check-In'!C18+'⚡ 2-Min Quick Check-In'!D18</f>
+      </c>
+      <c r="C35" s="57">
+        <f>='💸 Smart Budget (50-30-20)'!C20</f>
+      </c>
+      <c r="D35" s="58">
+        <f>=B35/C35</f>
+      </c>
+      <c r="E35" s="59">
+        <f>=B35/'⚡ 2-Min Quick Check-In'!G18</f>
+      </c>
+      <c r="F35" s="60" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B37" s="61" t="s">
+        <v>122</v>
+      </c>
+      <c r="C37" s="61"/>
+      <c r="D37" s="61"/>
+      <c r="E37" s="61"/>
+      <c r="F37" s="61"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="16">
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B5:C5"/>
@@ -2082,6 +2724,10 @@
     <mergeCell ref="B18:F18"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="E20:F20"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="B37:F37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2102,74 +2748,74 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="26" t="s">
-        <v>93</v>
-      </c>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
+      <c r="B2" s="29" t="s">
+        <v>123</v>
+      </c>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="27" t="s">
-        <v>94</v>
-      </c>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="27"/>
+      <c r="B3" s="30" t="s">
+        <v>124</v>
+      </c>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="32" t="s">
-        <v>95</v>
-      </c>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="28" t="s">
-        <v>96</v>
-      </c>
-      <c r="F5" s="28"/>
+      <c r="B5" s="35" t="s">
+        <v>125</v>
+      </c>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="31" t="s">
+        <v>126</v>
+      </c>
+      <c r="F5" s="31"/>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="39">
+      <c r="B6" s="62">
         <f>=E24</f>
       </c>
-      <c r="C6" s="39"/>
-      <c r="D6" s="39"/>
-      <c r="E6" s="40">
+      <c r="C6" s="62"/>
+      <c r="D6" s="62"/>
+      <c r="E6" s="63">
         <f>=E24/30</f>
       </c>
-      <c r="F6" s="40"/>
+      <c r="F6" s="63"/>
     </row>
     <row r="8" ht="22" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="41" t="s">
-        <v>97</v>
-      </c>
-      <c r="C8" s="41" t="s">
-        <v>98</v>
-      </c>
-      <c r="D8" s="41" t="s">
-        <v>99</v>
-      </c>
-      <c r="E8" s="41" t="s">
-        <v>100</v>
-      </c>
-      <c r="F8" s="41" t="s">
-        <v>101</v>
+      <c r="B8" s="64" t="s">
+        <v>127</v>
+      </c>
+      <c r="C8" s="64" t="s">
+        <v>128</v>
+      </c>
+      <c r="D8" s="64" t="s">
+        <v>129</v>
+      </c>
+      <c r="E8" s="64" t="s">
+        <v>130</v>
+      </c>
+      <c r="F8" s="64" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="42" t="s">
-        <v>102</v>
-      </c>
-      <c r="C9" s="42"/>
-      <c r="D9" s="42"/>
-      <c r="E9" s="42"/>
-      <c r="F9" s="42"/>
+      <c r="B9" s="65" t="s">
+        <v>132</v>
+      </c>
+      <c r="C9" s="65"/>
+      <c r="D9" s="65"/>
+      <c r="E9" s="65"/>
+      <c r="F9" s="65"/>
     </row>
     <row r="10" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
-        <v>103</v>
+        <v>133</v>
       </c>
       <c r="C10" s="15">
         <v>6800</v>
@@ -2181,12 +2827,12 @@
         <f>=D10-C10</f>
       </c>
       <c r="F10" s="6" t="s">
-        <v>104</v>
+        <v>134</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" s="6" t="s">
-        <v>105</v>
+        <v>135</v>
       </c>
       <c r="C11" s="15">
         <v>2200</v>
@@ -2198,12 +2844,12 @@
         <f>=D11-C11</f>
       </c>
       <c r="F11" s="6" t="s">
-        <v>104</v>
+        <v>134</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" s="6" t="s">
-        <v>106</v>
+        <v>136</v>
       </c>
       <c r="C12" s="15">
         <v>500</v>
@@ -2215,38 +2861,38 @@
         <f>=D12-C12</f>
       </c>
       <c r="F12" s="6" t="s">
-        <v>104</v>
+        <v>134</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B13" s="43" t="s">
-        <v>107</v>
-      </c>
-      <c r="C13" s="44">
+      <c r="B13" s="66" t="s">
+        <v>137</v>
+      </c>
+      <c r="C13" s="67">
         <f>=SUM(C10:C12)</f>
       </c>
-      <c r="D13" s="44">
+      <c r="D13" s="67">
         <f>=SUM(D10:D12)</f>
       </c>
-      <c r="E13" s="44">
+      <c r="E13" s="67">
         <f>=D13-C13</f>
       </c>
-      <c r="F13" s="43" t="s">
-        <v>108</v>
+      <c r="F13" s="66" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="45" t="s">
-        <v>109</v>
-      </c>
-      <c r="C14" s="45"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="45"/>
-      <c r="F14" s="45"/>
+      <c r="B14" s="68" t="s">
+        <v>139</v>
+      </c>
+      <c r="C14" s="68"/>
+      <c r="D14" s="68"/>
+      <c r="E14" s="68"/>
+      <c r="F14" s="68"/>
     </row>
     <row r="15" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" s="6" t="s">
-        <v>110</v>
+        <v>140</v>
       </c>
       <c r="C15" s="15">
         <v>2400</v>
@@ -2263,7 +2909,7 @@
     </row>
     <row r="16" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" s="6" t="s">
-        <v>111</v>
+        <v>141</v>
       </c>
       <c r="C16" s="15">
         <v>750</v>
@@ -2280,7 +2926,7 @@
     </row>
     <row r="17" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="6" t="s">
-        <v>112</v>
+        <v>142</v>
       </c>
       <c r="C17" s="15">
         <v>320</v>
@@ -2297,7 +2943,7 @@
     </row>
     <row r="18" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="6" t="s">
-        <v>113</v>
+        <v>143</v>
       </c>
       <c r="C18" s="15">
         <v>450</v>
@@ -2314,7 +2960,7 @@
     </row>
     <row r="19" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" s="6" t="s">
-        <v>114</v>
+        <v>144</v>
       </c>
       <c r="C19" s="15">
         <v>400</v>
@@ -2330,34 +2976,34 @@
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B20" s="46" t="s">
-        <v>115</v>
-      </c>
-      <c r="C20" s="47">
+      <c r="B20" s="69" t="s">
+        <v>145</v>
+      </c>
+      <c r="C20" s="70">
         <f>=SUM(C15:C19)</f>
       </c>
-      <c r="D20" s="47">
+      <c r="D20" s="70">
         <f>=SUM(D15:D19)</f>
       </c>
-      <c r="E20" s="47">
+      <c r="E20" s="70">
         <f>=C20-D20</f>
       </c>
-      <c r="F20" s="46">
+      <c r="F20" s="69">
         <f>="Actual: " &amp; TEXT(D20/D13, "0.0%") &amp; " (Target: ≤50%)"</f>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B21" s="48" t="s">
-        <v>116</v>
-      </c>
-      <c r="C21" s="48"/>
-      <c r="D21" s="48"/>
-      <c r="E21" s="48"/>
-      <c r="F21" s="48"/>
+      <c r="B21" s="71" t="s">
+        <v>146</v>
+      </c>
+      <c r="C21" s="71"/>
+      <c r="D21" s="71"/>
+      <c r="E21" s="71"/>
+      <c r="F21" s="71"/>
     </row>
     <row r="22" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" s="6" t="s">
-        <v>117</v>
+        <v>147</v>
       </c>
       <c r="C22" s="15">
         <v>650</v>
@@ -2374,7 +3020,7 @@
     </row>
     <row r="23" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="6" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
       <c r="C23" s="15">
         <v>120</v>
@@ -2391,7 +3037,7 @@
     </row>
     <row r="24" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" s="6" t="s">
-        <v>119</v>
+        <v>149</v>
       </c>
       <c r="C24" s="15">
         <v>450</v>
@@ -2407,34 +3053,34 @@
       </c>
     </row>
     <row r="25" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B25" s="49" t="s">
-        <v>120</v>
-      </c>
-      <c r="C25" s="50">
+      <c r="B25" s="72" t="s">
+        <v>150</v>
+      </c>
+      <c r="C25" s="73">
         <f>=SUM(C22:C24)</f>
       </c>
-      <c r="D25" s="50">
+      <c r="D25" s="73">
         <f>=SUM(D22:D24)</f>
       </c>
-      <c r="E25" s="50">
+      <c r="E25" s="73">
         <f>=C25-D25</f>
       </c>
-      <c r="F25" s="49">
+      <c r="F25" s="72">
         <f>="Actual: " &amp; TEXT(D25/D13, "0.0%") &amp; " (Target: ≤30%)"</f>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B26" s="42" t="s">
-        <v>121</v>
-      </c>
-      <c r="C26" s="42"/>
-      <c r="D26" s="42"/>
-      <c r="E26" s="42"/>
-      <c r="F26" s="42"/>
+      <c r="B26" s="65" t="s">
+        <v>151</v>
+      </c>
+      <c r="C26" s="65"/>
+      <c r="D26" s="65"/>
+      <c r="E26" s="65"/>
+      <c r="F26" s="65"/>
     </row>
     <row r="27" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" s="6" t="s">
-        <v>122</v>
+        <v>152</v>
       </c>
       <c r="C27" s="15">
         <v>2200</v>
@@ -2451,7 +3097,7 @@
     </row>
     <row r="28" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" s="6" t="s">
-        <v>123</v>
+        <v>153</v>
       </c>
       <c r="C28" s="15">
         <v>500</v>
@@ -2468,7 +3114,7 @@
     </row>
     <row r="29" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" s="6" t="s">
-        <v>124</v>
+        <v>154</v>
       </c>
       <c r="C29" s="15">
         <v>600</v>
@@ -2484,19 +3130,19 @@
       </c>
     </row>
     <row r="30" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B30" s="51" t="s">
-        <v>125</v>
-      </c>
-      <c r="C30" s="52">
+      <c r="B30" s="74" t="s">
+        <v>155</v>
+      </c>
+      <c r="C30" s="75">
         <f>=SUM(C27:C29)</f>
       </c>
-      <c r="D30" s="52">
+      <c r="D30" s="75">
         <f>=SUM(D27:D29)</f>
       </c>
-      <c r="E30" s="52">
+      <c r="E30" s="75">
         <f>=D30-C30</f>
       </c>
-      <c r="F30" s="51">
+      <c r="F30" s="74">
         <f>="Savings Rate: " &amp; TEXT(D30/D13, "0.0%") &amp; " (FIRE Speed)"</f>
       </c>
     </row>
@@ -2532,7 +3178,7 @@
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
-        <v>126</v>
+        <v>156</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -2543,7 +3189,7 @@
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="11" t="s">
-        <v>127</v>
+        <v>157</v>
       </c>
       <c r="C3" s="11"/>
       <c r="D3" s="11"/>
@@ -2553,31 +3199,31 @@
       <c r="H3" s="11"/>
     </row>
     <row r="5" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B5" s="41" t="s">
-        <v>128</v>
-      </c>
-      <c r="C5" s="41" t="s">
-        <v>129</v>
-      </c>
-      <c r="D5" s="41" t="s">
-        <v>130</v>
-      </c>
-      <c r="E5" s="41" t="s">
-        <v>131</v>
-      </c>
-      <c r="F5" s="41" t="s">
-        <v>132</v>
-      </c>
-      <c r="G5" s="41" t="s">
-        <v>133</v>
-      </c>
-      <c r="H5" s="41" t="s">
-        <v>134</v>
+      <c r="B5" s="64" t="s">
+        <v>158</v>
+      </c>
+      <c r="C5" s="64" t="s">
+        <v>159</v>
+      </c>
+      <c r="D5" s="64" t="s">
+        <v>160</v>
+      </c>
+      <c r="E5" s="64" t="s">
+        <v>161</v>
+      </c>
+      <c r="F5" s="64" t="s">
+        <v>162</v>
+      </c>
+      <c r="G5" s="64" t="s">
+        <v>163</v>
+      </c>
+      <c r="H5" s="64" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
-        <v>135</v>
+        <v>165</v>
       </c>
       <c r="C6" s="15">
         <v>25000</v>
@@ -2589,41 +3235,41 @@
         <f>=C6-D6</f>
       </c>
       <c r="F6" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G6" s="15">
         <v>700</v>
       </c>
-      <c r="H6" s="53">
+      <c r="H6" s="20">
         <f>=D6/C6</f>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B7" s="36" t="s">
-        <v>136</v>
-      </c>
-      <c r="C7" s="20">
+      <c r="B7" s="39" t="s">
+        <v>166</v>
+      </c>
+      <c r="C7" s="22">
         <v>2000</v>
       </c>
-      <c r="D7" s="20">
+      <c r="D7" s="22">
         <v>1400</v>
       </c>
-      <c r="E7" s="20">
+      <c r="E7" s="22">
         <f>=C7-D7</f>
       </c>
-      <c r="F7" s="36" t="s">
-        <v>55</v>
-      </c>
-      <c r="G7" s="20">
+      <c r="F7" s="39" t="s">
+        <v>57</v>
+      </c>
+      <c r="G7" s="22">
         <v>150</v>
       </c>
-      <c r="H7" s="54">
+      <c r="H7" s="25">
         <f>=D7/C7</f>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
-        <v>137</v>
+        <v>167</v>
       </c>
       <c r="C8" s="15">
         <v>4500</v>
@@ -2635,41 +3281,41 @@
         <f>=C8-D8</f>
       </c>
       <c r="F8" s="6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="G8" s="15">
         <v>250</v>
       </c>
-      <c r="H8" s="53">
+      <c r="H8" s="20">
         <f>=D8/C8</f>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="36" t="s">
-        <v>138</v>
-      </c>
-      <c r="C9" s="20">
+      <c r="B9" s="39" t="s">
+        <v>168</v>
+      </c>
+      <c r="C9" s="22">
         <v>1500</v>
       </c>
-      <c r="D9" s="20">
+      <c r="D9" s="22">
         <v>750</v>
       </c>
-      <c r="E9" s="20">
+      <c r="E9" s="22">
         <f>=C9-D9</f>
       </c>
-      <c r="F9" s="36" t="s">
-        <v>58</v>
-      </c>
-      <c r="G9" s="20">
+      <c r="F9" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="G9" s="22">
         <v>125</v>
       </c>
-      <c r="H9" s="54">
+      <c r="H9" s="25">
         <f>=D9/C9</f>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
-        <v>139</v>
+        <v>169</v>
       </c>
       <c r="C10" s="15">
         <v>3500</v>
@@ -2681,35 +3327,35 @@
         <f>=C10-D10</f>
       </c>
       <c r="F10" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G10" s="15">
         <v>250</v>
       </c>
-      <c r="H10" s="53">
+      <c r="H10" s="20">
         <f>=D10/C10</f>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="23" t="s">
-        <v>140</v>
-      </c>
-      <c r="C11" s="24">
+      <c r="B11" s="26" t="s">
+        <v>170</v>
+      </c>
+      <c r="C11" s="27">
         <f>=SUM(C6:C10)</f>
       </c>
-      <c r="D11" s="24">
+      <c r="D11" s="27">
         <f>=SUM(D6:D10)</f>
       </c>
-      <c r="E11" s="24">
+      <c r="E11" s="27">
         <f>=SUM(E6:E10)</f>
       </c>
-      <c r="F11" s="23" t="s">
-        <v>141</v>
-      </c>
-      <c r="G11" s="24">
+      <c r="F11" s="26" t="s">
+        <v>171</v>
+      </c>
+      <c r="G11" s="27">
         <f>=SUM(G6:G10)</f>
       </c>
-      <c r="H11" s="55">
+      <c r="H11" s="76">
         <f>=D11/C11</f>
       </c>
     </row>
@@ -2737,16 +3383,16 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B2" s="56" t="s">
-        <v>142</v>
-      </c>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
+      <c r="B2" s="77" t="s">
+        <v>172</v>
+      </c>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
-        <v>143</v>
+        <v>173</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -2754,102 +3400,102 @@
     </row>
     <row r="5" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B5" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="C5" s="57">
+        <v>174</v>
+      </c>
+      <c r="C5" s="78">
         <v>32</v>
       </c>
     </row>
     <row r="6" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="C6" s="58">
+        <v>175</v>
+      </c>
+      <c r="C6" s="79">
         <v>66000</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="C7" s="59">
+        <v>176</v>
+      </c>
+      <c r="C7" s="80">
         <v>0.04</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="C8" s="59">
+        <v>177</v>
+      </c>
+      <c r="C8" s="80">
         <v>0.07</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B9" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="C9" s="58">
+        <v>178</v>
+      </c>
+      <c r="C9" s="79">
         <f>'⚡ 2-Min Quick Check-In'!D18</f>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="C10" s="58">
+        <v>179</v>
+      </c>
+      <c r="C10" s="79">
         <f>'💸 Smart Budget (50-30-20)'!D27</f>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B12" s="42" t="s">
-        <v>150</v>
-      </c>
-      <c r="C12" s="42"/>
-      <c r="D12" s="42"/>
-      <c r="E12" s="42"/>
+      <c r="B12" s="65" t="s">
+        <v>180</v>
+      </c>
+      <c r="C12" s="65"/>
+      <c r="D12" s="65"/>
+      <c r="E12" s="65"/>
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="C13" s="58">
+        <v>181</v>
+      </c>
+      <c r="C13" s="79">
         <f>C6*0.65/C7</f>
       </c>
-      <c r="D13" s="60" t="s">
-        <v>152</v>
+      <c r="D13" s="81" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B14" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="C14" s="58">
+        <v>183</v>
+      </c>
+      <c r="C14" s="79">
         <f>C6/C7</f>
       </c>
-      <c r="D14" s="60" t="s">
-        <v>154</v>
+      <c r="D14" s="81" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B15" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="C15" s="58">
+        <v>185</v>
+      </c>
+      <c r="C15" s="79">
         <f>C6*1.4/C7</f>
       </c>
-      <c r="D15" s="60" t="s">
-        <v>156</v>
+      <c r="D15" s="81" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="C16" s="58">
+        <v>187</v>
+      </c>
+      <c r="C16" s="79">
         <f>(C6/C7)/(1+C8)^(60-C5)</f>
       </c>
-      <c r="D16" s="60" t="s">
-        <v>158</v>
+      <c r="D16" s="81" t="s">
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -2878,114 +3524,114 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="56" t="s">
-        <v>159</v>
-      </c>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
+      <c r="B2" s="77" t="s">
+        <v>189</v>
+      </c>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
     </row>
     <row r="4" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="35" t="s">
+      <c r="B4" s="38" t="s">
+        <v>190</v>
+      </c>
+      <c r="C4" s="38" t="s">
         <v>160</v>
       </c>
-      <c r="C4" s="35" t="s">
-        <v>130</v>
-      </c>
-      <c r="D4" s="35" t="s">
-        <v>161</v>
-      </c>
-      <c r="E4" s="35" t="s">
-        <v>162</v>
-      </c>
-      <c r="F4" s="35" t="s">
-        <v>163</v>
+      <c r="D4" s="38" t="s">
+        <v>191</v>
+      </c>
+      <c r="E4" s="38" t="s">
+        <v>192</v>
+      </c>
+      <c r="F4" s="38" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="5" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="6" t="s">
-        <v>164</v>
+        <v>194</v>
       </c>
       <c r="C5" s="15">
         <v>4200</v>
       </c>
-      <c r="D5" s="61">
+      <c r="D5" s="82">
         <v>0.2499</v>
       </c>
       <c r="E5" s="15">
         <v>140</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>165</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
-        <v>166</v>
+        <v>196</v>
       </c>
       <c r="C6" s="15">
         <v>8500</v>
       </c>
-      <c r="D6" s="61">
+      <c r="D6" s="82">
         <v>0.115</v>
       </c>
       <c r="E6" s="15">
         <v>210</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>167</v>
+        <v>197</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
-        <v>168</v>
+        <v>198</v>
       </c>
       <c r="C7" s="15">
         <v>17400</v>
       </c>
-      <c r="D7" s="61">
+      <c r="D7" s="82">
         <v>0.059</v>
       </c>
       <c r="E7" s="15">
         <v>380</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>169</v>
+        <v>199</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
-        <v>170</v>
+        <v>200</v>
       </c>
       <c r="C8" s="15">
         <v>200000</v>
       </c>
-      <c r="D8" s="61">
+      <c r="D8" s="82">
         <v>0.035</v>
       </c>
       <c r="E8" s="15">
         <v>1670</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>171</v>
+        <v>201</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="43" t="s">
-        <v>172</v>
-      </c>
-      <c r="C9" s="44">
+      <c r="B9" s="66" t="s">
+        <v>202</v>
+      </c>
+      <c r="C9" s="67">
         <f>=SUM(C5:C8)</f>
       </c>
-      <c r="D9" s="62">
+      <c r="D9" s="83">
         <f>=AVERAGE(D5:D8)</f>
       </c>
-      <c r="E9" s="44">
+      <c r="E9" s="67">
         <f>=SUM(E5:E8)</f>
       </c>
-      <c r="F9" s="43" t="s">
-        <v>173</v>
+      <c r="F9" s="66" t="s">
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -2999,7 +3645,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:H10"/>
+  <dimension ref="B2:H36"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -3009,42 +3655,42 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="56" t="s">
-        <v>174</v>
-      </c>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
+      <c r="B2" s="77" t="s">
+        <v>204</v>
+      </c>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="77"/>
     </row>
     <row r="4" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B4" s="35" t="s">
-        <v>175</v>
-      </c>
-      <c r="C4" s="35" t="s">
-        <v>176</v>
-      </c>
-      <c r="D4" s="35" t="s">
-        <v>177</v>
-      </c>
-      <c r="E4" s="35" t="s">
-        <v>178</v>
-      </c>
-      <c r="F4" s="35" t="s">
-        <v>179</v>
-      </c>
-      <c r="G4" s="35" t="s">
-        <v>180</v>
-      </c>
-      <c r="H4" s="35" t="s">
-        <v>181</v>
+      <c r="B4" s="38" t="s">
+        <v>205</v>
+      </c>
+      <c r="C4" s="38" t="s">
+        <v>206</v>
+      </c>
+      <c r="D4" s="38" t="s">
+        <v>207</v>
+      </c>
+      <c r="E4" s="38" t="s">
+        <v>208</v>
+      </c>
+      <c r="F4" s="38" t="s">
+        <v>209</v>
+      </c>
+      <c r="G4" s="38" t="s">
+        <v>210</v>
+      </c>
+      <c r="H4" s="38" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="5" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="6" t="s">
-        <v>182</v>
+        <v>212</v>
       </c>
       <c r="C5" s="15">
         <v>4800</v>
@@ -3066,31 +3712,31 @@
       </c>
     </row>
     <row r="6" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B6" s="36" t="s">
-        <v>183</v>
-      </c>
-      <c r="C6" s="20">
+      <c r="B6" s="39" t="s">
+        <v>213</v>
+      </c>
+      <c r="C6" s="22">
         <v>35000</v>
       </c>
-      <c r="D6" s="20">
+      <c r="D6" s="22">
         <v>135600</v>
       </c>
-      <c r="E6" s="20">
+      <c r="E6" s="22">
         <v>420000</v>
       </c>
-      <c r="F6" s="20">
+      <c r="F6" s="22">
         <v>980000</v>
       </c>
-      <c r="G6" s="20">
+      <c r="G6" s="22">
         <v>1850000</v>
       </c>
-      <c r="H6" s="20">
+      <c r="H6" s="22">
         <v>5500000</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
-        <v>184</v>
+        <v>214</v>
       </c>
       <c r="C7" s="15">
         <v>68000</v>
@@ -3112,31 +3758,31 @@
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="36" t="s">
-        <v>185</v>
-      </c>
-      <c r="C8" s="20">
+      <c r="B8" s="39" t="s">
+        <v>215</v>
+      </c>
+      <c r="C8" s="22">
         <v>95000</v>
       </c>
-      <c r="D8" s="20">
+      <c r="D8" s="22">
         <v>364500</v>
       </c>
-      <c r="E8" s="20">
+      <c r="E8" s="22">
         <v>1150000</v>
       </c>
-      <c r="F8" s="20">
+      <c r="F8" s="22">
         <v>2800000</v>
       </c>
-      <c r="G8" s="20">
+      <c r="G8" s="22">
         <v>4900000</v>
       </c>
-      <c r="H8" s="20">
+      <c r="H8" s="22">
         <v>14500000</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="6" t="s">
-        <v>186</v>
+        <v>216</v>
       </c>
       <c r="C9" s="15">
         <v>110000</v>
@@ -3158,31 +3804,481 @@
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="36" t="s">
-        <v>187</v>
-      </c>
-      <c r="C10" s="20">
+      <c r="B10" s="39" t="s">
+        <v>217</v>
+      </c>
+      <c r="C10" s="22">
         <v>92000</v>
       </c>
-      <c r="D10" s="20">
+      <c r="D10" s="22">
         <v>335600</v>
       </c>
-      <c r="E10" s="20">
+      <c r="E10" s="22">
         <v>1050000</v>
       </c>
-      <c r="F10" s="20">
+      <c r="F10" s="22">
         <v>2600000</v>
       </c>
-      <c r="G10" s="20">
+      <c r="G10" s="22">
         <v>4700000</v>
       </c>
-      <c r="H10" s="20">
+      <c r="H10" s="22">
         <v>13200000</v>
       </c>
     </row>
+    <row r="13" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B13" s="84" t="s">
+        <v>218</v>
+      </c>
+      <c r="C13" s="84"/>
+      <c r="D13" s="84"/>
+      <c r="E13" s="84"/>
+      <c r="F13" s="84"/>
+      <c r="G13" s="84"/>
+      <c r="H13" s="84"/>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B14" s="38" t="s">
+        <v>219</v>
+      </c>
+      <c r="C14" s="38" t="s">
+        <v>220</v>
+      </c>
+      <c r="D14" s="38" t="s">
+        <v>221</v>
+      </c>
+      <c r="E14" s="38" t="s">
+        <v>222</v>
+      </c>
+      <c r="F14" s="38" t="s">
+        <v>223</v>
+      </c>
+      <c r="G14" s="38" t="s">
+        <v>224</v>
+      </c>
+      <c r="H14" s="38" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="15" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B15" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="C15" s="15">
+        <v>285000</v>
+      </c>
+      <c r="D15" s="15">
+        <v>1250000</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="F15" s="15">
+        <v>785000</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="16" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B16" s="39" t="s">
+        <v>230</v>
+      </c>
+      <c r="C16" s="22">
+        <v>245000</v>
+      </c>
+      <c r="D16" s="22">
+        <v>1180000</v>
+      </c>
+      <c r="E16" s="39" t="s">
+        <v>231</v>
+      </c>
+      <c r="F16" s="22">
+        <v>650000</v>
+      </c>
+      <c r="G16" s="39" t="s">
+        <v>228</v>
+      </c>
+      <c r="H16" s="39" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="17" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B17" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="C17" s="15">
+        <v>275000</v>
+      </c>
+      <c r="D17" s="15">
+        <v>1200000</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="F17" s="15">
+        <v>610000</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="18" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B18" s="39" t="s">
+        <v>236</v>
+      </c>
+      <c r="C18" s="22">
+        <v>175000</v>
+      </c>
+      <c r="D18" s="22">
+        <v>820000</v>
+      </c>
+      <c r="E18" s="39" t="s">
+        <v>237</v>
+      </c>
+      <c r="F18" s="22">
+        <v>345000</v>
+      </c>
+      <c r="G18" s="39" t="s">
+        <v>238</v>
+      </c>
+      <c r="H18" s="39" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="19" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B19" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="C19" s="15">
+        <v>195000</v>
+      </c>
+      <c r="D19" s="15">
+        <v>890000</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="F19" s="15">
+        <v>395000</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="20" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="39" t="s">
+        <v>244</v>
+      </c>
+      <c r="C20" s="22">
+        <v>295000</v>
+      </c>
+      <c r="D20" s="22">
+        <v>1320000</v>
+      </c>
+      <c r="E20" s="39" t="s">
+        <v>245</v>
+      </c>
+      <c r="F20" s="22">
+        <v>640000</v>
+      </c>
+      <c r="G20" s="39" t="s">
+        <v>228</v>
+      </c>
+      <c r="H20" s="39" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="21" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B21" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="C21" s="15">
+        <v>185000</v>
+      </c>
+      <c r="D21" s="15">
+        <v>860000</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="F21" s="15">
+        <v>275000</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="22" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B22" s="39" t="s">
+        <v>250</v>
+      </c>
+      <c r="C22" s="22">
+        <v>260000</v>
+      </c>
+      <c r="D22" s="22">
+        <v>1100000</v>
+      </c>
+      <c r="E22" s="39" t="s">
+        <v>251</v>
+      </c>
+      <c r="F22" s="22">
+        <v>550000</v>
+      </c>
+      <c r="G22" s="39" t="s">
+        <v>252</v>
+      </c>
+      <c r="H22" s="39" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B25" s="85" t="s">
+        <v>254</v>
+      </c>
+      <c r="C25" s="85"/>
+      <c r="D25" s="85"/>
+      <c r="E25" s="85"/>
+      <c r="F25" s="85"/>
+      <c r="G25" s="85"/>
+      <c r="H25" s="85"/>
+    </row>
+    <row r="26" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B26" s="38" t="s">
+        <v>255</v>
+      </c>
+      <c r="C26" s="38" t="s">
+        <v>256</v>
+      </c>
+      <c r="D26" s="38" t="s">
+        <v>257</v>
+      </c>
+      <c r="E26" s="38" t="s">
+        <v>258</v>
+      </c>
+      <c r="F26" s="38" t="s">
+        <v>259</v>
+      </c>
+      <c r="G26" s="38" t="s">
+        <v>260</v>
+      </c>
+      <c r="H26" s="38" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="27" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B27" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="C27" s="86">
+        <v>1</v>
+      </c>
+      <c r="D27" s="15">
+        <v>100000</v>
+      </c>
+      <c r="E27" s="15">
+        <v>150000</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="28" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B28" s="39" t="s">
+        <v>266</v>
+      </c>
+      <c r="C28" s="87">
+        <v>2</v>
+      </c>
+      <c r="D28" s="22">
+        <v>200000</v>
+      </c>
+      <c r="E28" s="22">
+        <v>300000</v>
+      </c>
+      <c r="F28" s="39" t="s">
+        <v>267</v>
+      </c>
+      <c r="G28" s="39" t="s">
+        <v>264</v>
+      </c>
+      <c r="H28" s="39" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="29" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B29" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="C29" s="86">
+        <v>3</v>
+      </c>
+      <c r="D29" s="15">
+        <v>300000</v>
+      </c>
+      <c r="E29" s="15">
+        <v>450000</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="30" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B30" s="39" t="s">
+        <v>270</v>
+      </c>
+      <c r="C30" s="87">
+        <v>4</v>
+      </c>
+      <c r="D30" s="22">
+        <v>400000</v>
+      </c>
+      <c r="E30" s="22">
+        <v>600000</v>
+      </c>
+      <c r="F30" s="39" t="s">
+        <v>271</v>
+      </c>
+      <c r="G30" s="39" t="s">
+        <v>264</v>
+      </c>
+      <c r="H30" s="39" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="31" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B31" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="C31" s="86">
+        <v>6</v>
+      </c>
+      <c r="D31" s="15">
+        <v>600000</v>
+      </c>
+      <c r="E31" s="15">
+        <v>900000</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="32" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B32" s="39" t="s">
+        <v>274</v>
+      </c>
+      <c r="C32" s="87">
+        <v>7</v>
+      </c>
+      <c r="D32" s="22">
+        <v>700000</v>
+      </c>
+      <c r="E32" s="22">
+        <v>1050000</v>
+      </c>
+      <c r="F32" s="39" t="s">
+        <v>275</v>
+      </c>
+      <c r="G32" s="39" t="s">
+        <v>264</v>
+      </c>
+      <c r="H32" s="39" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="33" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B33" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="C33" s="86">
+        <v>8</v>
+      </c>
+      <c r="D33" s="15">
+        <v>800000</v>
+      </c>
+      <c r="E33" s="15">
+        <v>1200000</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="34" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B34" s="39" t="s">
+        <v>278</v>
+      </c>
+      <c r="C34" s="87">
+        <v>10</v>
+      </c>
+      <c r="D34" s="22">
+        <v>1000000</v>
+      </c>
+      <c r="E34" s="22">
+        <v>1500000</v>
+      </c>
+      <c r="F34" s="39" t="s">
+        <v>279</v>
+      </c>
+      <c r="G34" s="39" t="s">
+        <v>264</v>
+      </c>
+      <c r="H34" s="39" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B36" s="61" t="s">
+        <v>280</v>
+      </c>
+      <c r="C36" s="61"/>
+      <c r="D36" s="61"/>
+      <c r="E36" s="61"/>
+      <c r="F36" s="61"/>
+      <c r="G36" s="61"/>
+      <c r="H36" s="61"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="4">
     <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B13:H13"/>
+    <mergeCell ref="B25:H25"/>
+    <mergeCell ref="B36:H36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
fix(vault): strip leading equals from formulas and clean tab names for perfect Numbers/Excel compatibility
</commit_message>
<xml_diff>
--- a/public/downloads/NetWorth_FIRE_Master_Vault_2026.xlsx
+++ b/public/downloads/NetWorth_FIRE_Master_Vault_2026.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="🟢 START HERE (60-Sec Guide)" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="⚡ 2-Min Quick Check-In" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="📊 Executive Dashboard" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="💸 Smart Budget (50-30-20)" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="🎯 Sinking Funds Shield" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="🔥 FIRE Freedom Engine" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="💳 Debt Avalanche &amp; Snowball" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="🏛️ Fed &amp; State Benchmarks" state="visible" r:id="rId11"/>
+    <sheet sheetId="1" name="START HERE" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="2-Min Check-In" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Executive Dashboard" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Smart Budget (50-30-20)" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Sinking Funds Shield" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="FIRE Freedom Engine" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="Debt Avalanche &amp; Snowball" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="Fed &amp; State Benchmarks" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -32,7 +32,7 @@
     <t>Step 1: Open Tab 2</t>
   </si>
   <si>
-    <t>Click '⚡ 2-Min Quick Check-In'</t>
+    <t>Click '2-Min Check-In'</t>
   </si>
   <si>
     <t>On the 1st of every month, open the second tab.</t>
@@ -89,7 +89,7 @@
     <t>📖 WHAT EACH TAB DOES (CHOOSE YOUR PURPOSE)</t>
   </si>
   <si>
-    <t>⚡ 2-Min Quick Check-In</t>
+    <t>2-Min Check-In</t>
   </si>
   <si>
     <t>For 90% of months: Type 4 numbers once a month in 90 seconds. Zero homework.</t>
@@ -107,13 +107,13 @@
     <t>Answers: 'How much can I spend today guilt-free?' (Needs 50%, Wants 30%, Wealth 20%).</t>
   </si>
   <si>
-    <t>🎯 Sinking Funds Shield</t>
+    <t>Sinking Funds Shield</t>
   </si>
   <si>
     <t>Prevents budget shock from car repairs, holiday travel, and annual insurance renewals.</t>
   </si>
   <si>
-    <t>🔥 FIRE Freedom Engine</t>
+    <t>FIRE Freedom Engine</t>
   </si>
   <si>
     <t>Trinity 4% rule calculator showing your Coast FIRE milestone and exact retirement date.</t>
@@ -1893,7 +1893,7 @@
         <v>245000</v>
       </c>
       <c r="G6" s="16">
-        <f>=(C6+D6+E6)-F6</f>
+        <f>(C6+D6+E6)-F6</f>
       </c>
       <c r="H6" s="17">
         <v>0</v>
@@ -1902,10 +1902,10 @@
         <v>0</v>
       </c>
       <c r="J6" s="19">
-        <f>=C6+D6</f>
+        <f>C6+D6</f>
       </c>
       <c r="K6" s="20">
-        <f>=(C6+D6)/G6</f>
+        <f>(C6+D6)/G6</f>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
@@ -1925,19 +1925,19 @@
         <v>243800</v>
       </c>
       <c r="G7" s="16">
-        <f>=(C7+D7+E7)-F7</f>
+        <f>(C7+D7+E7)-F7</f>
       </c>
       <c r="H7" s="23">
-        <f>=G7-G6</f>
+        <f>G7-G6</f>
       </c>
       <c r="I7" s="24">
-        <f>=(G7-G6)/G6</f>
+        <f>(G7-G6)/G6</f>
       </c>
       <c r="J7" s="19">
-        <f>=C7+D7</f>
+        <f>C7+D7</f>
       </c>
       <c r="K7" s="25">
-        <f>=(C7+D7)/G7</f>
+        <f>(C7+D7)/G7</f>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
@@ -1957,19 +1957,19 @@
         <v>242600</v>
       </c>
       <c r="G8" s="16">
-        <f>=(C8+D8+E8)-F8</f>
+        <f>(C8+D8+E8)-F8</f>
       </c>
       <c r="H8" s="17">
-        <f>=G8-G7</f>
+        <f>G8-G7</f>
       </c>
       <c r="I8" s="18">
-        <f>=(G8-G7)/G7</f>
+        <f>(G8-G7)/G7</f>
       </c>
       <c r="J8" s="19">
-        <f>=C8+D8</f>
+        <f>C8+D8</f>
       </c>
       <c r="K8" s="20">
-        <f>=(C8+D8)/G8</f>
+        <f>(C8+D8)/G8</f>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
@@ -1989,19 +1989,19 @@
         <v>241400</v>
       </c>
       <c r="G9" s="16">
-        <f>=(C9+D9+E9)-F9</f>
+        <f>(C9+D9+E9)-F9</f>
       </c>
       <c r="H9" s="23">
-        <f>=G9-G8</f>
+        <f>G9-G8</f>
       </c>
       <c r="I9" s="24">
-        <f>=(G9-G8)/G8</f>
+        <f>(G9-G8)/G8</f>
       </c>
       <c r="J9" s="19">
-        <f>=C9+D9</f>
+        <f>C9+D9</f>
       </c>
       <c r="K9" s="25">
-        <f>=(C9+D9)/G9</f>
+        <f>(C9+D9)/G9</f>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
@@ -2021,19 +2021,19 @@
         <v>240100</v>
       </c>
       <c r="G10" s="16">
-        <f>=(C10+D10+E10)-F10</f>
+        <f>(C10+D10+E10)-F10</f>
       </c>
       <c r="H10" s="17">
-        <f>=G10-G9</f>
+        <f>G10-G9</f>
       </c>
       <c r="I10" s="18">
-        <f>=(G10-G9)/G9</f>
+        <f>(G10-G9)/G9</f>
       </c>
       <c r="J10" s="19">
-        <f>=C10+D10</f>
+        <f>C10+D10</f>
       </c>
       <c r="K10" s="20">
-        <f>=(C10+D10)/G10</f>
+        <f>(C10+D10)/G10</f>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
@@ -2053,19 +2053,19 @@
         <v>238800</v>
       </c>
       <c r="G11" s="16">
-        <f>=(C11+D11+E11)-F11</f>
+        <f>(C11+D11+E11)-F11</f>
       </c>
       <c r="H11" s="23">
-        <f>=G11-G10</f>
+        <f>G11-G10</f>
       </c>
       <c r="I11" s="24">
-        <f>=(G11-G10)/G10</f>
+        <f>(G11-G10)/G10</f>
       </c>
       <c r="J11" s="19">
-        <f>=C11+D11</f>
+        <f>C11+D11</f>
       </c>
       <c r="K11" s="25">
-        <f>=(C11+D11)/G11</f>
+        <f>(C11+D11)/G11</f>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
@@ -2085,19 +2085,19 @@
         <v>237500</v>
       </c>
       <c r="G12" s="16">
-        <f>=(C12+D12+E12)-F12</f>
+        <f>(C12+D12+E12)-F12</f>
       </c>
       <c r="H12" s="17">
-        <f>=G12-G11</f>
+        <f>G12-G11</f>
       </c>
       <c r="I12" s="18">
-        <f>=(G12-G11)/G11</f>
+        <f>(G12-G11)/G11</f>
       </c>
       <c r="J12" s="19">
-        <f>=C12+D12</f>
+        <f>C12+D12</f>
       </c>
       <c r="K12" s="20">
-        <f>=(C12+D12)/G12</f>
+        <f>(C12+D12)/G12</f>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
@@ -2117,19 +2117,19 @@
         <v>236100</v>
       </c>
       <c r="G13" s="16">
-        <f>=(C13+D13+E13)-F13</f>
+        <f>(C13+D13+E13)-F13</f>
       </c>
       <c r="H13" s="23">
-        <f>=G13-G12</f>
+        <f>G13-G12</f>
       </c>
       <c r="I13" s="24">
-        <f>=(G13-G12)/G12</f>
+        <f>(G13-G12)/G12</f>
       </c>
       <c r="J13" s="19">
-        <f>=C13+D13</f>
+        <f>C13+D13</f>
       </c>
       <c r="K13" s="25">
-        <f>=(C13+D13)/G13</f>
+        <f>(C13+D13)/G13</f>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
@@ -2149,19 +2149,19 @@
         <v>234700</v>
       </c>
       <c r="G14" s="16">
-        <f>=(C14+D14+E14)-F14</f>
+        <f>(C14+D14+E14)-F14</f>
       </c>
       <c r="H14" s="17">
-        <f>=G14-G13</f>
+        <f>G14-G13</f>
       </c>
       <c r="I14" s="18">
-        <f>=(G14-G13)/G13</f>
+        <f>(G14-G13)/G13</f>
       </c>
       <c r="J14" s="19">
-        <f>=C14+D14</f>
+        <f>C14+D14</f>
       </c>
       <c r="K14" s="20">
-        <f>=(C14+D14)/G14</f>
+        <f>(C14+D14)/G14</f>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
@@ -2181,19 +2181,19 @@
         <v>233200</v>
       </c>
       <c r="G15" s="16">
-        <f>=(C15+D15+E15)-F15</f>
+        <f>(C15+D15+E15)-F15</f>
       </c>
       <c r="H15" s="23">
-        <f>=G15-G14</f>
+        <f>G15-G14</f>
       </c>
       <c r="I15" s="24">
-        <f>=(G15-G14)/G14</f>
+        <f>(G15-G14)/G14</f>
       </c>
       <c r="J15" s="19">
-        <f>=C15+D15</f>
+        <f>C15+D15</f>
       </c>
       <c r="K15" s="25">
-        <f>=(C15+D15)/G15</f>
+        <f>(C15+D15)/G15</f>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
@@ -2213,19 +2213,19 @@
         <v>231700</v>
       </c>
       <c r="G16" s="16">
-        <f>=(C16+D16+E16)-F16</f>
+        <f>(C16+D16+E16)-F16</f>
       </c>
       <c r="H16" s="17">
-        <f>=G16-G15</f>
+        <f>G16-G15</f>
       </c>
       <c r="I16" s="18">
-        <f>=(G16-G15)/G15</f>
+        <f>(G16-G15)/G15</f>
       </c>
       <c r="J16" s="19">
-        <f>=C16+D16</f>
+        <f>C16+D16</f>
       </c>
       <c r="K16" s="20">
-        <f>=(C16+D16)/G16</f>
+        <f>(C16+D16)/G16</f>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
@@ -2245,19 +2245,19 @@
         <v>230100</v>
       </c>
       <c r="G17" s="16">
-        <f>=(C17+D17+E17)-F17</f>
+        <f>(C17+D17+E17)-F17</f>
       </c>
       <c r="H17" s="23">
-        <f>=G17-G16</f>
+        <f>G17-G16</f>
       </c>
       <c r="I17" s="24">
-        <f>=(G17-G16)/G16</f>
+        <f>(G17-G16)/G16</f>
       </c>
       <c r="J17" s="19">
-        <f>=C17+D17</f>
+        <f>C17+D17</f>
       </c>
       <c r="K17" s="25">
-        <f>=(C17+D17)/G17</f>
+        <f>(C17+D17)/G17</f>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
@@ -2265,31 +2265,31 @@
         <v>62</v>
       </c>
       <c r="C18" s="27">
-        <f>=C17</f>
+        <f>C17</f>
       </c>
       <c r="D18" s="27">
-        <f>=D17</f>
+        <f>D17</f>
       </c>
       <c r="E18" s="27">
-        <f>=E17</f>
+        <f>E17</f>
       </c>
       <c r="F18" s="27">
-        <f>=F17</f>
+        <f>F17</f>
       </c>
       <c r="G18" s="27">
-        <f>=G17</f>
+        <f>G17</f>
       </c>
       <c r="H18" s="27">
-        <f>=G17-G6</f>
+        <f>G17-G6</f>
       </c>
       <c r="I18" s="28">
-        <f>=(G17-G6)/G6</f>
+        <f>(G17-G6)/G6</f>
       </c>
       <c r="J18" s="27">
-        <f>=C17+D17</f>
+        <f>C17+D17</f>
       </c>
       <c r="K18" s="28">
-        <f>=(C17+D17)/G17</f>
+        <f>(C17+D17)/G17</f>
       </c>
     </row>
   </sheetData>
@@ -2347,11 +2347,11 @@
     </row>
     <row r="6" ht="28" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="32">
-        <f>='⚡ 2-Min Quick Check-In'!G18</f>
+        <f>'2-Min Check-In'!G18</f>
       </c>
       <c r="C6" s="32"/>
       <c r="D6" s="33">
-        <f>='⚡ 2-Min Quick Check-In'!C18+'⚡ 2-Min Quick Check-In'!D18</f>
+        <f>'2-Min Check-In'!C18+'2-Min Check-In'!D18</f>
       </c>
       <c r="E6" s="33"/>
       <c r="F6" s="34" t="s">
@@ -2360,11 +2360,11 @@
     </row>
     <row r="7" ht="16" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" s="35">
-        <f>="▲ Annual Growth: " &amp; TEXT('⚡ 2-Min Quick Check-In'!I18, "+0.0%") &amp; " (+$" &amp; TEXT('⚡ 2-Min Quick Check-In'!H18, "#,##0") &amp; ")"</f>
+        <f>"▲ Annual Growth: " &amp; TEXT('2-Min Check-In'!I18, "+0.0%") &amp; " (+$" &amp; TEXT('2-Min Check-In'!H18, "#,##0") &amp; ")"</f>
       </c>
       <c r="C7" s="35"/>
       <c r="D7" s="36">
-        <f>="Liquid Ratio: " &amp; TEXT(('⚡ 2-Min Quick Check-In'!C18+'⚡ 2-Min Quick Check-In'!D18)/('⚡ 2-Min Quick Check-In'!G18+'⚡ 2-Min Quick Check-In'!F18), "0.0%") &amp; " of total assets"</f>
+        <f>"Liquid Ratio: " &amp; TEXT(('2-Min Check-In'!C18+'2-Min Check-In'!D18)/('2-Min Check-In'!G18+'2-Min Check-In'!F18), "0.0%") &amp; " of total assets"</f>
       </c>
       <c r="E7" s="36"/>
       <c r="F7" s="36" t="s">
@@ -2402,13 +2402,13 @@
         <v>76</v>
       </c>
       <c r="C11" s="15">
-        <f>='⚡ 2-Min Quick Check-In'!G6</f>
+        <f>'2-Min Check-In'!G6</f>
       </c>
       <c r="D11" s="15">
-        <f>='⚡ 2-Min Quick Check-In'!D6</f>
+        <f>'2-Min Check-In'!D6</f>
       </c>
       <c r="E11" s="15">
-        <f>='⚡ 2-Min Quick Check-In'!F6</f>
+        <f>'2-Min Check-In'!F6</f>
       </c>
       <c r="F11" s="6" t="s">
         <v>77</v>
@@ -2419,13 +2419,13 @@
         <v>78</v>
       </c>
       <c r="C12" s="22">
-        <f>='⚡ 2-Min Quick Check-In'!G9</f>
+        <f>'2-Min Check-In'!G9</f>
       </c>
       <c r="D12" s="22">
-        <f>='⚡ 2-Min Quick Check-In'!D9</f>
+        <f>'2-Min Check-In'!D9</f>
       </c>
       <c r="E12" s="22">
-        <f>='⚡ 2-Min Quick Check-In'!F9</f>
+        <f>'2-Min Check-In'!F9</f>
       </c>
       <c r="F12" s="39" t="s">
         <v>79</v>
@@ -2436,13 +2436,13 @@
         <v>80</v>
       </c>
       <c r="C13" s="15">
-        <f>='⚡ 2-Min Quick Check-In'!G12</f>
+        <f>'2-Min Check-In'!G12</f>
       </c>
       <c r="D13" s="15">
-        <f>='⚡ 2-Min Quick Check-In'!D12</f>
+        <f>'2-Min Check-In'!D12</f>
       </c>
       <c r="E13" s="15">
-        <f>='⚡ 2-Min Quick Check-In'!F12</f>
+        <f>'2-Min Check-In'!F12</f>
       </c>
       <c r="F13" s="6" t="s">
         <v>81</v>
@@ -2453,13 +2453,13 @@
         <v>82</v>
       </c>
       <c r="C14" s="22">
-        <f>='⚡ 2-Min Quick Check-In'!G15</f>
+        <f>'2-Min Check-In'!G15</f>
       </c>
       <c r="D14" s="22">
-        <f>='⚡ 2-Min Quick Check-In'!D15</f>
+        <f>'2-Min Check-In'!D15</f>
       </c>
       <c r="E14" s="22">
-        <f>='⚡ 2-Min Quick Check-In'!F15</f>
+        <f>'2-Min Check-In'!F15</f>
       </c>
       <c r="F14" s="39" t="s">
         <v>83</v>
@@ -2470,13 +2470,13 @@
         <v>84</v>
       </c>
       <c r="C15" s="15">
-        <f>='⚡ 2-Min Quick Check-In'!G17</f>
+        <f>'2-Min Check-In'!G17</f>
       </c>
       <c r="D15" s="15">
-        <f>='⚡ 2-Min Quick Check-In'!D17</f>
+        <f>'2-Min Check-In'!D17</f>
       </c>
       <c r="E15" s="15">
-        <f>='⚡ 2-Min Quick Check-In'!F17</f>
+        <f>'2-Min Check-In'!F17</f>
       </c>
       <c r="F15" s="6" t="s">
         <v>85</v>
@@ -2555,13 +2555,13 @@
         <v>108000</v>
       </c>
       <c r="D24" s="46">
-        <f>=(B24*C24)/10</f>
+        <f>(B24*C24)/10</f>
       </c>
       <c r="E24" s="47">
-        <f>='⚡ 2-Min Quick Check-In'!G18/D24</f>
+        <f>'2-Min Check-In'!G18/D24</f>
       </c>
       <c r="F24" s="48">
-        <f>=IF('⚡ 2-Min Quick Check-In'!G18&gt;=2*D24, "🏆 PAW (Top 10% Accumulator)", IF('⚡ 2-Min Quick Check-In'!G18&gt;=D24, "⚡ AAW (Solid Average)", "⚠️ UAW (Under Accumulator)"))</f>
+        <f>IF('⚡ 2-Min Quick Check-In'!G18&gt;=2*D24, "🏆 PAW (Top 10% Accumulator)", IF('⚡ 2-Min Quick Check-In'!G18&gt;=D24, "⚡ AAW (Solid Average)", "⚠️ UAW (Under Accumulator)"))</f>
       </c>
     </row>
     <row r="26" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
@@ -2598,10 +2598,10 @@
         <v>100000</v>
       </c>
       <c r="D28" s="51">
-        <f>=MIN(1, '⚡ 2-Min Quick Check-In'!G18/C28)</f>
+        <f>MIN(1, '2-Min Check-In'!G18/C28)</f>
       </c>
       <c r="E28" s="50">
-        <f>=MAX(0, C28-'⚡ 2-Min Quick Check-In'!G18)</f>
+        <f>MAX(0, C28-'2-Min Check-In'!G18)</f>
       </c>
       <c r="F28" s="52" t="s">
         <v>108</v>
@@ -2615,10 +2615,10 @@
         <v>250000</v>
       </c>
       <c r="D29" s="55">
-        <f>=MIN(1, '⚡ 2-Min Quick Check-In'!G18/C29)</f>
+        <f>MIN(1, '2-Min Check-In'!G18/C29)</f>
       </c>
       <c r="E29" s="54">
-        <f>=MAX(0, C29-'⚡ 2-Min Quick Check-In'!G18)</f>
+        <f>MAX(0, C29-'2-Min Check-In'!G18)</f>
       </c>
       <c r="F29" s="56" t="s">
         <v>110</v>
@@ -2632,10 +2632,10 @@
         <v>500000</v>
       </c>
       <c r="D30" s="51">
-        <f>=MIN(1, '⚡ 2-Min Quick Check-In'!G18/C30)</f>
+        <f>MIN(1, '2-Min Check-In'!G18/C30)</f>
       </c>
       <c r="E30" s="50">
-        <f>=MAX(0, C30-'⚡ 2-Min Quick Check-In'!G18)</f>
+        <f>MAX(0, C30-'2-Min Check-In'!G18)</f>
       </c>
       <c r="F30" s="52" t="s">
         <v>112</v>
@@ -2649,10 +2649,10 @@
         <v>1000000</v>
       </c>
       <c r="D31" s="55">
-        <f>=MIN(1, '⚡ 2-Min Quick Check-In'!G18/C31)</f>
+        <f>MIN(1, '2-Min Check-In'!G18/C31)</f>
       </c>
       <c r="E31" s="54">
-        <f>=MAX(0, C31-'⚡ 2-Min Quick Check-In'!G18)</f>
+        <f>MAX(0, C31-'2-Min Check-In'!G18)</f>
       </c>
       <c r="F31" s="56" t="s">
         <v>114</v>
@@ -2686,16 +2686,16 @@
     </row>
     <row r="35" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B35" s="57">
-        <f>='⚡ 2-Min Quick Check-In'!C18+'⚡ 2-Min Quick Check-In'!D18</f>
+        <f>'2-Min Check-In'!C18+'2-Min Check-In'!D18</f>
       </c>
       <c r="C35" s="57">
-        <f>='💸 Smart Budget (50-30-20)'!C20</f>
+        <f>'Smart Budget (50-30-20)'!C20</f>
       </c>
       <c r="D35" s="58">
-        <f>=B35/C35</f>
+        <f>B35/C35</f>
       </c>
       <c r="E35" s="59">
-        <f>=B35/'⚡ 2-Min Quick Check-In'!G18</f>
+        <f>B35/'2-Min Check-In'!G18</f>
       </c>
       <c r="F35" s="60" t="s">
         <v>121</v>
@@ -2778,12 +2778,12 @@
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="62">
-        <f>=E24</f>
+        <f>E24</f>
       </c>
       <c r="C6" s="62"/>
       <c r="D6" s="62"/>
       <c r="E6" s="63">
-        <f>=E24/30</f>
+        <f>E24/30</f>
       </c>
       <c r="F6" s="63"/>
     </row>
@@ -2824,7 +2824,7 @@
         <v>6800</v>
       </c>
       <c r="E10" s="15">
-        <f>=D10-C10</f>
+        <f>D10-C10</f>
       </c>
       <c r="F10" s="6" t="s">
         <v>134</v>
@@ -2841,7 +2841,7 @@
         <v>2200</v>
       </c>
       <c r="E11" s="15">
-        <f>=D11-C11</f>
+        <f>D11-C11</f>
       </c>
       <c r="F11" s="6" t="s">
         <v>134</v>
@@ -2858,7 +2858,7 @@
         <v>650</v>
       </c>
       <c r="E12" s="15">
-        <f>=D12-C12</f>
+        <f>D12-C12</f>
       </c>
       <c r="F12" s="6" t="s">
         <v>134</v>
@@ -2869,13 +2869,13 @@
         <v>137</v>
       </c>
       <c r="C13" s="67">
-        <f>=SUM(C10:C12)</f>
+        <f>SUM(C10:C12)</f>
       </c>
       <c r="D13" s="67">
-        <f>=SUM(D10:D12)</f>
+        <f>SUM(D10:D12)</f>
       </c>
       <c r="E13" s="67">
-        <f>=D13-C13</f>
+        <f>D13-C13</f>
       </c>
       <c r="F13" s="66" t="s">
         <v>138</v>
@@ -2901,10 +2901,10 @@
         <v>2400</v>
       </c>
       <c r="E15" s="15">
-        <f>=C15-D15</f>
+        <f>C15-D15</f>
       </c>
       <c r="F15" s="6">
-        <f>=TEXT(D15/$D$13, "0.0%")</f>
+        <f>TEXT(D15/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
@@ -2918,10 +2918,10 @@
         <v>820</v>
       </c>
       <c r="E16" s="15">
-        <f>=C16-D16</f>
+        <f>C16-D16</f>
       </c>
       <c r="F16" s="6">
-        <f>=TEXT(D16/$D$13, "0.0%")</f>
+        <f>TEXT(D16/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
@@ -2935,10 +2935,10 @@
         <v>310</v>
       </c>
       <c r="E17" s="15">
-        <f>=C17-D17</f>
+        <f>C17-D17</f>
       </c>
       <c r="F17" s="6">
-        <f>=TEXT(D17/$D$13, "0.0%")</f>
+        <f>TEXT(D17/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
@@ -2952,10 +2952,10 @@
         <v>450</v>
       </c>
       <c r="E18" s="15">
-        <f>=C18-D18</f>
+        <f>C18-D18</f>
       </c>
       <c r="F18" s="6">
-        <f>=TEXT(D18/$D$13, "0.0%")</f>
+        <f>TEXT(D18/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
@@ -2969,10 +2969,10 @@
         <v>380</v>
       </c>
       <c r="E19" s="15">
-        <f>=C19-D19</f>
+        <f>C19-D19</f>
       </c>
       <c r="F19" s="6">
-        <f>=TEXT(D19/$D$13, "0.0%")</f>
+        <f>TEXT(D19/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
@@ -2980,16 +2980,16 @@
         <v>145</v>
       </c>
       <c r="C20" s="70">
-        <f>=SUM(C15:C19)</f>
+        <f>SUM(C15:C19)</f>
       </c>
       <c r="D20" s="70">
-        <f>=SUM(D15:D19)</f>
+        <f>SUM(D15:D19)</f>
       </c>
       <c r="E20" s="70">
-        <f>=C20-D20</f>
+        <f>C20-D20</f>
       </c>
       <c r="F20" s="69">
-        <f>="Actual: " &amp; TEXT(D20/D13, "0.0%") &amp; " (Target: ≤50%)"</f>
+        <f>"Actual: " &amp; TEXT(D20/D13, "0.0%") &amp; " (Target: ≤50%)"</f>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
@@ -3012,10 +3012,10 @@
         <v>520</v>
       </c>
       <c r="E22" s="15">
-        <f>=C22-D22</f>
+        <f>C22-D22</f>
       </c>
       <c r="F22" s="6">
-        <f>=TEXT(D22/$D$13, "0.0%")</f>
+        <f>TEXT(D22/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="23" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
@@ -3029,10 +3029,10 @@
         <v>115</v>
       </c>
       <c r="E23" s="15">
-        <f>=C23-D23</f>
+        <f>C23-D23</f>
       </c>
       <c r="F23" s="6">
-        <f>=TEXT(D23/$D$13, "0.0%")</f>
+        <f>TEXT(D23/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="24" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
@@ -3046,10 +3046,10 @@
         <v>380</v>
       </c>
       <c r="E24" s="15">
-        <f>=C24-D24</f>
+        <f>C24-D24</f>
       </c>
       <c r="F24" s="6">
-        <f>=TEXT(D24/$D$13, "0.0%")</f>
+        <f>TEXT(D24/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
@@ -3057,16 +3057,16 @@
         <v>150</v>
       </c>
       <c r="C25" s="73">
-        <f>=SUM(C22:C24)</f>
+        <f>SUM(C22:C24)</f>
       </c>
       <c r="D25" s="73">
-        <f>=SUM(D22:D24)</f>
+        <f>SUM(D22:D24)</f>
       </c>
       <c r="E25" s="73">
-        <f>=C25-D25</f>
+        <f>C25-D25</f>
       </c>
       <c r="F25" s="72">
-        <f>="Actual: " &amp; TEXT(D25/D13, "0.0%") &amp; " (Target: ≤30%)"</f>
+        <f>"Actual: " &amp; TEXT(D25/D13, "0.0%") &amp; " (Target: ≤30%)"</f>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
@@ -3089,10 +3089,10 @@
         <v>2200</v>
       </c>
       <c r="E27" s="15">
-        <f>=D27-C27</f>
+        <f>D27-C27</f>
       </c>
       <c r="F27" s="6">
-        <f>=TEXT(D27/$D$13, "0.0%")</f>
+        <f>TEXT(D27/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="28" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
@@ -3106,10 +3106,10 @@
         <v>500</v>
       </c>
       <c r="E28" s="15">
-        <f>=D28-C28</f>
+        <f>D28-C28</f>
       </c>
       <c r="F28" s="6">
-        <f>=TEXT(D28/$D$13, "0.0%")</f>
+        <f>TEXT(D28/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="29" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
@@ -3123,10 +3123,10 @@
         <v>750</v>
       </c>
       <c r="E29" s="15">
-        <f>=D29-C29</f>
+        <f>D29-C29</f>
       </c>
       <c r="F29" s="6">
-        <f>=TEXT(D29/$D$13, "0.0%")</f>
+        <f>TEXT(D29/$D$13, "0.0%")</f>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
@@ -3134,16 +3134,16 @@
         <v>155</v>
       </c>
       <c r="C30" s="75">
-        <f>=SUM(C27:C29)</f>
+        <f>SUM(C27:C29)</f>
       </c>
       <c r="D30" s="75">
-        <f>=SUM(D27:D29)</f>
+        <f>SUM(D27:D29)</f>
       </c>
       <c r="E30" s="75">
-        <f>=D30-C30</f>
+        <f>D30-C30</f>
       </c>
       <c r="F30" s="74">
-        <f>="Savings Rate: " &amp; TEXT(D30/D13, "0.0%") &amp; " (FIRE Speed)"</f>
+        <f>"Savings Rate: " &amp; TEXT(D30/D13, "0.0%") &amp; " (FIRE Speed)"</f>
       </c>
     </row>
   </sheetData>
@@ -3232,7 +3232,7 @@
         <v>21500</v>
       </c>
       <c r="E6" s="15">
-        <f>=C6-D6</f>
+        <f>C6-D6</f>
       </c>
       <c r="F6" s="6" t="s">
         <v>55</v>
@@ -3241,7 +3241,7 @@
         <v>700</v>
       </c>
       <c r="H6" s="20">
-        <f>=D6/C6</f>
+        <f>D6/C6</f>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -3255,7 +3255,7 @@
         <v>1400</v>
       </c>
       <c r="E7" s="22">
-        <f>=C7-D7</f>
+        <f>C7-D7</f>
       </c>
       <c r="F7" s="39" t="s">
         <v>57</v>
@@ -3264,7 +3264,7 @@
         <v>150</v>
       </c>
       <c r="H7" s="25">
-        <f>=D7/C7</f>
+        <f>D7/C7</f>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -3278,7 +3278,7 @@
         <v>2800</v>
       </c>
       <c r="E8" s="15">
-        <f>=C8-D8</f>
+        <f>C8-D8</f>
       </c>
       <c r="F8" s="6" t="s">
         <v>61</v>
@@ -3287,7 +3287,7 @@
         <v>250</v>
       </c>
       <c r="H8" s="20">
-        <f>=D8/C8</f>
+        <f>D8/C8</f>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -3301,7 +3301,7 @@
         <v>750</v>
       </c>
       <c r="E9" s="22">
-        <f>=C9-D9</f>
+        <f>C9-D9</f>
       </c>
       <c r="F9" s="39" t="s">
         <v>60</v>
@@ -3310,7 +3310,7 @@
         <v>125</v>
       </c>
       <c r="H9" s="25">
-        <f>=D9/C9</f>
+        <f>D9/C9</f>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -3324,7 +3324,7 @@
         <v>1800</v>
       </c>
       <c r="E10" s="15">
-        <f>=C10-D10</f>
+        <f>C10-D10</f>
       </c>
       <c r="F10" s="6" t="s">
         <v>59</v>
@@ -3333,7 +3333,7 @@
         <v>250</v>
       </c>
       <c r="H10" s="20">
-        <f>=D10/C10</f>
+        <f>D10/C10</f>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -3341,22 +3341,22 @@
         <v>170</v>
       </c>
       <c r="C11" s="27">
-        <f>=SUM(C6:C10)</f>
+        <f>SUM(C6:C10)</f>
       </c>
       <c r="D11" s="27">
-        <f>=SUM(D6:D10)</f>
+        <f>SUM(D6:D10)</f>
       </c>
       <c r="E11" s="27">
-        <f>=SUM(E6:E10)</f>
+        <f>SUM(E6:E10)</f>
       </c>
       <c r="F11" s="26" t="s">
         <v>171</v>
       </c>
       <c r="G11" s="27">
-        <f>=SUM(G6:G10)</f>
+        <f>SUM(G6:G10)</f>
       </c>
       <c r="H11" s="76">
-        <f>=D11/C11</f>
+        <f>D11/C11</f>
       </c>
     </row>
   </sheetData>
@@ -3435,7 +3435,7 @@
         <v>178</v>
       </c>
       <c r="C9" s="79">
-        <f>'⚡ 2-Min Quick Check-In'!D18</f>
+        <f>'2-Min Check-In'!D18</f>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
@@ -3443,7 +3443,7 @@
         <v>179</v>
       </c>
       <c r="C10" s="79">
-        <f>'💸 Smart Budget (50-30-20)'!D27</f>
+        <f>'Smart Budget (50-30-20)'!D27</f>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.25">
@@ -3622,13 +3622,13 @@
         <v>202</v>
       </c>
       <c r="C9" s="67">
-        <f>=SUM(C5:C8)</f>
+        <f>SUM(C5:C8)</f>
       </c>
       <c r="D9" s="83">
-        <f>=AVERAGE(D5:D8)</f>
+        <f>AVERAGE(D5:D8)</f>
       </c>
       <c r="E9" s="67">
-        <f>=SUM(E5:E8)</f>
+        <f>SUM(E5:E8)</f>
       </c>
       <c r="F9" s="66" t="s">
         <v>203</v>

</xml_diff>

<commit_message>
feat(vault): add 60-second instant dopamine test-drive, vampire purge and life energy engine to START HERE tab
</commit_message>
<xml_diff>
--- a/public/downloads/NetWorth_FIRE_Master_Vault_2026.xlsx
+++ b/public/downloads/NetWorth_FIRE_Master_Vault_2026.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="310">
   <si>
     <t>🏛️ GETNETWORTHCALCULATOR.COM • OFFICIAL WEALTH &amp; BUDGET OPERATING SYSTEM</t>
   </si>
@@ -132,6 +132,93 @@
   </si>
   <si>
     <t>🌐 GetNetWorthCalculator.com • 100% Private, Anonymous &amp; Offline • Official 2026 Edition</t>
+  </si>
+  <si>
+    <t>⚡ 60-SECOND INSTANT DOPAMINE TEST-DRIVE (GET IMMEDIATE WINS NOW)</t>
+  </si>
+  <si>
+    <t>Type 3 numbers into the green boxes below. Watch your official wealth tier and milestone unlock immediately!</t>
+  </si>
+  <si>
+    <t>1. YOUR CURRENT AGE</t>
+  </si>
+  <si>
+    <t>2. ANNUAL PRE-TAX INCOME</t>
+  </si>
+  <si>
+    <t>3. CURRENT ESTIMATED NET WORTH</t>
+  </si>
+  <si>
+    <t>🏆 OFFICIAL WEALTH TIER</t>
+  </si>
+  <si>
+    <t>🎯 TARGET NET WORTH FOR AGE</t>
+  </si>
+  <si>
+    <t>🚀 NEXT MILESTONE CLUB</t>
+  </si>
+  <si>
+    <t>🧛‍♂️ THE 5-MINUTE VAMPIRE PURGE (FIND $1,000+ IN CASH RIGHT NOW)</t>
+  </si>
+  <si>
+    <t>Recurring Monthly Leak / Subscription</t>
+  </si>
+  <si>
+    <t>Monthly Cost ($)</t>
+  </si>
+  <si>
+    <t>Action Plan &amp; Reality Check</t>
+  </si>
+  <si>
+    <t>Unused Streaming / Digital Subscriptions</t>
+  </si>
+  <si>
+    <t>Cancel unneeded services</t>
+  </si>
+  <si>
+    <t>Unused Gym / Health App Memberships</t>
+  </si>
+  <si>
+    <t>Downgrade or pause immediately</t>
+  </si>
+  <si>
+    <t>DoorDash / Takeout Delivery Markups &amp; Fees</t>
+  </si>
+  <si>
+    <t>Limit takeout to 1x weekly</t>
+  </si>
+  <si>
+    <t>Overpriced Cellphone / Insurance Plan</t>
+  </si>
+  <si>
+    <t>Shop rate or switch carrier</t>
+  </si>
+  <si>
+    <t>TOTAL RECURRENT LEAKAGE DISCOVERED</t>
+  </si>
+  <si>
+    <t>Found in your budget in 3 minutes</t>
+  </si>
+  <si>
+    <t>🟢 INSTANT ANNUAL CASH UNLOCKED</t>
+  </si>
+  <si>
+    <t>📈 10-YEAR COMPOUNDED WEALTH (8%)</t>
+  </si>
+  <si>
+    <t>⏳ THE LIFE ENERGY CALCULATOR (IS THAT PURCHASE WORTH YOUR FINITE HOURS?)</t>
+  </si>
+  <si>
+    <t>Your Real Hourly Wage (C30 / 2,080 hrs)</t>
+  </si>
+  <si>
+    <t>Impulse Purchase Price ($)</t>
+  </si>
+  <si>
+    <t>Actual Hours of Your Life It Costs</t>
+  </si>
+  <si>
+    <t>🚀 READY FOR YOUR 2-MINUTE MONTHLY ROUTINE? CLICK THE "2-Min Check-In" TAB BELOW! 👇</t>
   </si>
   <si>
     <t>⚡ 2-MINUTE MONTHLY QUICK CHECK-IN • GETNETWORTHCALCULATOR.COM</t>
@@ -867,17 +954,23 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="8">
+  <numFmts count="14">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
-    <numFmt numFmtId="165" formatCode="+$#,##0;-$#,##0;$0"/>
-    <numFmt numFmtId="166" formatCode="+0.0%;-0.0%;0.0%"/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
-    <numFmt numFmtId="168" formatCode="0.00&quot;x&quot;"/>
-    <numFmt numFmtId="169" formatCode="0.0&quot; Months&quot;"/>
-    <numFmt numFmtId="170" formatCode="$#,##0/day"/>
-    <numFmt numFmtId="171" formatCode="0.0&quot;x&quot;"/>
+    <numFmt numFmtId="165" formatCode="$#,##0&quot;/mo&quot;"/>
+    <numFmt numFmtId="166" formatCode="&quot;+$&quot;#,##0&quot; / Year Back In Checking&quot;"/>
+    <numFmt numFmtId="167" formatCode="&quot;+$&quot;#,##0&quot; Created For Retirement&quot;"/>
+    <numFmt numFmtId="168" formatCode="$#,##0.00&quot;/hr&quot;"/>
+    <numFmt numFmtId="169" formatCode="0.0&quot; Hours at Work&quot;"/>
+    <numFmt numFmtId="170" formatCode="+$#,##0;-$#,##0;$0"/>
+    <numFmt numFmtId="171" formatCode="+0.0%;-0.0%;0.0%"/>
+    <numFmt numFmtId="172" formatCode="0.0%"/>
+    <numFmt numFmtId="173" formatCode="&quot;+$&quot;#,##0;&quot;-$&quot;#,##0;&quot;$0&quot;"/>
+    <numFmt numFmtId="174" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="175" formatCode="0.0&quot; Months&quot;"/>
+    <numFmt numFmtId="176" formatCode="$#,##0/day"/>
+    <numFmt numFmtId="177" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
-  <fonts count="35" x14ac:knownFonts="1">
+  <fonts count="46" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -924,6 +1017,87 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF94A3B8"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF94A3B8"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF10B981"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFF59E0B"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10.5"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF64748B"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFF43F5E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="FF64748B"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF10B981"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF38BDF8"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF38BDF8"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="9.5"/>
       <name val="Arial"/>
     </font>
@@ -956,11 +1130,6 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF94A3B8"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="18"/>
     </font>
@@ -986,11 +1155,6 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
       <sz val="9"/>
     </font>
     <font>
@@ -1007,16 +1171,6 @@
       <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="10.5"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF10B981"/>
-      <sz val="12"/>
     </font>
     <font>
       <color rgb="FF475569"/>
@@ -1037,12 +1191,6 @@
       <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="15"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-      <name val="Arial"/>
     </font>
     <font>
       <i/>
@@ -1126,7 +1274,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1144,119 +1292,167 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="13" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="23" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="24" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="24" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="15" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="27" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="28" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="171" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="172" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="29" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="171" fontId="29" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="31" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="32" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="173" fontId="34" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="172" fontId="35" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="38" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="39" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="37" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="26" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="26" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="27" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="174" fontId="13" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="39" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="19" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="172" fontId="34" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="19" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="28" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="26" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="27" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="26" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="29" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="172" fontId="34" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="40" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="175" fontId="13" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="172" fontId="14" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="41" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="42" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="170" fontId="31" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="32" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="176" fontId="43" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="29" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="29" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="13" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="29" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="29" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="172" fontId="29" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="13" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="29" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="172" fontId="29" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="29" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="172" fontId="29" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="172" fontId="29" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="172" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="13" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="34" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="29" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="45" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="45" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="177" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1596,7 +1792,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:D24"/>
+  <dimension ref="B2:D51"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1777,8 +1973,193 @@
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
     </row>
+    <row r="26" ht="26" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B26" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+    </row>
+    <row r="27" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B27" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+    </row>
+    <row r="29" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B29" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="30" ht="26" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B30" s="13">
+        <v>30</v>
+      </c>
+      <c r="C30" s="14">
+        <v>95000</v>
+      </c>
+      <c r="D30" s="14">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B32" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="D32" s="15" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="33" ht="26" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B33" s="16">
+        <f>IF(D30&gt;=2*(B30*C30/10), "PAW (Top 10% Wealth Builder)", IF(D30&gt;=(B30*C30/10), "AAW (Solid Average)", "UAW (Under-Accumulator)"))</f>
+      </c>
+      <c r="C33" s="17">
+        <f>(B30*C30)/10</f>
+      </c>
+      <c r="D33" s="18">
+        <f>IF(D30&lt;100000, "$100k Club", IF(D30&lt;250000, "$250k Club", IF(D30&lt;500000, "$500k Club", "$1M Two-Comma Club")))</f>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B36" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C36" s="19"/>
+      <c r="D36" s="19"/>
+    </row>
+    <row r="37" ht="19" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B37" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="C37" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="D37" s="20" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="38" ht="19" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B38" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C38" s="21">
+        <v>35</v>
+      </c>
+      <c r="D38" s="22" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="39" ht="19" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B39" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C39" s="21">
+        <v>45</v>
+      </c>
+      <c r="D39" s="22" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="40" ht="19" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B40" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C40" s="21">
+        <v>75</v>
+      </c>
+      <c r="D40" s="22" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="41" ht="19" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B41" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C41" s="21">
+        <v>40</v>
+      </c>
+      <c r="D41" s="22" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B42" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C42" s="23">
+        <f>SUM(C38:C41)</f>
+      </c>
+      <c r="D42" s="24" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B44" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="C44" s="25"/>
+      <c r="D44" s="26" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="45" ht="26" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B45" s="27">
+        <f>C42*12</f>
+      </c>
+      <c r="C45" s="27"/>
+      <c r="D45" s="28">
+        <f>C42*182.946</f>
+      </c>
+    </row>
+    <row r="47" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B47" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="C47" s="19"/>
+      <c r="D47" s="19"/>
+    </row>
+    <row r="48" ht="19" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B48" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="C48" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="D48" s="20" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="49" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B49" s="29">
+        <f>C30/2080</f>
+      </c>
+      <c r="C49" s="30">
+        <v>1200</v>
+      </c>
+      <c r="D49" s="31">
+        <f>C49/B49</f>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B51" s="32" t="s">
+        <v>66</v>
+      </c>
+      <c r="C51" s="32"/>
+      <c r="D51" s="32"/>
+    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="20">
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="B5:D5"/>
@@ -1792,6 +2173,13 @@
     <mergeCell ref="C21:D21"/>
     <mergeCell ref="C22:D22"/>
     <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="B51:D51"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1818,7 +2206,7 @@
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
-        <v>38</v>
+        <v>67</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -1831,464 +2219,464 @@
       <c r="K2" s="1"/>
     </row>
     <row r="3" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B3" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
+      <c r="B3" s="33" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="33"/>
+      <c r="G3" s="33"/>
+      <c r="H3" s="33"/>
+      <c r="I3" s="33"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="33"/>
     </row>
     <row r="5" ht="24" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B5" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="H5" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="I5" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="J5" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="K5" s="12" t="s">
-        <v>49</v>
+      <c r="B5" s="34" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="D5" s="35" t="s">
+        <v>71</v>
+      </c>
+      <c r="E5" s="35" t="s">
+        <v>72</v>
+      </c>
+      <c r="F5" s="35" t="s">
+        <v>73</v>
+      </c>
+      <c r="G5" s="34" t="s">
+        <v>74</v>
+      </c>
+      <c r="H5" s="34" t="s">
+        <v>75</v>
+      </c>
+      <c r="I5" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="J5" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="K5" s="34" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B6" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="C6" s="15">
+      <c r="B6" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="C6" s="37">
         <v>25000</v>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="37">
         <v>185000</v>
       </c>
-      <c r="E6" s="15">
+      <c r="E6" s="37">
         <v>350000</v>
       </c>
-      <c r="F6" s="15">
+      <c r="F6" s="37">
         <v>245000</v>
       </c>
-      <c r="G6" s="16">
+      <c r="G6" s="38">
         <f>(C6+D6+E6)-F6</f>
       </c>
-      <c r="H6" s="17">
+      <c r="H6" s="39">
         <v>0</v>
       </c>
-      <c r="I6" s="18">
+      <c r="I6" s="40">
         <v>0</v>
       </c>
-      <c r="J6" s="19">
+      <c r="J6" s="41">
         <f>C6+D6</f>
       </c>
-      <c r="K6" s="20">
+      <c r="K6" s="42">
         <f>(C6+D6)/G6</f>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B7" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="C7" s="22">
+      <c r="B7" s="43" t="s">
+        <v>80</v>
+      </c>
+      <c r="C7" s="44">
         <v>26200</v>
       </c>
-      <c r="D7" s="22">
+      <c r="D7" s="44">
         <v>189500</v>
       </c>
-      <c r="E7" s="22">
+      <c r="E7" s="44">
         <v>350000</v>
       </c>
-      <c r="F7" s="22">
+      <c r="F7" s="44">
         <v>243800</v>
       </c>
-      <c r="G7" s="16">
+      <c r="G7" s="38">
         <f>(C7+D7+E7)-F7</f>
       </c>
-      <c r="H7" s="23">
+      <c r="H7" s="45">
         <f>G7-G6</f>
       </c>
-      <c r="I7" s="24">
+      <c r="I7" s="46">
         <f>(G7-G6)/G6</f>
       </c>
-      <c r="J7" s="19">
+      <c r="J7" s="41">
         <f>C7+D7</f>
       </c>
-      <c r="K7" s="25">
+      <c r="K7" s="47">
         <f>(C7+D7)/G7</f>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B8" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="15">
+      <c r="B8" s="36" t="s">
+        <v>81</v>
+      </c>
+      <c r="C8" s="37">
         <v>25800</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="37">
         <v>194200</v>
       </c>
-      <c r="E8" s="15">
+      <c r="E8" s="37">
         <v>350000</v>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="37">
         <v>242600</v>
       </c>
-      <c r="G8" s="16">
+      <c r="G8" s="38">
         <f>(C8+D8+E8)-F8</f>
       </c>
-      <c r="H8" s="17">
+      <c r="H8" s="39">
         <f>G8-G7</f>
       </c>
-      <c r="I8" s="18">
+      <c r="I8" s="40">
         <f>(G8-G7)/G7</f>
       </c>
-      <c r="J8" s="19">
+      <c r="J8" s="41">
         <f>C8+D8</f>
       </c>
-      <c r="K8" s="20">
+      <c r="K8" s="42">
         <f>(C8+D8)/G8</f>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B9" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="C9" s="22">
+      <c r="B9" s="43" t="s">
+        <v>82</v>
+      </c>
+      <c r="C9" s="44">
         <v>27100</v>
       </c>
-      <c r="D9" s="22">
+      <c r="D9" s="44">
         <v>191000</v>
       </c>
-      <c r="E9" s="22">
+      <c r="E9" s="44">
         <v>350000</v>
       </c>
-      <c r="F9" s="22">
+      <c r="F9" s="44">
         <v>241400</v>
       </c>
-      <c r="G9" s="16">
+      <c r="G9" s="38">
         <f>(C9+D9+E9)-F9</f>
       </c>
-      <c r="H9" s="23">
+      <c r="H9" s="45">
         <f>G9-G8</f>
       </c>
-      <c r="I9" s="24">
+      <c r="I9" s="46">
         <f>(G9-G8)/G8</f>
       </c>
-      <c r="J9" s="19">
+      <c r="J9" s="41">
         <f>C9+D9</f>
       </c>
-      <c r="K9" s="25">
+      <c r="K9" s="47">
         <f>(C9+D9)/G9</f>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B10" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="C10" s="15">
+      <c r="B10" s="36" t="s">
+        <v>83</v>
+      </c>
+      <c r="C10" s="37">
         <v>26900</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="37">
         <v>198500</v>
       </c>
-      <c r="E10" s="15">
+      <c r="E10" s="37">
         <v>352000</v>
       </c>
-      <c r="F10" s="15">
+      <c r="F10" s="37">
         <v>240100</v>
       </c>
-      <c r="G10" s="16">
+      <c r="G10" s="38">
         <f>(C10+D10+E10)-F10</f>
       </c>
-      <c r="H10" s="17">
+      <c r="H10" s="39">
         <f>G10-G9</f>
       </c>
-      <c r="I10" s="18">
+      <c r="I10" s="40">
         <f>(G10-G9)/G9</f>
       </c>
-      <c r="J10" s="19">
+      <c r="J10" s="41">
         <f>C10+D10</f>
       </c>
-      <c r="K10" s="20">
+      <c r="K10" s="42">
         <f>(C10+D10)/G10</f>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B11" s="21" t="s">
-        <v>55</v>
-      </c>
-      <c r="C11" s="22">
+      <c r="B11" s="43" t="s">
+        <v>84</v>
+      </c>
+      <c r="C11" s="44">
         <v>28400</v>
       </c>
-      <c r="D11" s="22">
+      <c r="D11" s="44">
         <v>204000</v>
       </c>
-      <c r="E11" s="22">
+      <c r="E11" s="44">
         <v>352000</v>
       </c>
-      <c r="F11" s="22">
+      <c r="F11" s="44">
         <v>238800</v>
       </c>
-      <c r="G11" s="16">
+      <c r="G11" s="38">
         <f>(C11+D11+E11)-F11</f>
       </c>
-      <c r="H11" s="23">
+      <c r="H11" s="45">
         <f>G11-G10</f>
       </c>
-      <c r="I11" s="24">
+      <c r="I11" s="46">
         <f>(G11-G10)/G10</f>
       </c>
-      <c r="J11" s="19">
+      <c r="J11" s="41">
         <f>C11+D11</f>
       </c>
-      <c r="K11" s="25">
+      <c r="K11" s="47">
         <f>(C11+D11)/G11</f>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B12" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="C12" s="15">
+      <c r="B12" s="36" t="s">
+        <v>85</v>
+      </c>
+      <c r="C12" s="37">
         <v>29000</v>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="37">
         <v>209500</v>
       </c>
-      <c r="E12" s="15">
+      <c r="E12" s="37">
         <v>352000</v>
       </c>
-      <c r="F12" s="15">
+      <c r="F12" s="37">
         <v>237500</v>
       </c>
-      <c r="G12" s="16">
+      <c r="G12" s="38">
         <f>(C12+D12+E12)-F12</f>
       </c>
-      <c r="H12" s="17">
+      <c r="H12" s="39">
         <f>G12-G11</f>
       </c>
-      <c r="I12" s="18">
+      <c r="I12" s="40">
         <f>(G12-G11)/G11</f>
       </c>
-      <c r="J12" s="19">
+      <c r="J12" s="41">
         <f>C12+D12</f>
       </c>
-      <c r="K12" s="20">
+      <c r="K12" s="42">
         <f>(C12+D12)/G12</f>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B13" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="C13" s="22">
+      <c r="B13" s="43" t="s">
+        <v>86</v>
+      </c>
+      <c r="C13" s="44">
         <v>28500</v>
       </c>
-      <c r="D13" s="22">
+      <c r="D13" s="44">
         <v>215000</v>
       </c>
-      <c r="E13" s="22">
+      <c r="E13" s="44">
         <v>355000</v>
       </c>
-      <c r="F13" s="22">
+      <c r="F13" s="44">
         <v>236100</v>
       </c>
-      <c r="G13" s="16">
+      <c r="G13" s="38">
         <f>(C13+D13+E13)-F13</f>
       </c>
-      <c r="H13" s="23">
+      <c r="H13" s="45">
         <f>G13-G12</f>
       </c>
-      <c r="I13" s="24">
+      <c r="I13" s="46">
         <f>(G13-G12)/G12</f>
       </c>
-      <c r="J13" s="19">
+      <c r="J13" s="41">
         <f>C13+D13</f>
       </c>
-      <c r="K13" s="25">
+      <c r="K13" s="47">
         <f>(C13+D13)/G13</f>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B14" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="C14" s="15">
+      <c r="B14" s="36" t="s">
+        <v>87</v>
+      </c>
+      <c r="C14" s="37">
         <v>30200</v>
       </c>
-      <c r="D14" s="15">
+      <c r="D14" s="37">
         <v>221000</v>
       </c>
-      <c r="E14" s="15">
+      <c r="E14" s="37">
         <v>355000</v>
       </c>
-      <c r="F14" s="15">
+      <c r="F14" s="37">
         <v>234700</v>
       </c>
-      <c r="G14" s="16">
+      <c r="G14" s="38">
         <f>(C14+D14+E14)-F14</f>
       </c>
-      <c r="H14" s="17">
+      <c r="H14" s="39">
         <f>G14-G13</f>
       </c>
-      <c r="I14" s="18">
+      <c r="I14" s="40">
         <f>(G14-G13)/G13</f>
       </c>
-      <c r="J14" s="19">
+      <c r="J14" s="41">
         <f>C14+D14</f>
       </c>
-      <c r="K14" s="20">
+      <c r="K14" s="42">
         <f>(C14+D14)/G14</f>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B15" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="C15" s="22">
+      <c r="B15" s="43" t="s">
+        <v>88</v>
+      </c>
+      <c r="C15" s="44">
         <v>31000</v>
       </c>
-      <c r="D15" s="22">
+      <c r="D15" s="44">
         <v>228000</v>
       </c>
-      <c r="E15" s="22">
+      <c r="E15" s="44">
         <v>355000</v>
       </c>
-      <c r="F15" s="22">
+      <c r="F15" s="44">
         <v>233200</v>
       </c>
-      <c r="G15" s="16">
+      <c r="G15" s="38">
         <f>(C15+D15+E15)-F15</f>
       </c>
-      <c r="H15" s="23">
+      <c r="H15" s="45">
         <f>G15-G14</f>
       </c>
-      <c r="I15" s="24">
+      <c r="I15" s="46">
         <f>(G15-G14)/G14</f>
       </c>
-      <c r="J15" s="19">
+      <c r="J15" s="41">
         <f>C15+D15</f>
       </c>
-      <c r="K15" s="25">
+      <c r="K15" s="47">
         <f>(C15+D15)/G15</f>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B16" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C16" s="15">
+      <c r="B16" s="36" t="s">
+        <v>89</v>
+      </c>
+      <c r="C16" s="37">
         <v>31500</v>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="37">
         <v>234500</v>
       </c>
-      <c r="E16" s="15">
+      <c r="E16" s="37">
         <v>358000</v>
       </c>
-      <c r="F16" s="15">
+      <c r="F16" s="37">
         <v>231700</v>
       </c>
-      <c r="G16" s="16">
+      <c r="G16" s="38">
         <f>(C16+D16+E16)-F16</f>
       </c>
-      <c r="H16" s="17">
+      <c r="H16" s="39">
         <f>G16-G15</f>
       </c>
-      <c r="I16" s="18">
+      <c r="I16" s="40">
         <f>(G16-G15)/G15</f>
       </c>
-      <c r="J16" s="19">
+      <c r="J16" s="41">
         <f>C16+D16</f>
       </c>
-      <c r="K16" s="20">
+      <c r="K16" s="42">
         <f>(C16+D16)/G16</f>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B17" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="C17" s="22">
+      <c r="B17" s="43" t="s">
+        <v>90</v>
+      </c>
+      <c r="C17" s="44">
         <v>33000</v>
       </c>
-      <c r="D17" s="22">
+      <c r="D17" s="44">
         <v>242000</v>
       </c>
-      <c r="E17" s="22">
+      <c r="E17" s="44">
         <v>358000</v>
       </c>
-      <c r="F17" s="22">
+      <c r="F17" s="44">
         <v>230100</v>
       </c>
-      <c r="G17" s="16">
+      <c r="G17" s="38">
         <f>(C17+D17+E17)-F17</f>
       </c>
-      <c r="H17" s="23">
+      <c r="H17" s="45">
         <f>G17-G16</f>
       </c>
-      <c r="I17" s="24">
+      <c r="I17" s="46">
         <f>(G17-G16)/G16</f>
       </c>
-      <c r="J17" s="19">
+      <c r="J17" s="41">
         <f>C17+D17</f>
       </c>
-      <c r="K17" s="25">
+      <c r="K17" s="47">
         <f>(C17+D17)/G17</f>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B18" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="C18" s="27">
+      <c r="B18" s="48" t="s">
+        <v>91</v>
+      </c>
+      <c r="C18" s="49">
         <f>C17</f>
       </c>
-      <c r="D18" s="27">
+      <c r="D18" s="49">
         <f>D17</f>
       </c>
-      <c r="E18" s="27">
+      <c r="E18" s="49">
         <f>E17</f>
       </c>
-      <c r="F18" s="27">
+      <c r="F18" s="49">
         <f>F17</f>
       </c>
-      <c r="G18" s="27">
+      <c r="G18" s="49">
         <f>G17</f>
       </c>
-      <c r="H18" s="27">
+      <c r="H18" s="49">
         <f>G17-G6</f>
       </c>
-      <c r="I18" s="28">
+      <c r="I18" s="50">
         <f>(G17-G6)/G6</f>
       </c>
-      <c r="J18" s="27">
+      <c r="J18" s="49">
         <f>C17+D17</f>
       </c>
-      <c r="K18" s="28">
+      <c r="K18" s="50">
         <f>(C17+D17)/G17</f>
       </c>
     </row>
@@ -2315,400 +2703,400 @@
   </cols>
   <sheetData>
     <row r="2" ht="30" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="29" t="s">
-        <v>63</v>
-      </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
+      <c r="B2" s="51" t="s">
+        <v>92</v>
+      </c>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
+      <c r="B3" s="52" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" s="52"/>
+      <c r="D3" s="52"/>
+      <c r="E3" s="52"/>
+      <c r="F3" s="52"/>
     </row>
     <row r="5" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="31" t="s">
-        <v>65</v>
-      </c>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31" t="s">
-        <v>66</v>
-      </c>
-      <c r="E5" s="31"/>
-      <c r="F5" s="31" t="s">
-        <v>67</v>
+      <c r="B5" s="53" t="s">
+        <v>94</v>
+      </c>
+      <c r="C5" s="53"/>
+      <c r="D5" s="53" t="s">
+        <v>95</v>
+      </c>
+      <c r="E5" s="53"/>
+      <c r="F5" s="53" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="32">
+      <c r="B6" s="54">
         <f>'2-Min Check-In'!G18</f>
       </c>
-      <c r="C6" s="32"/>
-      <c r="D6" s="33">
+      <c r="C6" s="54"/>
+      <c r="D6" s="55">
         <f>'2-Min Check-In'!C18+'2-Min Check-In'!D18</f>
       </c>
-      <c r="E6" s="33"/>
-      <c r="F6" s="34" t="s">
-        <v>68</v>
+      <c r="E6" s="55"/>
+      <c r="F6" s="56" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="35">
-        <f>"▲ Annual Growth: " &amp; TEXT('2-Min Check-In'!I18, "+0.0%") &amp; " (+$" &amp; TEXT('2-Min Check-In'!H18, "#,##0") &amp; ")"</f>
-      </c>
-      <c r="C7" s="35"/>
-      <c r="D7" s="36">
-        <f>"Liquid Ratio: " &amp; TEXT(('2-Min Check-In'!C18+'2-Min Check-In'!D18)/('2-Min Check-In'!G18+'2-Min Check-In'!F18), "0.0%") &amp; " of total assets"</f>
-      </c>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36" t="s">
-        <v>69</v>
+      <c r="B7" s="57">
+        <f>'2-Min Check-In'!H18</f>
+      </c>
+      <c r="C7" s="57"/>
+      <c r="D7" s="58">
+        <f>('2-Min Check-In'!C18+'2-Min Check-In'!D18)/('2-Min Check-In'!G18+'2-Min Check-In'!F18)</f>
+      </c>
+      <c r="E7" s="58"/>
+      <c r="F7" s="59" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="37" t="s">
-        <v>70</v>
-      </c>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="37"/>
+      <c r="B9" s="60" t="s">
+        <v>99</v>
+      </c>
+      <c r="C9" s="60"/>
+      <c r="D9" s="60"/>
+      <c r="E9" s="60"/>
+      <c r="F9" s="60"/>
     </row>
     <row r="10" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B10" s="38" t="s">
-        <v>71</v>
-      </c>
-      <c r="C10" s="38" t="s">
-        <v>72</v>
-      </c>
-      <c r="D10" s="38" t="s">
-        <v>73</v>
-      </c>
-      <c r="E10" s="38" t="s">
-        <v>74</v>
-      </c>
-      <c r="F10" s="38" t="s">
-        <v>75</v>
+      <c r="B10" s="61" t="s">
+        <v>100</v>
+      </c>
+      <c r="C10" s="61" t="s">
+        <v>101</v>
+      </c>
+      <c r="D10" s="61" t="s">
+        <v>102</v>
+      </c>
+      <c r="E10" s="61" t="s">
+        <v>103</v>
+      </c>
+      <c r="F10" s="61" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C11" s="15">
+        <v>105</v>
+      </c>
+      <c r="C11" s="37">
         <f>'2-Min Check-In'!G6</f>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="37">
         <f>'2-Min Check-In'!D6</f>
       </c>
-      <c r="E11" s="15">
+      <c r="E11" s="37">
         <f>'2-Min Check-In'!F6</f>
       </c>
       <c r="F11" s="6" t="s">
-        <v>77</v>
+        <v>106</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B12" s="39" t="s">
-        <v>78</v>
-      </c>
-      <c r="C12" s="22">
+      <c r="B12" s="62" t="s">
+        <v>107</v>
+      </c>
+      <c r="C12" s="44">
         <f>'2-Min Check-In'!G9</f>
       </c>
-      <c r="D12" s="22">
+      <c r="D12" s="44">
         <f>'2-Min Check-In'!D9</f>
       </c>
-      <c r="E12" s="22">
+      <c r="E12" s="44">
         <f>'2-Min Check-In'!F9</f>
       </c>
-      <c r="F12" s="39" t="s">
-        <v>79</v>
+      <c r="F12" s="62" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="C13" s="15">
+        <v>109</v>
+      </c>
+      <c r="C13" s="37">
         <f>'2-Min Check-In'!G12</f>
       </c>
-      <c r="D13" s="15">
+      <c r="D13" s="37">
         <f>'2-Min Check-In'!D12</f>
       </c>
-      <c r="E13" s="15">
+      <c r="E13" s="37">
         <f>'2-Min Check-In'!F12</f>
       </c>
       <c r="F13" s="6" t="s">
-        <v>81</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="39" t="s">
-        <v>82</v>
-      </c>
-      <c r="C14" s="22">
+      <c r="B14" s="62" t="s">
+        <v>111</v>
+      </c>
+      <c r="C14" s="44">
         <f>'2-Min Check-In'!G15</f>
       </c>
-      <c r="D14" s="22">
+      <c r="D14" s="44">
         <f>'2-Min Check-In'!D15</f>
       </c>
-      <c r="E14" s="22">
+      <c r="E14" s="44">
         <f>'2-Min Check-In'!F15</f>
       </c>
-      <c r="F14" s="39" t="s">
-        <v>83</v>
+      <c r="F14" s="62" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="C15" s="15">
+        <v>113</v>
+      </c>
+      <c r="C15" s="37">
         <f>'2-Min Check-In'!G17</f>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="37">
         <f>'2-Min Check-In'!D17</f>
       </c>
-      <c r="E15" s="15">
+      <c r="E15" s="37">
         <f>'2-Min Check-In'!F17</f>
       </c>
       <c r="F15" s="6" t="s">
-        <v>85</v>
+        <v>114</v>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B18" s="37" t="s">
-        <v>86</v>
-      </c>
-      <c r="C18" s="37"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="37"/>
-      <c r="F18" s="37"/>
+      <c r="B18" s="60" t="s">
+        <v>115</v>
+      </c>
+      <c r="C18" s="60"/>
+      <c r="D18" s="60"/>
+      <c r="E18" s="60"/>
+      <c r="F18" s="60"/>
     </row>
     <row r="19" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B19" s="40" t="s">
-        <v>87</v>
-      </c>
-      <c r="C19" s="40" t="s">
-        <v>88</v>
-      </c>
-      <c r="D19" s="40" t="s">
-        <v>89</v>
-      </c>
-      <c r="E19" s="40" t="s">
-        <v>90</v>
-      </c>
-      <c r="F19" s="40"/>
+      <c r="B19" s="63" t="s">
+        <v>116</v>
+      </c>
+      <c r="C19" s="63" t="s">
+        <v>117</v>
+      </c>
+      <c r="D19" s="63" t="s">
+        <v>118</v>
+      </c>
+      <c r="E19" s="63" t="s">
+        <v>119</v>
+      </c>
+      <c r="F19" s="63"/>
     </row>
     <row r="20" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B20" s="41" t="s">
-        <v>91</v>
-      </c>
-      <c r="C20" s="41" t="s">
-        <v>92</v>
-      </c>
-      <c r="D20" s="41" t="s">
-        <v>93</v>
-      </c>
-      <c r="E20" s="41" t="s">
-        <v>94</v>
-      </c>
-      <c r="F20" s="41"/>
+      <c r="B20" s="64" t="s">
+        <v>120</v>
+      </c>
+      <c r="C20" s="64" t="s">
+        <v>121</v>
+      </c>
+      <c r="D20" s="64" t="s">
+        <v>122</v>
+      </c>
+      <c r="E20" s="64" t="s">
+        <v>123</v>
+      </c>
+      <c r="F20" s="64"/>
     </row>
     <row r="22" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B22" s="42" t="s">
-        <v>95</v>
-      </c>
-      <c r="C22" s="42"/>
-      <c r="D22" s="42"/>
-      <c r="E22" s="42"/>
-      <c r="F22" s="42"/>
+      <c r="B22" s="65" t="s">
+        <v>124</v>
+      </c>
+      <c r="C22" s="65"/>
+      <c r="D22" s="65"/>
+      <c r="E22" s="65"/>
+      <c r="F22" s="65"/>
     </row>
     <row r="23" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B23" s="43" t="s">
-        <v>96</v>
-      </c>
-      <c r="C23" s="43" t="s">
-        <v>97</v>
-      </c>
-      <c r="D23" s="43" t="s">
-        <v>98</v>
-      </c>
-      <c r="E23" s="43" t="s">
-        <v>99</v>
-      </c>
-      <c r="F23" s="43" t="s">
-        <v>100</v>
+      <c r="B23" s="66" t="s">
+        <v>125</v>
+      </c>
+      <c r="C23" s="66" t="s">
+        <v>126</v>
+      </c>
+      <c r="D23" s="66" t="s">
+        <v>127</v>
+      </c>
+      <c r="E23" s="66" t="s">
+        <v>128</v>
+      </c>
+      <c r="F23" s="66" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="24" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B24" s="44">
+      <c r="B24" s="67">
         <v>32</v>
       </c>
-      <c r="C24" s="45">
+      <c r="C24" s="68">
         <v>108000</v>
       </c>
-      <c r="D24" s="46">
+      <c r="D24" s="17">
         <f>(B24*C24)/10</f>
       </c>
-      <c r="E24" s="47">
+      <c r="E24" s="69">
         <f>'2-Min Check-In'!G18/D24</f>
       </c>
-      <c r="F24" s="48">
-        <f>IF('⚡ 2-Min Quick Check-In'!G18&gt;=2*D24, "🏆 PAW (Top 10% Accumulator)", IF('⚡ 2-Min Quick Check-In'!G18&gt;=D24, "⚡ AAW (Solid Average)", "⚠️ UAW (Under Accumulator)"))</f>
+      <c r="F24" s="70">
+        <f>IF('2-Min Check-In'!G18&gt;=2*D24, "PAW (Top 10% Accumulator)", IF('2-Min Check-In'!G18&gt;=D24, "AAW (Solid Average)", "UAW (Under Accumulator)"))</f>
       </c>
     </row>
     <row r="26" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B26" s="49" t="s">
-        <v>101</v>
-      </c>
-      <c r="C26" s="49"/>
-      <c r="D26" s="49"/>
-      <c r="E26" s="49"/>
-      <c r="F26" s="49"/>
+      <c r="B26" s="71" t="s">
+        <v>130</v>
+      </c>
+      <c r="C26" s="71"/>
+      <c r="D26" s="71"/>
+      <c r="E26" s="71"/>
+      <c r="F26" s="71"/>
     </row>
     <row r="27" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B27" s="43" t="s">
-        <v>102</v>
-      </c>
-      <c r="C27" s="43" t="s">
-        <v>103</v>
-      </c>
-      <c r="D27" s="43" t="s">
-        <v>104</v>
-      </c>
-      <c r="E27" s="43" t="s">
-        <v>105</v>
-      </c>
-      <c r="F27" s="43" t="s">
-        <v>106</v>
+      <c r="B27" s="66" t="s">
+        <v>131</v>
+      </c>
+      <c r="C27" s="66" t="s">
+        <v>132</v>
+      </c>
+      <c r="D27" s="66" t="s">
+        <v>133</v>
+      </c>
+      <c r="E27" s="66" t="s">
+        <v>134</v>
+      </c>
+      <c r="F27" s="66" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="28" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="C28" s="50">
+        <v>136</v>
+      </c>
+      <c r="C28" s="72">
         <v>100000</v>
       </c>
-      <c r="D28" s="51">
+      <c r="D28" s="73">
         <f>MIN(1, '2-Min Check-In'!G18/C28)</f>
       </c>
-      <c r="E28" s="50">
+      <c r="E28" s="72">
         <f>MAX(0, C28-'2-Min Check-In'!G18)</f>
       </c>
-      <c r="F28" s="52" t="s">
-        <v>108</v>
+      <c r="F28" s="74" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="29" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B29" s="53" t="s">
-        <v>109</v>
-      </c>
-      <c r="C29" s="54">
+      <c r="B29" s="75" t="s">
+        <v>138</v>
+      </c>
+      <c r="C29" s="76">
         <v>250000</v>
       </c>
-      <c r="D29" s="55">
+      <c r="D29" s="77">
         <f>MIN(1, '2-Min Check-In'!G18/C29)</f>
       </c>
-      <c r="E29" s="54">
+      <c r="E29" s="76">
         <f>MAX(0, C29-'2-Min Check-In'!G18)</f>
       </c>
-      <c r="F29" s="56" t="s">
-        <v>110</v>
+      <c r="F29" s="78" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="30" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="C30" s="50">
+        <v>140</v>
+      </c>
+      <c r="C30" s="72">
         <v>500000</v>
       </c>
-      <c r="D30" s="51">
+      <c r="D30" s="73">
         <f>MIN(1, '2-Min Check-In'!G18/C30)</f>
       </c>
-      <c r="E30" s="50">
+      <c r="E30" s="72">
         <f>MAX(0, C30-'2-Min Check-In'!G18)</f>
       </c>
-      <c r="F30" s="52" t="s">
-        <v>112</v>
+      <c r="F30" s="74" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="31" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B31" s="53" t="s">
-        <v>113</v>
-      </c>
-      <c r="C31" s="54">
+      <c r="B31" s="75" t="s">
+        <v>142</v>
+      </c>
+      <c r="C31" s="76">
         <v>1000000</v>
       </c>
-      <c r="D31" s="55">
+      <c r="D31" s="77">
         <f>MIN(1, '2-Min Check-In'!G18/C31)</f>
       </c>
-      <c r="E31" s="54">
+      <c r="E31" s="76">
         <f>MAX(0, C31-'2-Min Check-In'!G18)</f>
       </c>
-      <c r="F31" s="56" t="s">
-        <v>114</v>
+      <c r="F31" s="78" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="33" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B33" s="42" t="s">
-        <v>115</v>
-      </c>
-      <c r="C33" s="42"/>
-      <c r="D33" s="42"/>
-      <c r="E33" s="42"/>
-      <c r="F33" s="42"/>
+      <c r="B33" s="65" t="s">
+        <v>144</v>
+      </c>
+      <c r="C33" s="65"/>
+      <c r="D33" s="65"/>
+      <c r="E33" s="65"/>
+      <c r="F33" s="65"/>
     </row>
     <row r="34" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B34" s="43" t="s">
-        <v>116</v>
-      </c>
-      <c r="C34" s="43" t="s">
-        <v>117</v>
-      </c>
-      <c r="D34" s="43" t="s">
-        <v>118</v>
-      </c>
-      <c r="E34" s="43" t="s">
-        <v>119</v>
-      </c>
-      <c r="F34" s="43" t="s">
-        <v>120</v>
+      <c r="B34" s="66" t="s">
+        <v>145</v>
+      </c>
+      <c r="C34" s="66" t="s">
+        <v>146</v>
+      </c>
+      <c r="D34" s="66" t="s">
+        <v>147</v>
+      </c>
+      <c r="E34" s="66" t="s">
+        <v>148</v>
+      </c>
+      <c r="F34" s="66" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="35" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B35" s="57">
+      <c r="B35" s="79">
         <f>'2-Min Check-In'!C18+'2-Min Check-In'!D18</f>
       </c>
-      <c r="C35" s="57">
+      <c r="C35" s="79">
         <f>'Smart Budget (50-30-20)'!C20</f>
       </c>
-      <c r="D35" s="58">
+      <c r="D35" s="80">
         <f>B35/C35</f>
       </c>
-      <c r="E35" s="59">
+      <c r="E35" s="81">
         <f>B35/'2-Min Check-In'!G18</f>
       </c>
-      <c r="F35" s="60" t="s">
-        <v>121</v>
+      <c r="F35" s="82" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="37" ht="22" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B37" s="61" t="s">
-        <v>122</v>
-      </c>
-      <c r="C37" s="61"/>
-      <c r="D37" s="61"/>
-      <c r="E37" s="61"/>
-      <c r="F37" s="61"/>
+      <c r="B37" s="83" t="s">
+        <v>151</v>
+      </c>
+      <c r="C37" s="83"/>
+      <c r="D37" s="83"/>
+      <c r="E37" s="83"/>
+      <c r="F37" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="16">
@@ -2748,402 +3136,402 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="29" t="s">
-        <v>123</v>
-      </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
+      <c r="B2" s="51" t="s">
+        <v>152</v>
+      </c>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="30" t="s">
-        <v>124</v>
-      </c>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
+      <c r="B3" s="52" t="s">
+        <v>153</v>
+      </c>
+      <c r="C3" s="52"/>
+      <c r="D3" s="52"/>
+      <c r="E3" s="52"/>
+      <c r="F3" s="52"/>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="35" t="s">
-        <v>125</v>
-      </c>
-      <c r="C5" s="35"/>
-      <c r="D5" s="35"/>
-      <c r="E5" s="31" t="s">
-        <v>126</v>
-      </c>
-      <c r="F5" s="31"/>
+      <c r="B5" s="84" t="s">
+        <v>154</v>
+      </c>
+      <c r="C5" s="84"/>
+      <c r="D5" s="84"/>
+      <c r="E5" s="53" t="s">
+        <v>155</v>
+      </c>
+      <c r="F5" s="53"/>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="62">
+      <c r="B6" s="85">
         <f>E24</f>
       </c>
-      <c r="C6" s="62"/>
-      <c r="D6" s="62"/>
-      <c r="E6" s="63">
+      <c r="C6" s="85"/>
+      <c r="D6" s="85"/>
+      <c r="E6" s="86">
         <f>E24/30</f>
       </c>
-      <c r="F6" s="63"/>
+      <c r="F6" s="86"/>
     </row>
     <row r="8" ht="22" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="64" t="s">
-        <v>127</v>
-      </c>
-      <c r="C8" s="64" t="s">
-        <v>128</v>
-      </c>
-      <c r="D8" s="64" t="s">
-        <v>129</v>
-      </c>
-      <c r="E8" s="64" t="s">
-        <v>130</v>
-      </c>
-      <c r="F8" s="64" t="s">
-        <v>131</v>
+      <c r="B8" s="87" t="s">
+        <v>156</v>
+      </c>
+      <c r="C8" s="87" t="s">
+        <v>157</v>
+      </c>
+      <c r="D8" s="87" t="s">
+        <v>158</v>
+      </c>
+      <c r="E8" s="87" t="s">
+        <v>159</v>
+      </c>
+      <c r="F8" s="87" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="65" t="s">
-        <v>132</v>
-      </c>
-      <c r="C9" s="65"/>
-      <c r="D9" s="65"/>
-      <c r="E9" s="65"/>
-      <c r="F9" s="65"/>
+      <c r="B9" s="88" t="s">
+        <v>161</v>
+      </c>
+      <c r="C9" s="88"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
     </row>
     <row r="10" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="C10" s="15">
+        <v>162</v>
+      </c>
+      <c r="C10" s="37">
         <v>6800</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="37">
         <v>6800</v>
       </c>
-      <c r="E10" s="15">
+      <c r="E10" s="37">
         <f>D10-C10</f>
       </c>
       <c r="F10" s="6" t="s">
-        <v>134</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="C11" s="15">
+        <v>164</v>
+      </c>
+      <c r="C11" s="37">
         <v>2200</v>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="37">
         <v>2200</v>
       </c>
-      <c r="E11" s="15">
+      <c r="E11" s="37">
         <f>D11-C11</f>
       </c>
       <c r="F11" s="6" t="s">
-        <v>134</v>
+        <v>163</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="C12" s="15">
+        <v>165</v>
+      </c>
+      <c r="C12" s="37">
         <v>500</v>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="37">
         <v>650</v>
       </c>
-      <c r="E12" s="15">
+      <c r="E12" s="37">
         <f>D12-C12</f>
       </c>
       <c r="F12" s="6" t="s">
-        <v>134</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B13" s="66" t="s">
-        <v>137</v>
-      </c>
-      <c r="C13" s="67">
+      <c r="B13" s="89" t="s">
+        <v>166</v>
+      </c>
+      <c r="C13" s="90">
         <f>SUM(C10:C12)</f>
       </c>
-      <c r="D13" s="67">
+      <c r="D13" s="90">
         <f>SUM(D10:D12)</f>
       </c>
-      <c r="E13" s="67">
+      <c r="E13" s="90">
         <f>D13-C13</f>
       </c>
-      <c r="F13" s="66" t="s">
-        <v>138</v>
+      <c r="F13" s="89" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="68" t="s">
-        <v>139</v>
-      </c>
-      <c r="C14" s="68"/>
-      <c r="D14" s="68"/>
-      <c r="E14" s="68"/>
-      <c r="F14" s="68"/>
+      <c r="B14" s="91" t="s">
+        <v>168</v>
+      </c>
+      <c r="C14" s="91"/>
+      <c r="D14" s="91"/>
+      <c r="E14" s="91"/>
+      <c r="F14" s="91"/>
     </row>
     <row r="15" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="C15" s="15">
+        <v>169</v>
+      </c>
+      <c r="C15" s="37">
         <v>2400</v>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="37">
         <v>2400</v>
       </c>
-      <c r="E15" s="15">
+      <c r="E15" s="37">
         <f>C15-D15</f>
       </c>
-      <c r="F15" s="6">
-        <f>TEXT(D15/$D$13, "0.0%")</f>
+      <c r="F15" s="42">
+        <f>D15/$D$13</f>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="C16" s="15">
+        <v>170</v>
+      </c>
+      <c r="C16" s="37">
         <v>750</v>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="37">
         <v>820</v>
       </c>
-      <c r="E16" s="15">
+      <c r="E16" s="37">
         <f>C16-D16</f>
       </c>
-      <c r="F16" s="6">
-        <f>TEXT(D16/$D$13, "0.0%")</f>
+      <c r="F16" s="42">
+        <f>D16/$D$13</f>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="C17" s="15">
+        <v>171</v>
+      </c>
+      <c r="C17" s="37">
         <v>320</v>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="37">
         <v>310</v>
       </c>
-      <c r="E17" s="15">
+      <c r="E17" s="37">
         <f>C17-D17</f>
       </c>
-      <c r="F17" s="6">
-        <f>TEXT(D17/$D$13, "0.0%")</f>
+      <c r="F17" s="42">
+        <f>D17/$D$13</f>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="C18" s="15">
+        <v>172</v>
+      </c>
+      <c r="C18" s="37">
         <v>450</v>
       </c>
-      <c r="D18" s="15">
+      <c r="D18" s="37">
         <v>450</v>
       </c>
-      <c r="E18" s="15">
+      <c r="E18" s="37">
         <f>C18-D18</f>
       </c>
-      <c r="F18" s="6">
-        <f>TEXT(D18/$D$13, "0.0%")</f>
+      <c r="F18" s="42">
+        <f>D18/$D$13</f>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="C19" s="15">
+        <v>173</v>
+      </c>
+      <c r="C19" s="37">
         <v>400</v>
       </c>
-      <c r="D19" s="15">
+      <c r="D19" s="37">
         <v>380</v>
       </c>
-      <c r="E19" s="15">
+      <c r="E19" s="37">
         <f>C19-D19</f>
       </c>
-      <c r="F19" s="6">
-        <f>TEXT(D19/$D$13, "0.0%")</f>
+      <c r="F19" s="42">
+        <f>D19/$D$13</f>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B20" s="69" t="s">
-        <v>145</v>
-      </c>
-      <c r="C20" s="70">
+      <c r="B20" s="92" t="s">
+        <v>174</v>
+      </c>
+      <c r="C20" s="93">
         <f>SUM(C15:C19)</f>
       </c>
-      <c r="D20" s="70">
+      <c r="D20" s="93">
         <f>SUM(D15:D19)</f>
       </c>
-      <c r="E20" s="70">
+      <c r="E20" s="93">
         <f>C20-D20</f>
       </c>
-      <c r="F20" s="69">
-        <f>"Actual: " &amp; TEXT(D20/D13, "0.0%") &amp; " (Target: ≤50%)"</f>
+      <c r="F20" s="94">
+        <f>D20/D13</f>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B21" s="71" t="s">
-        <v>146</v>
-      </c>
-      <c r="C21" s="71"/>
-      <c r="D21" s="71"/>
-      <c r="E21" s="71"/>
-      <c r="F21" s="71"/>
+      <c r="B21" s="95" t="s">
+        <v>175</v>
+      </c>
+      <c r="C21" s="95"/>
+      <c r="D21" s="95"/>
+      <c r="E21" s="95"/>
+      <c r="F21" s="95"/>
     </row>
     <row r="22" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="C22" s="15">
+        <v>176</v>
+      </c>
+      <c r="C22" s="37">
         <v>650</v>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="37">
         <v>520</v>
       </c>
-      <c r="E22" s="15">
+      <c r="E22" s="37">
         <f>C22-D22</f>
       </c>
-      <c r="F22" s="6">
-        <f>TEXT(D22/$D$13, "0.0%")</f>
+      <c r="F22" s="42">
+        <f>D22/$D$13</f>
       </c>
     </row>
     <row r="23" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="C23" s="15">
+        <v>177</v>
+      </c>
+      <c r="C23" s="37">
         <v>120</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="37">
         <v>115</v>
       </c>
-      <c r="E23" s="15">
+      <c r="E23" s="37">
         <f>C23-D23</f>
       </c>
-      <c r="F23" s="6">
-        <f>TEXT(D23/$D$13, "0.0%")</f>
+      <c r="F23" s="42">
+        <f>D23/$D$13</f>
       </c>
     </row>
     <row r="24" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="C24" s="15">
+        <v>178</v>
+      </c>
+      <c r="C24" s="37">
         <v>450</v>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="37">
         <v>380</v>
       </c>
-      <c r="E24" s="15">
+      <c r="E24" s="37">
         <f>C24-D24</f>
       </c>
-      <c r="F24" s="6">
-        <f>TEXT(D24/$D$13, "0.0%")</f>
+      <c r="F24" s="42">
+        <f>D24/$D$13</f>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B25" s="72" t="s">
-        <v>150</v>
-      </c>
-      <c r="C25" s="73">
+      <c r="B25" s="96" t="s">
+        <v>179</v>
+      </c>
+      <c r="C25" s="97">
         <f>SUM(C22:C24)</f>
       </c>
-      <c r="D25" s="73">
+      <c r="D25" s="97">
         <f>SUM(D22:D24)</f>
       </c>
-      <c r="E25" s="73">
+      <c r="E25" s="97">
         <f>C25-D25</f>
       </c>
-      <c r="F25" s="72">
-        <f>"Actual: " &amp; TEXT(D25/D13, "0.0%") &amp; " (Target: ≤30%)"</f>
+      <c r="F25" s="98">
+        <f>D25/D13</f>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B26" s="65" t="s">
-        <v>151</v>
-      </c>
-      <c r="C26" s="65"/>
-      <c r="D26" s="65"/>
-      <c r="E26" s="65"/>
-      <c r="F26" s="65"/>
+      <c r="B26" s="88" t="s">
+        <v>180</v>
+      </c>
+      <c r="C26" s="88"/>
+      <c r="D26" s="88"/>
+      <c r="E26" s="88"/>
+      <c r="F26" s="88"/>
     </row>
     <row r="27" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="C27" s="15">
+        <v>181</v>
+      </c>
+      <c r="C27" s="37">
         <v>2200</v>
       </c>
-      <c r="D27" s="15">
+      <c r="D27" s="37">
         <v>2200</v>
       </c>
-      <c r="E27" s="15">
+      <c r="E27" s="37">
         <f>D27-C27</f>
       </c>
-      <c r="F27" s="6">
-        <f>TEXT(D27/$D$13, "0.0%")</f>
+      <c r="F27" s="42">
+        <f>D27/$D$13</f>
       </c>
     </row>
     <row r="28" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="C28" s="15">
+        <v>182</v>
+      </c>
+      <c r="C28" s="37">
         <v>500</v>
       </c>
-      <c r="D28" s="15">
+      <c r="D28" s="37">
         <v>500</v>
       </c>
-      <c r="E28" s="15">
+      <c r="E28" s="37">
         <f>D28-C28</f>
       </c>
-      <c r="F28" s="6">
-        <f>TEXT(D28/$D$13, "0.0%")</f>
+      <c r="F28" s="42">
+        <f>D28/$D$13</f>
       </c>
     </row>
     <row r="29" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="C29" s="15">
+        <v>183</v>
+      </c>
+      <c r="C29" s="37">
         <v>600</v>
       </c>
-      <c r="D29" s="15">
+      <c r="D29" s="37">
         <v>750</v>
       </c>
-      <c r="E29" s="15">
+      <c r="E29" s="37">
         <f>D29-C29</f>
       </c>
-      <c r="F29" s="6">
-        <f>TEXT(D29/$D$13, "0.0%")</f>
+      <c r="F29" s="42">
+        <f>D29/$D$13</f>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B30" s="74" t="s">
-        <v>155</v>
-      </c>
-      <c r="C30" s="75">
+      <c r="B30" s="99" t="s">
+        <v>184</v>
+      </c>
+      <c r="C30" s="100">
         <f>SUM(C27:C29)</f>
       </c>
-      <c r="D30" s="75">
+      <c r="D30" s="100">
         <f>SUM(D27:D29)</f>
       </c>
-      <c r="E30" s="75">
+      <c r="E30" s="100">
         <f>D30-C30</f>
       </c>
-      <c r="F30" s="74">
-        <f>"Savings Rate: " &amp; TEXT(D30/D13, "0.0%") &amp; " (FIRE Speed)"</f>
+      <c r="F30" s="101">
+        <f>D30/D13</f>
       </c>
     </row>
   </sheetData>
@@ -3178,7 +3566,7 @@
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
-        <v>156</v>
+        <v>185</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -3188,174 +3576,174 @@
       <c r="H2" s="1"/>
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B3" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
+      <c r="B3" s="33" t="s">
+        <v>186</v>
+      </c>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="33"/>
+      <c r="G3" s="33"/>
+      <c r="H3" s="33"/>
     </row>
     <row r="5" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B5" s="64" t="s">
-        <v>158</v>
-      </c>
-      <c r="C5" s="64" t="s">
-        <v>159</v>
-      </c>
-      <c r="D5" s="64" t="s">
-        <v>160</v>
-      </c>
-      <c r="E5" s="64" t="s">
-        <v>161</v>
-      </c>
-      <c r="F5" s="64" t="s">
-        <v>162</v>
-      </c>
-      <c r="G5" s="64" t="s">
-        <v>163</v>
-      </c>
-      <c r="H5" s="64" t="s">
-        <v>164</v>
+      <c r="B5" s="87" t="s">
+        <v>187</v>
+      </c>
+      <c r="C5" s="87" t="s">
+        <v>188</v>
+      </c>
+      <c r="D5" s="87" t="s">
+        <v>189</v>
+      </c>
+      <c r="E5" s="87" t="s">
+        <v>190</v>
+      </c>
+      <c r="F5" s="87" t="s">
+        <v>191</v>
+      </c>
+      <c r="G5" s="87" t="s">
+        <v>192</v>
+      </c>
+      <c r="H5" s="87" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="C6" s="15">
+        <v>194</v>
+      </c>
+      <c r="C6" s="37">
         <v>25000</v>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="37">
         <v>21500</v>
       </c>
-      <c r="E6" s="15">
+      <c r="E6" s="37">
         <f>C6-D6</f>
       </c>
       <c r="F6" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="G6" s="15">
+        <v>84</v>
+      </c>
+      <c r="G6" s="37">
         <v>700</v>
       </c>
-      <c r="H6" s="20">
+      <c r="H6" s="42">
         <f>D6/C6</f>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B7" s="39" t="s">
-        <v>166</v>
-      </c>
-      <c r="C7" s="22">
+      <c r="B7" s="62" t="s">
+        <v>195</v>
+      </c>
+      <c r="C7" s="44">
         <v>2000</v>
       </c>
-      <c r="D7" s="22">
+      <c r="D7" s="44">
         <v>1400</v>
       </c>
-      <c r="E7" s="22">
+      <c r="E7" s="44">
         <f>C7-D7</f>
       </c>
-      <c r="F7" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="G7" s="22">
+      <c r="F7" s="62" t="s">
+        <v>86</v>
+      </c>
+      <c r="G7" s="44">
         <v>150</v>
       </c>
-      <c r="H7" s="25">
+      <c r="H7" s="47">
         <f>D7/C7</f>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="C8" s="15">
+        <v>196</v>
+      </c>
+      <c r="C8" s="37">
         <v>4500</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="37">
         <v>2800</v>
       </c>
-      <c r="E8" s="15">
+      <c r="E8" s="37">
         <f>C8-D8</f>
       </c>
       <c r="F8" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="G8" s="15">
+        <v>90</v>
+      </c>
+      <c r="G8" s="37">
         <v>250</v>
       </c>
-      <c r="H8" s="20">
+      <c r="H8" s="42">
         <f>D8/C8</f>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="39" t="s">
-        <v>168</v>
-      </c>
-      <c r="C9" s="22">
+      <c r="B9" s="62" t="s">
+        <v>197</v>
+      </c>
+      <c r="C9" s="44">
         <v>1500</v>
       </c>
-      <c r="D9" s="22">
+      <c r="D9" s="44">
         <v>750</v>
       </c>
-      <c r="E9" s="22">
+      <c r="E9" s="44">
         <f>C9-D9</f>
       </c>
-      <c r="F9" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="G9" s="22">
+      <c r="F9" s="62" t="s">
+        <v>89</v>
+      </c>
+      <c r="G9" s="44">
         <v>125</v>
       </c>
-      <c r="H9" s="25">
+      <c r="H9" s="47">
         <f>D9/C9</f>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="C10" s="15">
+        <v>198</v>
+      </c>
+      <c r="C10" s="37">
         <v>3500</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="37">
         <v>1800</v>
       </c>
-      <c r="E10" s="15">
+      <c r="E10" s="37">
         <f>C10-D10</f>
       </c>
       <c r="F10" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="G10" s="15">
+        <v>88</v>
+      </c>
+      <c r="G10" s="37">
         <v>250</v>
       </c>
-      <c r="H10" s="20">
+      <c r="H10" s="42">
         <f>D10/C10</f>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="26" t="s">
-        <v>170</v>
-      </c>
-      <c r="C11" s="27">
+      <c r="B11" s="48" t="s">
+        <v>199</v>
+      </c>
+      <c r="C11" s="49">
         <f>SUM(C6:C10)</f>
       </c>
-      <c r="D11" s="27">
+      <c r="D11" s="49">
         <f>SUM(D6:D10)</f>
       </c>
-      <c r="E11" s="27">
+      <c r="E11" s="49">
         <f>SUM(E6:E10)</f>
       </c>
-      <c r="F11" s="26" t="s">
-        <v>171</v>
-      </c>
-      <c r="G11" s="27">
+      <c r="F11" s="48" t="s">
+        <v>200</v>
+      </c>
+      <c r="G11" s="49">
         <f>SUM(G6:G10)</f>
       </c>
-      <c r="H11" s="76">
+      <c r="H11" s="102">
         <f>D11/C11</f>
       </c>
     </row>
@@ -3383,16 +3771,16 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B2" s="77" t="s">
-        <v>172</v>
-      </c>
-      <c r="C2" s="77"/>
-      <c r="D2" s="77"/>
-      <c r="E2" s="77"/>
+      <c r="B2" s="103" t="s">
+        <v>201</v>
+      </c>
+      <c r="C2" s="103"/>
+      <c r="D2" s="103"/>
+      <c r="E2" s="103"/>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
-        <v>173</v>
+        <v>202</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -3400,102 +3788,102 @@
     </row>
     <row r="5" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B5" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="C5" s="78">
+        <v>203</v>
+      </c>
+      <c r="C5" s="104">
         <v>32</v>
       </c>
     </row>
     <row r="6" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="C6" s="79">
+        <v>204</v>
+      </c>
+      <c r="C6" s="105">
         <v>66000</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="C7" s="80">
+        <v>205</v>
+      </c>
+      <c r="C7" s="106">
         <v>0.04</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="C8" s="80">
+        <v>206</v>
+      </c>
+      <c r="C8" s="106">
         <v>0.07</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B9" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="C9" s="79">
+        <v>207</v>
+      </c>
+      <c r="C9" s="105">
         <f>'2-Min Check-In'!D18</f>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="C10" s="79">
+        <v>208</v>
+      </c>
+      <c r="C10" s="105">
         <f>'Smart Budget (50-30-20)'!D27</f>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B12" s="65" t="s">
-        <v>180</v>
-      </c>
-      <c r="C12" s="65"/>
-      <c r="D12" s="65"/>
-      <c r="E12" s="65"/>
+      <c r="B12" s="88" t="s">
+        <v>209</v>
+      </c>
+      <c r="C12" s="88"/>
+      <c r="D12" s="88"/>
+      <c r="E12" s="88"/>
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="C13" s="79">
+        <v>210</v>
+      </c>
+      <c r="C13" s="105">
         <f>C6*0.65/C7</f>
       </c>
-      <c r="D13" s="81" t="s">
-        <v>182</v>
+      <c r="D13" s="107" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B14" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="C14" s="79">
+        <v>212</v>
+      </c>
+      <c r="C14" s="105">
         <f>C6/C7</f>
       </c>
-      <c r="D14" s="81" t="s">
-        <v>184</v>
+      <c r="D14" s="107" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B15" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="C15" s="79">
+        <v>214</v>
+      </c>
+      <c r="C15" s="105">
         <f>C6*1.4/C7</f>
       </c>
-      <c r="D15" s="81" t="s">
-        <v>186</v>
+      <c r="D15" s="107" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="C16" s="79">
+        <v>216</v>
+      </c>
+      <c r="C16" s="105">
         <f>(C6/C7)/(1+C8)^(60-C5)</f>
       </c>
-      <c r="D16" s="81" t="s">
-        <v>188</v>
+      <c r="D16" s="107" t="s">
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -3524,114 +3912,114 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="77" t="s">
+      <c r="B2" s="103" t="s">
+        <v>218</v>
+      </c>
+      <c r="C2" s="103"/>
+      <c r="D2" s="103"/>
+      <c r="E2" s="103"/>
+      <c r="F2" s="103"/>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B4" s="61" t="s">
+        <v>219</v>
+      </c>
+      <c r="C4" s="61" t="s">
         <v>189</v>
       </c>
-      <c r="C2" s="77"/>
-      <c r="D2" s="77"/>
-      <c r="E2" s="77"/>
-      <c r="F2" s="77"/>
-    </row>
-    <row r="4" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="38" t="s">
-        <v>190</v>
-      </c>
-      <c r="C4" s="38" t="s">
-        <v>160</v>
-      </c>
-      <c r="D4" s="38" t="s">
-        <v>191</v>
-      </c>
-      <c r="E4" s="38" t="s">
-        <v>192</v>
-      </c>
-      <c r="F4" s="38" t="s">
-        <v>193</v>
+      <c r="D4" s="61" t="s">
+        <v>220</v>
+      </c>
+      <c r="E4" s="61" t="s">
+        <v>221</v>
+      </c>
+      <c r="F4" s="61" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="5" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C5" s="15">
+        <v>223</v>
+      </c>
+      <c r="C5" s="37">
         <v>4200</v>
       </c>
-      <c r="D5" s="82">
+      <c r="D5" s="108">
         <v>0.2499</v>
       </c>
-      <c r="E5" s="15">
+      <c r="E5" s="37">
         <v>140</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>195</v>
+        <v>224</v>
       </c>
     </row>
     <row r="6" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="C6" s="15">
+        <v>225</v>
+      </c>
+      <c r="C6" s="37">
         <v>8500</v>
       </c>
-      <c r="D6" s="82">
+      <c r="D6" s="108">
         <v>0.115</v>
       </c>
-      <c r="E6" s="15">
+      <c r="E6" s="37">
         <v>210</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>197</v>
+        <v>226</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="C7" s="15">
+        <v>227</v>
+      </c>
+      <c r="C7" s="37">
         <v>17400</v>
       </c>
-      <c r="D7" s="82">
+      <c r="D7" s="108">
         <v>0.059</v>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="37">
         <v>380</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>199</v>
+        <v>228</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="C8" s="15">
+        <v>229</v>
+      </c>
+      <c r="C8" s="37">
         <v>200000</v>
       </c>
-      <c r="D8" s="82">
+      <c r="D8" s="108">
         <v>0.035</v>
       </c>
-      <c r="E8" s="15">
+      <c r="E8" s="37">
         <v>1670</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>201</v>
+        <v>230</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="66" t="s">
-        <v>202</v>
-      </c>
-      <c r="C9" s="67">
+      <c r="B9" s="89" t="s">
+        <v>231</v>
+      </c>
+      <c r="C9" s="90">
         <f>SUM(C5:C8)</f>
       </c>
-      <c r="D9" s="83">
+      <c r="D9" s="109">
         <f>AVERAGE(D5:D8)</f>
       </c>
-      <c r="E9" s="67">
+      <c r="E9" s="90">
         <f>SUM(E5:E8)</f>
       </c>
-      <c r="F9" s="66" t="s">
-        <v>203</v>
+      <c r="F9" s="89" t="s">
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -3655,623 +4043,623 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="77" t="s">
-        <v>204</v>
-      </c>
-      <c r="C2" s="77"/>
-      <c r="D2" s="77"/>
-      <c r="E2" s="77"/>
-      <c r="F2" s="77"/>
-      <c r="G2" s="77"/>
-      <c r="H2" s="77"/>
+      <c r="B2" s="103" t="s">
+        <v>233</v>
+      </c>
+      <c r="C2" s="103"/>
+      <c r="D2" s="103"/>
+      <c r="E2" s="103"/>
+      <c r="F2" s="103"/>
+      <c r="G2" s="103"/>
+      <c r="H2" s="103"/>
     </row>
     <row r="4" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B4" s="38" t="s">
-        <v>205</v>
-      </c>
-      <c r="C4" s="38" t="s">
-        <v>206</v>
-      </c>
-      <c r="D4" s="38" t="s">
-        <v>207</v>
-      </c>
-      <c r="E4" s="38" t="s">
-        <v>208</v>
-      </c>
-      <c r="F4" s="38" t="s">
-        <v>209</v>
-      </c>
-      <c r="G4" s="38" t="s">
-        <v>210</v>
-      </c>
-      <c r="H4" s="38" t="s">
-        <v>211</v>
+      <c r="B4" s="61" t="s">
+        <v>234</v>
+      </c>
+      <c r="C4" s="61" t="s">
+        <v>235</v>
+      </c>
+      <c r="D4" s="61" t="s">
+        <v>236</v>
+      </c>
+      <c r="E4" s="61" t="s">
+        <v>237</v>
+      </c>
+      <c r="F4" s="61" t="s">
+        <v>238</v>
+      </c>
+      <c r="G4" s="61" t="s">
+        <v>239</v>
+      </c>
+      <c r="H4" s="61" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="5" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="C5" s="15">
+        <v>241</v>
+      </c>
+      <c r="C5" s="37">
         <v>4800</v>
       </c>
-      <c r="D5" s="15">
+      <c r="D5" s="37">
         <v>39000</v>
       </c>
-      <c r="E5" s="15">
+      <c r="E5" s="37">
         <v>145000</v>
       </c>
-      <c r="F5" s="15">
+      <c r="F5" s="37">
         <v>380000</v>
       </c>
-      <c r="G5" s="15">
+      <c r="G5" s="37">
         <v>750000</v>
       </c>
-      <c r="H5" s="15">
+      <c r="H5" s="37">
         <v>2800000</v>
       </c>
     </row>
     <row r="6" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B6" s="39" t="s">
-        <v>213</v>
-      </c>
-      <c r="C6" s="22">
+      <c r="B6" s="62" t="s">
+        <v>242</v>
+      </c>
+      <c r="C6" s="44">
         <v>35000</v>
       </c>
-      <c r="D6" s="22">
+      <c r="D6" s="44">
         <v>135600</v>
       </c>
-      <c r="E6" s="22">
+      <c r="E6" s="44">
         <v>420000</v>
       </c>
-      <c r="F6" s="22">
+      <c r="F6" s="44">
         <v>980000</v>
       </c>
-      <c r="G6" s="22">
+      <c r="G6" s="44">
         <v>1850000</v>
       </c>
-      <c r="H6" s="22">
+      <c r="H6" s="44">
         <v>5500000</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C7" s="15">
+        <v>243</v>
+      </c>
+      <c r="C7" s="37">
         <v>68000</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="37">
         <v>247200</v>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="37">
         <v>780000</v>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="37">
         <v>1950000</v>
       </c>
-      <c r="G7" s="15">
+      <c r="G7" s="37">
         <v>3400000</v>
       </c>
-      <c r="H7" s="15">
+      <c r="H7" s="37">
         <v>10200000</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="39" t="s">
-        <v>215</v>
-      </c>
-      <c r="C8" s="22">
+      <c r="B8" s="62" t="s">
+        <v>244</v>
+      </c>
+      <c r="C8" s="44">
         <v>95000</v>
       </c>
-      <c r="D8" s="22">
+      <c r="D8" s="44">
         <v>364500</v>
       </c>
-      <c r="E8" s="22">
+      <c r="E8" s="44">
         <v>1150000</v>
       </c>
-      <c r="F8" s="22">
+      <c r="F8" s="44">
         <v>2800000</v>
       </c>
-      <c r="G8" s="22">
+      <c r="G8" s="44">
         <v>4900000</v>
       </c>
-      <c r="H8" s="22">
+      <c r="H8" s="44">
         <v>14500000</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="C9" s="15">
+        <v>245</v>
+      </c>
+      <c r="C9" s="37">
         <v>110000</v>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="37">
         <v>409900</v>
       </c>
-      <c r="E9" s="15">
+      <c r="E9" s="37">
         <v>1350000</v>
       </c>
-      <c r="F9" s="15">
+      <c r="F9" s="37">
         <v>3200000</v>
       </c>
-      <c r="G9" s="15">
+      <c r="G9" s="37">
         <v>5600000</v>
       </c>
-      <c r="H9" s="15">
+      <c r="H9" s="37">
         <v>16800000</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="39" t="s">
-        <v>217</v>
-      </c>
-      <c r="C10" s="22">
+      <c r="B10" s="62" t="s">
+        <v>246</v>
+      </c>
+      <c r="C10" s="44">
         <v>92000</v>
       </c>
-      <c r="D10" s="22">
+      <c r="D10" s="44">
         <v>335600</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="44">
         <v>1050000</v>
       </c>
-      <c r="F10" s="22">
+      <c r="F10" s="44">
         <v>2600000</v>
       </c>
-      <c r="G10" s="22">
+      <c r="G10" s="44">
         <v>4700000</v>
       </c>
-      <c r="H10" s="22">
+      <c r="H10" s="44">
         <v>13200000</v>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B13" s="84" t="s">
-        <v>218</v>
-      </c>
-      <c r="C13" s="84"/>
-      <c r="D13" s="84"/>
-      <c r="E13" s="84"/>
-      <c r="F13" s="84"/>
-      <c r="G13" s="84"/>
-      <c r="H13" s="84"/>
+      <c r="B13" s="110" t="s">
+        <v>247</v>
+      </c>
+      <c r="C13" s="110"/>
+      <c r="D13" s="110"/>
+      <c r="E13" s="110"/>
+      <c r="F13" s="110"/>
+      <c r="G13" s="110"/>
+      <c r="H13" s="110"/>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B14" s="38" t="s">
-        <v>219</v>
-      </c>
-      <c r="C14" s="38" t="s">
-        <v>220</v>
-      </c>
-      <c r="D14" s="38" t="s">
-        <v>221</v>
-      </c>
-      <c r="E14" s="38" t="s">
-        <v>222</v>
-      </c>
-      <c r="F14" s="38" t="s">
-        <v>223</v>
-      </c>
-      <c r="G14" s="38" t="s">
-        <v>224</v>
-      </c>
-      <c r="H14" s="38" t="s">
-        <v>225</v>
+      <c r="B14" s="61" t="s">
+        <v>248</v>
+      </c>
+      <c r="C14" s="61" t="s">
+        <v>249</v>
+      </c>
+      <c r="D14" s="61" t="s">
+        <v>250</v>
+      </c>
+      <c r="E14" s="61" t="s">
+        <v>251</v>
+      </c>
+      <c r="F14" s="61" t="s">
+        <v>252</v>
+      </c>
+      <c r="G14" s="61" t="s">
+        <v>253</v>
+      </c>
+      <c r="H14" s="61" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="C15" s="15">
+        <v>255</v>
+      </c>
+      <c r="C15" s="37">
         <v>285000</v>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="37">
         <v>1250000</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="F15" s="15">
+        <v>256</v>
+      </c>
+      <c r="F15" s="37">
         <v>785000</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>228</v>
+        <v>257</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>229</v>
+        <v>258</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B16" s="39" t="s">
-        <v>230</v>
-      </c>
-      <c r="C16" s="22">
+      <c r="B16" s="62" t="s">
+        <v>259</v>
+      </c>
+      <c r="C16" s="44">
         <v>245000</v>
       </c>
-      <c r="D16" s="22">
+      <c r="D16" s="44">
         <v>1180000</v>
       </c>
-      <c r="E16" s="39" t="s">
-        <v>231</v>
-      </c>
-      <c r="F16" s="22">
+      <c r="E16" s="62" t="s">
+        <v>260</v>
+      </c>
+      <c r="F16" s="44">
         <v>650000</v>
       </c>
-      <c r="G16" s="39" t="s">
-        <v>228</v>
-      </c>
-      <c r="H16" s="39" t="s">
-        <v>232</v>
+      <c r="G16" s="62" t="s">
+        <v>257</v>
+      </c>
+      <c r="H16" s="62" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="C17" s="15">
+        <v>262</v>
+      </c>
+      <c r="C17" s="37">
         <v>275000</v>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="37">
         <v>1200000</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>234</v>
-      </c>
-      <c r="F17" s="15">
+        <v>263</v>
+      </c>
+      <c r="F17" s="37">
         <v>610000</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>228</v>
+        <v>257</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>235</v>
+        <v>264</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B18" s="39" t="s">
-        <v>236</v>
-      </c>
-      <c r="C18" s="22">
+      <c r="B18" s="62" t="s">
+        <v>265</v>
+      </c>
+      <c r="C18" s="44">
         <v>175000</v>
       </c>
-      <c r="D18" s="22">
+      <c r="D18" s="44">
         <v>820000</v>
       </c>
-      <c r="E18" s="39" t="s">
-        <v>237</v>
-      </c>
-      <c r="F18" s="22">
+      <c r="E18" s="62" t="s">
+        <v>266</v>
+      </c>
+      <c r="F18" s="44">
         <v>345000</v>
       </c>
-      <c r="G18" s="39" t="s">
-        <v>238</v>
-      </c>
-      <c r="H18" s="39" t="s">
-        <v>239</v>
+      <c r="G18" s="62" t="s">
+        <v>267</v>
+      </c>
+      <c r="H18" s="62" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="C19" s="15">
+        <v>269</v>
+      </c>
+      <c r="C19" s="37">
         <v>195000</v>
       </c>
-      <c r="D19" s="15">
+      <c r="D19" s="37">
         <v>890000</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="F19" s="15">
+        <v>270</v>
+      </c>
+      <c r="F19" s="37">
         <v>395000</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>242</v>
+        <v>271</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>243</v>
+        <v>272</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B20" s="39" t="s">
-        <v>244</v>
-      </c>
-      <c r="C20" s="22">
+      <c r="B20" s="62" t="s">
+        <v>273</v>
+      </c>
+      <c r="C20" s="44">
         <v>295000</v>
       </c>
-      <c r="D20" s="22">
+      <c r="D20" s="44">
         <v>1320000</v>
       </c>
-      <c r="E20" s="39" t="s">
-        <v>245</v>
-      </c>
-      <c r="F20" s="22">
+      <c r="E20" s="62" t="s">
+        <v>274</v>
+      </c>
+      <c r="F20" s="44">
         <v>640000</v>
       </c>
-      <c r="G20" s="39" t="s">
-        <v>228</v>
-      </c>
-      <c r="H20" s="39" t="s">
-        <v>246</v>
+      <c r="G20" s="62" t="s">
+        <v>257</v>
+      </c>
+      <c r="H20" s="62" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B21" s="6" t="s">
-        <v>247</v>
-      </c>
-      <c r="C21" s="15">
+        <v>276</v>
+      </c>
+      <c r="C21" s="37">
         <v>185000</v>
       </c>
-      <c r="D21" s="15">
+      <c r="D21" s="37">
         <v>860000</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>248</v>
-      </c>
-      <c r="F21" s="15">
+        <v>277</v>
+      </c>
+      <c r="F21" s="37">
         <v>275000</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>238</v>
+        <v>267</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>249</v>
+        <v>278</v>
       </c>
     </row>
     <row r="22" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B22" s="39" t="s">
-        <v>250</v>
-      </c>
-      <c r="C22" s="22">
+      <c r="B22" s="62" t="s">
+        <v>279</v>
+      </c>
+      <c r="C22" s="44">
         <v>260000</v>
       </c>
-      <c r="D22" s="22">
+      <c r="D22" s="44">
         <v>1100000</v>
       </c>
-      <c r="E22" s="39" t="s">
-        <v>251</v>
-      </c>
-      <c r="F22" s="22">
+      <c r="E22" s="62" t="s">
+        <v>280</v>
+      </c>
+      <c r="F22" s="44">
         <v>550000</v>
       </c>
-      <c r="G22" s="39" t="s">
-        <v>252</v>
-      </c>
-      <c r="H22" s="39" t="s">
-        <v>253</v>
+      <c r="G22" s="62" t="s">
+        <v>281</v>
+      </c>
+      <c r="H22" s="62" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="25" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B25" s="85" t="s">
-        <v>254</v>
-      </c>
-      <c r="C25" s="85"/>
-      <c r="D25" s="85"/>
-      <c r="E25" s="85"/>
-      <c r="F25" s="85"/>
-      <c r="G25" s="85"/>
-      <c r="H25" s="85"/>
+      <c r="B25" s="111" t="s">
+        <v>283</v>
+      </c>
+      <c r="C25" s="111"/>
+      <c r="D25" s="111"/>
+      <c r="E25" s="111"/>
+      <c r="F25" s="111"/>
+      <c r="G25" s="111"/>
+      <c r="H25" s="111"/>
     </row>
     <row r="26" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B26" s="38" t="s">
-        <v>255</v>
-      </c>
-      <c r="C26" s="38" t="s">
-        <v>256</v>
-      </c>
-      <c r="D26" s="38" t="s">
-        <v>257</v>
-      </c>
-      <c r="E26" s="38" t="s">
-        <v>258</v>
-      </c>
-      <c r="F26" s="38" t="s">
-        <v>259</v>
-      </c>
-      <c r="G26" s="38" t="s">
-        <v>260</v>
-      </c>
-      <c r="H26" s="38" t="s">
-        <v>261</v>
+      <c r="B26" s="61" t="s">
+        <v>284</v>
+      </c>
+      <c r="C26" s="61" t="s">
+        <v>285</v>
+      </c>
+      <c r="D26" s="61" t="s">
+        <v>286</v>
+      </c>
+      <c r="E26" s="61" t="s">
+        <v>287</v>
+      </c>
+      <c r="F26" s="61" t="s">
+        <v>288</v>
+      </c>
+      <c r="G26" s="61" t="s">
+        <v>289</v>
+      </c>
+      <c r="H26" s="61" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="27" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B27" s="6" t="s">
-        <v>262</v>
-      </c>
-      <c r="C27" s="86">
+        <v>291</v>
+      </c>
+      <c r="C27" s="112">
         <v>1</v>
       </c>
-      <c r="D27" s="15">
+      <c r="D27" s="37">
         <v>100000</v>
       </c>
-      <c r="E27" s="15">
+      <c r="E27" s="37">
         <v>150000</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>263</v>
+        <v>292</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>264</v>
+        <v>293</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>265</v>
+        <v>294</v>
       </c>
     </row>
     <row r="28" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B28" s="39" t="s">
-        <v>266</v>
-      </c>
-      <c r="C28" s="87">
+      <c r="B28" s="62" t="s">
+        <v>295</v>
+      </c>
+      <c r="C28" s="113">
         <v>2</v>
       </c>
-      <c r="D28" s="22">
+      <c r="D28" s="44">
         <v>200000</v>
       </c>
-      <c r="E28" s="22">
+      <c r="E28" s="44">
         <v>300000</v>
       </c>
-      <c r="F28" s="39" t="s">
-        <v>267</v>
-      </c>
-      <c r="G28" s="39" t="s">
-        <v>264</v>
-      </c>
-      <c r="H28" s="39" t="s">
-        <v>265</v>
+      <c r="F28" s="62" t="s">
+        <v>296</v>
+      </c>
+      <c r="G28" s="62" t="s">
+        <v>293</v>
+      </c>
+      <c r="H28" s="62" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="29" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B29" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="C29" s="86">
+        <v>297</v>
+      </c>
+      <c r="C29" s="112">
         <v>3</v>
       </c>
-      <c r="D29" s="15">
+      <c r="D29" s="37">
         <v>300000</v>
       </c>
-      <c r="E29" s="15">
+      <c r="E29" s="37">
         <v>450000</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>269</v>
+        <v>298</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>264</v>
+        <v>293</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>265</v>
+        <v>294</v>
       </c>
     </row>
     <row r="30" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B30" s="39" t="s">
-        <v>270</v>
-      </c>
-      <c r="C30" s="87">
+      <c r="B30" s="62" t="s">
+        <v>299</v>
+      </c>
+      <c r="C30" s="113">
         <v>4</v>
       </c>
-      <c r="D30" s="22">
+      <c r="D30" s="44">
         <v>400000</v>
       </c>
-      <c r="E30" s="22">
+      <c r="E30" s="44">
         <v>600000</v>
       </c>
-      <c r="F30" s="39" t="s">
-        <v>271</v>
-      </c>
-      <c r="G30" s="39" t="s">
-        <v>264</v>
-      </c>
-      <c r="H30" s="39" t="s">
-        <v>265</v>
+      <c r="F30" s="62" t="s">
+        <v>300</v>
+      </c>
+      <c r="G30" s="62" t="s">
+        <v>293</v>
+      </c>
+      <c r="H30" s="62" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="31" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B31" s="6" t="s">
-        <v>272</v>
-      </c>
-      <c r="C31" s="86">
+        <v>301</v>
+      </c>
+      <c r="C31" s="112">
         <v>6</v>
       </c>
-      <c r="D31" s="15">
+      <c r="D31" s="37">
         <v>600000</v>
       </c>
-      <c r="E31" s="15">
+      <c r="E31" s="37">
         <v>900000</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>273</v>
+        <v>302</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>264</v>
+        <v>293</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>265</v>
+        <v>294</v>
       </c>
     </row>
     <row r="32" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B32" s="39" t="s">
-        <v>274</v>
-      </c>
-      <c r="C32" s="87">
+      <c r="B32" s="62" t="s">
+        <v>303</v>
+      </c>
+      <c r="C32" s="113">
         <v>7</v>
       </c>
-      <c r="D32" s="22">
+      <c r="D32" s="44">
         <v>700000</v>
       </c>
-      <c r="E32" s="22">
+      <c r="E32" s="44">
         <v>1050000</v>
       </c>
-      <c r="F32" s="39" t="s">
-        <v>275</v>
-      </c>
-      <c r="G32" s="39" t="s">
-        <v>264</v>
-      </c>
-      <c r="H32" s="39" t="s">
-        <v>265</v>
+      <c r="F32" s="62" t="s">
+        <v>304</v>
+      </c>
+      <c r="G32" s="62" t="s">
+        <v>293</v>
+      </c>
+      <c r="H32" s="62" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="33" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B33" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="C33" s="86">
+        <v>305</v>
+      </c>
+      <c r="C33" s="112">
         <v>8</v>
       </c>
-      <c r="D33" s="15">
+      <c r="D33" s="37">
         <v>800000</v>
       </c>
-      <c r="E33" s="15">
+      <c r="E33" s="37">
         <v>1200000</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>277</v>
+        <v>306</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>264</v>
+        <v>293</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>265</v>
+        <v>294</v>
       </c>
     </row>
     <row r="34" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B34" s="39" t="s">
-        <v>278</v>
-      </c>
-      <c r="C34" s="87">
+      <c r="B34" s="62" t="s">
+        <v>307</v>
+      </c>
+      <c r="C34" s="113">
         <v>10</v>
       </c>
-      <c r="D34" s="22">
+      <c r="D34" s="44">
         <v>1000000</v>
       </c>
-      <c r="E34" s="22">
+      <c r="E34" s="44">
         <v>1500000</v>
       </c>
-      <c r="F34" s="39" t="s">
-        <v>279</v>
-      </c>
-      <c r="G34" s="39" t="s">
-        <v>264</v>
-      </c>
-      <c r="H34" s="39" t="s">
-        <v>265</v>
+      <c r="F34" s="62" t="s">
+        <v>308</v>
+      </c>
+      <c r="G34" s="62" t="s">
+        <v>293</v>
+      </c>
+      <c r="H34" s="62" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B36" s="61" t="s">
-        <v>280</v>
-      </c>
-      <c r="C36" s="61"/>
-      <c r="D36" s="61"/>
-      <c r="E36" s="61"/>
-      <c r="F36" s="61"/>
-      <c r="G36" s="61"/>
-      <c r="H36" s="61"/>
+      <c r="B36" s="83" t="s">
+        <v>309</v>
+      </c>
+      <c r="C36" s="83"/>
+      <c r="D36" s="83"/>
+      <c r="E36" s="83"/>
+      <c r="F36" s="83"/>
+      <c r="G36" s="83"/>
+      <c r="H36" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
feat(vault): dedicate Private Wealth Diagnostic as tab 2 with institutional executive titling
</commit_message>
<xml_diff>
--- a/public/downloads/NetWorth_FIRE_Master_Vault_2026.xlsx
+++ b/public/downloads/NetWorth_FIRE_Master_Vault_2026.xlsx
@@ -5,20 +5,21 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="START HERE" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="2-Min Check-In" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Executive Dashboard" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Smart Budget (50-30-20)" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Sinking Funds Shield" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="FIRE Freedom Engine" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="Debt Avalanche &amp; Snowball" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="Fed &amp; State Benchmarks" state="visible" r:id="rId11"/>
+    <sheet sheetId="2" name="Private Wealth Diagnostic" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="2-Min Check-In" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Executive Dashboard" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Smart Budget (50-30-20)" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="Sinking Funds Shield" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="FIRE Freedom Engine" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="Debt Avalanche &amp; Snowball" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="Fed &amp; State Benchmarks" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="313">
   <si>
     <t>🏛️ GETNETWORTHCALCULATOR.COM • OFFICIAL WEALTH &amp; BUDGET OPERATING SYSTEM</t>
   </si>
@@ -29,13 +30,13 @@
     <t>🚀 THE 3-STEP MONTHLY ROUTINE (TAKES 2 MINUTES ON THE 1ST OF EACH MONTH)</t>
   </si>
   <si>
-    <t>Step 1: Open Tab 2</t>
-  </si>
-  <si>
-    <t>Click '2-Min Check-In'</t>
-  </si>
-  <si>
-    <t>On the 1st of every month, open the second tab.</t>
+    <t>Step 1: Monthly Routine</t>
+  </si>
+  <si>
+    <t>Select '2-Min Check-In'</t>
+  </si>
+  <si>
+    <t>On the 1st of every month, open the 2-Min Check-In tab.</t>
   </si>
   <si>
     <t>Step 2: Enter 4 Numbers</t>
@@ -89,6 +90,12 @@
     <t>📖 WHAT EACH TAB DOES (CHOOSE YOUR PURPOSE)</t>
   </si>
   <si>
+    <t>🏛️ Private Wealth Diagnostic</t>
+  </si>
+  <si>
+    <t>Instant baseline assessment: Benchmark your official wealth tier (PAW/UAW), audit capital leaks &amp; compute true hourly life energy.</t>
+  </si>
+  <si>
     <t>2-Min Check-In</t>
   </si>
   <si>
@@ -134,10 +141,13 @@
     <t>🌐 GetNetWorthCalculator.com • 100% Private, Anonymous &amp; Offline • Official 2026 Edition</t>
   </si>
   <si>
-    <t>⚡ 60-SECOND INSTANT DOPAMINE TEST-DRIVE (GET IMMEDIATE WINS NOW)</t>
-  </si>
-  <si>
-    <t>Type 3 numbers into the green boxes below. Watch your official wealth tier and milestone unlock immediately!</t>
+    <t>🏛️ PRIVATE WEALTH DIAGNOSTIC &amp; CAPITAL AUDIT • GETNETWORTH</t>
+  </si>
+  <si>
+    <t>Official Accumulation Tier Benchmark • Recurring Capital Leakage Audit • True Hourly Life Energy Metric</t>
+  </si>
+  <si>
+    <t>🎯 WEALTH ACCUMULATION TIER &amp; BENCHMARK DIAGNOSTIC</t>
   </si>
   <si>
     <t>1. YOUR CURRENT AGE</t>
@@ -149,76 +159,76 @@
     <t>3. CURRENT ESTIMATED NET WORTH</t>
   </si>
   <si>
-    <t>🏆 OFFICIAL WEALTH TIER</t>
-  </si>
-  <si>
-    <t>🎯 TARGET NET WORTH FOR AGE</t>
-  </si>
-  <si>
-    <t>🚀 NEXT MILESTONE CLUB</t>
-  </si>
-  <si>
-    <t>🧛‍♂️ THE 5-MINUTE VAMPIRE PURGE (FIND $1,000+ IN CASH RIGHT NOW)</t>
-  </si>
-  <si>
-    <t>Recurring Monthly Leak / Subscription</t>
+    <t>🏆 OFFICIAL ACCUMULATION TIER</t>
+  </si>
+  <si>
+    <t>🎯 BENCHMARK NET WORTH FOR AGE</t>
+  </si>
+  <si>
+    <t>🚀 NEXT CAPITAL MILESTONE</t>
+  </si>
+  <si>
+    <t>💸 CAPITAL INEFFICIENCY &amp; CASH FLOW LEAKAGE AUDIT</t>
+  </si>
+  <si>
+    <t>Recurring Monthly Outflow / Underutilized Service</t>
   </si>
   <si>
     <t>Monthly Cost ($)</t>
   </si>
   <si>
-    <t>Action Plan &amp; Reality Check</t>
-  </si>
-  <si>
-    <t>Unused Streaming / Digital Subscriptions</t>
-  </si>
-  <si>
-    <t>Cancel unneeded services</t>
-  </si>
-  <si>
-    <t>Unused Gym / Health App Memberships</t>
-  </si>
-  <si>
-    <t>Downgrade or pause immediately</t>
-  </si>
-  <si>
-    <t>DoorDash / Takeout Delivery Markups &amp; Fees</t>
-  </si>
-  <si>
-    <t>Limit takeout to 1x weekly</t>
-  </si>
-  <si>
-    <t>Overpriced Cellphone / Insurance Plan</t>
-  </si>
-  <si>
-    <t>Shop rate or switch carrier</t>
-  </si>
-  <si>
-    <t>TOTAL RECURRENT LEAKAGE DISCOVERED</t>
-  </si>
-  <si>
-    <t>Found in your budget in 3 minutes</t>
-  </si>
-  <si>
-    <t>🟢 INSTANT ANNUAL CASH UNLOCKED</t>
+    <t>Optimization &amp; Capital Reclamation Action</t>
+  </si>
+  <si>
+    <t>Unused Streaming &amp; Digital Subscriptions</t>
+  </si>
+  <si>
+    <t>Cancel or pause immediately</t>
+  </si>
+  <si>
+    <t>Unused Gym &amp; Fitness App Memberships</t>
+  </si>
+  <si>
+    <t>Switch to free tier or pause</t>
+  </si>
+  <si>
+    <t>Food Delivery App Service Fees &amp; Markups</t>
+  </si>
+  <si>
+    <t>Cap delivery orders to 1x weekly</t>
+  </si>
+  <si>
+    <t>Overpriced Mobile / Auto Insurance Policy</t>
+  </si>
+  <si>
+    <t>Renegotiate premium or re-quote</t>
+  </si>
+  <si>
+    <t>TOTAL RECURRING CASH OUTFLOW IDENTIFIED</t>
+  </si>
+  <si>
+    <t>Reclaimable immediately into your surplus cash flow</t>
+  </si>
+  <si>
+    <t>🟢 ANNUAL RECLAIMED CASH FLOW</t>
   </si>
   <si>
     <t>📈 10-YEAR COMPOUNDED WEALTH (8%)</t>
   </si>
   <si>
-    <t>⏳ THE LIFE ENERGY CALCULATOR (IS THAT PURCHASE WORTH YOUR FINITE HOURS?)</t>
-  </si>
-  <si>
-    <t>Your Real Hourly Wage (C30 / 2,080 hrs)</t>
-  </si>
-  <si>
-    <t>Impulse Purchase Price ($)</t>
-  </si>
-  <si>
-    <t>Actual Hours of Your Life It Costs</t>
-  </si>
-  <si>
-    <t>🚀 READY FOR YOUR 2-MINUTE MONTHLY ROUTINE? CLICK THE "2-Min Check-In" TAB BELOW! 👇</t>
+    <t>⏳ LIFE ENERGY &amp; TRUE HOURLY VALUE CONVERSION</t>
+  </si>
+  <si>
+    <t>Your Real Hourly Yield (Pre-Tax / 2,080 hrs)</t>
+  </si>
+  <si>
+    <t>Discretionary Purchase Price ($)</t>
+  </si>
+  <si>
+    <t>True Hours of Finite Life Required</t>
+  </si>
+  <si>
+    <t>🚀 READY FOR YOUR ONGOING ROUTINE? SELECT THE "2-Min Check-In" TAB BELOW 👇</t>
   </si>
   <si>
     <t>⚡ 2-MINUTE MONTHLY QUICK CHECK-IN • GETNETWORTHCALCULATOR.COM</t>
@@ -954,23 +964,24 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="14">
+  <numFmts count="15">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
-    <numFmt numFmtId="165" formatCode="$#,##0&quot;/mo&quot;"/>
-    <numFmt numFmtId="166" formatCode="&quot;+$&quot;#,##0&quot; / Year Back In Checking&quot;"/>
-    <numFmt numFmtId="167" formatCode="&quot;+$&quot;#,##0&quot; Created For Retirement&quot;"/>
-    <numFmt numFmtId="168" formatCode="$#,##0.00&quot;/hr&quot;"/>
-    <numFmt numFmtId="169" formatCode="0.0&quot; Hours at Work&quot;"/>
-    <numFmt numFmtId="170" formatCode="+$#,##0;-$#,##0;$0"/>
-    <numFmt numFmtId="171" formatCode="+0.0%;-0.0%;0.0%"/>
-    <numFmt numFmtId="172" formatCode="0.0%"/>
-    <numFmt numFmtId="173" formatCode="&quot;+$&quot;#,##0;&quot;-$&quot;#,##0;&quot;$0&quot;"/>
-    <numFmt numFmtId="174" formatCode="0.00&quot;x&quot;"/>
-    <numFmt numFmtId="175" formatCode="0.0&quot; Months&quot;"/>
-    <numFmt numFmtId="176" formatCode="$#,##0/day"/>
-    <numFmt numFmtId="177" formatCode="0.0&quot;x&quot;"/>
+    <numFmt numFmtId="165" formatCode="&quot;Remaining Capital to Next Milestone: $&quot;#,##0"/>
+    <numFmt numFmtId="166" formatCode="$#,##0&quot;/mo&quot;"/>
+    <numFmt numFmtId="167" formatCode="&quot;+$&quot;#,##0&quot; / Year Added To Net Worth&quot;"/>
+    <numFmt numFmtId="168" formatCode="&quot;+$&quot;#,##0&quot; (10-Yr Compounded Value)&quot;"/>
+    <numFmt numFmtId="169" formatCode="$#,##0.00&quot;/hr&quot;"/>
+    <numFmt numFmtId="170" formatCode="0.0&quot; Hours of Work&quot;"/>
+    <numFmt numFmtId="171" formatCode="+$#,##0;-$#,##0;$0"/>
+    <numFmt numFmtId="172" formatCode="+0.0%;-0.0%;0.0%"/>
+    <numFmt numFmtId="173" formatCode="0.0%"/>
+    <numFmt numFmtId="174" formatCode="&quot;+$&quot;#,##0;&quot;-$&quot;#,##0;&quot;$0&quot;"/>
+    <numFmt numFmtId="175" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="176" formatCode="0.0&quot; Months&quot;"/>
+    <numFmt numFmtId="177" formatCode="$#,##0/day"/>
+    <numFmt numFmtId="178" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
-  <fonts count="46" x14ac:knownFonts="1">
+  <fonts count="47" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -1017,7 +1028,7 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
+      <sz val="10.5"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -1052,9 +1063,8 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="10.5"/>
-      <name val="Arial"/>
+      <color rgb="FFCBD5E1"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <b/>
@@ -1088,7 +1098,7 @@
     <font>
       <b/>
       <color rgb="FF38BDF8"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
     <font>
       <b/>
@@ -1193,6 +1203,12 @@
       <sz val="15"/>
     </font>
     <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <name val="Arial"/>
+    </font>
+    <font>
       <i/>
       <color rgb="FF64748B"/>
       <sz val="9"/>
@@ -1292,10 +1308,10 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1316,25 +1332,29 @@
     <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="16" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="19" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="13" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="23" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="24" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="13" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="23" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="24" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="15" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="15" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1352,20 +1372,20 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="27" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="171" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="28" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="26" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="171" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="172" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="173" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="29" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="29" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="29" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="172" fontId="29" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1382,8 +1402,8 @@
     <xf numFmtId="0" fontId="33" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="34" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="172" fontId="35" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="174" fontId="34" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="173" fontId="35" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="35" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="24" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="36" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1398,7 +1418,7 @@
     <xf numFmtId="164" fontId="14" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="174" fontId="13" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="175" fontId="13" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1406,15 +1426,15 @@
     </xf>
     <xf numFmtId="0" fontId="39" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="34" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="173" fontId="34" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="40" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="34" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="173" fontId="34" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="40" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="14" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="175" fontId="13" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="14" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="13" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="173" fontId="14" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="41" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1423,7 +1443,7 @@
     </xf>
     <xf numFmtId="0" fontId="34" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="32" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="176" fontId="43" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="177" fontId="43" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="36" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="29" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1431,28 +1451,28 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="29" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="29" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="29" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="173" fontId="29" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="29" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="29" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="29" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="173" fontId="29" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="29" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="29" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="29" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="29" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="173" fontId="29" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="173" fontId="29" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="44" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="173" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="29" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="45" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="45" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="46" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="46" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="178" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1792,7 +1812,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:D51"/>
+  <dimension ref="B2:D25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1966,200 +1986,24 @@
       </c>
       <c r="D22" s="9"/>
     </row>
-    <row r="24" ht="26" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B24" s="10" t="s">
+    <row r="23" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B23" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
-    </row>
-    <row r="26" ht="26" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B26" s="11" t="s">
+      <c r="C23" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-    </row>
-    <row r="27" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B27" s="2" t="s">
+      <c r="D23" s="9"/>
+    </row>
+    <row r="25" ht="26" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B25" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-    </row>
-    <row r="29" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B29" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C29" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="D29" s="12" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="30" ht="26" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B30" s="13">
-        <v>30</v>
-      </c>
-      <c r="C30" s="14">
-        <v>95000</v>
-      </c>
-      <c r="D30" s="14">
-        <v>85000</v>
-      </c>
-    </row>
-    <row r="32" ht="18" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B32" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="C32" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="D32" s="15" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="33" ht="26" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B33" s="16">
-        <f>IF(D30&gt;=2*(B30*C30/10), "PAW (Top 10% Wealth Builder)", IF(D30&gt;=(B30*C30/10), "AAW (Solid Average)", "UAW (Under-Accumulator)"))</f>
-      </c>
-      <c r="C33" s="17">
-        <f>(B30*C30)/10</f>
-      </c>
-      <c r="D33" s="18">
-        <f>IF(D30&lt;100000, "$100k Club", IF(D30&lt;250000, "$250k Club", IF(D30&lt;500000, "$500k Club", "$1M Two-Comma Club")))</f>
-      </c>
-    </row>
-    <row r="36" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B36" s="19" t="s">
-        <v>46</v>
-      </c>
-      <c r="C36" s="19"/>
-      <c r="D36" s="19"/>
-    </row>
-    <row r="37" ht="19" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B37" s="20" t="s">
-        <v>47</v>
-      </c>
-      <c r="C37" s="20" t="s">
-        <v>48</v>
-      </c>
-      <c r="D37" s="20" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="38" ht="19" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B38" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="C38" s="21">
-        <v>35</v>
-      </c>
-      <c r="D38" s="22" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="39" ht="19" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B39" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="C39" s="21">
-        <v>45</v>
-      </c>
-      <c r="D39" s="22" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="40" ht="19" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B40" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="C40" s="21">
-        <v>75</v>
-      </c>
-      <c r="D40" s="22" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="41" ht="19" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B41" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="C41" s="21">
-        <v>40</v>
-      </c>
-      <c r="D41" s="22" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="42" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B42" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="C42" s="23">
-        <f>SUM(C38:C41)</f>
-      </c>
-      <c r="D42" s="24" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="44" ht="18" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B44" s="25" t="s">
-        <v>60</v>
-      </c>
-      <c r="C44" s="25"/>
-      <c r="D44" s="26" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="45" ht="26" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B45" s="27">
-        <f>C42*12</f>
-      </c>
-      <c r="C45" s="27"/>
-      <c r="D45" s="28">
-        <f>C42*182.946</f>
-      </c>
-    </row>
-    <row r="47" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B47" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="C47" s="19"/>
-      <c r="D47" s="19"/>
-    </row>
-    <row r="48" ht="19" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B48" s="20" t="s">
-        <v>63</v>
-      </c>
-      <c r="C48" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="D48" s="20" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="49" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B49" s="29">
-        <f>C30/2080</f>
-      </c>
-      <c r="C49" s="30">
-        <v>1200</v>
-      </c>
-      <c r="D49" s="31">
-        <f>C49/B49</f>
-      </c>
-    </row>
-    <row r="51" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B51" s="32" t="s">
-        <v>66</v>
-      </c>
-      <c r="C51" s="32"/>
-      <c r="D51" s="32"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="14">
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="B5:D5"/>
@@ -2172,14 +2016,8 @@
     <mergeCell ref="C20:D20"/>
     <mergeCell ref="C21:D21"/>
     <mergeCell ref="C22:D22"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B47:D47"/>
-    <mergeCell ref="B51:D51"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="B25:D25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2187,6 +2025,234 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B2:D32"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="4" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="38" customWidth="1"/>
+    <col min="5" max="5" width="4" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+    </row>
+    <row r="5" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B5" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+    </row>
+    <row r="6" ht="19" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B6" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" ht="26" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B7" s="13">
+        <v>30</v>
+      </c>
+      <c r="C7" s="14">
+        <v>95000</v>
+      </c>
+      <c r="D7" s="14">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B9" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B10" s="16">
+        <f>IF(D7&gt;=2*(B7*C7/10), "PAW (Top 10% Wealth Builder)", IF(D7&gt;=(B7*C7/10), "AAW (Solid Average Accumulator)", "UAW (Under-Accumulator)"))</f>
+      </c>
+      <c r="C10" s="17">
+        <f>(B7*C7)/10</f>
+      </c>
+      <c r="D10" s="18">
+        <f>IF(D7&lt;100000, "$100k Club", IF(D7&lt;250000, "$250k Club", IF(D7&lt;500000, "$500k Club", "$1M Two-Comma Club")))</f>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B12" s="19">
+        <f>MAX(0, IF(D7&lt;100000, 100000-D7, IF(D7&lt;250000, 250000-D7, IF(D7&lt;500000, 500000-D7, 1000000-D7))))</f>
+      </c>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+    </row>
+    <row r="15" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B15" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+    </row>
+    <row r="16" ht="19" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B16" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" ht="19" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B17" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C17" s="21">
+        <v>35</v>
+      </c>
+      <c r="D17" s="22" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="18" ht="19" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B18" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" s="21">
+        <v>45</v>
+      </c>
+      <c r="D18" s="22" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="19" ht="19" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B19" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" s="21">
+        <v>75</v>
+      </c>
+      <c r="D19" s="22" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="20" ht="19" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B20" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" s="21">
+        <v>40</v>
+      </c>
+      <c r="D20" s="22" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B21" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="23">
+        <f>SUM(C17:C20)</f>
+      </c>
+      <c r="D21" s="24" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B23" s="25" t="s">
+        <v>63</v>
+      </c>
+      <c r="C23" s="25"/>
+      <c r="D23" s="26" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B24" s="27">
+        <f>C21*12</f>
+      </c>
+      <c r="C24" s="27"/>
+      <c r="D24" s="28">
+        <f>C21*182.946</f>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B27" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+    </row>
+    <row r="28" ht="19" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B28" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="C28" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="D28" s="20" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B29" s="29">
+        <f>C7/2080</f>
+      </c>
+      <c r="C29" s="30">
+        <v>1200</v>
+      </c>
+      <c r="D29" s="31">
+        <f>C29/B29</f>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B32" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B32:D32"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:K18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -2206,7 +2272,7 @@
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -2220,7 +2286,7 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="33" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C3" s="33"/>
       <c r="D3" s="33"/>
@@ -2234,39 +2300,39 @@
     </row>
     <row r="5" ht="24" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" s="34" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C5" s="35" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D5" s="35" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E5" s="35" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="F5" s="35" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="G5" s="34" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="H5" s="34" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I5" s="34" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="J5" s="34" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="K5" s="34" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" s="36" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C6" s="37">
         <v>25000</v>
@@ -2298,7 +2364,7 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" s="43" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C7" s="44">
         <v>26200</v>
@@ -2330,7 +2396,7 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B8" s="36" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C8" s="37">
         <v>25800</v>
@@ -2362,7 +2428,7 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B9" s="43" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C9" s="44">
         <v>27100</v>
@@ -2394,7 +2460,7 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B10" s="36" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C10" s="37">
         <v>26900</v>
@@ -2426,7 +2492,7 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B11" s="43" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C11" s="44">
         <v>28400</v>
@@ -2458,7 +2524,7 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B12" s="36" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C12" s="37">
         <v>29000</v>
@@ -2490,7 +2556,7 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B13" s="43" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C13" s="44">
         <v>28500</v>
@@ -2522,7 +2588,7 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B14" s="36" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C14" s="37">
         <v>30200</v>
@@ -2554,7 +2620,7 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B15" s="43" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C15" s="44">
         <v>31000</v>
@@ -2586,7 +2652,7 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B16" s="36" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C16" s="37">
         <v>31500</v>
@@ -2618,7 +2684,7 @@
     </row>
     <row r="17" ht="20" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B17" s="43" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C17" s="44">
         <v>33000</v>
@@ -2650,7 +2716,7 @@
     </row>
     <row r="18" ht="22" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B18" s="48" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C18" s="49">
         <f>C17</f>
@@ -2690,7 +2756,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:F37"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -2704,7 +2770,7 @@
   <sheetData>
     <row r="2" ht="30" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B2" s="51" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C2" s="51"/>
       <c r="D2" s="51"/>
@@ -2713,7 +2779,7 @@
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B3" s="52" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C3" s="52"/>
       <c r="D3" s="52"/>
@@ -2722,15 +2788,15 @@
     </row>
     <row r="5" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="53" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C5" s="53"/>
       <c r="D5" s="53" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="E5" s="53"/>
       <c r="F5" s="53" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
@@ -2743,7 +2809,7 @@
       </c>
       <c r="E6" s="55"/>
       <c r="F6" s="56" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
@@ -2756,12 +2822,12 @@
       </c>
       <c r="E7" s="58"/>
       <c r="F7" s="59" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" s="60" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C9" s="60"/>
       <c r="D9" s="60"/>
@@ -2770,24 +2836,24 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" s="61" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C10" s="61" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D10" s="61" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E10" s="61" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="F10" s="61" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" s="6" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C11" s="37">
         <f>'2-Min Check-In'!G6</f>
@@ -2799,12 +2865,12 @@
         <f>'2-Min Check-In'!F6</f>
       </c>
       <c r="F11" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" s="62" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C12" s="44">
         <f>'2-Min Check-In'!G9</f>
@@ -2816,12 +2882,12 @@
         <f>'2-Min Check-In'!F9</f>
       </c>
       <c r="F12" s="62" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" s="6" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C13" s="37">
         <f>'2-Min Check-In'!G12</f>
@@ -2833,12 +2899,12 @@
         <f>'2-Min Check-In'!F12</f>
       </c>
       <c r="F13" s="6" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14" s="62" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C14" s="44">
         <f>'2-Min Check-In'!G15</f>
@@ -2850,12 +2916,12 @@
         <f>'2-Min Check-In'!F15</f>
       </c>
       <c r="F14" s="62" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" s="6" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C15" s="37">
         <f>'2-Min Check-In'!G17</f>
@@ -2867,12 +2933,12 @@
         <f>'2-Min Check-In'!F17</f>
       </c>
       <c r="F15" s="6" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="60" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C18" s="60"/>
       <c r="D18" s="60"/>
@@ -2881,37 +2947,37 @@
     </row>
     <row r="19" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" s="63" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C19" s="63" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D19" s="63" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E19" s="63" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F19" s="63"/>
     </row>
     <row r="20" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" s="64" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C20" s="64" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D20" s="64" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="E20" s="64" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F20" s="64"/>
     </row>
     <row r="22" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" s="65" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C22" s="65"/>
       <c r="D22" s="65"/>
@@ -2920,19 +2986,19 @@
     </row>
     <row r="23" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="66" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C23" s="66" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D23" s="66" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E23" s="66" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="F23" s="66" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
     <row r="24" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
@@ -2954,7 +3020,7 @@
     </row>
     <row r="26" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" s="71" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C26" s="71"/>
       <c r="D26" s="71"/>
@@ -2963,24 +3029,24 @@
     </row>
     <row r="27" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" s="66" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C27" s="66" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="D27" s="66" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E27" s="66" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F27" s="66" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="28" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" s="8" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C28" s="72">
         <v>100000</v>
@@ -2992,12 +3058,12 @@
         <f>MAX(0, C28-'2-Min Check-In'!G18)</f>
       </c>
       <c r="F28" s="74" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="29" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" s="75" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C29" s="76">
         <v>250000</v>
@@ -3009,12 +3075,12 @@
         <f>MAX(0, C29-'2-Min Check-In'!G18)</f>
       </c>
       <c r="F29" s="78" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="30" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" s="8" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C30" s="72">
         <v>500000</v>
@@ -3026,12 +3092,12 @@
         <f>MAX(0, C30-'2-Min Check-In'!G18)</f>
       </c>
       <c r="F30" s="74" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="31" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B31" s="75" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C31" s="76">
         <v>1000000</v>
@@ -3043,12 +3109,12 @@
         <f>MAX(0, C31-'2-Min Check-In'!G18)</f>
       </c>
       <c r="F31" s="78" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="33" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B33" s="65" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C33" s="65"/>
       <c r="D33" s="65"/>
@@ -3057,19 +3123,19 @@
     </row>
     <row r="34" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B34" s="66" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C34" s="66" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D34" s="66" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="E34" s="66" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="F34" s="66" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="35" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
@@ -3086,12 +3152,12 @@
         <f>B35/'2-Min Check-In'!G18</f>
       </c>
       <c r="F35" s="82" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="37" ht="22" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B37" s="83" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C37" s="83"/>
       <c r="D37" s="83"/>
@@ -3122,7 +3188,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:F30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -3137,7 +3203,7 @@
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B2" s="51" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C2" s="51"/>
       <c r="D2" s="51"/>
@@ -3146,7 +3212,7 @@
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B3" s="52" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="C3" s="52"/>
       <c r="D3" s="52"/>
@@ -3155,12 +3221,12 @@
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="84" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="C5" s="84"/>
       <c r="D5" s="84"/>
       <c r="E5" s="53" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="F5" s="53"/>
     </row>
@@ -3177,24 +3243,24 @@
     </row>
     <row r="8" ht="22" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="87" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C8" s="87" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D8" s="87" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="E8" s="87" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="F8" s="87" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" s="88" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C9" s="88"/>
       <c r="D9" s="88"/>
@@ -3203,7 +3269,7 @@
     </row>
     <row r="10" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="C10" s="37">
         <v>6800</v>
@@ -3215,12 +3281,12 @@
         <f>D10-C10</f>
       </c>
       <c r="F10" s="6" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" s="6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C11" s="37">
         <v>2200</v>
@@ -3232,12 +3298,12 @@
         <f>D11-C11</f>
       </c>
       <c r="F11" s="6" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" s="6" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C12" s="37">
         <v>500</v>
@@ -3249,12 +3315,12 @@
         <f>D12-C12</f>
       </c>
       <c r="F12" s="6" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" s="89" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C13" s="90">
         <f>SUM(C10:C12)</f>
@@ -3266,12 +3332,12 @@
         <f>D13-C13</f>
       </c>
       <c r="F13" s="89" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14" s="91" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C14" s="91"/>
       <c r="D14" s="91"/>
@@ -3280,7 +3346,7 @@
     </row>
     <row r="15" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" s="6" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C15" s="37">
         <v>2400</v>
@@ -3297,7 +3363,7 @@
     </row>
     <row r="16" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" s="6" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C16" s="37">
         <v>750</v>
@@ -3314,7 +3380,7 @@
     </row>
     <row r="17" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="6" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="C17" s="37">
         <v>320</v>
@@ -3331,7 +3397,7 @@
     </row>
     <row r="18" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="6" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C18" s="37">
         <v>450</v>
@@ -3348,7 +3414,7 @@
     </row>
     <row r="19" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" s="6" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C19" s="37">
         <v>400</v>
@@ -3365,7 +3431,7 @@
     </row>
     <row r="20" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" s="92" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="C20" s="93">
         <f>SUM(C15:C19)</f>
@@ -3382,7 +3448,7 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" s="95" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="C21" s="95"/>
       <c r="D21" s="95"/>
@@ -3391,7 +3457,7 @@
     </row>
     <row r="22" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" s="6" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C22" s="37">
         <v>650</v>
@@ -3408,7 +3474,7 @@
     </row>
     <row r="23" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="6" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C23" s="37">
         <v>120</v>
@@ -3425,7 +3491,7 @@
     </row>
     <row r="24" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" s="6" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C24" s="37">
         <v>450</v>
@@ -3442,7 +3508,7 @@
     </row>
     <row r="25" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" s="96" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="C25" s="97">
         <f>SUM(C22:C24)</f>
@@ -3459,7 +3525,7 @@
     </row>
     <row r="26" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" s="88" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C26" s="88"/>
       <c r="D26" s="88"/>
@@ -3468,7 +3534,7 @@
     </row>
     <row r="27" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" s="6" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C27" s="37">
         <v>2200</v>
@@ -3485,7 +3551,7 @@
     </row>
     <row r="28" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" s="6" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C28" s="37">
         <v>500</v>
@@ -3502,7 +3568,7 @@
     </row>
     <row r="29" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" s="6" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C29" s="37">
         <v>600</v>
@@ -3519,7 +3585,7 @@
     </row>
     <row r="30" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" s="99" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C30" s="100">
         <f>SUM(C27:C29)</f>
@@ -3552,7 +3618,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:H11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -3566,7 +3632,7 @@
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -3577,7 +3643,7 @@
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="33" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C3" s="33"/>
       <c r="D3" s="33"/>
@@ -3588,30 +3654,30 @@
     </row>
     <row r="5" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="87" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C5" s="87" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D5" s="87" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="E5" s="87" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F5" s="87" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="G5" s="87" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="H5" s="87" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C6" s="37">
         <v>25000</v>
@@ -3623,7 +3689,7 @@
         <f>C6-D6</f>
       </c>
       <c r="F6" s="6" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="G6" s="37">
         <v>700</v>
@@ -3634,7 +3700,7 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="62" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C7" s="44">
         <v>2000</v>
@@ -3646,7 +3712,7 @@
         <f>C7-D7</f>
       </c>
       <c r="F7" s="62" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="G7" s="44">
         <v>150</v>
@@ -3657,7 +3723,7 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C8" s="37">
         <v>4500</v>
@@ -3669,7 +3735,7 @@
         <f>C8-D8</f>
       </c>
       <c r="F8" s="6" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G8" s="37">
         <v>250</v>
@@ -3680,7 +3746,7 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="62" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="C9" s="44">
         <v>1500</v>
@@ -3692,7 +3758,7 @@
         <f>C9-D9</f>
       </c>
       <c r="F9" s="62" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="G9" s="44">
         <v>125</v>
@@ -3703,7 +3769,7 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C10" s="37">
         <v>3500</v>
@@ -3715,7 +3781,7 @@
         <f>C10-D10</f>
       </c>
       <c r="F10" s="6" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G10" s="37">
         <v>250</v>
@@ -3726,7 +3792,7 @@
     </row>
     <row r="11" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" s="48" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C11" s="49">
         <f>SUM(C6:C10)</f>
@@ -3738,7 +3804,7 @@
         <f>SUM(E6:E10)</f>
       </c>
       <c r="F11" s="48" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="G11" s="49">
         <f>SUM(G6:G10)</f>
@@ -3757,7 +3823,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:E16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -3772,7 +3838,7 @@
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B2" s="103" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="C2" s="103"/>
       <c r="D2" s="103"/>
@@ -3780,7 +3846,7 @@
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -3788,7 +3854,7 @@
     </row>
     <row r="5" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B5" s="6" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C5" s="104">
         <v>32</v>
@@ -3796,7 +3862,7 @@
     </row>
     <row r="6" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="C6" s="105">
         <v>66000</v>
@@ -3804,7 +3870,7 @@
     </row>
     <row r="7" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C7" s="106">
         <v>0.04</v>
@@ -3812,7 +3878,7 @@
     </row>
     <row r="8" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C8" s="106">
         <v>0.07</v>
@@ -3820,7 +3886,7 @@
     </row>
     <row r="9" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B9" s="6" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C9" s="105">
         <f>'2-Min Check-In'!D18</f>
@@ -3828,7 +3894,7 @@
     </row>
     <row r="10" ht="19" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="C10" s="105">
         <f>'Smart Budget (50-30-20)'!D27</f>
@@ -3836,7 +3902,7 @@
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B12" s="88" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="C12" s="88"/>
       <c r="D12" s="88"/>
@@ -3844,46 +3910,46 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="6" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="C13" s="105">
         <f>C6*0.65/C7</f>
       </c>
       <c r="D13" s="107" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B14" s="6" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="C14" s="105">
         <f>C6/C7</f>
       </c>
       <c r="D14" s="107" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B15" s="6" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="C15" s="105">
         <f>C6*1.4/C7</f>
       </c>
       <c r="D15" s="107" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="6" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="C16" s="105">
         <f>(C6/C7)/(1+C8)^(60-C5)</f>
       </c>
       <c r="D16" s="107" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
   </sheetData>
@@ -3897,7 +3963,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:F9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -3913,7 +3979,7 @@
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B2" s="103" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C2" s="103"/>
       <c r="D2" s="103"/>
@@ -3922,24 +3988,24 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" s="61" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="C4" s="61" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="D4" s="61" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="E4" s="61" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="F4" s="61" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="5" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="6" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C5" s="37">
         <v>4200</v>
@@ -3951,12 +4017,12 @@
         <v>140</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="6" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="C6" s="37">
         <v>8500</v>
@@ -3968,12 +4034,12 @@
         <v>210</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="C7" s="37">
         <v>17400</v>
@@ -3985,12 +4051,12 @@
         <v>380</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="C8" s="37">
         <v>200000</v>
@@ -4002,12 +4068,12 @@
         <v>1670</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" s="89" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="C9" s="90">
         <f>SUM(C5:C8)</f>
@@ -4019,7 +4085,7 @@
         <f>SUM(E5:E8)</f>
       </c>
       <c r="F9" s="89" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -4031,7 +4097,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:H36"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -4044,7 +4110,7 @@
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="103" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="C2" s="103"/>
       <c r="D2" s="103"/>
@@ -4055,30 +4121,30 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4" s="61" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="C4" s="61" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="D4" s="61" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="E4" s="61" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="F4" s="61" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="G4" s="61" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H4" s="61" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="5" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="6" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C5" s="37">
         <v>4800</v>
@@ -4101,7 +4167,7 @@
     </row>
     <row r="6" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="62" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="C6" s="44">
         <v>35000</v>
@@ -4124,7 +4190,7 @@
     </row>
     <row r="7" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="C7" s="37">
         <v>68000</v>
@@ -4147,7 +4213,7 @@
     </row>
     <row r="8" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="62" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="C8" s="44">
         <v>95000</v>
@@ -4170,7 +4236,7 @@
     </row>
     <row r="9" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="6" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C9" s="37">
         <v>110000</v>
@@ -4193,7 +4259,7 @@
     </row>
     <row r="10" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="62" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="C10" s="44">
         <v>92000</v>
@@ -4216,7 +4282,7 @@
     </row>
     <row r="13" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" s="110" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="C13" s="110"/>
       <c r="D13" s="110"/>
@@ -4227,30 +4293,30 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B14" s="61" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="C14" s="61" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="D14" s="61" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="E14" s="61" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="F14" s="61" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="G14" s="61" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="H14" s="61" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" s="6" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="C15" s="37">
         <v>285000</v>
@@ -4259,21 +4325,21 @@
         <v>1250000</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="F15" s="37">
         <v>785000</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B16" s="62" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C16" s="44">
         <v>245000</v>
@@ -4282,21 +4348,21 @@
         <v>1180000</v>
       </c>
       <c r="E16" s="62" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="F16" s="44">
         <v>650000</v>
       </c>
       <c r="G16" s="62" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="H16" s="62" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" s="6" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="C17" s="37">
         <v>275000</v>
@@ -4305,21 +4371,21 @@
         <v>1200000</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="F17" s="37">
         <v>610000</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" s="62" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C18" s="44">
         <v>175000</v>
@@ -4328,21 +4394,21 @@
         <v>820000</v>
       </c>
       <c r="E18" s="62" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="F18" s="44">
         <v>345000</v>
       </c>
       <c r="G18" s="62" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="H18" s="62" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" s="6" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="C19" s="37">
         <v>195000</v>
@@ -4351,21 +4417,21 @@
         <v>890000</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="F19" s="37">
         <v>395000</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B20" s="62" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="C20" s="44">
         <v>295000</v>
@@ -4374,21 +4440,21 @@
         <v>1320000</v>
       </c>
       <c r="E20" s="62" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="F20" s="44">
         <v>640000</v>
       </c>
       <c r="G20" s="62" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="H20" s="62" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B21" s="6" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C21" s="37">
         <v>185000</v>
@@ -4397,21 +4463,21 @@
         <v>860000</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="F21" s="37">
         <v>275000</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
     </row>
     <row r="22" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B22" s="62" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C22" s="44">
         <v>260000</v>
@@ -4420,21 +4486,21 @@
         <v>1100000</v>
       </c>
       <c r="E22" s="62" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="F22" s="44">
         <v>550000</v>
       </c>
       <c r="G22" s="62" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="H22" s="62" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
     </row>
     <row r="25" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B25" s="111" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="C25" s="111"/>
       <c r="D25" s="111"/>
@@ -4445,30 +4511,30 @@
     </row>
     <row r="26" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B26" s="61" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="C26" s="61" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="D26" s="61" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="E26" s="61" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="F26" s="61" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="G26" s="61" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="H26" s="61" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="27" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B27" s="6" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="C27" s="112">
         <v>1</v>
@@ -4480,18 +4546,18 @@
         <v>150000</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="28" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B28" s="62" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="C28" s="113">
         <v>2</v>
@@ -4503,18 +4569,18 @@
         <v>300000</v>
       </c>
       <c r="F28" s="62" t="s">
+        <v>299</v>
+      </c>
+      <c r="G28" s="62" t="s">
         <v>296</v>
       </c>
-      <c r="G28" s="62" t="s">
-        <v>293</v>
-      </c>
       <c r="H28" s="62" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="29" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B29" s="6" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="C29" s="112">
         <v>3</v>
@@ -4526,18 +4592,18 @@
         <v>450000</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="30" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B30" s="62" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="C30" s="113">
         <v>4</v>
@@ -4549,18 +4615,18 @@
         <v>600000</v>
       </c>
       <c r="F30" s="62" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="G30" s="62" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="H30" s="62" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="31" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B31" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="C31" s="112">
         <v>6</v>
@@ -4572,18 +4638,18 @@
         <v>900000</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="32" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B32" s="62" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="C32" s="113">
         <v>7</v>
@@ -4595,18 +4661,18 @@
         <v>1050000</v>
       </c>
       <c r="F32" s="62" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="G32" s="62" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="H32" s="62" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="33" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B33" s="6" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="C33" s="112">
         <v>8</v>
@@ -4618,18 +4684,18 @@
         <v>1200000</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="34" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B34" s="62" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="C34" s="113">
         <v>10</v>
@@ -4641,18 +4707,18 @@
         <v>1500000</v>
       </c>
       <c r="F34" s="62" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="G34" s="62" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="H34" s="62" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B36" s="83" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="C36" s="83"/>
       <c r="D36" s="83"/>

</xml_diff>

<commit_message>
fix(excel): resolve all formula references, cell coordinates, and statement ledger KPI cards across all 10 sheets
</commit_message>
<xml_diff>
--- a/public/downloads/NetWorth_FIRE_Master_Vault_2026.xlsx
+++ b/public/downloads/NetWorth_FIRE_Master_Vault_2026.xlsx
@@ -25,27 +25,32 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="18">
+  <numFmts count="23">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.00&quot;x&quot;"/>
-    <numFmt numFmtId="167" formatCode="#,##0 hrs"/>
-    <numFmt numFmtId="168" formatCode="$#,##0.00/hr"/>
+    <numFmt numFmtId="167" formatCode="#,##0 &quot;hrs&quot;"/>
+    <numFmt numFmtId="168" formatCode="$#,##0.00&quot;/hr&quot;"/>
     <numFmt numFmtId="169" formatCode="mmm yyyy"/>
     <numFmt numFmtId="170" formatCode="+$#,##0;-$#,##0;$0"/>
     <numFmt numFmtId="171" formatCode="+0.0%;-0.0%;0.0%"/>
-    <numFmt numFmtId="172" formatCode="0.0%&quot; Liquid&quot;"/>
-    <numFmt numFmtId="173" formatCode="&quot;Age Cohort: &quot;0&quot; Years&quot;"/>
-    <numFmt numFmtId="174" formatCode="mmmm yyyy"/>
-    <numFmt numFmtId="175" formatCode="$#,##0/day"/>
-    <numFmt numFmtId="176" formatCode="0.0%&quot; (Target ≤50%)&quot;"/>
-    <numFmt numFmtId="177" formatCode="0.0%&quot; (Target ≤30%)&quot;"/>
-    <numFmt numFmtId="178" formatCode="0.0%&quot; (Target ≥20%)&quot;"/>
-    <numFmt numFmtId="179" formatCode="$#,##0.00"/>
-    <numFmt numFmtId="180" formatCode="0.0%&quot; Funded&quot;"/>
-    <numFmt numFmtId="181" formatCode="0.0&quot; Years&quot;"/>
+    <numFmt numFmtId="172" formatCode="+$#,##0;-$#,##0;&quot;$0&quot; Annual Gain"/>
+    <numFmt numFmtId="173" formatCode="0.0%&quot; Liquid&quot;"/>
+    <numFmt numFmtId="174" formatCode="&quot;Age Cohort: &quot;0&quot; Years&quot;"/>
+    <numFmt numFmtId="175" formatCode="0.0%&quot; Funded&quot;"/>
+    <numFmt numFmtId="176" formatCode="mmmm yyyy"/>
+    <numFmt numFmtId="177" formatCode="0.0&quot; Years Remaining&quot;"/>
+    <numFmt numFmtId="178" formatCode="$#,##0/day"/>
+    <numFmt numFmtId="179" formatCode="0.0%&quot; (Target ≤50%)&quot;"/>
+    <numFmt numFmtId="180" formatCode="0.0%&quot; (Target ≤30%)&quot;"/>
+    <numFmt numFmtId="181" formatCode="0.0%&quot; (Target ≥20%)&quot;"/>
+    <numFmt numFmtId="182" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="183" formatCode="0.0%&quot; of Outflows&quot;"/>
+    <numFmt numFmtId="184" formatCode="0.0&quot; Years&quot;"/>
+    <numFmt numFmtId="185" formatCode="0&quot; mos&quot;"/>
+    <numFmt numFmtId="186" formatCode="0&quot; mos saved&quot;"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="27">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -133,12 +138,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="0010B981"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <color rgb="00F59E0B"/>
       <sz val="14"/>
     </font>
@@ -157,8 +156,32 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="0010B981"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="15"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0010B981"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0010B981"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -191,7 +214,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -232,12 +255,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F8FAFC"/>
         <bgColor rgb="00F8FAFC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="008B5CF6"/>
-        <bgColor rgb="008B5CF6"/>
       </patternFill>
     </fill>
   </fills>
@@ -281,7 +298,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -289,36 +306,36 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="8" fillId="5" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="8" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="5" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="165" fontId="8" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -337,21 +354,25 @@
     <xf numFmtId="167" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="5" fillId="5" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="168" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="169" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -396,59 +417,77 @@
     <xf numFmtId="164" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="14" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="172" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="173" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="174" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="176" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="174" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="175" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="177" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="13" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="175" fontId="18" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="178" fontId="18" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="176" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="177" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="178" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="179" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="180" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="181" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="20" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="21" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="179" fontId="5" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="182" fontId="5" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -465,7 +504,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="175" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -475,31 +514,33 @@
     <xf numFmtId="165" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="184" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="174" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="176" fontId="25" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="8" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="10" fontId="23" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="26" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="185" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="186" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1200,8 +1241,8 @@
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
     <col width="3" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -1277,7 +1318,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1">
+    <row r="10" ht="22" customHeight="1">
       <c r="B10" s="7" t="inlineStr">
         <is>
           <t>⚙️ MASTER SETUP &amp; PROFILE (ENTER ONCE — POWERS ALL 8 TABS)</t>
@@ -1290,7 +1331,7 @@
           <t>Setup Parameter</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Your Value (Green Input)</t>
         </is>
@@ -1301,13 +1342,13 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1">
+    <row r="12" ht="20" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Your Current Age</t>
         </is>
       </c>
-      <c r="C12" s="10" t="n">
+      <c r="C12" s="9" t="n">
         <v>32</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -1316,13 +1357,13 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1">
+    <row r="13" ht="20" customHeight="1">
       <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Pre-Tax Annual Household Income</t>
         </is>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="10" t="n">
         <v>108000</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1331,13 +1372,13 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
+    <row r="14" ht="20" customHeight="1">
       <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Target Retirement / Independence Age</t>
         </is>
       </c>
-      <c r="C14" s="10" t="n">
+      <c r="C14" s="9" t="n">
         <v>60</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1346,13 +1387,13 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
+    <row r="15" ht="20" customHeight="1">
       <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Target Annual Spending in Retirement</t>
         </is>
       </c>
-      <c r="C15" s="11" t="n">
+      <c r="C15" s="10" t="n">
         <v>66000</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1361,13 +1402,13 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
+    <row r="16" ht="20" customHeight="1">
       <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Safe Withdrawal Rate (SWR)</t>
         </is>
       </c>
-      <c r="C16" s="12" t="n">
+      <c r="C16" s="11" t="n">
         <v>0.04</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -1376,13 +1417,13 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
+    <row r="17" ht="20" customHeight="1">
       <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Expected Real Return After Inflation</t>
         </is>
       </c>
-      <c r="C17" s="12" t="n">
+      <c r="C17" s="11" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -1391,13 +1432,13 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
+    <row r="18" ht="20" customHeight="1">
       <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Lean FIRE Spending Ratio</t>
         </is>
       </c>
-      <c r="C18" s="12" t="n">
+      <c r="C18" s="11" t="n">
         <v>0.65</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -1406,13 +1447,13 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
+    <row r="19" ht="20" customHeight="1">
       <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Check-In Start Year</t>
         </is>
       </c>
-      <c r="C19" s="10" t="n">
+      <c r="C19" s="9" t="n">
         <v>2026</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -1421,13 +1462,13 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
+    <row r="20" ht="20" customHeight="1">
       <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Check-In Start Month (1 = Jan, 10 = Oct)</t>
         </is>
       </c>
-      <c r="C20" s="10" t="n">
+      <c r="C20" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -1437,13 +1478,13 @@
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>🎨 WORKBOOK GUARDRAILS &amp; COLOR CODES</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="20" customHeight="1">
+    <row r="23" ht="19" customHeight="1">
       <c r="B23" s="4" t="inlineStr">
         <is>
           <t>🟩 GREEN CELLS</t>
@@ -1460,7 +1501,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="20" customHeight="1">
+    <row r="24" ht="19" customHeight="1">
       <c r="B24" s="4" t="inlineStr">
         <is>
           <t>⬛ DARK / SLATE CELLS</t>
@@ -1477,7 +1518,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="20" customHeight="1">
+    <row r="25" ht="19" customHeight="1">
       <c r="B25" s="4" t="inlineStr">
         <is>
           <t>🟨 GOLD / AMBER CELLS</t>
@@ -1495,7 +1536,7 @@
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>📖 TAB DIRECTORY &amp; WORKFLOW</t>
         </is>
@@ -1512,7 +1553,7 @@
           <t>Master setup area, user manual, methodology citations &amp; legal notices.</t>
         </is>
       </c>
-      <c r="D28" s="14" t="n"/>
+      <c r="D28" s="13" t="n"/>
     </row>
     <row r="29" ht="19" customHeight="1">
       <c r="B29" s="4" t="inlineStr">
@@ -1525,7 +1566,7 @@
           <t>Instant baseline: Stanley &amp; Danko PAW tier, leak audit &amp; true hourly wage.</t>
         </is>
       </c>
-      <c r="D29" s="14" t="n"/>
+      <c r="D29" s="13" t="n"/>
     </row>
     <row r="30" ht="19" customHeight="1">
       <c r="B30" s="4" t="inlineStr">
@@ -1538,7 +1579,7 @@
           <t>Monthly routine: 4 numbers once a month with rolling open-ended calendar.</t>
         </is>
       </c>
-      <c r="D30" s="14" t="n"/>
+      <c r="D30" s="13" t="n"/>
     </row>
     <row r="31" ht="19" customHeight="1">
       <c r="B31" s="4" t="inlineStr">
@@ -1551,7 +1592,7 @@
           <t>Visual dashboard with dynamic Fed rank, FIRE counters, and trajectory chart.</t>
         </is>
       </c>
-      <c r="D31" s="14" t="n"/>
+      <c r="D31" s="13" t="n"/>
     </row>
     <row r="32" ht="19" customHeight="1">
       <c r="B32" s="4" t="inlineStr">
@@ -1564,7 +1605,7 @@
           <t>Answers 'How much can I spend today guilt-free?' with live spending buffer.</t>
         </is>
       </c>
-      <c r="D32" s="14" t="n"/>
+      <c r="D32" s="13" t="n"/>
     </row>
     <row r="33" ht="19" customHeight="1">
       <c r="B33" s="4" t="inlineStr">
@@ -1574,10 +1615,10 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Private drop-zone for bank statements converted via our web utility.</t>
-        </is>
-      </c>
-      <c r="D33" s="14" t="n"/>
+          <t>Private drop-zone for bank statements with live 50/30/20 summary cards.</t>
+        </is>
+      </c>
+      <c r="D33" s="13" t="n"/>
     </row>
     <row r="34" ht="19" customHeight="1">
       <c r="B34" s="4" t="inlineStr">
@@ -1590,7 +1631,7 @@
           <t>Target funds protecting against car repairs, travel, and annual shocks.</t>
         </is>
       </c>
-      <c r="D34" s="14" t="n"/>
+      <c r="D34" s="13" t="n"/>
     </row>
     <row r="35" ht="19" customHeight="1">
       <c r="B35" s="4" t="inlineStr">
@@ -1603,7 +1644,7 @@
           <t>Coast, Lean, Standard &amp; Fat FIRE milestones with dynamic freedom date.</t>
         </is>
       </c>
-      <c r="D35" s="14" t="n"/>
+      <c r="D35" s="13" t="n"/>
     </row>
     <row r="36" ht="19" customHeight="1">
       <c r="B36" s="4" t="inlineStr">
@@ -1616,7 +1657,7 @@
           <t>Ranked Avalanche vs Snowball schedule with exact interest savings.</t>
         </is>
       </c>
-      <c r="D36" s="14" t="n"/>
+      <c r="D36" s="13" t="n"/>
     </row>
     <row r="37" ht="19" customHeight="1">
       <c r="B37" s="4" t="inlineStr">
@@ -1629,17 +1670,17 @@
           <t>Raw 2022 Federal Reserve SCF survey tables &amp; state cost-of-living index.</t>
         </is>
       </c>
-      <c r="D37" s="14" t="n"/>
+      <c r="D37" s="13" t="n"/>
     </row>
     <row r="39" ht="22" customHeight="1">
-      <c r="B39" s="13" t="inlineStr">
+      <c r="B39" s="7" t="inlineStr">
         <is>
           <t>⚖️ DATA SOURCING &amp; EDUCATIONAL DISCLAIMER</t>
         </is>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1">
-      <c r="B40" s="15" t="inlineStr">
+      <c r="B40" s="14" t="inlineStr">
         <is>
           <t>1. Federal Reserve Benchmarks are derived from the 2022 Survey of Consumer Finances (SCF), the latest official triennial release by the Federal Reserve Board. State wealth indices are illustrative estimates modeled using Fed SCF regional microdata and US Census Bureau median income ratios.
 2. This spreadsheet is strictly for personal budgeting, educational, and organizational purposes. It does not constitute financial, investment, accounting, tax, or legal advice. Consult a licensed CFP or CPA for specific financial planning.</t>
@@ -1707,44 +1748,44 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="B4" s="8" t="inlineStr">
+    <row r="4" ht="22" customHeight="1">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Age Bracket</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>25th Pct</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>50th (Median)</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="15" t="inlineStr">
         <is>
           <t>75th Pct</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F4" s="15" t="inlineStr">
         <is>
           <t>90th Pct</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
+      <c r="G4" s="15" t="inlineStr">
         <is>
           <t>95th Pct</t>
         </is>
       </c>
-      <c r="H4" s="8" t="inlineStr">
+      <c r="H4" s="15" t="inlineStr">
         <is>
           <t>Top 1% (99th)</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="19" customHeight="1">
+    <row r="5" ht="20" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Under 35</t>
@@ -1769,7 +1810,7 @@
         <v>2800000</v>
       </c>
     </row>
-    <row r="6" ht="19" customHeight="1">
+    <row r="6" ht="20" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
           <t>35 - 44</t>
@@ -1794,7 +1835,7 @@
         <v>5500000</v>
       </c>
     </row>
-    <row r="7" ht="19" customHeight="1">
+    <row r="7" ht="20" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
           <t>45 - 54</t>
@@ -1819,7 +1860,7 @@
         <v>10200000</v>
       </c>
     </row>
-    <row r="8" ht="19" customHeight="1">
+    <row r="8" ht="20" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
           <t>55 - 64</t>
@@ -1844,7 +1885,7 @@
         <v>14500000</v>
       </c>
     </row>
-    <row r="9" ht="19" customHeight="1">
+    <row r="9" ht="20" customHeight="1">
       <c r="B9" s="4" t="inlineStr">
         <is>
           <t>65 - 74</t>
@@ -1869,7 +1910,7 @@
         <v>16800000</v>
       </c>
     </row>
-    <row r="10" ht="19" customHeight="1">
+    <row r="10" ht="20" customHeight="1">
       <c r="B10" s="4" t="inlineStr">
         <is>
           <t>75+</t>
@@ -1894,52 +1935,52 @@
         <v>13200000</v>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="57" t="inlineStr">
+    <row r="13" ht="22" customHeight="1">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>📍 US STATES WEALTH &amp; COST-OF-LIVING INDEX (ILLUSTRATIVE ESTIMATES)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="91" t="inlineStr">
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Modeled using Fed SCF regional microdata combined with US Census Bureau state median income ratios.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="B15" s="46" t="inlineStr">
+      <c r="B15" s="48" t="inlineStr">
         <is>
           <t>US State</t>
         </is>
       </c>
-      <c r="C15" s="46" t="inlineStr">
+      <c r="C15" s="48" t="inlineStr">
         <is>
           <t>Median NW (Est)</t>
         </is>
       </c>
-      <c r="D15" s="46" t="inlineStr">
+      <c r="D15" s="48" t="inlineStr">
         <is>
           <t>Top 10% NW (Est)</t>
         </is>
       </c>
-      <c r="E15" s="46" t="inlineStr">
+      <c r="E15" s="48" t="inlineStr">
         <is>
           <t>COL Index</t>
         </is>
       </c>
-      <c r="F15" s="46" t="inlineStr">
+      <c r="F15" s="48" t="inlineStr">
         <is>
           <t>Median Home</t>
         </is>
       </c>
-      <c r="G15" s="46" t="inlineStr">
+      <c r="G15" s="48" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="H15" s="46" t="inlineStr">
+      <c r="H15" s="48" t="inlineStr">
         <is>
           <t>Source Model</t>
         </is>
@@ -1951,21 +1992,21 @@
           <t>California (CA)</t>
         </is>
       </c>
-      <c r="C16" s="92" t="n">
+      <c r="C16" s="101" t="n">
         <v>285000</v>
       </c>
-      <c r="D16" s="92" t="n">
+      <c r="D16" s="101" t="n">
         <v>1250000</v>
       </c>
-      <c r="E16" s="93" t="inlineStr">
+      <c r="E16" s="102" t="inlineStr">
         <is>
           <t>138.5 (HCOL)</t>
         </is>
       </c>
-      <c r="F16" s="92" t="n">
+      <c r="F16" s="101" t="n">
         <v>785000</v>
       </c>
-      <c r="G16" s="93" t="inlineStr">
+      <c r="G16" s="102" t="inlineStr">
         <is>
           <t>Top Tier</t>
         </is>
@@ -1982,21 +2023,21 @@
           <t>New York (NY)</t>
         </is>
       </c>
-      <c r="C17" s="92" t="n">
+      <c r="C17" s="101" t="n">
         <v>245000</v>
       </c>
-      <c r="D17" s="92" t="n">
+      <c r="D17" s="101" t="n">
         <v>1180000</v>
       </c>
-      <c r="E17" s="93" t="inlineStr">
+      <c r="E17" s="102" t="inlineStr">
         <is>
           <t>134.2 (HCOL)</t>
         </is>
       </c>
-      <c r="F17" s="92" t="n">
+      <c r="F17" s="101" t="n">
         <v>650000</v>
       </c>
-      <c r="G17" s="93" t="inlineStr">
+      <c r="G17" s="102" t="inlineStr">
         <is>
           <t>Top Tier</t>
         </is>
@@ -2013,21 +2054,21 @@
           <t>Washington (WA)</t>
         </is>
       </c>
-      <c r="C18" s="92" t="n">
+      <c r="C18" s="101" t="n">
         <v>275000</v>
       </c>
-      <c r="D18" s="92" t="n">
+      <c r="D18" s="101" t="n">
         <v>1200000</v>
       </c>
-      <c r="E18" s="93" t="inlineStr">
+      <c r="E18" s="102" t="inlineStr">
         <is>
           <t>115.1 (MCOL+)</t>
         </is>
       </c>
-      <c r="F18" s="92" t="n">
+      <c r="F18" s="101" t="n">
         <v>610000</v>
       </c>
-      <c r="G18" s="93" t="inlineStr">
+      <c r="G18" s="102" t="inlineStr">
         <is>
           <t>Top Tier</t>
         </is>
@@ -2044,21 +2085,21 @@
           <t>Texas (TX)</t>
         </is>
       </c>
-      <c r="C19" s="92" t="n">
+      <c r="C19" s="101" t="n">
         <v>175000</v>
       </c>
-      <c r="D19" s="92" t="n">
+      <c r="D19" s="101" t="n">
         <v>820000</v>
       </c>
-      <c r="E19" s="93" t="inlineStr">
+      <c r="E19" s="102" t="inlineStr">
         <is>
           <t>92.5 (LCOL)</t>
         </is>
       </c>
-      <c r="F19" s="92" t="n">
+      <c r="F19" s="101" t="n">
         <v>345000</v>
       </c>
-      <c r="G19" s="93" t="inlineStr">
+      <c r="G19" s="102" t="inlineStr">
         <is>
           <t>High Value</t>
         </is>
@@ -2075,21 +2116,21 @@
           <t>Florida (FL)</t>
         </is>
       </c>
-      <c r="C20" s="92" t="n">
+      <c r="C20" s="101" t="n">
         <v>195000</v>
       </c>
-      <c r="D20" s="92" t="n">
+      <c r="D20" s="101" t="n">
         <v>890000</v>
       </c>
-      <c r="E20" s="93" t="inlineStr">
+      <c r="E20" s="102" t="inlineStr">
         <is>
           <t>102.8 (Avg)</t>
         </is>
       </c>
-      <c r="F20" s="92" t="n">
+      <c r="F20" s="101" t="n">
         <v>395000</v>
       </c>
-      <c r="G20" s="93" t="inlineStr">
+      <c r="G20" s="102" t="inlineStr">
         <is>
           <t>Growing</t>
         </is>
@@ -2106,21 +2147,21 @@
           <t>Massachusetts (MA)</t>
         </is>
       </c>
-      <c r="C21" s="92" t="n">
+      <c r="C21" s="101" t="n">
         <v>295000</v>
       </c>
-      <c r="D21" s="92" t="n">
+      <c r="D21" s="101" t="n">
         <v>1320000</v>
       </c>
-      <c r="E21" s="93" t="inlineStr">
+      <c r="E21" s="102" t="inlineStr">
         <is>
           <t>148.0 (HCOL)</t>
         </is>
       </c>
-      <c r="F21" s="92" t="n">
+      <c r="F21" s="101" t="n">
         <v>640000</v>
       </c>
-      <c r="G21" s="93" t="inlineStr">
+      <c r="G21" s="102" t="inlineStr">
         <is>
           <t>Top Tier</t>
         </is>
@@ -2137,21 +2178,21 @@
           <t>Illinois (IL)</t>
         </is>
       </c>
-      <c r="C22" s="92" t="n">
+      <c r="C22" s="101" t="n">
         <v>185000</v>
       </c>
-      <c r="D22" s="92" t="n">
+      <c r="D22" s="101" t="n">
         <v>860000</v>
       </c>
-      <c r="E22" s="93" t="inlineStr">
+      <c r="E22" s="102" t="inlineStr">
         <is>
           <t>91.8 (LCOL)</t>
         </is>
       </c>
-      <c r="F22" s="92" t="n">
+      <c r="F22" s="101" t="n">
         <v>275000</v>
       </c>
-      <c r="G22" s="93" t="inlineStr">
+      <c r="G22" s="102" t="inlineStr">
         <is>
           <t>High Value</t>
         </is>
@@ -2168,21 +2209,21 @@
           <t>Colorado (CO)</t>
         </is>
       </c>
-      <c r="C23" s="92" t="n">
+      <c r="C23" s="101" t="n">
         <v>260000</v>
       </c>
-      <c r="D23" s="92" t="n">
+      <c r="D23" s="101" t="n">
         <v>1100000</v>
       </c>
-      <c r="E23" s="93" t="inlineStr">
+      <c r="E23" s="102" t="inlineStr">
         <is>
           <t>105.4 (Avg)</t>
         </is>
       </c>
-      <c r="F23" s="92" t="n">
+      <c r="F23" s="101" t="n">
         <v>550000</v>
       </c>
-      <c r="G23" s="93" t="inlineStr">
+      <c r="G23" s="102" t="inlineStr">
         <is>
           <t>High Growth</t>
         </is>
@@ -2215,7 +2256,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
     <col width="3" customWidth="1" min="5" max="5"/>
@@ -2236,24 +2277,24 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>🎯 WEALTH ACCUMULATION TIER (READS FROM MASTER SETUP)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>1. CURRENT AGE (FROM SETUP)</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>2. ANNUAL PRE-TAX INCOME</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>3. CURRENT NET WORTH (FROM CHECK-IN)</t>
         </is>
@@ -2274,17 +2315,17 @@
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>🏆 STANLEY &amp; DANKO WEALTH CLASS</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>🎯 EXPECTED NET WORTH (AGE×INC/10)</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>🚀 ACCUMULATION MULTIPLIER</t>
         </is>
@@ -2292,7 +2333,7 @@
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="B10" s="18">
-        <f>IF(C10&lt;=0, "N/A", IF(D10&gt;=2.0, "PAW (Prodigious Accumulator of Wealth)", IF(D10&gt;=0.5, "AAW (Average Accumulator of Wealth)", "UAW (Under-Accumulator of Wealth)")))</f>
+        <f>IF(B7&lt;=0, "Setup Required", IF(C10&lt;=0, "N/A", IF(D10&gt;=2.0, "PAW (Prodigious Accumulator of Wealth)", IF(D10&gt;=0.5, "AAW (Average Accumulator of Wealth)", "UAW (Under-Accumulator of Wealth)"))))</f>
         <v/>
       </c>
       <c r="C10" s="17">
@@ -2305,7 +2346,7 @@
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>⏳ TRUE HOURLY WAGE &amp; LIFE ENERGY ENGINE (YOUR REAL PAY RATE)</t>
         </is>
@@ -2333,12 +2374,12 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="22" t="inlineStr">
         <is>
           <t>Annual Work Commute Hours</t>
         </is>
       </c>
-      <c r="C16" s="22" t="n">
+      <c r="C16" s="23" t="n">
         <v>250</v>
       </c>
     </row>
@@ -2349,17 +2390,17 @@
         </is>
       </c>
       <c r="C17" s="20">
-        <f>B14*0.25</f>
+        <f>C14*0.25</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="22" t="inlineStr">
         <is>
           <t>Annual Work-Related Expenses (Commute, Clothes, Food)</t>
         </is>
       </c>
-      <c r="C18" s="23" t="n">
+      <c r="C18" s="24" t="n">
         <v>4800</v>
       </c>
     </row>
@@ -2370,7 +2411,7 @@
         </is>
       </c>
       <c r="C19" s="20">
-        <f>B14-B17-B18</f>
+        <f>C14-C17-C18</f>
         <v/>
       </c>
     </row>
@@ -2381,7 +2422,7 @@
         </is>
       </c>
       <c r="C20" s="21">
-        <f>B15+B16</f>
+        <f>C15+C16</f>
         <v/>
       </c>
     </row>
@@ -2391,8 +2432,8 @@
           <t>⭐ TRUE HOURLY LIFE ENERGY WAGE</t>
         </is>
       </c>
-      <c r="C21" s="24">
-        <f>IFERROR(B19/B20, 0)</f>
+      <c r="C21" s="25">
+        <f>IFERROR(C19/C20, 0)</f>
         <v/>
       </c>
     </row>
@@ -2446,119 +2487,119 @@
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>Month / Period</t>
         </is>
       </c>
-      <c r="C5" s="26" t="inlineStr">
+      <c r="C5" s="27" t="inlineStr">
         <is>
           <t>💵 Cash &amp; Savings</t>
         </is>
       </c>
-      <c r="D5" s="26" t="inlineStr">
+      <c r="D5" s="27" t="inlineStr">
         <is>
           <t>📈 Invested Portfolio</t>
         </is>
       </c>
-      <c r="E5" s="26" t="inlineStr">
+      <c r="E5" s="27" t="inlineStr">
         <is>
           <t>🏠 Property &amp; Assets</t>
         </is>
       </c>
-      <c r="F5" s="26" t="inlineStr">
+      <c r="F5" s="27" t="inlineStr">
         <is>
           <t>💳 Total Debts</t>
         </is>
       </c>
-      <c r="G5" s="25" t="inlineStr">
+      <c r="G5" s="28" t="inlineStr">
         <is>
           <t>🏛️ TOTAL NET WORTH</t>
         </is>
       </c>
-      <c r="H5" s="25" t="inlineStr">
+      <c r="H5" s="26" t="inlineStr">
         <is>
           <t>MoM Gain ($)</t>
         </is>
       </c>
-      <c r="I5" s="25" t="inlineStr">
+      <c r="I5" s="26" t="inlineStr">
         <is>
           <t>Growth (%)</t>
         </is>
       </c>
-      <c r="J5" s="25" t="inlineStr">
+      <c r="J5" s="26" t="inlineStr">
         <is>
           <t>💧 Liquid Net Worth</t>
         </is>
       </c>
-      <c r="K5" s="25" t="inlineStr">
+      <c r="K5" s="26" t="inlineStr">
         <is>
           <t>Liquid Ratio</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="B6" s="27">
+      <c r="B6" s="29">
         <f>DATE('START HERE'!C19, 'START HERE'!C20, 1)</f>
         <v/>
       </c>
-      <c r="C6" s="28" t="n">
+      <c r="C6" s="30" t="n">
         <v>25000</v>
       </c>
-      <c r="D6" s="28" t="n">
+      <c r="D6" s="30" t="n">
         <v>185000</v>
       </c>
-      <c r="E6" s="28" t="n">
+      <c r="E6" s="30" t="n">
         <v>350000</v>
       </c>
-      <c r="F6" s="28" t="n">
+      <c r="F6" s="30" t="n">
         <v>245000</v>
       </c>
-      <c r="G6" s="29">
+      <c r="G6" s="31">
         <f>(C6+D6+E6)-F6</f>
         <v/>
       </c>
-      <c r="H6" s="30" t="n">
+      <c r="H6" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="31" t="n">
+      <c r="I6" s="33" t="n">
         <v>0</v>
       </c>
       <c r="J6" s="20">
         <f>C6+D6</f>
         <v/>
       </c>
-      <c r="K6" s="32">
+      <c r="K6" s="34">
         <f>IFERROR(J6/G6, 0)</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="B7" s="27">
+      <c r="B7" s="29">
         <f>EDATE(B6, 1)</f>
         <v/>
       </c>
-      <c r="C7" s="28" t="n">
+      <c r="C7" s="30" t="n">
         <v>26200</v>
       </c>
-      <c r="D7" s="28" t="n">
+      <c r="D7" s="30" t="n">
         <v>189500</v>
       </c>
-      <c r="E7" s="28" t="n">
+      <c r="E7" s="30" t="n">
         <v>350000</v>
       </c>
-      <c r="F7" s="28" t="n">
+      <c r="F7" s="30" t="n">
         <v>243800</v>
       </c>
-      <c r="G7" s="29">
+      <c r="G7" s="31">
         <f>(C7+D7+E7)-F7</f>
         <v/>
       </c>
-      <c r="H7" s="30">
+      <c r="H7" s="32">
         <f>G7-G6</f>
         <v/>
       </c>
-      <c r="I7" s="31">
+      <c r="I7" s="33">
         <f>IFERROR((G7-G6)/G6, 0)</f>
         <v/>
       </c>
@@ -2566,37 +2607,37 @@
         <f>C7+D7</f>
         <v/>
       </c>
-      <c r="K7" s="32">
+      <c r="K7" s="34">
         <f>IFERROR(J7/G7, 0)</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="B8" s="27">
+      <c r="B8" s="29">
         <f>EDATE(B7, 1)</f>
         <v/>
       </c>
-      <c r="C8" s="28" t="n">
+      <c r="C8" s="30" t="n">
         <v>25800</v>
       </c>
-      <c r="D8" s="28" t="n">
+      <c r="D8" s="30" t="n">
         <v>194200</v>
       </c>
-      <c r="E8" s="28" t="n">
+      <c r="E8" s="30" t="n">
         <v>350000</v>
       </c>
-      <c r="F8" s="28" t="n">
+      <c r="F8" s="30" t="n">
         <v>242600</v>
       </c>
-      <c r="G8" s="29">
+      <c r="G8" s="31">
         <f>(C8+D8+E8)-F8</f>
         <v/>
       </c>
-      <c r="H8" s="30">
+      <c r="H8" s="32">
         <f>G8-G7</f>
         <v/>
       </c>
-      <c r="I8" s="31">
+      <c r="I8" s="33">
         <f>IFERROR((G8-G7)/G7, 0)</f>
         <v/>
       </c>
@@ -2604,37 +2645,37 @@
         <f>C8+D8</f>
         <v/>
       </c>
-      <c r="K8" s="32">
+      <c r="K8" s="34">
         <f>IFERROR(J8/G8, 0)</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="B9" s="27">
+      <c r="B9" s="29">
         <f>EDATE(B8, 1)</f>
         <v/>
       </c>
-      <c r="C9" s="28" t="n">
+      <c r="C9" s="30" t="n">
         <v>27100</v>
       </c>
-      <c r="D9" s="28" t="n">
+      <c r="D9" s="30" t="n">
         <v>191000</v>
       </c>
-      <c r="E9" s="28" t="n">
+      <c r="E9" s="30" t="n">
         <v>350000</v>
       </c>
-      <c r="F9" s="28" t="n">
+      <c r="F9" s="30" t="n">
         <v>241400</v>
       </c>
-      <c r="G9" s="29">
+      <c r="G9" s="31">
         <f>(C9+D9+E9)-F9</f>
         <v/>
       </c>
-      <c r="H9" s="30">
+      <c r="H9" s="32">
         <f>G9-G8</f>
         <v/>
       </c>
-      <c r="I9" s="31">
+      <c r="I9" s="33">
         <f>IFERROR((G9-G8)/G8, 0)</f>
         <v/>
       </c>
@@ -2642,37 +2683,37 @@
         <f>C9+D9</f>
         <v/>
       </c>
-      <c r="K9" s="32">
+      <c r="K9" s="34">
         <f>IFERROR(J9/G9, 0)</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="B10" s="27">
+      <c r="B10" s="29">
         <f>EDATE(B9, 1)</f>
         <v/>
       </c>
-      <c r="C10" s="28" t="n">
+      <c r="C10" s="30" t="n">
         <v>26900</v>
       </c>
-      <c r="D10" s="28" t="n">
+      <c r="D10" s="30" t="n">
         <v>198500</v>
       </c>
-      <c r="E10" s="28" t="n">
+      <c r="E10" s="30" t="n">
         <v>352000</v>
       </c>
-      <c r="F10" s="28" t="n">
+      <c r="F10" s="30" t="n">
         <v>240100</v>
       </c>
-      <c r="G10" s="29">
+      <c r="G10" s="31">
         <f>(C10+D10+E10)-F10</f>
         <v/>
       </c>
-      <c r="H10" s="30">
+      <c r="H10" s="32">
         <f>G10-G9</f>
         <v/>
       </c>
-      <c r="I10" s="31">
+      <c r="I10" s="33">
         <f>IFERROR((G10-G9)/G9, 0)</f>
         <v/>
       </c>
@@ -2680,37 +2721,37 @@
         <f>C10+D10</f>
         <v/>
       </c>
-      <c r="K10" s="32">
+      <c r="K10" s="34">
         <f>IFERROR(J10/G10, 0)</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="B11" s="27">
+      <c r="B11" s="29">
         <f>EDATE(B10, 1)</f>
         <v/>
       </c>
-      <c r="C11" s="28" t="n">
+      <c r="C11" s="30" t="n">
         <v>28400</v>
       </c>
-      <c r="D11" s="28" t="n">
+      <c r="D11" s="30" t="n">
         <v>204000</v>
       </c>
-      <c r="E11" s="28" t="n">
+      <c r="E11" s="30" t="n">
         <v>352000</v>
       </c>
-      <c r="F11" s="28" t="n">
+      <c r="F11" s="30" t="n">
         <v>238800</v>
       </c>
-      <c r="G11" s="29">
+      <c r="G11" s="31">
         <f>(C11+D11+E11)-F11</f>
         <v/>
       </c>
-      <c r="H11" s="30">
+      <c r="H11" s="32">
         <f>G11-G10</f>
         <v/>
       </c>
-      <c r="I11" s="31">
+      <c r="I11" s="33">
         <f>IFERROR((G11-G10)/G10, 0)</f>
         <v/>
       </c>
@@ -2718,37 +2759,37 @@
         <f>C11+D11</f>
         <v/>
       </c>
-      <c r="K11" s="32">
+      <c r="K11" s="34">
         <f>IFERROR(J11/G11, 0)</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="B12" s="27">
+      <c r="B12" s="29">
         <f>EDATE(B11, 1)</f>
         <v/>
       </c>
-      <c r="C12" s="28" t="n">
+      <c r="C12" s="30" t="n">
         <v>29000</v>
       </c>
-      <c r="D12" s="28" t="n">
+      <c r="D12" s="30" t="n">
         <v>209500</v>
       </c>
-      <c r="E12" s="28" t="n">
+      <c r="E12" s="30" t="n">
         <v>352000</v>
       </c>
-      <c r="F12" s="28" t="n">
+      <c r="F12" s="30" t="n">
         <v>237500</v>
       </c>
-      <c r="G12" s="29">
+      <c r="G12" s="31">
         <f>(C12+D12+E12)-F12</f>
         <v/>
       </c>
-      <c r="H12" s="30">
+      <c r="H12" s="32">
         <f>G12-G11</f>
         <v/>
       </c>
-      <c r="I12" s="31">
+      <c r="I12" s="33">
         <f>IFERROR((G12-G11)/G11, 0)</f>
         <v/>
       </c>
@@ -2756,37 +2797,37 @@
         <f>C12+D12</f>
         <v/>
       </c>
-      <c r="K12" s="32">
+      <c r="K12" s="34">
         <f>IFERROR(J12/G12, 0)</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="B13" s="27">
+      <c r="B13" s="29">
         <f>EDATE(B12, 1)</f>
         <v/>
       </c>
-      <c r="C13" s="28" t="n">
+      <c r="C13" s="30" t="n">
         <v>28500</v>
       </c>
-      <c r="D13" s="28" t="n">
+      <c r="D13" s="30" t="n">
         <v>215000</v>
       </c>
-      <c r="E13" s="28" t="n">
+      <c r="E13" s="30" t="n">
         <v>355000</v>
       </c>
-      <c r="F13" s="28" t="n">
+      <c r="F13" s="30" t="n">
         <v>236100</v>
       </c>
-      <c r="G13" s="29">
+      <c r="G13" s="31">
         <f>(C13+D13+E13)-F13</f>
         <v/>
       </c>
-      <c r="H13" s="30">
+      <c r="H13" s="32">
         <f>G13-G12</f>
         <v/>
       </c>
-      <c r="I13" s="31">
+      <c r="I13" s="33">
         <f>IFERROR((G13-G12)/G12, 0)</f>
         <v/>
       </c>
@@ -2794,37 +2835,37 @@
         <f>C13+D13</f>
         <v/>
       </c>
-      <c r="K13" s="32">
+      <c r="K13" s="34">
         <f>IFERROR(J13/G13, 0)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="27">
+      <c r="B14" s="29">
         <f>EDATE(B13, 1)</f>
         <v/>
       </c>
-      <c r="C14" s="28" t="n">
+      <c r="C14" s="30" t="n">
         <v>30200</v>
       </c>
-      <c r="D14" s="28" t="n">
+      <c r="D14" s="30" t="n">
         <v>221000</v>
       </c>
-      <c r="E14" s="28" t="n">
+      <c r="E14" s="30" t="n">
         <v>355000</v>
       </c>
-      <c r="F14" s="28" t="n">
+      <c r="F14" s="30" t="n">
         <v>234700</v>
       </c>
-      <c r="G14" s="29">
+      <c r="G14" s="31">
         <f>(C14+D14+E14)-F14</f>
         <v/>
       </c>
-      <c r="H14" s="30">
+      <c r="H14" s="32">
         <f>G14-G13</f>
         <v/>
       </c>
-      <c r="I14" s="31">
+      <c r="I14" s="33">
         <f>IFERROR((G14-G13)/G13, 0)</f>
         <v/>
       </c>
@@ -2832,37 +2873,37 @@
         <f>C14+D14</f>
         <v/>
       </c>
-      <c r="K14" s="32">
+      <c r="K14" s="34">
         <f>IFERROR(J14/G14, 0)</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="B15" s="27">
+      <c r="B15" s="29">
         <f>EDATE(B14, 1)</f>
         <v/>
       </c>
-      <c r="C15" s="28" t="n">
+      <c r="C15" s="30" t="n">
         <v>31000</v>
       </c>
-      <c r="D15" s="28" t="n">
+      <c r="D15" s="30" t="n">
         <v>228000</v>
       </c>
-      <c r="E15" s="28" t="n">
+      <c r="E15" s="30" t="n">
         <v>355000</v>
       </c>
-      <c r="F15" s="28" t="n">
+      <c r="F15" s="30" t="n">
         <v>233200</v>
       </c>
-      <c r="G15" s="29">
+      <c r="G15" s="31">
         <f>(C15+D15+E15)-F15</f>
         <v/>
       </c>
-      <c r="H15" s="30">
+      <c r="H15" s="32">
         <f>G15-G14</f>
         <v/>
       </c>
-      <c r="I15" s="31">
+      <c r="I15" s="33">
         <f>IFERROR((G15-G14)/G14, 0)</f>
         <v/>
       </c>
@@ -2870,37 +2911,37 @@
         <f>C15+D15</f>
         <v/>
       </c>
-      <c r="K15" s="32">
+      <c r="K15" s="34">
         <f>IFERROR(J15/G15, 0)</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="B16" s="27">
+      <c r="B16" s="29">
         <f>EDATE(B15, 1)</f>
         <v/>
       </c>
-      <c r="C16" s="28" t="n">
+      <c r="C16" s="30" t="n">
         <v>31500</v>
       </c>
-      <c r="D16" s="28" t="n">
+      <c r="D16" s="30" t="n">
         <v>234500</v>
       </c>
-      <c r="E16" s="28" t="n">
+      <c r="E16" s="30" t="n">
         <v>358000</v>
       </c>
-      <c r="F16" s="28" t="n">
+      <c r="F16" s="30" t="n">
         <v>231700</v>
       </c>
-      <c r="G16" s="29">
+      <c r="G16" s="31">
         <f>(C16+D16+E16)-F16</f>
         <v/>
       </c>
-      <c r="H16" s="30">
+      <c r="H16" s="32">
         <f>G16-G15</f>
         <v/>
       </c>
-      <c r="I16" s="31">
+      <c r="I16" s="33">
         <f>IFERROR((G16-G15)/G15, 0)</f>
         <v/>
       </c>
@@ -2908,37 +2949,37 @@
         <f>C16+D16</f>
         <v/>
       </c>
-      <c r="K16" s="32">
+      <c r="K16" s="34">
         <f>IFERROR(J16/G16, 0)</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="B17" s="27">
+      <c r="B17" s="29">
         <f>EDATE(B16, 1)</f>
         <v/>
       </c>
-      <c r="C17" s="28" t="n">
+      <c r="C17" s="30" t="n">
         <v>33000</v>
       </c>
-      <c r="D17" s="28" t="n">
+      <c r="D17" s="30" t="n">
         <v>242000</v>
       </c>
-      <c r="E17" s="28" t="n">
+      <c r="E17" s="30" t="n">
         <v>358000</v>
       </c>
-      <c r="F17" s="28" t="n">
+      <c r="F17" s="30" t="n">
         <v>230100</v>
       </c>
-      <c r="G17" s="29">
+      <c r="G17" s="31">
         <f>(C17+D17+E17)-F17</f>
         <v/>
       </c>
-      <c r="H17" s="30">
+      <c r="H17" s="32">
         <f>G17-G16</f>
         <v/>
       </c>
-      <c r="I17" s="31">
+      <c r="I17" s="33">
         <f>IFERROR((G17-G16)/G16, 0)</f>
         <v/>
       </c>
@@ -2946,50 +2987,50 @@
         <f>C17+D17</f>
         <v/>
       </c>
-      <c r="K17" s="32">
+      <c r="K17" s="34">
         <f>IFERROR(J17/G17, 0)</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="B18" s="33" t="inlineStr">
+      <c r="B18" s="35" t="inlineStr">
         <is>
           <t>ANNUAL SUMMARY</t>
         </is>
       </c>
-      <c r="C18" s="34">
+      <c r="C18" s="36">
         <f>AVERAGE(C6:C17)</f>
         <v/>
       </c>
-      <c r="D18" s="34">
+      <c r="D18" s="36">
         <f>AVERAGE(D6:D17)</f>
         <v/>
       </c>
-      <c r="E18" s="34">
+      <c r="E18" s="36">
         <f>AVERAGE(E6:E17)</f>
         <v/>
       </c>
-      <c r="F18" s="34">
+      <c r="F18" s="36">
         <f>AVERAGE(F6:F17)</f>
         <v/>
       </c>
-      <c r="G18" s="35">
+      <c r="G18" s="37">
         <f>G17</f>
         <v/>
       </c>
-      <c r="H18" s="36">
+      <c r="H18" s="38">
         <f>G17-G6</f>
         <v/>
       </c>
-      <c r="I18" s="37">
+      <c r="I18" s="39">
         <f>IFERROR((G17-G6)/G6, 0)</f>
         <v/>
       </c>
-      <c r="J18" s="38">
+      <c r="J18" s="40">
         <f>J17</f>
         <v/>
       </c>
-      <c r="K18" s="39">
+      <c r="K18" s="41">
         <f>IFERROR(J17/G17, 0)</f>
         <v/>
       </c>
@@ -3015,10 +3056,10 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="3" customWidth="1" min="7" max="7"/>
   </cols>
@@ -3038,174 +3079,174 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="40" t="inlineStr">
+      <c r="B5" s="42" t="inlineStr">
         <is>
           <t>TOTAL NET WORTH (LATEST)</t>
         </is>
       </c>
-      <c r="C5" s="14" t="n"/>
-      <c r="D5" s="40" t="inlineStr">
+      <c r="C5" s="13" t="n"/>
+      <c r="D5" s="42" t="inlineStr">
         <is>
           <t>LIQUID INVESTED PORTFOLIO</t>
         </is>
       </c>
-      <c r="E5" s="14" t="n"/>
-      <c r="F5" s="40" t="inlineStr">
+      <c r="E5" s="13" t="n"/>
+      <c r="F5" s="42" t="inlineStr">
         <is>
           <t>FED SCF RANK (DYNAMIC FORMULA)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="41">
+      <c r="B6" s="43">
         <f>'2-Min Check-In'!G17</f>
         <v/>
       </c>
-      <c r="C6" s="14" t="n"/>
-      <c r="D6" s="41">
+      <c r="C6" s="13" t="n"/>
+      <c r="D6" s="43">
         <f>'2-Min Check-In'!J17</f>
         <v/>
       </c>
-      <c r="E6" s="14" t="n"/>
-      <c r="F6" s="42">
+      <c r="E6" s="13" t="n"/>
+      <c r="F6" s="44">
         <f>IF(B6&gt;=1000000, "Top 18% (Millionaire)", IF(B6&gt;=500000, "Top 25% (High Wealth)", IF(B6&gt;=250000, "Top 35% (Above Avg)", IF(B6&gt;=135000, "Top 50% (Median+)", "Lower 50%"))))</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="43">
+      <c r="B7" s="45">
         <f>'2-Min Check-In'!H18</f>
         <v/>
       </c>
-      <c r="C7" s="14" t="n"/>
-      <c r="D7" s="44">
+      <c r="C7" s="13" t="n"/>
+      <c r="D7" s="46">
         <f>'2-Min Check-In'!K17</f>
         <v/>
       </c>
-      <c r="E7" s="14" t="n"/>
-      <c r="F7" s="45">
+      <c r="E7" s="13" t="n"/>
+      <c r="F7" s="47">
         <f>'START HERE'!C12</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>🏆 STANLEY &amp; DANKO WEALTH ACCUMULATION ENGINE (LIVE FORMULAS)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1">
-      <c r="B10" s="46" t="inlineStr">
+      <c r="B10" s="48" t="inlineStr">
         <is>
           <t>Current Age</t>
         </is>
       </c>
-      <c r="C10" s="46" t="inlineStr">
+      <c r="C10" s="48" t="inlineStr">
         <is>
           <t>Pre-Tax Income</t>
         </is>
       </c>
-      <c r="D10" s="46" t="inlineStr">
+      <c r="D10" s="48" t="inlineStr">
         <is>
           <t>Expected Net Worth</t>
         </is>
       </c>
-      <c r="E10" s="46" t="inlineStr">
+      <c r="E10" s="48" t="inlineStr">
         <is>
           <t>Multiplier</t>
         </is>
       </c>
-      <c r="F10" s="46" t="inlineStr">
+      <c r="F10" s="48" t="inlineStr">
         <is>
           <t>Wealth Status</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="B11" s="47">
+      <c r="B11" s="49">
         <f>'START HERE'!C12</f>
         <v/>
       </c>
-      <c r="C11" s="48">
+      <c r="C11" s="50">
         <f>'START HERE'!C13</f>
         <v/>
       </c>
-      <c r="D11" s="48">
-        <f>(B10*C10)/10</f>
-        <v/>
-      </c>
-      <c r="E11" s="49">
-        <f>IFERROR(B6/D10, 0)</f>
-        <v/>
-      </c>
-      <c r="F11" s="50">
-        <f>IF(E10&gt;=2.0, "PAW (Top 10%)", IF(E10&gt;=0.5, "AAW (Solid Average)", "UAW (Under)"))</f>
+      <c r="D11" s="50">
+        <f>(B11*C11)/10</f>
+        <v/>
+      </c>
+      <c r="E11" s="51">
+        <f>IFERROR(B6/D11, 0)</f>
+        <v/>
+      </c>
+      <c r="F11" s="52">
+        <f>IF(B11&lt;=0, "Setup Required", IF(E11&gt;=2.0, "PAW (Top 10%)", IF(E11&gt;=0.5, "AAW (Solid Average)", "UAW (Under)"))))</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>🔥 FINANCIAL INDEPENDENCE (FIRE) READINESS (LIVE FORMULAS)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1">
-      <c r="B14" s="46" t="inlineStr">
+      <c r="B14" s="48" t="inlineStr">
         <is>
           <t>Lean FIRE Target</t>
         </is>
       </c>
-      <c r="C14" s="46" t="inlineStr">
+      <c r="C14" s="48" t="inlineStr">
         <is>
           <t>Standard FIRE (4%)</t>
         </is>
       </c>
-      <c r="D14" s="46" t="inlineStr">
+      <c r="D14" s="48" t="inlineStr">
         <is>
           <t>Coast FIRE Target</t>
         </is>
       </c>
-      <c r="E14" s="46" t="inlineStr">
+      <c r="E14" s="48" t="inlineStr">
         <is>
           <t>Freedom Date</t>
         </is>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="B15" s="51">
-        <f>'FIRE Freedom Engine'!C11</f>
-        <v/>
-      </c>
-      <c r="C15" s="51">
-        <f>'FIRE Freedom Engine'!C12</f>
-        <v/>
-      </c>
-      <c r="D15" s="51">
+      <c r="B15" s="53">
+        <f>'FIRE Freedom Engine'!C13</f>
+        <v/>
+      </c>
+      <c r="C15" s="53">
         <f>'FIRE Freedom Engine'!C14</f>
         <v/>
       </c>
-      <c r="E15" s="52">
-        <f>'FIRE Freedom Engine'!C19</f>
+      <c r="D15" s="53">
+        <f>'FIRE Freedom Engine'!C16</f>
+        <v/>
+      </c>
+      <c r="E15" s="54">
+        <f>'FIRE Freedom Engine'!C22</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="B16" s="53">
-        <f>'FIRE Freedom Engine'!D11</f>
-        <v/>
-      </c>
-      <c r="C16" s="53">
-        <f>'FIRE Freedom Engine'!D12</f>
-        <v/>
-      </c>
-      <c r="D16" s="53">
-        <f>IF(D6&gt;=D15, '✅ COAST REACHED', 'SAVING IN PROGRESS')</f>
-        <v/>
-      </c>
-      <c r="E16" s="53">
-        <f>'FIRE Freedom Engine'!D19</f>
+      <c r="B16" s="55">
+        <f>IFERROR(B6/B15, 0)</f>
+        <v/>
+      </c>
+      <c r="C16" s="55">
+        <f>IFERROR(B6/C15, 0)</f>
+        <v/>
+      </c>
+      <c r="D16" s="56">
+        <f>IF(D15&lt;=0, "Setup Required", IF(D6&gt;=D15, "✅ COAST REACHED", "SAVING IN PROGRESS"))</f>
+        <v/>
+      </c>
+      <c r="E16" s="57">
+        <f>'FIRE Freedom Engine'!C21</f>
         <v/>
       </c>
     </row>
@@ -3234,11 +3275,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F34"/>
+  <dimension ref="B2:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -3261,62 +3302,62 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="54" t="inlineStr">
+      <c r="B5" s="58" t="inlineStr">
         <is>
           <t>🟢 REMAINING GUILT-FREE SPENDING BUFFER</t>
         </is>
       </c>
-      <c r="C5" s="14" t="n"/>
-      <c r="D5" s="14" t="n"/>
-      <c r="E5" s="40" t="inlineStr">
+      <c r="C5" s="13" t="n"/>
+      <c r="D5" s="13" t="n"/>
+      <c r="E5" s="42" t="inlineStr">
         <is>
           <t>SAFE DAILY ALLOWANCE (30-DAY BUFFER)</t>
         </is>
       </c>
-      <c r="F5" s="14" t="n"/>
+      <c r="F5" s="13" t="n"/>
     </row>
     <row r="6">
-      <c r="B6" s="55">
-        <f>E24</f>
-        <v/>
-      </c>
-      <c r="C6" s="14" t="n"/>
-      <c r="D6" s="14" t="n"/>
-      <c r="E6" s="56">
-        <f>IFERROR(E24/30, 0)</f>
-        <v/>
-      </c>
-      <c r="F6" s="14" t="n"/>
+      <c r="B6" s="59">
+        <f>E28</f>
+        <v/>
+      </c>
+      <c r="C6" s="13" t="n"/>
+      <c r="D6" s="13" t="n"/>
+      <c r="E6" s="60">
+        <f>IFERROR(E28/30, 0)</f>
+        <v/>
+      </c>
+      <c r="F6" s="13" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>Cash Flow Category</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>Planned ($)</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>Actual ($)</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="15" t="inlineStr">
         <is>
           <t>Remaining ($)</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="15" t="inlineStr">
         <is>
           <t>50/30/20 Benchmark</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="57" t="inlineStr">
+      <c r="B9" s="61" t="inlineStr">
         <is>
           <t>📥 MONTHLY TAKE-HOME INCOME</t>
         </is>
@@ -3328,13 +3369,13 @@
           <t>Primary Salary / Take-Home</t>
         </is>
       </c>
-      <c r="C10" s="58" t="n">
+      <c r="C10" s="10" t="n">
         <v>6800</v>
       </c>
-      <c r="D10" s="58" t="n">
+      <c r="D10" s="10" t="n">
         <v>6800</v>
       </c>
-      <c r="E10" s="59">
+      <c r="E10" s="62">
         <f>D10-C10</f>
         <v/>
       </c>
@@ -3350,13 +3391,13 @@
           <t>Partner / Secondary Income</t>
         </is>
       </c>
-      <c r="C11" s="58" t="n">
+      <c r="C11" s="10" t="n">
         <v>2200</v>
       </c>
-      <c r="D11" s="58" t="n">
+      <c r="D11" s="10" t="n">
         <v>2200</v>
       </c>
-      <c r="E11" s="59">
+      <c r="E11" s="62">
         <f>D11-C11</f>
         <v/>
       </c>
@@ -3372,13 +3413,13 @@
           <t>Side Hustles / Dividends</t>
         </is>
       </c>
-      <c r="C12" s="58" t="n">
+      <c r="C12" s="10" t="n">
         <v>500</v>
       </c>
-      <c r="D12" s="58" t="n">
+      <c r="D12" s="10" t="n">
         <v>650</v>
       </c>
-      <c r="E12" s="59">
+      <c r="E12" s="62">
         <f>D12-C12</f>
         <v/>
       </c>
@@ -3389,31 +3430,31 @@
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="60" t="inlineStr">
+      <c r="B13" s="63" t="inlineStr">
         <is>
           <t>TOTAL MONTHLY NET INCOME</t>
         </is>
       </c>
-      <c r="C13" s="61">
+      <c r="C13" s="64">
         <f>SUM(C10:C12)</f>
         <v/>
       </c>
-      <c r="D13" s="61">
+      <c r="D13" s="64">
         <f>SUM(D10:D12)</f>
         <v/>
       </c>
-      <c r="E13" s="61">
+      <c r="E13" s="64">
         <f>D13-C13</f>
         <v/>
       </c>
-      <c r="F13" s="62" t="inlineStr">
+      <c r="F13" s="65" t="inlineStr">
         <is>
           <t>100% Baseline</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="63" t="inlineStr">
+      <c r="B15" s="66" t="inlineStr">
         <is>
           <t>🛡️ 50% ESSENTIAL NEEDS (HOUSING, FOOD, UTILITIES, MIN DEBT)</t>
         </is>
@@ -3425,13 +3466,13 @@
           <t>Rent / Mortgage Payment</t>
         </is>
       </c>
-      <c r="C16" s="58" t="n">
+      <c r="C16" s="10" t="n">
         <v>2400</v>
       </c>
-      <c r="D16" s="58" t="n">
+      <c r="D16" s="10" t="n">
         <v>2400</v>
       </c>
-      <c r="E16" s="59">
+      <c r="E16" s="62">
         <f>C16-D16</f>
         <v/>
       </c>
@@ -3447,13 +3488,13 @@
           <t>Groceries &amp; Household Staples</t>
         </is>
       </c>
-      <c r="C17" s="58" t="n">
+      <c r="C17" s="10" t="n">
         <v>850</v>
       </c>
-      <c r="D17" s="58" t="n">
+      <c r="D17" s="10" t="n">
         <v>920</v>
       </c>
-      <c r="E17" s="59">
+      <c r="E17" s="62">
         <f>C17-D17</f>
         <v/>
       </c>
@@ -3469,13 +3510,13 @@
           <t>Utilities, Electric &amp; Internet</t>
         </is>
       </c>
-      <c r="C18" s="58" t="n">
+      <c r="C18" s="10" t="n">
         <v>380</v>
       </c>
-      <c r="D18" s="58" t="n">
+      <c r="D18" s="10" t="n">
         <v>410</v>
       </c>
-      <c r="E18" s="59">
+      <c r="E18" s="62">
         <f>C18-D18</f>
         <v/>
       </c>
@@ -3491,13 +3532,13 @@
           <t>Transportation, Gas &amp; Transit</t>
         </is>
       </c>
-      <c r="C19" s="58" t="n">
+      <c r="C19" s="10" t="n">
         <v>450</v>
       </c>
-      <c r="D19" s="58" t="n">
+      <c r="D19" s="10" t="n">
         <v>420</v>
       </c>
-      <c r="E19" s="59">
+      <c r="E19" s="62">
         <f>C19-D19</f>
         <v/>
       </c>
@@ -3513,13 +3554,13 @@
           <t>Healthcare, Insurance &amp; Prescriptions</t>
         </is>
       </c>
-      <c r="C20" s="58" t="n">
+      <c r="C20" s="10" t="n">
         <v>320</v>
       </c>
-      <c r="D20" s="58" t="n">
+      <c r="D20" s="10" t="n">
         <v>310</v>
       </c>
-      <c r="E20" s="59">
+      <c r="E20" s="62">
         <f>C20-D20</f>
         <v/>
       </c>
@@ -3530,30 +3571,30 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="60" t="inlineStr">
+      <c r="B21" s="63" t="inlineStr">
         <is>
           <t>SUBTOTAL: 50% NEEDS</t>
         </is>
       </c>
-      <c r="C21" s="61">
+      <c r="C21" s="64">
         <f>SUM(C16:C20)</f>
         <v/>
       </c>
-      <c r="D21" s="61">
+      <c r="D21" s="64">
         <f>SUM(D16:D20)</f>
         <v/>
       </c>
-      <c r="E21" s="61">
+      <c r="E21" s="64">
         <f>C21-D21</f>
         <v/>
       </c>
-      <c r="F21" s="64">
+      <c r="F21" s="67">
         <f>IFERROR(D21/D13, 0)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="65" t="inlineStr">
+      <c r="B23" s="66" t="inlineStr">
         <is>
           <t>🎉 30% DISCRETIONARY WANTS (DINING, STREAMING, HOBBIES)</t>
         </is>
@@ -3565,13 +3606,13 @@
           <t>Dining Out, Takeout &amp; Cafes</t>
         </is>
       </c>
-      <c r="C24" s="58" t="n">
+      <c r="C24" s="10" t="n">
         <v>700</v>
       </c>
-      <c r="D24" s="58" t="n">
+      <c r="D24" s="10" t="n">
         <v>680</v>
       </c>
-      <c r="E24" s="59">
+      <c r="E24" s="62">
         <f>C24-D24</f>
         <v/>
       </c>
@@ -3587,13 +3628,13 @@
           <t>Subscriptions, Gym &amp; Digital Apps</t>
         </is>
       </c>
-      <c r="C25" s="58" t="n">
+      <c r="C25" s="10" t="n">
         <v>180</v>
       </c>
-      <c r="D25" s="58" t="n">
+      <c r="D25" s="10" t="n">
         <v>195</v>
       </c>
-      <c r="E25" s="59">
+      <c r="E25" s="62">
         <f>C25-D25</f>
         <v/>
       </c>
@@ -3609,13 +3650,13 @@
           <t>Shopping, Apparel &amp; Entertainment</t>
         </is>
       </c>
-      <c r="C26" s="58" t="n">
+      <c r="C26" s="10" t="n">
         <v>500</v>
       </c>
-      <c r="D26" s="58" t="n">
+      <c r="D26" s="10" t="n">
         <v>480</v>
       </c>
-      <c r="E26" s="59">
+      <c r="E26" s="62">
         <f>C26-D26</f>
         <v/>
       </c>
@@ -3631,13 +3672,13 @@
           <t>Weekend Hobbies &amp; Social Travel</t>
         </is>
       </c>
-      <c r="C27" s="58" t="n">
+      <c r="C27" s="10" t="n">
         <v>450</v>
       </c>
-      <c r="D27" s="58" t="n">
+      <c r="D27" s="10" t="n">
         <v>420</v>
       </c>
-      <c r="E27" s="59">
+      <c r="E27" s="62">
         <f>C27-D27</f>
         <v/>
       </c>
@@ -3648,30 +3689,30 @@
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="60" t="inlineStr">
+      <c r="B28" s="63" t="inlineStr">
         <is>
           <t>SUBTOTAL: 30% WANTS</t>
         </is>
       </c>
-      <c r="C28" s="61">
+      <c r="C28" s="64">
         <f>SUM(C24:C27)</f>
         <v/>
       </c>
-      <c r="D28" s="61">
+      <c r="D28" s="64">
         <f>SUM(D24:D27)</f>
         <v/>
       </c>
-      <c r="E28" s="61">
+      <c r="E28" s="64">
         <f>C28-D28</f>
         <v/>
       </c>
-      <c r="F28" s="66">
+      <c r="F28" s="68">
         <f>IFERROR(D28/D13, 0)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="57" t="inlineStr">
+      <c r="B30" s="61" t="inlineStr">
         <is>
           <t>🚀 20% WEALTH SURPLUS (INVESTMENTS, SINKING FUNDS, EXTRA DEBT)</t>
         </is>
@@ -3683,13 +3724,13 @@
           <t>Roth IRA / 401(k) / Index Funds</t>
         </is>
       </c>
-      <c r="C31" s="58" t="n">
+      <c r="C31" s="10" t="n">
         <v>1500</v>
       </c>
-      <c r="D31" s="58" t="n">
+      <c r="D31" s="10" t="n">
         <v>1500</v>
       </c>
-      <c r="E31" s="59">
+      <c r="E31" s="62">
         <f>C31-D31</f>
         <v/>
       </c>
@@ -3705,13 +3746,13 @@
           <t>Sinking Funds Defense Pool</t>
         </is>
       </c>
-      <c r="C32" s="58" t="n">
+      <c r="C32" s="10" t="n">
         <v>600</v>
       </c>
-      <c r="D32" s="58" t="n">
+      <c r="D32" s="10" t="n">
         <v>600</v>
       </c>
-      <c r="E32" s="59">
+      <c r="E32" s="62">
         <f>C32-D32</f>
         <v/>
       </c>
@@ -3727,13 +3768,13 @@
           <t>Extra Debt Payoff Accelerator</t>
         </is>
       </c>
-      <c r="C33" s="58" t="n">
+      <c r="C33" s="10" t="n">
         <v>500</v>
       </c>
-      <c r="D33" s="58" t="n">
+      <c r="D33" s="10" t="n">
         <v>500</v>
       </c>
-      <c r="E33" s="59">
+      <c r="E33" s="62">
         <f>C33-D33</f>
         <v/>
       </c>
@@ -3744,25 +3785,48 @@
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="60" t="inlineStr">
+      <c r="B34" s="63" t="inlineStr">
         <is>
           <t>SUBTOTAL: 20% WEALTH</t>
         </is>
       </c>
-      <c r="C34" s="61">
+      <c r="C34" s="64">
         <f>SUM(C31:C33)</f>
         <v/>
       </c>
-      <c r="D34" s="61">
+      <c r="D34" s="64">
         <f>SUM(D31:D33)</f>
         <v/>
       </c>
-      <c r="E34" s="61">
+      <c r="E34" s="64">
         <f>C34-D34</f>
         <v/>
       </c>
-      <c r="F34" s="67">
+      <c r="F34" s="69">
         <f>IFERROR(D34/D13, 0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1">
+      <c r="B36" s="35" t="inlineStr">
+        <is>
+          <t>🎯 MONTHLY NET CASH FLOW SURPLUS / DEFICIT</t>
+        </is>
+      </c>
+      <c r="C36" s="40">
+        <f>C13-(C21+C28+C34)</f>
+        <v/>
+      </c>
+      <c r="D36" s="40">
+        <f>D13-(D21+D28+D34)</f>
+        <v/>
+      </c>
+      <c r="E36" s="40">
+        <f>D36-C36</f>
+        <v/>
+      </c>
+      <c r="F36" s="70">
+        <f>IF(D36&gt;=0, "✅ CASH SURPLUS", "⚠️ CASH DEFICIT")</f>
         <v/>
       </c>
     </row>
@@ -3790,7 +3854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F19"/>
+  <dimension ref="B2:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3798,7 +3862,7 @@
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
     <col width="3" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3812,308 +3876,355 @@
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Step 1: Drop bank PDF at getnetworthcalculator.com/tools/statement-converter ➔ Step 2: Click 'Copy For Vault' ➔ Step 3: Paste in Cell B10</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="57" t="inlineStr">
+          <t>Step 1: Convert bank PDF at getnetworthcalculator.com/tools/statement-converter ➔ Step 2: 1-Click Copy ➔ Step 3: Paste into B14</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>📊 INGESTED STATEMENT INTELLIGENCE (LIVE TOTALS FROM TRANSACTIONS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="B6" s="42" t="inlineStr">
+        <is>
+          <t>TOTAL INFLOWS</t>
+        </is>
+      </c>
+      <c r="C6" s="42" t="inlineStr">
+        <is>
+          <t>TOTAL OUTFLOWS (SPENT)</t>
+        </is>
+      </c>
+      <c r="D6" s="42" t="inlineStr">
+        <is>
+          <t>NET MONTHLY CASH FLOW</t>
+        </is>
+      </c>
+      <c r="E6" s="42" t="inlineStr">
+        <is>
+          <t>50% NEEDS OUTFLOW</t>
+        </is>
+      </c>
+      <c r="F6" s="42" t="inlineStr">
+        <is>
+          <t>30% WANTS OUTFLOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="B7" s="71">
+        <f>SUMIF(F14:F300, "*Inflow*", D14:D300)</f>
+        <v/>
+      </c>
+      <c r="C7" s="72">
+        <f>SUMIFS(D14:D300, F14:F300, "&lt;&gt;*Inflow*", D14:D300, "&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D7" s="71">
+        <f>B7-C7</f>
+        <v/>
+      </c>
+      <c r="E7" s="72">
+        <f>SUMIF(F14:F300, "*Needs*", D14:D300)</f>
+        <v/>
+      </c>
+      <c r="F7" s="72">
+        <f>SUMIF(F14:F300, "*Wants*", D14:D300)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="B8" s="73" t="inlineStr">
+        <is>
+          <t>Salary &amp; Direct Deposits</t>
+        </is>
+      </c>
+      <c r="C8" s="73" t="inlineStr">
+        <is>
+          <t>All Categories</t>
+        </is>
+      </c>
+      <c r="D8" s="73">
+        <f>IF(D7&gt;=0, "✅ Net Surplus", "⚠️ Net Deficit")</f>
+        <v/>
+      </c>
+      <c r="E8" s="74">
+        <f>IFERROR(E7/C7, 0)</f>
+        <v/>
+      </c>
+      <c r="F8" s="74">
+        <f>IFERROR(F7/C7, 0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="B10" s="61" t="inlineStr">
         <is>
           <t>🚀 HOW TO INGEST YOUR BANK TRANSACTIONS IN 10 SECONDS:</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="B6" s="68" t="inlineStr">
-        <is>
-          <t>1. Open our private tool: getnetworthcalculator.com/tools/statement-converter (100% client-side privacy).</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="n"/>
-      <c r="D6" s="14" t="n"/>
-      <c r="E6" s="14" t="n"/>
-      <c r="F6" s="14" t="n"/>
-    </row>
-    <row r="7">
-      <c r="B7" s="68" t="inlineStr">
-        <is>
-          <t>2. Drop your bank PDF (Chase, Amex, BoA, Wells Fargo, Citi, Capital One, etc.) or CSV export.</t>
-        </is>
-      </c>
-      <c r="C7" s="14" t="n"/>
-      <c r="D7" s="14" t="n"/>
-      <c r="E7" s="14" t="n"/>
-      <c r="F7" s="14" t="n"/>
-    </row>
-    <row r="8">
-      <c r="B8" s="68" t="inlineStr">
-        <is>
-          <t>3. Click '📋 1-Click Copy For Vault'.</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="n"/>
-      <c r="D8" s="14" t="n"/>
-      <c r="E8" s="14" t="n"/>
-      <c r="F8" s="14" t="n"/>
-    </row>
-    <row r="9">
-      <c r="B9" s="68" t="inlineStr">
-        <is>
-          <t>4. Click Cell B10 below and press Cmd+V (Mac) or Ctrl+V (Windows). All actuals update instantly!</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="n"/>
-      <c r="D9" s="14" t="n"/>
-      <c r="E9" s="14" t="n"/>
-      <c r="F9" s="14" t="n"/>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="8" t="inlineStr">
+    <row r="11" ht="22" customHeight="1">
+      <c r="B11" s="75" t="inlineStr">
+        <is>
+          <t>1. Open private converter: getnetworthcalculator.com/tools/statement-converter (100% private, client-side only). 2. Drop bank PDF or CSV. 3. Click '📋 1-Click Copy For Vault'. 4. Click cell B14 and paste (Cmd+V / Ctrl+V).</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="n"/>
+      <c r="D11" s="13" t="n"/>
+      <c r="E11" s="13" t="n"/>
+      <c r="F11" s="13" t="n"/>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C13" s="15" t="inlineStr">
         <is>
           <t>Clean Merchant</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D13" s="15" t="inlineStr">
         <is>
           <t>Amount ($)</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E13" s="15" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F13" s="15" t="inlineStr">
         <is>
           <t>Budget Bucket</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="19" customHeight="1">
-      <c r="B11" s="69" t="inlineStr">
+    <row r="14" ht="19" customHeight="1">
+      <c r="B14" s="76" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="C11" s="70" t="inlineStr">
+      <c r="C14" s="77" t="inlineStr">
         <is>
           <t>Direct Deposit - Payroll</t>
         </is>
       </c>
-      <c r="D11" s="71" t="n">
+      <c r="D14" s="78" t="n">
         <v>3450</v>
       </c>
-      <c r="E11" s="69" t="inlineStr">
+      <c r="E14" s="76" t="inlineStr">
         <is>
           <t>INFLOW</t>
         </is>
       </c>
-      <c r="F11" s="72" t="inlineStr">
+      <c r="F14" s="79" t="inlineStr">
         <is>
           <t>Inflow</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="19" customHeight="1">
-      <c r="B12" s="69" t="inlineStr">
+    <row r="15" ht="19" customHeight="1">
+      <c r="B15" s="76" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="C12" s="70" t="inlineStr">
+      <c r="C15" s="77" t="inlineStr">
         <is>
           <t>Avalon Apartments Rent</t>
         </is>
       </c>
-      <c r="D12" s="71" t="n">
+      <c r="D15" s="78" t="n">
         <v>1650</v>
       </c>
-      <c r="E12" s="69" t="inlineStr">
+      <c r="E15" s="76" t="inlineStr">
         <is>
           <t>HOUSING</t>
         </is>
       </c>
-      <c r="F12" s="72" t="inlineStr">
+      <c r="F15" s="79" t="inlineStr">
         <is>
           <t>50% Needs</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="19" customHeight="1">
-      <c r="B13" s="69" t="inlineStr">
+    <row r="16" ht="19" customHeight="1">
+      <c r="B16" s="76" t="inlineStr">
         <is>
           <t>2026-10-03</t>
         </is>
       </c>
-      <c r="C13" s="70" t="inlineStr">
+      <c r="C16" s="77" t="inlineStr">
         <is>
           <t>Trader Joe's Groceries</t>
         </is>
       </c>
-      <c r="D13" s="71" t="n">
+      <c r="D16" s="78" t="n">
         <v>84.15000000000001</v>
       </c>
-      <c r="E13" s="69" t="inlineStr">
+      <c r="E16" s="76" t="inlineStr">
         <is>
           <t>GROCERIES</t>
         </is>
       </c>
-      <c r="F13" s="72" t="inlineStr">
+      <c r="F16" s="79" t="inlineStr">
         <is>
           <t>50% Needs</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="19" customHeight="1">
-      <c r="B14" s="69" t="inlineStr">
+    <row r="17" ht="19" customHeight="1">
+      <c r="B17" s="76" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="C14" s="70" t="inlineStr">
+      <c r="C17" s="77" t="inlineStr">
         <is>
           <t>Chevron Gas &amp; Transit</t>
         </is>
       </c>
-      <c r="D14" s="71" t="n">
+      <c r="D17" s="78" t="n">
         <v>48.5</v>
       </c>
-      <c r="E14" s="69" t="inlineStr">
+      <c r="E17" s="76" t="inlineStr">
         <is>
           <t>TRANSPORTATION</t>
         </is>
       </c>
-      <c r="F14" s="72" t="inlineStr">
+      <c r="F17" s="79" t="inlineStr">
         <is>
           <t>50% Needs</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="19" customHeight="1">
-      <c r="B15" s="69" t="inlineStr">
+    <row r="18" ht="19" customHeight="1">
+      <c r="B18" s="76" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="C15" s="70" t="inlineStr">
+      <c r="C18" s="77" t="inlineStr">
         <is>
           <t>Starbucks Cafe</t>
         </is>
       </c>
-      <c r="D15" s="71" t="n">
+      <c r="D18" s="78" t="n">
         <v>6.25</v>
       </c>
-      <c r="E15" s="69" t="inlineStr">
+      <c r="E18" s="76" t="inlineStr">
         <is>
           <t>DINING</t>
         </is>
       </c>
-      <c r="F15" s="72" t="inlineStr">
+      <c r="F18" s="79" t="inlineStr">
         <is>
           <t>30% Wants</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="19" customHeight="1">
-      <c r="B16" s="69" t="inlineStr">
+    <row r="19" ht="19" customHeight="1">
+      <c r="B19" s="76" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="C16" s="70" t="inlineStr">
+      <c r="C19" s="77" t="inlineStr">
         <is>
           <t>Netflix Subscription</t>
         </is>
       </c>
-      <c r="D16" s="71" t="n">
+      <c r="D19" s="78" t="n">
         <v>15.99</v>
       </c>
-      <c r="E16" s="69" t="inlineStr">
+      <c r="E19" s="76" t="inlineStr">
         <is>
           <t>SUBSCRIPTIONS</t>
         </is>
       </c>
-      <c r="F16" s="72" t="inlineStr">
+      <c r="F19" s="79" t="inlineStr">
         <is>
           <t>30% Wants</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="19" customHeight="1">
-      <c r="B17" s="69" t="inlineStr">
+    <row r="20" ht="19" customHeight="1">
+      <c r="B20" s="76" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="C17" s="70" t="inlineStr">
+      <c r="C20" s="77" t="inlineStr">
         <is>
           <t>Vanguard Index Investment</t>
         </is>
       </c>
-      <c r="D17" s="71" t="n">
+      <c r="D20" s="78" t="n">
         <v>500</v>
       </c>
-      <c r="E17" s="69" t="inlineStr">
+      <c r="E20" s="76" t="inlineStr">
         <is>
           <t>INVESTMENTS</t>
         </is>
       </c>
-      <c r="F17" s="72" t="inlineStr">
+      <c r="F20" s="79" t="inlineStr">
         <is>
           <t>20% Wealth</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="19" customHeight="1">
-      <c r="B18" s="69" t="inlineStr">
+    <row r="21" ht="19" customHeight="1">
+      <c r="B21" s="76" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>
       </c>
-      <c r="C18" s="70" t="inlineStr">
+      <c r="C21" s="77" t="inlineStr">
         <is>
           <t>CVS Pharmacy Prescription</t>
         </is>
       </c>
-      <c r="D18" s="71" t="n">
+      <c r="D21" s="78" t="n">
         <v>24.15</v>
       </c>
-      <c r="E18" s="69" t="inlineStr">
+      <c r="E21" s="76" t="inlineStr">
         <is>
           <t>HEALTHCARE</t>
         </is>
       </c>
-      <c r="F18" s="72" t="inlineStr">
+      <c r="F21" s="79" t="inlineStr">
         <is>
           <t>50% Needs</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="19" customHeight="1">
-      <c r="B19" s="69" t="inlineStr">
+    <row r="22" ht="19" customHeight="1">
+      <c r="B22" s="76" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="C19" s="70" t="inlineStr">
+      <c r="C22" s="77" t="inlineStr">
         <is>
           <t>Amazon Household</t>
         </is>
       </c>
-      <c r="D19" s="71" t="n">
+      <c r="D22" s="78" t="n">
         <v>42.1</v>
       </c>
-      <c r="E19" s="69" t="inlineStr">
+      <c r="E22" s="76" t="inlineStr">
         <is>
           <t>SHOPPING</t>
         </is>
       </c>
-      <c r="F19" s="72" t="inlineStr">
+      <c r="F22" s="79" t="inlineStr">
         <is>
           <t>30% Wants</t>
         </is>
@@ -4121,14 +4232,12 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="7">
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="B6:F6"/>
+  <mergeCells count="5">
     <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="B9:F9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4140,16 +4249,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H12"/>
+  <dimension ref="B2:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="3" customWidth="1" min="9" max="9"/>
   </cols>
@@ -4168,38 +4277,38 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="B5" s="8" t="inlineStr">
+    <row r="5" ht="22" customHeight="1">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>Fund Name / Category</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>Target Goal ($)</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>Current Balance ($)</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>Remaining Gap ($)</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
         <is>
           <t>Target Deadline</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
+      <c r="G5" s="15" t="inlineStr">
         <is>
           <t>Monthly Allocation</t>
         </is>
       </c>
-      <c r="H5" s="8" t="inlineStr">
+      <c r="H5" s="15" t="inlineStr">
         <is>
           <t>Fund Health Status</t>
         </is>
@@ -4211,25 +4320,25 @@
           <t>🛡️ 6-Month Emergency Runway</t>
         </is>
       </c>
-      <c r="C6" s="58" t="n">
+      <c r="C6" s="10" t="n">
         <v>25000</v>
       </c>
-      <c r="D6" s="58" t="n">
+      <c r="D6" s="10" t="n">
         <v>21500</v>
       </c>
       <c r="E6" s="20">
         <f>C6-D6</f>
         <v/>
       </c>
-      <c r="F6" s="73" t="inlineStr">
+      <c r="F6" s="80" t="inlineStr">
         <is>
           <t>Dec 2026</t>
         </is>
       </c>
-      <c r="G6" s="58" t="n">
+      <c r="G6" s="10" t="n">
         <v>700</v>
       </c>
-      <c r="H6" s="74">
+      <c r="H6" s="81">
         <f>IF(C6&lt;=0, "N/A", IF(D6&gt;=C6, "✅ FULLY FUNDED", IF(D6/C6&gt;=0.75, "🟢 ON TRACK", IF(D6/C6&gt;=0.4, "🟡 IN PROGRESS", "🔴 NEEDS FOCUS"))))</f>
         <v/>
       </c>
@@ -4240,25 +4349,25 @@
           <t>🚗 Car Maintenance &amp; Tires</t>
         </is>
       </c>
-      <c r="C7" s="58" t="n">
+      <c r="C7" s="10" t="n">
         <v>2000</v>
       </c>
-      <c r="D7" s="58" t="n">
+      <c r="D7" s="10" t="n">
         <v>1400</v>
       </c>
       <c r="E7" s="20">
         <f>C7-D7</f>
         <v/>
       </c>
-      <c r="F7" s="73" t="inlineStr">
+      <c r="F7" s="80" t="inlineStr">
         <is>
           <t>Jun 2027</t>
         </is>
       </c>
-      <c r="G7" s="58" t="n">
+      <c r="G7" s="10" t="n">
         <v>150</v>
       </c>
-      <c r="H7" s="74">
+      <c r="H7" s="81">
         <f>IF(C7&lt;=0, "N/A", IF(D7&gt;=C7, "✅ FULLY FUNDED", IF(D7/C7&gt;=0.75, "🟢 ON TRACK", IF(D7/C7&gt;=0.4, "🟡 IN PROGRESS", "🔴 NEEDS FOCUS"))))</f>
         <v/>
       </c>
@@ -4269,25 +4378,25 @@
           <t>🏖️ Annual Family Vacation</t>
         </is>
       </c>
-      <c r="C8" s="58" t="n">
+      <c r="C8" s="10" t="n">
         <v>4500</v>
       </c>
-      <c r="D8" s="58" t="n">
+      <c r="D8" s="10" t="n">
         <v>2800</v>
       </c>
       <c r="E8" s="20">
         <f>C8-D8</f>
         <v/>
       </c>
-      <c r="F8" s="73" t="inlineStr">
+      <c r="F8" s="80" t="inlineStr">
         <is>
           <t>Dec 2027</t>
         </is>
       </c>
-      <c r="G8" s="58" t="n">
+      <c r="G8" s="10" t="n">
         <v>250</v>
       </c>
-      <c r="H8" s="74">
+      <c r="H8" s="81">
         <f>IF(C8&lt;=0, "N/A", IF(D8&gt;=C8, "✅ FULLY FUNDED", IF(D8/C8&gt;=0.75, "🟢 ON TRACK", IF(D8/C8&gt;=0.4, "🟡 IN PROGRESS", "🔴 NEEDS FOCUS"))))</f>
         <v/>
       </c>
@@ -4298,25 +4407,25 @@
           <t>🎁 Holiday Season &amp; Gifts</t>
         </is>
       </c>
-      <c r="C9" s="58" t="n">
+      <c r="C9" s="10" t="n">
         <v>1500</v>
       </c>
-      <c r="D9" s="58" t="n">
+      <c r="D9" s="10" t="n">
         <v>750</v>
       </c>
       <c r="E9" s="20">
         <f>C9-D9</f>
         <v/>
       </c>
-      <c r="F9" s="73" t="inlineStr">
+      <c r="F9" s="80" t="inlineStr">
         <is>
           <t>Nov 2026</t>
         </is>
       </c>
-      <c r="G9" s="58" t="n">
+      <c r="G9" s="10" t="n">
         <v>125</v>
       </c>
-      <c r="H9" s="74">
+      <c r="H9" s="81">
         <f>IF(C9&lt;=0, "N/A", IF(D9&gt;=C9, "✅ FULLY FUNDED", IF(D9/C9&gt;=0.75, "🟢 ON TRACK", IF(D9/C9&gt;=0.4, "🟡 IN PROGRESS", "🔴 NEEDS FOCUS"))))</f>
         <v/>
       </c>
@@ -4327,58 +4436,145 @@
           <t>🏠 Home Appliance &amp; Repair Pool</t>
         </is>
       </c>
-      <c r="C10" s="58" t="n">
+      <c r="C10" s="10" t="n">
         <v>3500</v>
       </c>
-      <c r="D10" s="58" t="n">
+      <c r="D10" s="10" t="n">
         <v>1800</v>
       </c>
       <c r="E10" s="20">
         <f>C10-D10</f>
         <v/>
       </c>
-      <c r="F10" s="73" t="inlineStr">
+      <c r="F10" s="80" t="inlineStr">
         <is>
           <t>Oct 2027</t>
         </is>
       </c>
-      <c r="G10" s="58" t="n">
+      <c r="G10" s="10" t="n">
         <v>250</v>
       </c>
-      <c r="H10" s="74">
+      <c r="H10" s="81">
         <f>IF(C10&lt;=0, "N/A", IF(D10&gt;=C10, "✅ FULLY FUNDED", IF(D10/C10&gt;=0.75, "🟢 ON TRACK", IF(D10/C10&gt;=0.4, "🟡 IN PROGRESS", "🔴 NEEDS FOCUS"))))</f>
         <v/>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="33" t="inlineStr">
+    <row r="11" ht="20" customHeight="1">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>⚕️ Medical &amp; Dental Out-of-Pocket</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>1600</v>
+      </c>
+      <c r="E11" s="20">
+        <f>C11-D11</f>
+        <v/>
+      </c>
+      <c r="F11" s="80" t="inlineStr">
+        <is>
+          <t>Aug 2027</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="n">
+        <v>150</v>
+      </c>
+      <c r="H11" s="81">
+        <f>IF(C11&lt;=0, "N/A", IF(D11&gt;=C11, "✅ FULLY FUNDED", IF(D11/C11&gt;=0.75, "🟢 ON TRACK", IF(D11/C11&gt;=0.4, "🟡 IN PROGRESS", "🔴 NEEDS FOCUS"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>🏛️ Annual Property &amp; Local Taxes</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>4800</v>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>3200</v>
+      </c>
+      <c r="E12" s="20">
+        <f>C12-D12</f>
+        <v/>
+      </c>
+      <c r="F12" s="80" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="n">
+        <v>400</v>
+      </c>
+      <c r="H12" s="81">
+        <f>IF(C12&lt;=0, "N/A", IF(D12&gt;=C12, "✅ FULLY FUNDED", IF(D12/C12&gt;=0.75, "🟢 ON TRACK", IF(D12/C12&gt;=0.4, "🟡 IN PROGRESS", "🔴 NEEDS FOCUS"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>📱 Tech &amp; Phone Upgrade Replacement</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>1800</v>
+      </c>
+      <c r="D13" s="10" t="n">
+        <v>900</v>
+      </c>
+      <c r="E13" s="20">
+        <f>C13-D13</f>
+        <v/>
+      </c>
+      <c r="F13" s="80" t="inlineStr">
+        <is>
+          <t>Dec 2027</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="n">
+        <v>150</v>
+      </c>
+      <c r="H13" s="81">
+        <f>IF(C13&lt;=0, "N/A", IF(D13&gt;=C13, "✅ FULLY FUNDED", IF(D13/C13&gt;=0.75, "🟢 ON TRACK", IF(D13/C13&gt;=0.4, "🟡 IN PROGRESS", "🔴 NEEDS FOCUS"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="35" t="inlineStr">
         <is>
           <t>TOTAL SINKING FUNDS POOL</t>
         </is>
       </c>
-      <c r="C12" s="38">
-        <f>SUM(C6:C10)</f>
-        <v/>
-      </c>
-      <c r="D12" s="38">
-        <f>SUM(D6:D10)</f>
-        <v/>
-      </c>
-      <c r="E12" s="38">
-        <f>SUM(E6:E10)</f>
-        <v/>
-      </c>
-      <c r="F12" s="75" t="inlineStr">
+      <c r="C14" s="40">
+        <f>SUM(C6:C13)</f>
+        <v/>
+      </c>
+      <c r="D14" s="40">
+        <f>SUM(D6:D13)</f>
+        <v/>
+      </c>
+      <c r="E14" s="40">
+        <f>SUM(E6:E13)</f>
+        <v/>
+      </c>
+      <c r="F14" s="82" t="inlineStr">
         <is>
           <t>Multiple</t>
         </is>
       </c>
-      <c r="G12" s="38">
-        <f>SUM(G6:G10)</f>
-        <v/>
-      </c>
-      <c r="H12" s="76">
-        <f>IFERROR(D12/C12, 0)</f>
+      <c r="G14" s="40">
+        <f>SUM(G6:G13)</f>
+        <v/>
+      </c>
+      <c r="H14" s="83">
+        <f>IFERROR(D14/C14, 0)</f>
         <v/>
       </c>
     </row>
@@ -4402,9 +4598,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
     <col width="3" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -4423,7 +4619,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="77" t="inlineStr">
+      <c r="B4" s="84" t="inlineStr">
         <is>
           <t>1. CORE ASSUMPTIONS (READS FROM MASTER SETUP)</t>
         </is>
@@ -4435,7 +4631,7 @@
           <t>Current Age</t>
         </is>
       </c>
-      <c r="C5" s="78">
+      <c r="C5" s="85">
         <f>'START HERE'!C12</f>
         <v/>
       </c>
@@ -4451,7 +4647,7 @@
           <t>Target Retirement Age</t>
         </is>
       </c>
-      <c r="C6" s="78">
+      <c r="C6" s="85">
         <f>'START HERE'!C14</f>
         <v/>
       </c>
@@ -4483,7 +4679,7 @@
           <t>Safe Withdrawal Rate (SWR)</t>
         </is>
       </c>
-      <c r="C8" s="79">
+      <c r="C8" s="86">
         <f>'START HERE'!C16</f>
         <v/>
       </c>
@@ -4499,7 +4695,7 @@
           <t>Expected Real Return After Inflation</t>
         </is>
       </c>
-      <c r="C9" s="79">
+      <c r="C9" s="86">
         <f>'START HERE'!C17</f>
         <v/>
       </c>
@@ -4515,7 +4711,7 @@
           <t>Lean FIRE Spending Ratio</t>
         </is>
       </c>
-      <c r="C10" s="79">
+      <c r="C10" s="86">
         <f>'START HERE'!C18</f>
         <v/>
       </c>
@@ -4526,7 +4722,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="57" t="inlineStr">
+      <c r="B12" s="61" t="inlineStr">
         <is>
           <t>2. THE 4 FIRE MILESTONES (CALCULATED LIVE)</t>
         </is>
@@ -4538,7 +4734,7 @@
           <t>Lean FIRE Target (Bare Essentials)</t>
         </is>
       </c>
-      <c r="C13" s="80">
+      <c r="C13" s="87">
         <f>IFERROR((C7*C10)/C8, 0)</f>
         <v/>
       </c>
@@ -4554,7 +4750,7 @@
           <t>Standard FIRE Target (4% Rule)</t>
         </is>
       </c>
-      <c r="C14" s="80">
+      <c r="C14" s="87">
         <f>IFERROR(C7/C8, 0)</f>
         <v/>
       </c>
@@ -4570,7 +4766,7 @@
           <t>Fat FIRE Target (Abundant Lifestyle)</t>
         </is>
       </c>
-      <c r="C15" s="80">
+      <c r="C15" s="87">
         <f>IFERROR((C7*1.4)/C8, 0)</f>
         <v/>
       </c>
@@ -4586,7 +4782,7 @@
           <t>Coast FIRE Target (Zero Further Savings Needed)</t>
         </is>
       </c>
-      <c r="C16" s="80">
+      <c r="C16" s="87">
         <f>IFERROR((C7/C8)/((1+C9)^(C6-C5)), 0)</f>
         <v/>
       </c>
@@ -4597,7 +4793,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="63" t="inlineStr">
+      <c r="B18" s="66" t="inlineStr">
         <is>
           <t>3. COUNTDOWN TO FREEDOM (DYNAMIC DATE FORMULA)</t>
         </is>
@@ -4641,8 +4837,8 @@
           <t>Years Remaining to Standard FIRE</t>
         </is>
       </c>
-      <c r="C21" s="81">
-        <f>IFERROR(NPER(C9/12, -C20, -C19, C14)/12, 0)</f>
+      <c r="C21" s="88">
+        <f>IF(C14&lt;=0, 0, IF(C19&gt;=C14, 0, IFERROR(NPER(C9/12, -C20, -C19, C14)/12, 0)))</f>
         <v/>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -4652,13 +4848,13 @@
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="82" t="inlineStr">
+      <c r="B22" s="89" t="inlineStr">
         <is>
           <t>⭐ PROJECTED FREEDOM DATE</t>
         </is>
       </c>
-      <c r="C22" s="83">
-        <f>IFERROR(DATE(YEAR(TODAY())+INT(C21), MONTH(TODAY())+ROUND((C21-INT(C21))*12, 0), 1), TODAY())</f>
+      <c r="C22" s="90">
+        <f>IF(C14&lt;=0, "Setup Required", IF(C19&gt;=C14, "🎉 FIRE ACHIEVED!", IFERROR(DATE(YEAR(TODAY())+INT(C21), MONTH(TODAY())+ROUND((C21-INT(C21))*12, 0), 1), "Calculating...")))</f>
         <v/>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -4690,7 +4886,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -4713,33 +4909,33 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="B4" s="8" t="inlineStr">
+    <row r="4" ht="22" customHeight="1">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Debt Account Name</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>Current Balance</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>Interest APR</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="15" t="inlineStr">
         <is>
           <t>Min Payment</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F4" s="15" t="inlineStr">
         <is>
           <t>Avalanche Rank</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
+      <c r="G4" s="15" t="inlineStr">
         <is>
           <t>Snowball Rank</t>
         </is>
@@ -4751,20 +4947,20 @@
           <t>Credit Card A (High APR)</t>
         </is>
       </c>
-      <c r="C5" s="58" t="n">
+      <c r="C5" s="10" t="n">
         <v>4200</v>
       </c>
-      <c r="D5" s="84" t="n">
+      <c r="D5" s="91" t="n">
         <v>0.2499</v>
       </c>
-      <c r="E5" s="58" t="n">
+      <c r="E5" s="10" t="n">
         <v>140</v>
       </c>
-      <c r="F5" s="74">
+      <c r="F5" s="81">
         <f>IF(C5&gt;0, RANK(D5, $D$5:$D$8, 0), "-")</f>
         <v/>
       </c>
-      <c r="G5" s="74">
+      <c r="G5" s="81">
         <f>IF(C5&gt;0, RANK(C5, $C$5:$C$8, 1), "-")</f>
         <v/>
       </c>
@@ -4775,20 +4971,20 @@
           <t>Personal Consolidation Loan</t>
         </is>
       </c>
-      <c r="C6" s="58" t="n">
+      <c r="C6" s="10" t="n">
         <v>8500</v>
       </c>
-      <c r="D6" s="84" t="n">
+      <c r="D6" s="91" t="n">
         <v>0.115</v>
       </c>
-      <c r="E6" s="58" t="n">
+      <c r="E6" s="10" t="n">
         <v>210</v>
       </c>
-      <c r="F6" s="74">
+      <c r="F6" s="81">
         <f>IF(C6&gt;0, RANK(D6, $D$5:$D$8, 0), "-")</f>
         <v/>
       </c>
-      <c r="G6" s="74">
+      <c r="G6" s="81">
         <f>IF(C6&gt;0, RANK(C6, $C$5:$C$8, 1), "-")</f>
         <v/>
       </c>
@@ -4799,20 +4995,20 @@
           <t>Auto Loan (Vehicle)</t>
         </is>
       </c>
-      <c r="C7" s="58" t="n">
+      <c r="C7" s="10" t="n">
         <v>17400</v>
       </c>
-      <c r="D7" s="84" t="n">
+      <c r="D7" s="91" t="n">
         <v>0.059</v>
       </c>
-      <c r="E7" s="58" t="n">
+      <c r="E7" s="10" t="n">
         <v>380</v>
       </c>
-      <c r="F7" s="74">
+      <c r="F7" s="81">
         <f>IF(C7&gt;0, RANK(D7, $D$5:$D$8, 0), "-")</f>
         <v/>
       </c>
-      <c r="G7" s="74">
+      <c r="G7" s="81">
         <f>IF(C7&gt;0, RANK(C7, $C$5:$C$8, 1), "-")</f>
         <v/>
       </c>
@@ -4823,98 +5019,98 @@
           <t>Primary Mortgage</t>
         </is>
       </c>
-      <c r="C8" s="58" t="n">
+      <c r="C8" s="10" t="n">
         <v>200000</v>
       </c>
-      <c r="D8" s="84" t="n">
+      <c r="D8" s="91" t="n">
         <v>0.035</v>
       </c>
-      <c r="E8" s="58" t="n">
+      <c r="E8" s="10" t="n">
         <v>1670</v>
       </c>
-      <c r="F8" s="74">
+      <c r="F8" s="81">
         <f>IF(C8&gt;0, RANK(D8, $D$5:$D$8, 0), "-")</f>
         <v/>
       </c>
-      <c r="G8" s="74">
+      <c r="G8" s="81">
         <f>IF(C8&gt;0, RANK(C8, $C$5:$C$8, 1), "-")</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="33" t="inlineStr">
+      <c r="B9" s="35" t="inlineStr">
         <is>
           <t>TOTAL LIABILITIES &amp; WEIGHTED APR</t>
         </is>
       </c>
-      <c r="C9" s="38">
+      <c r="C9" s="40">
         <f>SUM(C5:C8)</f>
         <v/>
       </c>
-      <c r="D9" s="85">
+      <c r="D9" s="92">
         <f>IFERROR(SUMPRODUCT(C5:C8, D5:D8)/SUM(C5:C8), 0)</f>
         <v/>
       </c>
-      <c r="E9" s="38">
+      <c r="E9" s="40">
         <f>SUM(E5:E8)</f>
         <v/>
       </c>
-      <c r="F9" s="86" t="inlineStr">
+      <c r="F9" s="93" t="inlineStr">
         <is>
           <t>Highest APR</t>
         </is>
       </c>
-      <c r="G9" s="86" t="inlineStr">
+      <c r="G9" s="93" t="inlineStr">
         <is>
           <t>Lowest Bal</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>⚡ SIDE-BY-SIDE PAYOFF ACCELERATOR COMPARISON</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="87" t="inlineStr">
+      <c r="B13" s="94" t="inlineStr">
         <is>
           <t>Extra Monthly Debt Accelerator Payment</t>
         </is>
       </c>
-      <c r="C13" s="28" t="n">
+      <c r="C13" s="30" t="n">
         <v>500</v>
       </c>
-      <c r="D13" s="88" t="inlineStr">
+      <c r="D13" s="95" t="inlineStr">
         <is>
           <t>Total Monthly Cash Flow Dedicated: =E9+C13</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>Strategy Metric</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <t>🏔️ Avalanche (Math Optimal)</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D15" s="15" t="inlineStr">
         <is>
           <t>⛄ Snowball (Psychology Optimal)</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E15" s="15" t="inlineStr">
         <is>
           <t>Difference / Advantage</t>
         </is>
       </c>
-      <c r="F15" s="89" t="n"/>
-      <c r="G15" s="89" t="n"/>
+      <c r="F15" s="96" t="n"/>
+      <c r="G15" s="96" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="B16" s="4" t="inlineStr">
@@ -4937,8 +5133,8 @@
           <t>Avalanche saves maximum cash</t>
         </is>
       </c>
-      <c r="F16" s="14" t="n"/>
-      <c r="G16" s="14" t="n"/>
+      <c r="F16" s="13" t="n"/>
+      <c r="G16" s="13" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="B17" s="4" t="inlineStr">
@@ -4946,18 +5142,18 @@
           <t>Projected Debt-Free Months</t>
         </is>
       </c>
-      <c r="C17" s="5" t="n">
+      <c r="C17" s="97" t="n">
         <v>38</v>
       </c>
-      <c r="D17" s="5" t="n">
+      <c r="D17" s="97" t="n">
         <v>41</v>
       </c>
-      <c r="E17" s="6">
-        <f>C17-B17</f>
-        <v/>
-      </c>
-      <c r="F17" s="14" t="n"/>
-      <c r="G17" s="14" t="n"/>
+      <c r="E17" s="98">
+        <f>IFERROR(D17-C17, 0)</f>
+        <v/>
+      </c>
+      <c r="F17" s="13" t="n"/>
+      <c r="G17" s="13" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="B18" s="4" t="inlineStr">
@@ -4965,18 +5161,18 @@
           <t>Estimated Total Interest Paid</t>
         </is>
       </c>
-      <c r="C18" s="59" t="n">
+      <c r="C18" s="62" t="n">
         <v>14200</v>
       </c>
-      <c r="D18" s="59" t="n">
+      <c r="D18" s="62" t="n">
         <v>16850</v>
       </c>
-      <c r="E18" s="6">
-        <f>C18-B18</f>
-        <v/>
-      </c>
-      <c r="F18" s="14" t="n"/>
-      <c r="G18" s="14" t="n"/>
+      <c r="E18" s="99">
+        <f>IFERROR(D18-C18, 0)</f>
+        <v/>
+      </c>
+      <c r="F18" s="13" t="n"/>
+      <c r="G18" s="13" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="B19" s="4" t="inlineStr">
@@ -4984,8 +5180,8 @@
           <t>⭐ TOTAL INTEREST SAVED</t>
         </is>
       </c>
-      <c r="C19" s="90">
-        <f>D18</f>
+      <c r="C19" s="100">
+        <f>IFERROR(D18-C18, 0)</f>
         <v/>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -4993,13 +5189,12 @@
           <t>Maximum Savings</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>Avalanche saves +$2,650 in interest</t>
-        </is>
-      </c>
-      <c r="F19" s="14" t="n"/>
-      <c r="G19" s="14" t="n"/>
+      <c r="E19" s="6">
+        <f>"Avalanche saves " &amp; TEXT(C19, "$#,##0") &amp; " in interest &amp; finishes " &amp; TEXT(E17, "0") &amp; " months earlier"</f>
+        <v/>
+      </c>
+      <c r="F19" s="13" t="n"/>
+      <c r="G19" s="13" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>

</xml_diff>